<commit_message>
Batch original-file recovery checkpoint
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -4277,7 +4277,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -6380,7 +6380,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -6466,7 +6466,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.399153+00:00</t>
+          <t>2026-10-17T08:30:22.811991+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.400099+00:00</t>
+          <t>2026-10-17T08:30:22.813153+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.400122+00:00</t>
+          <t>2026-10-17T08:30:22.813181+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.400356+00:00</t>
+          <t>2026-10-17T08:30:22.813428+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.401443+00:00</t>
+          <t>2026-10-17T08:30:22.814635+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.401921+00:00</t>
+          <t>2026-10-17T08:30:22.815153+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.408803+00:00</t>
+          <t>2026-10-17T08:30:22.820691+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.411250+00:00</t>
+          <t>2026-10-17T08:30:22.823145+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.412226+00:00</t>
+          <t>2026-10-17T08:30:22.824089+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.412619+00:00</t>
+          <t>2026-10-17T08:30:22.824676+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.413356+00:00</t>
+          <t>2026-10-17T08:30:22.825398+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.414019+00:00</t>
+          <t>2026-10-17T08:30:22.826068+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.414915+00:00</t>
+          <t>2026-10-17T08:30:22.827017+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.415144+00:00</t>
+          <t>2026-10-17T08:30:22.827279+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.415998+00:00</t>
+          <t>2026-10-17T08:30:22.828154+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.424546+00:00</t>
+          <t>2026-10-17T08:30:22.837004+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.425262+00:00</t>
+          <t>2026-10-17T08:30:22.837782+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.426486+00:00</t>
+          <t>2026-10-17T08:30:22.839002+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.429285+00:00</t>
+          <t>2026-10-17T08:30:22.841840+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.430444+00:00</t>
+          <t>2026-10-17T08:30:22.843085+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.431844+00:00</t>
+          <t>2026-10-17T08:30:22.844299+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.436022+00:00</t>
+          <t>2026-10-17T08:30:22.848756+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.438310+00:00</t>
+          <t>2026-10-17T08:30:22.851190+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.440446+00:00</t>
+          <t>2026-10-17T08:30:22.853013+00:00</t>
         </is>
       </c>
     </row>
@@ -26859,13 +26859,21 @@
           <t>papers/R13558/main/0006612a5b75_R13558_2026_Redox_mediators_and_microaeration_overcoming_linear_alkylbenzene_sulfonate_recalcitrance.pdf</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13558_2026_Redox_mediators_and_microaeration_overcoming_linear_alkylbenzene_sulfonate_recalcitrance.pdf</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-current-run/fulltexts/R13558_2026_Redox_mediators_and_microaeration_overcoming_linear_alkylbenzene_sulfonate_recalcitrance.pdf</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13558_2026_Redox_mediators_and_microaeration_overcoming_linear_alkylbenzene_sulfonate_recalcitrance.pdf</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>pdf</t>
@@ -26881,12 +26889,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -26923,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.440476+00:00</t>
+          <t>2026-10-17T08:30:22.853701+00:00</t>
         </is>
       </c>
     </row>
@@ -26959,13 +26967,21 @@
           <t>papers/R04889/main/860a05325037_R04889_2019_Inoculum_Selection_and_Micro-Aeration_for_Biogas_Production_in_Two-Stage.pdf</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R04889_2019_Inoculum_Selection_and_Micro-Aeration_for_Biogas_Production_in_Two-Stage.pdf</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-current-run/fulltexts/R04889_2019_Inoculum_Selection_and_Micro-Aeration_for_Biogas_Production_in_Two-Stage.pdf</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R04889_2019_Inoculum_Selection_and_Micro-Aeration_for_Biogas_Production_in_Two-Stage.pdf</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>pdf</t>
@@ -26981,12 +26997,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -27023,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.440483+00:00</t>
+          <t>2026-10-17T08:30:22.854077+00:00</t>
         </is>
       </c>
     </row>
@@ -27131,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.442628+00:00</t>
+          <t>2026-10-17T08:30:22.856050+00:00</t>
         </is>
       </c>
     </row>
@@ -27239,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.443878+00:00</t>
+          <t>2026-10-17T08:30:22.857269+00:00</t>
         </is>
       </c>
     </row>
@@ -27347,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.445912+00:00</t>
+          <t>2026-10-17T08:30:22.859717+00:00</t>
         </is>
       </c>
     </row>
@@ -27455,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.447862+00:00</t>
+          <t>2026-10-17T08:30:22.861830+00:00</t>
         </is>
       </c>
     </row>
@@ -27555,7 +27571,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.447879+00:00</t>
+          <t>2026-10-17T08:30:22.861861+00:00</t>
         </is>
       </c>
     </row>
@@ -27591,13 +27607,21 @@
           <t>papers/R05542/main/735560cdb276_R05542_2020_Effect_of_micro-aerobic_process_on_improvement_of_anaerobic_digestion.pdf</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R05542_2020_Effect_of_micro-aerobic_process_on_improvement_of_anaerobic_digestion.pdf</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-current-run/fulltexts/R05542_2020_Effect_of_micro-aerobic_process_on_improvement_of_anaerobic_digestion.pdf</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R05542_2020_Effect_of_micro-aerobic_process_on_improvement_of_anaerobic_digestion.pdf</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
           <t>pdf</t>
@@ -27613,12 +27637,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -27655,7 +27679,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.447883+00:00</t>
+          <t>2026-10-17T08:30:22.862453+00:00</t>
         </is>
       </c>
     </row>
@@ -27763,7 +27787,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.449544+00:00</t>
+          <t>2026-10-17T08:30:22.864374+00:00</t>
         </is>
       </c>
     </row>
@@ -27871,7 +27895,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.452406+00:00</t>
+          <t>2026-10-17T08:30:22.867680+00:00</t>
         </is>
       </c>
     </row>
@@ -27907,13 +27931,21 @@
           <t>papers/R06611/main/b8eb8afdada2_R06611_2021_Effective_pretreatment_of_lignocellulosic_co-substrates_using_barley_straw-adapted_microbial.pdf</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R06611_2021_Effective_pretreatment_of_lignocellulosic_co-substrates_using_barley_straw-adapted_microbial.pdf</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-current-run/fulltexts/R06611_2021_Effective_pretreatment_of_lignocellulosic_co-substrates_using_barley_straw-adapted_microbial.pdf</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R06611_2021_Effective_pretreatment_of_lignocellulosic_co-substrates_using_barley_straw-adapted_microbial.pdf</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
           <t>pdf</t>
@@ -27929,12 +27961,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -27971,7 +28003,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.452425+00:00</t>
+          <t>2026-10-17T08:30:22.869860+00:00</t>
         </is>
       </c>
     </row>
@@ -28079,7 +28111,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.453644+00:00</t>
+          <t>2026-10-17T08:30:22.871044+00:00</t>
         </is>
       </c>
     </row>
@@ -28115,13 +28147,21 @@
           <t>papers/R07238/main/26c38d163174_R07238_2021_The_influence_of_combined_low-strength_ultrasonics_and_micro-aerobic_pretreatment.pdf</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R07238_2021_The_influence_of_combined_low-strength_ultrasonics_and_micro-aerobic_pretreatment.pdf</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-current-run/fulltexts/R07238_2021_The_influence_of_combined_low-strength_ultrasonics_and_micro-aerobic_pretreatment.pdf</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R07238_2021_The_influence_of_combined_low-strength_ultrasonics_and_micro-aerobic_pretreatment.pdf</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr">
         <is>
           <t>pdf</t>
@@ -28137,12 +28177,12 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -28179,7 +28219,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.453661+00:00</t>
+          <t>2026-10-17T08:30:22.873865+00:00</t>
         </is>
       </c>
     </row>
@@ -28287,7 +28327,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.454380+00:00</t>
+          <t>2026-10-17T08:30:22.874561+00:00</t>
         </is>
       </c>
     </row>
@@ -28395,7 +28435,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.455942+00:00</t>
+          <t>2026-10-17T08:30:22.876112+00:00</t>
         </is>
       </c>
     </row>
@@ -28503,7 +28543,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.456415+00:00</t>
+          <t>2026-10-17T08:30:22.876382+00:00</t>
         </is>
       </c>
     </row>
@@ -28603,7 +28643,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.456440+00:00</t>
+          <t>2026-10-17T08:30:22.876396+00:00</t>
         </is>
       </c>
     </row>
@@ -28711,7 +28751,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.459380+00:00</t>
+          <t>2026-10-17T08:30:22.879197+00:00</t>
         </is>
       </c>
     </row>
@@ -28811,7 +28851,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.459405+00:00</t>
+          <t>2026-10-17T08:30:22.879216+00:00</t>
         </is>
       </c>
     </row>
@@ -28919,7 +28959,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.459921+00:00</t>
+          <t>2026-10-17T08:30:22.879738+00:00</t>
         </is>
       </c>
     </row>
@@ -29019,7 +29059,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.459935+00:00</t>
+          <t>2026-10-17T08:30:22.879752+00:00</t>
         </is>
       </c>
     </row>
@@ -29119,7 +29159,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.459940+00:00</t>
+          <t>2026-10-17T08:30:22.879756+00:00</t>
         </is>
       </c>
     </row>
@@ -29219,7 +29259,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.459942+00:00</t>
+          <t>2026-10-17T08:30:22.879759+00:00</t>
         </is>
       </c>
     </row>
@@ -29327,7 +29367,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.461544+00:00</t>
+          <t>2026-10-17T08:30:22.881343+00:00</t>
         </is>
       </c>
     </row>
@@ -29427,7 +29467,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.461560+00:00</t>
+          <t>2026-10-17T08:30:22.881357+00:00</t>
         </is>
       </c>
     </row>
@@ -29527,7 +29567,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.461563+00:00</t>
+          <t>2026-10-17T08:30:22.881361+00:00</t>
         </is>
       </c>
     </row>
@@ -29635,7 +29675,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.461971+00:00</t>
+          <t>2026-10-17T08:30:22.881786+00:00</t>
         </is>
       </c>
     </row>
@@ -29735,7 +29775,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.461985+00:00</t>
+          <t>2026-10-17T08:30:22.881799+00:00</t>
         </is>
       </c>
     </row>
@@ -29843,7 +29883,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.463704+00:00</t>
+          <t>2026-10-17T08:30:22.883348+00:00</t>
         </is>
       </c>
     </row>
@@ -29951,7 +29991,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465195+00:00</t>
+          <t>2026-10-17T08:30:22.884628+00:00</t>
         </is>
       </c>
     </row>
@@ -30051,7 +30091,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465222+00:00</t>
+          <t>2026-10-17T08:30:22.884643+00:00</t>
         </is>
       </c>
     </row>
@@ -30151,7 +30191,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465227+00:00</t>
+          <t>2026-10-17T08:30:22.884647+00:00</t>
         </is>
       </c>
     </row>
@@ -30251,7 +30291,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465230+00:00</t>
+          <t>2026-10-17T08:30:22.884651+00:00</t>
         </is>
       </c>
     </row>
@@ -30351,7 +30391,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465232+00:00</t>
+          <t>2026-10-17T08:30:22.884653+00:00</t>
         </is>
       </c>
     </row>
@@ -30459,7 +30499,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465855+00:00</t>
+          <t>2026-10-17T08:30:22.885197+00:00</t>
         </is>
       </c>
     </row>
@@ -30559,7 +30599,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465981+00:00</t>
+          <t>2026-10-17T08:30:22.885210+00:00</t>
         </is>
       </c>
     </row>
@@ -30659,7 +30699,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465989+00:00</t>
+          <t>2026-10-17T08:30:22.885214+00:00</t>
         </is>
       </c>
     </row>
@@ -30759,7 +30799,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.465994+00:00</t>
+          <t>2026-10-17T08:30:22.885217+00:00</t>
         </is>
       </c>
     </row>
@@ -30859,7 +30899,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.466063+00:00</t>
+          <t>2026-10-17T08:30:22.885220+00:00</t>
         </is>
       </c>
     </row>
@@ -30959,7 +30999,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.466067+00:00</t>
+          <t>2026-10-17T08:30:22.885223+00:00</t>
         </is>
       </c>
     </row>
@@ -31067,7 +31107,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.466580+00:00</t>
+          <t>2026-10-17T08:30:22.885672+00:00</t>
         </is>
       </c>
     </row>
@@ -31175,7 +31215,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.467708+00:00</t>
+          <t>2026-10-17T08:30:22.886715+00:00</t>
         </is>
       </c>
     </row>
@@ -31283,7 +31323,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.470706+00:00</t>
+          <t>2026-10-17T08:30:22.889652+00:00</t>
         </is>
       </c>
     </row>
@@ -31383,7 +31423,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.470725+00:00</t>
+          <t>2026-10-17T08:30:22.889671+00:00</t>
         </is>
       </c>
     </row>
@@ -31491,7 +31531,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.474854+00:00</t>
+          <t>2026-10-17T08:30:22.893917+00:00</t>
         </is>
       </c>
     </row>
@@ -31591,7 +31631,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.474874+00:00</t>
+          <t>2026-10-17T08:30:22.893952+00:00</t>
         </is>
       </c>
     </row>
@@ -31699,7 +31739,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.476946+00:00</t>
+          <t>2026-10-17T08:30:22.896133+00:00</t>
         </is>
       </c>
     </row>
@@ -31807,7 +31847,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.478682+00:00</t>
+          <t>2026-10-17T08:30:22.897997+00:00</t>
         </is>
       </c>
     </row>
@@ -31907,7 +31947,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.478699+00:00</t>
+          <t>2026-10-17T08:30:22.898030+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32047,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.478703+00:00</t>
+          <t>2026-10-17T08:30:22.898035+00:00</t>
         </is>
       </c>
     </row>
@@ -32107,7 +32147,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.478707+00:00</t>
+          <t>2026-10-17T08:30:22.898038+00:00</t>
         </is>
       </c>
     </row>
@@ -32207,7 +32247,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.478709+00:00</t>
+          <t>2026-10-17T08:30:22.898041+00:00</t>
         </is>
       </c>
     </row>
@@ -32315,7 +32355,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.479956+00:00</t>
+          <t>2026-10-17T08:30:22.899307+00:00</t>
         </is>
       </c>
     </row>
@@ -32415,7 +32455,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.479979+00:00</t>
+          <t>2026-10-17T08:30:22.899337+00:00</t>
         </is>
       </c>
     </row>
@@ -32515,7 +32555,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.479983+00:00</t>
+          <t>2026-10-17T08:30:22.899343+00:00</t>
         </is>
       </c>
     </row>
@@ -32615,7 +32655,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.479986+00:00</t>
+          <t>2026-10-17T08:30:22.899347+00:00</t>
         </is>
       </c>
     </row>
@@ -32711,7 +32751,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.479990+00:00</t>
+          <t>2026-10-17T08:30:22.899352+00:00</t>
         </is>
       </c>
     </row>
@@ -32807,7 +32847,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.479993+00:00</t>
+          <t>2026-10-17T08:30:22.899356+00:00</t>
         </is>
       </c>
     </row>
@@ -32903,7 +32943,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.479995+00:00</t>
+          <t>2026-10-17T08:30:22.899360+00:00</t>
         </is>
       </c>
     </row>
@@ -32999,7 +33039,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.479999+00:00</t>
+          <t>2026-10-17T08:30:22.899365+00:00</t>
         </is>
       </c>
     </row>
@@ -33095,7 +33135,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.480001+00:00</t>
+          <t>2026-10-17T08:30:22.899368+00:00</t>
         </is>
       </c>
     </row>
@@ -33191,7 +33231,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.480004+00:00</t>
+          <t>2026-10-17T08:30:22.899372+00:00</t>
         </is>
       </c>
     </row>
@@ -33287,7 +33327,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.480007+00:00</t>
+          <t>2026-10-17T08:30:22.899376+00:00</t>
         </is>
       </c>
     </row>
@@ -33395,7 +33435,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.480698+00:00</t>
+          <t>2026-10-17T08:30:22.900155+00:00</t>
         </is>
       </c>
     </row>
@@ -33495,7 +33535,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.480715+00:00</t>
+          <t>2026-10-17T08:30:22.900177+00:00</t>
         </is>
       </c>
     </row>
@@ -33603,7 +33643,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.480766+00:00</t>
+          <t>2026-10-17T08:30:22.900231+00:00</t>
         </is>
       </c>
     </row>
@@ -33711,7 +33751,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.481177+00:00</t>
+          <t>2026-10-17T08:30:22.900571+00:00</t>
         </is>
       </c>
     </row>
@@ -33819,7 +33859,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.481353+00:00</t>
+          <t>2026-10-17T08:30:22.900873+00:00</t>
         </is>
       </c>
     </row>
@@ -33931,7 +33971,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.481500+00:00</t>
+          <t>2026-10-17T08:30:22.901038+00:00</t>
         </is>
       </c>
     </row>
@@ -34039,7 +34079,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.481870+00:00</t>
+          <t>2026-10-17T08:30:22.901461+00:00</t>
         </is>
       </c>
     </row>
@@ -34147,7 +34187,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482061+00:00</t>
+          <t>2026-10-17T08:30:22.901696+00:00</t>
         </is>
       </c>
     </row>
@@ -34259,7 +34299,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482111+00:00</t>
+          <t>2026-10-17T08:30:22.901753+00:00</t>
         </is>
       </c>
     </row>
@@ -34371,7 +34411,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482170+00:00</t>
+          <t>2026-10-17T08:30:22.901818+00:00</t>
         </is>
       </c>
     </row>
@@ -34483,7 +34523,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482322+00:00</t>
+          <t>2026-10-17T08:30:22.902135+00:00</t>
         </is>
       </c>
     </row>
@@ -34595,7 +34635,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482369+00:00</t>
+          <t>2026-10-17T08:30:22.902198+00:00</t>
         </is>
       </c>
     </row>
@@ -34703,7 +34743,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482814+00:00</t>
+          <t>2026-10-17T08:30:22.902780+00:00</t>
         </is>
       </c>
     </row>
@@ -34811,7 +34851,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482858+00:00</t>
+          <t>2026-10-17T08:30:22.902847+00:00</t>
         </is>
       </c>
     </row>
@@ -34911,7 +34951,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482868+00:00</t>
+          <t>2026-10-17T08:30:22.902875+00:00</t>
         </is>
       </c>
     </row>
@@ -35011,7 +35051,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482871+00:00</t>
+          <t>2026-10-17T08:30:22.902880+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35155,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482875+00:00</t>
+          <t>2026-10-17T08:30:22.902883+00:00</t>
         </is>
       </c>
     </row>
@@ -35215,7 +35255,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.482878+00:00</t>
+          <t>2026-10-17T08:30:22.902886+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35363,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.483148+00:00</t>
+          <t>2026-10-17T08:30:22.903118+00:00</t>
         </is>
       </c>
     </row>
@@ -35431,7 +35471,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484210+00:00</t>
+          <t>2026-10-17T08:30:22.904207+00:00</t>
         </is>
       </c>
     </row>
@@ -35525,7 +35565,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484234+00:00</t>
+          <t>2026-10-17T08:30:22.904232+00:00</t>
         </is>
       </c>
     </row>
@@ -35619,7 +35659,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484237+00:00</t>
+          <t>2026-10-17T08:30:22.904237+00:00</t>
         </is>
       </c>
     </row>
@@ -35713,7 +35753,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484240+00:00</t>
+          <t>2026-10-17T08:30:22.904240+00:00</t>
         </is>
       </c>
     </row>
@@ -35807,7 +35847,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484243+00:00</t>
+          <t>2026-10-17T08:30:22.904244+00:00</t>
         </is>
       </c>
     </row>
@@ -35901,7 +35941,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484246+00:00</t>
+          <t>2026-10-17T08:30:22.904246+00:00</t>
         </is>
       </c>
     </row>
@@ -35995,7 +36035,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484248+00:00</t>
+          <t>2026-10-17T08:30:22.904250+00:00</t>
         </is>
       </c>
     </row>
@@ -36089,7 +36129,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484251+00:00</t>
+          <t>2026-10-17T08:30:22.904253+00:00</t>
         </is>
       </c>
     </row>
@@ -36183,7 +36223,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484259+00:00</t>
+          <t>2026-10-17T08:30:22.904255+00:00</t>
         </is>
       </c>
     </row>
@@ -36277,7 +36317,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484262+00:00</t>
+          <t>2026-10-17T08:30:22.904258+00:00</t>
         </is>
       </c>
     </row>
@@ -36371,7 +36411,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484265+00:00</t>
+          <t>2026-10-17T08:30:22.904261+00:00</t>
         </is>
       </c>
     </row>
@@ -36465,7 +36505,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484269+00:00</t>
+          <t>2026-10-17T08:30:22.904264+00:00</t>
         </is>
       </c>
     </row>
@@ -36559,7 +36599,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484272+00:00</t>
+          <t>2026-10-17T08:30:22.904267+00:00</t>
         </is>
       </c>
     </row>
@@ -36653,7 +36693,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484275+00:00</t>
+          <t>2026-10-17T08:30:22.904270+00:00</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36787,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484277+00:00</t>
+          <t>2026-10-17T08:30:22.904273+00:00</t>
         </is>
       </c>
     </row>
@@ -36841,7 +36881,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484280+00:00</t>
+          <t>2026-10-17T08:30:22.904276+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36975,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484283+00:00</t>
+          <t>2026-10-17T08:30:22.904279+00:00</t>
         </is>
       </c>
     </row>
@@ -37029,7 +37069,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484285+00:00</t>
+          <t>2026-10-17T08:30:22.904425+00:00</t>
         </is>
       </c>
     </row>
@@ -37123,7 +37163,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484288+00:00</t>
+          <t>2026-10-17T08:30:22.904429+00:00</t>
         </is>
       </c>
     </row>
@@ -37217,7 +37257,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484290+00:00</t>
+          <t>2026-10-17T08:30:22.904433+00:00</t>
         </is>
       </c>
     </row>
@@ -37311,7 +37351,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484292+00:00</t>
+          <t>2026-10-17T08:30:22.904435+00:00</t>
         </is>
       </c>
     </row>
@@ -37405,7 +37445,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484322+00:00</t>
+          <t>2026-10-17T08:30:22.904439+00:00</t>
         </is>
       </c>
     </row>
@@ -37499,7 +37539,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484329+00:00</t>
+          <t>2026-10-17T08:30:22.904442+00:00</t>
         </is>
       </c>
     </row>
@@ -37593,7 +37633,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484333+00:00</t>
+          <t>2026-10-17T08:30:22.904445+00:00</t>
         </is>
       </c>
     </row>
@@ -37687,7 +37727,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484336+00:00</t>
+          <t>2026-10-17T08:30:22.904448+00:00</t>
         </is>
       </c>
     </row>
@@ -37781,7 +37821,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484339+00:00</t>
+          <t>2026-10-17T08:30:22.904451+00:00</t>
         </is>
       </c>
     </row>
@@ -37875,7 +37915,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484342+00:00</t>
+          <t>2026-10-17T08:30:22.904454+00:00</t>
         </is>
       </c>
     </row>
@@ -37969,7 +38009,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484346+00:00</t>
+          <t>2026-10-17T08:30:22.904458+00:00</t>
         </is>
       </c>
     </row>
@@ -38069,7 +38109,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T08:29:31.484349+00:00</t>
+          <t>2026-10-17T08:30:22.904461+00:00</t>
         </is>
       </c>
     </row>
@@ -38084,7 +38124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38172,12 +38212,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>R13558</t>
+          <t>R01212</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R13558.main.0006612a5b75c131</t>
+          <t>R01212.main.ef235fcb491d4749</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -38187,20 +38227,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0006612a5b75c131170aa335c1e8d9810b41dca937beefac6ea258e1920944ec</t>
+          <t>ef235fcb491d474970838cf59cfd36efaf9a37c84ddd225c06788beb77d497e3</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>974385</v>
+        <v>773976</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.scielo.br/j/esa/a/DPQswHpgKLty6wPLBbxGcCn/?lang=en&amp;format=pdf</t>
+          <t>https://www.eeer.org/upload/eer-19-1-59-9.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>R13558_2026_Redox_mediators_and_microaeration_overcoming_linear_alkylbenzene_sulfonate_recalcitrance.pdf</t>
+          <t>R01212_2014_Effects_of_Pre-aeration_on_the_Anaerobic_Digestion_of_Sewage.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -38212,12 +38252,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>R04889</t>
+          <t>R08646</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R04889.main.860a0532503787f8</t>
+          <t>R08646.main.7df5523334e7d1bb</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -38227,20 +38267,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>860a0532503787f8bb84a599bdbf923f690615b05121c8a78c21249f8de911cb</t>
+          <t>7df5523334e7d1bb513d2a3deb5b018c0c9b2a3ea9e49b7ff8f09a1fe853cd96</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>506684</v>
+        <v>3009960</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://journal.unnes.ac.id/nju/jbat/article/download/16318/9427</t>
+          <t>https://europepmc.org/api/getPdf?pmcid=PMC10559078</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>R04889_2019_Inoculum_Selection_and_Micro-Aeration_for_Biogas_Production_in_Two-Stage.pdf</t>
+          <t>R08646_2023_Approaches_to_mitigation_of_hydrogen_sulfide_during_anaerobic_digestion.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -38252,12 +38292,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>R01212</t>
+          <t>R10894</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R01212.main.ef235fcb491d4749</t>
+          <t>R10894.main.f9caf3b730e23f0d</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -38267,20 +38307,20 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ef235fcb491d474970838cf59cfd36efaf9a37c84ddd225c06788beb77d497e3</t>
+          <t>f9caf3b730e23f0d9d31d71069935c39e162415bbdac53ee97821305a81be9d2</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>773976</v>
+        <v>2030435</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.eeer.org/upload/eer-19-1-59-9.pdf</t>
+          <t>https://europepmc.org/api/getPdf?pmcid=PMC11499478</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>R01212_2014_Effects_of_Pre-aeration_on_the_Anaerobic_Digestion_of_Sewage.pdf</t>
+          <t>R10894_2024_The_effects_of_different_pretreatment_technologies_on_microbial_community.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -38292,12 +38332,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>R05542</t>
+          <t>R06737</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R05542.main.735560cdb2769e25</t>
+          <t>R06737.main.32eabc0a46b31862</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -38307,20 +38347,20 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>735560cdb2769e2517355c073dd51a95ac90b015a5b36f90dcc0dff360ae182b</t>
+          <t>32eabc0a46b31862fa95a7bcf29fc4e5b154b7ec51c11cd1d4f798bbad95b59a</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>836053</v>
+        <v>4126947</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://europepmc.org/api/getPdf?pmcid=PMC9056904</t>
+          <t>https://ira.lib.polyu.edu.hk/bitstream/10397/97386/1/Zhuang_Genomic_Driven_Factors.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>R05542_2020_Effect_of_micro-aerobic_process_on_improvement_of_anaerobic_digestion.pdf</t>
+          <t>R06737_2021_Genomic_driven_factors_enhance_biocatalyst-related_cellulolysis_potential_in_anaerobic.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -38332,12 +38372,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>R06611</t>
+          <t>R04119</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>R06611.main.b8eb8afdada2a2d0</t>
+          <t>R04119.main.c9b1902447e38978</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -38347,20 +38387,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>b8eb8afdada2a2d0d5151fd81489263cbfd0ccc3bbde8c5ca36a02af52cfa12f</t>
+          <t>c9b1902447e38978d2f6f25327940f80e825baee1ebabba8bd8a860ed1fa254c</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3320239</v>
+        <v>1726821</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://eprints.whiterose.ac.uk/id/eprint/168685/1/A_draft_BITE_paper.pdf</t>
+          <t>https://europepmc.org/api/getPdf?pmcid=PMC6197294</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>R06611_2021_Effective_pretreatment_of_lignocellulosic_co-substrates_using_barley_straw-adapted_microbial.pdf</t>
+          <t>R04119_2018_Microbial_pretreatment_of_lignocellulosic_biomass_for_enhanced_biomethanation_and.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -38372,12 +38412,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R00273</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R07238.main.26c38d1631747ddc</t>
+          <t>R00273.main.2059ae72be92bd0e</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -38387,20 +38427,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>26c38d1631747ddcb443b8d80d0070145f1968ff0f4b8e86dc2f69cc2bb968d8</t>
+          <t>2059ae72be92bd0e0928b31eb73f27d1f92ac15865050966ba9369eae1ac9c0c</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>4532295</v>
+        <v>5372083</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://europepmc.org/api/getPdf?pmcid=PMC8044681</t>
+          <t>https://lup.lub.lu.se/luur/download?func=downloadFile&amp;recordOId=5277171&amp;fileOId=5277177</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>R07238_2021_The_influence_of_combined_low-strength_ultrasonics_and_micro-aerobic_pretreatment.pdf</t>
+          <t>R00273_2012_Management_of_hydrogen_sulfide_in_anaerobic_digestion_of_enzyme.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -38412,12 +38452,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R08646</t>
+          <t>R04700</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>R08646.main.7df5523334e7d1bb</t>
+          <t>R04700.main.40ac0de29f75851c</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -38427,20 +38467,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>7df5523334e7d1bb513d2a3deb5b018c0c9b2a3ea9e49b7ff8f09a1fe853cd96</t>
+          <t>40ac0de29f75851cab1651e1e339d03329bb7ce0141519329487f0559ebd8297</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3009960</v>
+        <v>2892628</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://europepmc.org/api/getPdf?pmcid=PMC10559078</t>
+          <t>https://repository.tudelft.nl/file/File_d8b73973-6e26-4f66-9162-3212f6b93431</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>R08646_2023_Approaches_to_mitigation_of_hydrogen_sulfide_during_anaerobic_digestion.pdf</t>
+          <t>R04700_2019_Effect_of_aeration_by_micro_-_bubbles_on_methane.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -38452,12 +38492,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>R10894</t>
+          <t>R09568</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>R10894.main.f9caf3b730e23f0d</t>
+          <t>R09568.main.393322098ea47587</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -38467,20 +38507,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>f9caf3b730e23f0d9d31d71069935c39e162415bbdac53ee97821305a81be9d2</t>
+          <t>393322098ea4758738b0e338c3e0019bd8618611d25a41cf3535d9542a6c8d16</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2030435</v>
+        <v>1433947</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://europepmc.org/api/getPdf?pmcid=PMC11499478</t>
+          <t>https://repository.tudelft.nl/file/File_b3a1ee42-17d3-4f7d-82dc-616c91a5a6bf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>R10894_2024_The_effects_of_different_pretreatment_technologies_on_microbial_community.pdf</t>
+          <t>R09568_2023_The_fate_of_sulfamethoxazole_and_trimethoprim_in_a_micro-aerated.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -38492,12 +38532,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>R06737</t>
+          <t>R10290</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>R06737.main.32eabc0a46b31862</t>
+          <t>R10290.main.0a63bc6c89e8dff8</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -38507,20 +38547,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>32eabc0a46b31862fa95a7bcf29fc4e5b154b7ec51c11cd1d4f798bbad95b59a</t>
+          <t>0a63bc6c89e8dff87ff1b364322ce6738e4fc87f505478ef522e7c73b7db342f</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>4126947</v>
+        <v>530753</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://ira.lib.polyu.edu.hk/bitstream/10397/97386/1/Zhuang_Genomic_Driven_Factors.pdf</t>
+          <t>https://office.nbc-journal.org/index.php/NBC/article/download/2100/955</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>R06737_2021_Genomic_driven_factors_enhance_biocatalyst-related_cellulolysis_potential_in_anaerobic.pdf</t>
+          <t>R10290_2024_Gas_nanobubble_technology_in_wastewater_treatment_and_anaerobic_digestion.pdf</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -38532,12 +38572,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>R04119</t>
+          <t>R10724</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>R04119.main.c9b1902447e38978</t>
+          <t>R10724.main.cfdc1bcb235acdd7</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -38547,20 +38587,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>c9b1902447e38978d2f6f25327940f80e825baee1ebabba8bd8a860ed1fa254c</t>
+          <t>cfdc1bcb235acdd703e58447b30b31cb8c4e8d53d1c86999ee8ecdafbba1e8aa</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1726821</v>
+        <v>2366242</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://europepmc.org/api/getPdf?pmcid=PMC6197294</t>
+          <t>https://www.ecoeet.com/pdf-181210-105068?filename=Protection-of-the-Purific.pdf</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>R04119_2018_Microbial_pretreatment_of_lignocellulosic_biomass_for_enhanced_biomethanation_and.pdf</t>
+          <t>R10724_2024_Protection_of_the_Purification_Station_Thermal_Engines_Against_the.pdf</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -38572,12 +38612,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>R00273</t>
+          <t>R11658</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>R00273.main.2059ae72be92bd0e</t>
+          <t>R11658.main.83a514a4b04c73a0</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -38587,20 +38627,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2059ae72be92bd0e0928b31eb73f27d1f92ac15865050966ba9369eae1ac9c0c</t>
+          <t>83a514a4b04c73a09129c21d623d57eb798a3af7c20dc842d47308f889d7695f</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5372083</v>
+        <v>458052</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://lup.lub.lu.se/luur/download?func=downloadFile&amp;recordOId=5277171&amp;fileOId=5277177</t>
+          <t>https://bsuj.bsu.edu.az/readpdf.php?file=236e3d6763a43f726c9814e7b5de8bc1.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>R00273_2012_Management_of_hydrogen_sulfide_in_anaerobic_digestion_of_enzyme.pdf</t>
+          <t>R11658_2025_IMPACT_OF_MICRO-AERATION_ON_FUNGAL_COMMUNITY_FROM_ANAEROBIC_DIGESTION.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -38612,12 +38652,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>R04700</t>
+          <t>R12483</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>R04700.main.40ac0de29f75851c</t>
+          <t>R12483.main.b51428ca89e5bf95</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -38627,20 +38667,20 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>40ac0de29f75851cab1651e1e339d03329bb7ce0141519329487f0559ebd8297</t>
+          <t>b51428ca89e5bf95c17225fe2e0a08a920379629281ab76f33337561553f3b0f</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2892628</v>
+        <v>1807518</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://repository.tudelft.nl/file/File_d8b73973-6e26-4f66-9162-3212f6b93431</t>
+          <t>https://li01.tci-thaijo.org/index.php/TSAEJ/article/download/269146/181297</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>R04700_2019_Effect_of_aeration_by_micro_-_bubbles_on_methane.pdf</t>
+          <t>R12483_2025_การปรบสภาพชวมวลลกโนเซลลโลสดวยวสดเพาะเหดเหลอทง_แนวทางการเพมมล.pdf</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -38652,12 +38692,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>R09568</t>
+          <t>R13819</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>R09568.main.393322098ea47587</t>
+          <t>R13819.main.431f5e76781d3cef</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -38667,20 +38707,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>393322098ea4758738b0e338c3e0019bd8618611d25a41cf3535d9542a6c8d16</t>
+          <t>431f5e76781d3cef39588c258c5589b1c9cf01db486c503ba29ab166bc73f14a</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1433947</v>
+        <v>2172752</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://repository.tudelft.nl/file/File_b3a1ee42-17d3-4f7d-82dc-616c91a5a6bf</t>
+          <t>https://epublications.marquette.edu/cgi/viewcontent.cgi?article=1131&amp;context=civengin_fac</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>R09568_2023_The_fate_of_sulfamethoxazole_and_trimethoprim_in_a_micro-aerated.pdf</t>
+          <t>R13819_2015_Bioaugmentation_of_overloaded_anaerobic_digesters_restores_function_and_archaeal.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -38692,12 +38732,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>R10290</t>
+          <t>R13833</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R10290.main.0a63bc6c89e8dff8</t>
+          <t>R13833.main.1a4a4d5f8fd45de9</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -38707,20 +38747,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0a63bc6c89e8dff87ff1b364322ce6738e4fc87f505478ef522e7c73b7db342f</t>
+          <t>1a4a4d5f8fd45de924c78a7be11e1c032c630bd9341431d1d49135c8351cdaf7</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>530753</v>
+        <v>1463714</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://office.nbc-journal.org/index.php/NBC/article/download/2100/955</t>
+          <t>https://repositorium.uminho.pt/server/api/core/bitstreams/234ac4ff-f996-498f-8853-72ba22cb7700/content</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>R10290_2024_Gas_nanobubble_technology_in_wastewater_treatment_and_anaerobic_digestion.pdf</t>
+          <t>R13833_2018_Insight_into_the_Role_of_Facultative_Bacteria_Stimulated_by.pdf</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -38732,12 +38772,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>R10724</t>
+          <t>R13861</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R10724.main.cfdc1bcb235acdd7</t>
+          <t>R13861.main.ba6f44b77d79c4a0</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -38747,20 +38787,20 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>cfdc1bcb235acdd703e58447b30b31cb8c4e8d53d1c86999ee8ecdafbba1e8aa</t>
+          <t>ba6f44b77d79c4a07ba08602860bcf1bdbb36cb47b4527fa9d1f087825e394d8</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2366242</v>
+        <v>433474</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.ecoeet.com/pdf-181210-105068?filename=Protection-of-the-Purific.pdf</t>
+          <t>https://www.scielo.br/j/esa/a/BD6Bc5rMVrTsbkK7CZz6yVd/?format=pdf&amp;lang=en&amp;ilang=pt_BR</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>R10724_2024_Protection_of_the_Purification_Station_Thermal_Engines_Against_the.pdf</t>
+          <t>R13861_2019_Enhanced_removal_of_emerging_micropollutants_by_applying_microaeration_to.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -38772,12 +38812,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>R11658</t>
+          <t>R13871</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R11658.main.83a514a4b04c73a0</t>
+          <t>R13871.main.aeab3126b6e68775</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -38787,20 +38827,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>83a514a4b04c73a09129c21d623d57eb798a3af7c20dc842d47308f889d7695f</t>
+          <t>aeab3126b6e68775b9b316714633bd97c1f184cf9e308d75b404bca6b33be19f</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>458052</v>
+        <v>7983514</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://bsuj.bsu.edu.az/readpdf.php?file=236e3d6763a43f726c9814e7b5de8bc1.pdf</t>
+          <t>https://etheses.whiterose.ac.uk/id/eprint/4094/6/Mahmood_Khazzal_Hummadi_Al-Mashhadani._Reg._No._080243946_%28PhD_thesis%29_2013.pdf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>R11658_2025_IMPACT_OF_MICRO-AERATION_ON_FUNGAL_COMMUNITY_FROM_ANAEROBIC_DIGESTION.pdf</t>
+          <t>R13871_2013_Application_of_Microbubbles_Generated_by_Fluidic_Oscillation_in_the.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -38812,12 +38852,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>R12483</t>
+          <t>R13877</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R12483.main.b51428ca89e5bf95</t>
+          <t>R13877.main.04a76adc76fa9472</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -38827,20 +38867,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>b51428ca89e5bf95c17225fe2e0a08a920379629281ab76f33337561553f3b0f</t>
+          <t>04a76adc76fa947250861c95c93759c590dd3e02d7f80dc23ce0abedccb74510</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1807518</v>
+        <v>522402</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://li01.tci-thaijo.org/index.php/TSAEJ/article/download/269146/181297</t>
+          <t>https://escholarship.org/content/qt5572k7rw/qt5572k7rw.pdf</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>R12483_2025_การปรบสภาพชวมวลลกโนเซลลโลสดวยวสดเพาะเหดเหลอทง_แนวทางการเพมมล.pdf</t>
+          <t>R13877_2018_Microbial_community_response_and_SDS-PAGE_reveal_possible_mechanism_of.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -38852,12 +38892,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>R13819</t>
+          <t>R13862</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R13819.main.431f5e76781d3cef</t>
+          <t>R13862.main.64e03a9beb5813a0</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -38867,20 +38907,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>431f5e76781d3cef39588c258c5589b1c9cf01db486c503ba29ab166bc73f14a</t>
+          <t>64e03a9beb5813a0ce6d94272350217f12dac94293420969e3d2d9d7975e96e3</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2172752</v>
+        <v>833659</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://epublications.marquette.edu/cgi/viewcontent.cgi?article=1131&amp;context=civengin_fac</t>
+          <t>https://repositorium.uminho.pt/server/api/core/bitstreams/eb850f96-0570-4e0d-be55-73fcee5f1364/content</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>R13819_2015_Bioaugmentation_of_overloaded_anaerobic_digesters_restores_function_and_archaeal.pdf</t>
+          <t>R13862_2020_Multiple_and_flexible_roles_of_facultative_anaerobic_bacteria_in.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -38892,12 +38932,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>R13833</t>
+          <t>R13900</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R13833.main.1a4a4d5f8fd45de9</t>
+          <t>R13900.main.b2ba7df8c04ab66c</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -38907,20 +38947,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1a4a4d5f8fd45de924c78a7be11e1c032c630bd9341431d1d49135c8351cdaf7</t>
+          <t>b2ba7df8c04ab66c0e548f778e19c5764802c0da8408a3b8499547b3f6ef51b3</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1463714</v>
+        <v>299244</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://repositorium.uminho.pt/server/api/core/bitstreams/234ac4ff-f996-498f-8853-72ba22cb7700/content</t>
+          <t>https://www.research.unipd.it/bitstream/11577/3261852/1/Front.%20Environ.%20Sci.%20Eng%20Dongbei%202018.pdf</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>R13833_2018_Insight_into_the_Role_of_Facultative_Bacteria_Stimulated_by.pdf</t>
+          <t>R13900_2018_Effectiveness_of_aerobic_pretreatment_of_municipal_solid_waste_for.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -38932,12 +38972,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>R13861</t>
+          <t>R13903</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R13861.main.ba6f44b77d79c4a0</t>
+          <t>R13903.main.2cd9e7b409250e7b</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -38947,20 +38987,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ba6f44b77d79c4a07ba08602860bcf1bdbb36cb47b4527fa9d1f087825e394d8</t>
+          <t>2cd9e7b409250e7b104f489e139f57d4daa40d97133c6c57c937184c3ec73b71</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>433474</v>
+        <v>1107675</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.scielo.br/j/esa/a/BD6Bc5rMVrTsbkK7CZz6yVd/?format=pdf&amp;lang=en&amp;ilang=pt_BR</t>
+          <t>https://ijabe.org/index.php/ijabe/article/download/7975/pdf</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>R13861_2019_Enhanced_removal_of_emerging_micropollutants_by_applying_microaeration_to.pdf</t>
+          <t>R13903_2023_Effect_of_vacuum_negative_pressure_aerobic_hydrolysis_pretreatment_on.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -38972,12 +39012,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>R13871</t>
+          <t>R13931</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R13871.main.aeab3126b6e68775</t>
+          <t>R13931.main.6e898a403edac7b3</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -38987,20 +39027,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>aeab3126b6e68775b9b316714633bd97c1f184cf9e308d75b404bca6b33be19f</t>
+          <t>6e898a403edac7b3ae15ad88cf75788898cd84ea377b2572f7bab40d9c126f8c</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>7983514</v>
+        <v>1324593</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://etheses.whiterose.ac.uk/id/eprint/4094/6/Mahmood_Khazzal_Hummadi_Al-Mashhadani._Reg._No._080243946_%28PhD_thesis%29_2013.pdf</t>
+          <t>https://www.eeer.org/upload/eer-2020-470.pdf</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>R13871_2013_Application_of_Microbubbles_Generated_by_Fluidic_Oscillation_in_the.pdf</t>
+          <t>R13931_2020_Biogas_recovery_from_fresh_landfill_leachates_by_using_a.pdf</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -39012,12 +39052,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>R13877</t>
+          <t>R13945</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R13877.main.04a76adc76fa9472</t>
+          <t>R13945.main.67309ea094d2f9bb</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -39027,20 +39067,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>04a76adc76fa947250861c95c93759c590dd3e02d7f80dc23ce0abedccb74510</t>
+          <t>67309ea094d2f9bb088d605746ede869866819a733f53c44dc2d44af934e6be9</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>522402</v>
+        <v>2230958</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://escholarship.org/content/qt5572k7rw/qt5572k7rw.pdf</t>
+          <t>https://epublications.marquette.edu/cgi/viewcontent.cgi?article=1459&amp;context=theses_open</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>R13877_2018_Microbial_community_response_and_SDS-PAGE_reveal_possible_mechanism_of.pdf</t>
+          <t>R13945_2018_Effect_of_Low_Aeration_and_Heat_Drying_on_Anaerobic.pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -39052,12 +39092,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>R13862</t>
+          <t>R13950</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R13862.main.64e03a9beb5813a0</t>
+          <t>R13950.main.2bf9b46c448685b9</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -39067,20 +39107,20 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>64e03a9beb5813a0ce6d94272350217f12dac94293420969e3d2d9d7975e96e3</t>
+          <t>2bf9b46c448685b9e66f4064245c5840dc28ded79ee4d613ddd9efeb4805812e</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>833659</v>
+        <v>3508852</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://repositorium.uminho.pt/server/api/core/bitstreams/eb850f96-0570-4e0d-be55-73fcee5f1364/content</t>
+          <t>https://www.research.unipd.it/bitstream/11577/3425227/1/Thesis_Razieh_Rafieenia.pdf</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>R13862_2020_Multiple_and_flexible_roles_of_facultative_anaerobic_bacteria_in.pdf</t>
+          <t>R13950_2019_Enhancement_of_hydrogen_and_methane_production_through_anaerobic_digestion.pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -39092,12 +39132,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R13900</t>
+          <t>R13944</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R13900.main.b2ba7df8c04ab66c</t>
+          <t>R13944.main.7e22fbfd39ddfed0</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -39107,20 +39147,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>b2ba7df8c04ab66c0e548f778e19c5764802c0da8408a3b8499547b3f6ef51b3</t>
+          <t>7e22fbfd39ddfed09b9235fea5c6914cfbe5987d12564fc9cb799bf412ae6779</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>299244</v>
+        <v>12042699</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.research.unipd.it/bitstream/11577/3261852/1/Front.%20Environ.%20Sci.%20Eng%20Dongbei%202018.pdf</t>
+          <t>https://scholarspace.manoa.hawaii.edu/server/api/core/bitstreams/60c88164-f37f-492a-97bc-e34a2f2b1698/content</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>R13900_2018_Effectiveness_of_aerobic_pretreatment_of_municipal_solid_waste_for.pdf</t>
+          <t>R13944_2018_Oxidation-Reduction_Potential-Based_Micro-Aeration_Control_System_for_Anaerobic_Digestion.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -39132,12 +39172,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>R13903</t>
+          <t>R13967</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R13903.main.2cd9e7b409250e7b</t>
+          <t>R13967.main.5e9f84dbaf01dd19</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -39147,20 +39187,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2cd9e7b409250e7b104f489e139f57d4daa40d97133c6c57c937184c3ec73b71</t>
+          <t>5e9f84dbaf01dd19674f09cbce96f338f32fe21a37a883bb9658e49af7072194</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1107675</v>
+        <v>160020</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://ijabe.org/index.php/ijabe/article/download/7975/pdf</t>
+          <t>https://www.aceee.org/wp-content/uploads/proceedings-1980-2020/2012/0193-000342.pdf</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>R13903_2023_Effect_of_vacuum_negative_pressure_aerobic_hydrolysis_pretreatment_on.pdf</t>
+          <t>R13967_2012_An_Improved_Biomass_Waste_Anaerobic_Degradation_Technology_for_Producing.pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -39172,12 +39212,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>R13931</t>
+          <t>R13972</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>R13931.main.6e898a403edac7b3</t>
+          <t>R13972.main.ff4ee9377a7e227c</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -39187,20 +39227,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>6e898a403edac7b3ae15ad88cf75788898cd84ea377b2572f7bab40d9c126f8c</t>
+          <t>ff4ee9377a7e227c48a5bc64d301bfc1a989ee0e709c322eb90f254819d7b391</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1324593</v>
+        <v>1192569</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.eeer.org/upload/eer-2020-470.pdf</t>
+          <t>https://www.osti.gov/servlets/purl/2386939</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>R13931_2020_Biogas_recovery_from_fresh_landfill_leachates_by_using_a.pdf</t>
+          <t>R13972_2022_Enhancing_methane_production_of_anaerobic_digested_sewage_sludge_by.pdf</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -39212,12 +39252,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>R13945</t>
+          <t>R13957</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>R13945.main.67309ea094d2f9bb</t>
+          <t>R13957.main.3db804dcdefb7608</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -39227,20 +39267,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>67309ea094d2f9bb088d605746ede869866819a733f53c44dc2d44af934e6be9</t>
+          <t>3db804dcdefb7608eefc6bf166b0713cbbec8ac027b1c01831aec97b54253b82</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2230958</v>
+        <v>7806265</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://epublications.marquette.edu/cgi/viewcontent.cgi?article=1459&amp;context=theses_open</t>
+          <t>https://backoffice.biblio.ugent.be/download/8530499/8530500</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>R13945_2018_Effect_of_Low_Aeration_and_Heat_Drying_on_Anaerobic.pdf</t>
+          <t>R13957_2017_Microaeration_for_biogas_desulfurization_experimental_and_simulation_study_of.pdf</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -39252,12 +39292,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>R13950</t>
+          <t>R04510</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>R13950.main.2bf9b46c448685b9</t>
+          <t>R04510.main.c4520ca79e301bb6</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -39267,20 +39307,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2bf9b46c448685b9e66f4064245c5840dc28ded79ee4d613ddd9efeb4805812e</t>
+          <t>c4520ca79e301bb606a8ab1fef6cf4af9064c0d85f3c390a4cf31a877238e1c6</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3508852</v>
+        <v>492630</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.research.unipd.it/bitstream/11577/3425227/1/Thesis_Razieh_Rafieenia.pdf</t>
+          <t>https://digital.csic.es/bitstream/10261/196040/5/PostP_2019_JESH_V54_Iss10.pdf</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>R13950_2019_Enhancement_of_hydrogen_and_methane_production_through_anaerobic_digestion.pdf</t>
+          <t>R04510_2019_Anaerobic_digestion_of_wastewater_rich_in_sulfate_and_sulfide_effects_of_metallic_waste_addition_and.pdf</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -39292,12 +39332,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>R13944</t>
+          <t>R13889</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>R13944.main.7e22fbfd39ddfed0</t>
+          <t>R13889.main.8db0dcdf434e876e</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -39307,20 +39347,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>7e22fbfd39ddfed09b9235fea5c6914cfbe5987d12564fc9cb799bf412ae6779</t>
+          <t>8db0dcdf434e876e7cbff3cf342105807bdd41a900f74c0028cb14a6c6e56779</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>12042699</v>
+        <v>514378</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://scholarspace.manoa.hawaii.edu/server/api/core/bitstreams/60c88164-f37f-492a-97bc-e34a2f2b1698/content</t>
+          <t>https://digital.csic.es/bitstream/10261/178890/1/PotP_2018_RE_V123_P541.pdf</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>R13944_2018_Oxidation-Reduction_Potential-Based_Micro-Aeration_Control_System_for_Anaerobic_Digestion.pdf</t>
+          <t>R13889_2018_Increase_in_biogas_production_in_anaerobic_sludge_digestion_by_combining_aerobic_hydrolysis_and_addi.pdf</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -39332,12 +39372,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R13967</t>
+          <t>R02719</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>R13967.main.5e9f84dbaf01dd19</t>
+          <t>R02719.main.4bf5e309b2ef3431</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -39347,20 +39387,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>5e9f84dbaf01dd19674f09cbce96f338f32fe21a37a883bb9658e49af7072194</t>
+          <t>4bf5e309b2ef343162a9588383a7ae0254118c33cdf2e96bec1a05459fae1523</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>160020</v>
+        <v>583591</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.aceee.org/wp-content/uploads/proceedings-1980-2020/2012/0193-000342.pdf</t>
+          <t>https://digital.csic.es/bitstream/10261/137944/1/Post_2016_JEnvSciHealth_A_BorjaR.pdf</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>R13967_2012_An_Improved_Biomass_Waste_Anaerobic_Degradation_Technology_for_Producing.pdf</t>
+          <t>R02719_2016_Performance_evaluation_of_micro_aerobic_hydrolysis_of_mixed_sludge_Optimum_aeration_and_effect_on_it.pdf</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -39372,12 +39412,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R13972</t>
+          <t>R02282</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>R13972.main.ff4ee9377a7e227c</t>
+          <t>R02282.main.e709439b748e7938</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -39387,20 +39427,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ff4ee9377a7e227c48a5bc64d301bfc1a989ee0e709c322eb90f254819d7b391</t>
+          <t>e709439b748e793826102646c009aa10e1e9ac30627ac301fac7dd42276a2047</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1192569</v>
+        <v>1067465</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.osti.gov/servlets/purl/2386939</t>
+          <t>https://digital.csic.es/bitstream/10261/130093/1/Postprint_2016_EnviromRev_V24_P84.pdf</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>R13972_2022_Enhancing_methane_production_of_anaerobic_digested_sewage_sludge_by.pdf</t>
+          <t>R02282_2016_Advances_in_the_biological_removal_of_sulphides_from_aqueous_phase_in_anaerobic_processes_A_review.pdf</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -39412,12 +39452,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R13957</t>
+          <t>R13905</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>R13957.main.3db804dcdefb7608</t>
+          <t>R13905.main.c75b5084c2545bd9</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -39427,20 +39467,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3db804dcdefb7608eefc6bf166b0713cbbec8ac027b1c01831aec97b54253b82</t>
+          <t>c75b5084c2545bd939d3b1928be41fe0072c7302f26c25ba023c4bb6fc8a6970</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>7806265</v>
+        <v>2159708</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://backoffice.biblio.ugent.be/download/8530499/8530500</t>
+          <t>https://ddd.uab.cat/pub/artpub/2017/196242/wasbioval_a2017m7v8n5p1793.pdf</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>R13957_2017_Microaeration_for_biogas_desulfurization_experimental_and_simulation_study_of.pdf</t>
+          <t>R13905_2017_The_Effect_of_a_Short_Term_Aerobic_Pretreatment_Step_on_the_Anaerobic_Co_digestion_of_the_Organic_Fr.pdf</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -39452,12 +39492,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R04510</t>
+          <t>R13932</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>R04510.main.c4520ca79e301bb6</t>
+          <t>R13932.main.c15f49a3d617e1be</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -39467,20 +39507,20 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>c4520ca79e301bb606a8ab1fef6cf4af9064c0d85f3c390a4cf31a877238e1c6</t>
+          <t>c15f49a3d617e1be5e21578ebda1c2d855f8d460c1d66f446ad0d02856a40a13</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>492630</v>
+        <v>1258157</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://digital.csic.es/bitstream/10261/196040/5/PostP_2019_JESH_V54_Iss10.pdf</t>
+          <t>https://hal.inrae.fr/hal-02620984/document</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>R04510_2019_Anaerobic_digestion_of_wastewater_rich_in_sulfate_and_sulfide_effects_of_metallic_waste_addition_and.pdf</t>
+          <t>R13932_2018_Comparison_of_pre_and_inter_stage_aerobic_treatment_of_wastewater_sludge_Effects_on_biogas_productio.pdf</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -39492,12 +39532,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R13889</t>
+          <t>R13956</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>R13889.main.8db0dcdf434e876e</t>
+          <t>R13956.main.fedaffcdf5be81e2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -39507,20 +39547,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>8db0dcdf434e876e7cbff3cf342105807bdd41a900f74c0028cb14a6c6e56779</t>
+          <t>fedaffcdf5be81e2070b7edb0531c332e423578228eeb8c55a6afc4ba8fe1e18</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>514378</v>
+        <v>421626</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://digital.csic.es/bitstream/10261/178890/1/PotP_2018_RE_V123_P541.pdf</t>
+          <t>https://www.banglajol.info/index.php/BJSIR/article/download/25579/17152</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>R13889_2018_Increase_in_biogas_production_in_anaerobic_sludge_digestion_by_combining_aerobic_hydrolysis_and_addi.pdf</t>
+          <t>R13956_2015_Anaerobic_digestion_of_mixed_dried_fallen_leaves_by_mixing_with_cow_dung.pdf</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -39532,12 +39572,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R02719</t>
+          <t>R13955</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>R02719.main.4bf5e309b2ef3431</t>
+          <t>R13955.main.7549e1025985363e</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -39547,20 +39587,20 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>4bf5e309b2ef343162a9588383a7ae0254118c33cdf2e96bec1a05459fae1523</t>
+          <t>7549e1025985363e89542bbc1af6eaaa1150bbd62ea43bdd03d2c7b764631f9d</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>583591</v>
+        <v>14662438</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://digital.csic.es/bitstream/10261/137944/1/Post_2016_JEnvSciHealth_A_BorjaR.pdf</t>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>R02719_2016_Performance_evaluation_of_micro_aerobic_hydrolysis_of_mixed_sludge_Optimum_aeration_and_effect_on_it.pdf</t>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion_7549e1025985.pdf</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -39572,35 +39612,35 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R02282</t>
+          <t>R07238</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>R02282.main.e709439b748e7938</t>
+          <t>R07238.supplementary.0b7925ad1ed9c793</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>supplementary</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>e709439b748e793826102646c009aa10e1e9ac30627ac301fac7dd42276a2047</t>
+          <t>0b7925ad1ed9c7939a79ba6294d17abc4b23fca77e52ec50df5463d050940d1e</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1067465</v>
+        <v>49526</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://digital.csic.es/bitstream/10261/130093/1/Postprint_2016_EnviromRev_V24_P84.pdf</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>R02282_2016_Advances_in_the_biological_removal_of_sulphides_from_aqueous_phase_in_anaerobic_processes_A_review.pdf</t>
+          <t>mmc1.docx</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -39612,35 +39652,35 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R13905</t>
+          <t>R07238</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>R13905.main.c75b5084c2545bd9</t>
+          <t>R07238.supplementary.f346f9bdcc964013</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>supplementary</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>c75b5084c2545bd939d3b1928be41fe0072c7302f26c25ba023c4bb6fc8a6970</t>
+          <t>f346f9bdcc964013ecb7c4282d6b30f1ab334e035d98adcc653de1447fbe9a9a</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2159708</v>
+        <v>14286928</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://ddd.uab.cat/pub/artpub/2017/196242/wasbioval_a2017m7v8n5p1793.pdf</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>R13905_2017_The_Effect_of_a_Short_Term_Aerobic_Pretreatment_Step_on_the_Anaerobic_Co_digestion_of_the_Organic_Fr.pdf</t>
+          <t>mmc2.zip</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -39652,35 +39692,35 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R13932</t>
+          <t>R07238</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>R13932.main.c15f49a3d617e1be</t>
+          <t>R07238.derived.49b84e369d4bb31b</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>c15f49a3d617e1be5e21578ebda1c2d855f8d460c1d66f446ad0d02856a40a13</t>
+          <t>49b84e369d4bb31b4ebdcd25265be3174105c3433e6fbb865f34a445775516a1</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1258157</v>
+        <v>34855493</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://hal.inrae.fr/hal-02620984/document</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>R13932_2018_Comparison_of_pre_and_inter_stage_aerobic_treatment_of_wastewater_sludge_Effects_on_biogas_productio.pdf</t>
+          <t>g a.skp</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -39692,35 +39732,35 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R13956</t>
+          <t>R08646</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>R13956.main.fedaffcdf5be81e2</t>
+          <t>R08646.supplementary.cfda7e29b12b9784</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>supplementary</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>fedaffcdf5be81e2070b7edb0531c332e423578228eeb8c55a6afc4ba8fe1e18</t>
+          <t>cfda7e29b12b97846343963f9f3b64e784bc79644fb1ee1ca31170be78d75327</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>421626</v>
+        <v>42279</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://www.banglajol.info/index.php/BJSIR/article/download/25579/17152</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>R13956_2015_Anaerobic_digestion_of_mixed_dried_fallen_leaves_by_mixing_with_cow_dung.pdf</t>
+          <t>mmc1.docx</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -39732,35 +39772,35 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R13955</t>
+          <t>R03161</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>R13955.main.7549e1025985363e</t>
+          <t>R03161.evidence_xml.466f3a1e78e8b0f1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>7549e1025985363e89542bbc1af6eaaa1150bbd62ea43bdd03d2c7b764631f9d</t>
+          <t>466f3a1e78e8b0f148b1f28f97b61f7134c61488c837c5c5a26ef7316cebc1e9</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>14662438</v>
+        <v>59018</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/fullTextXML</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion_7549e1025985.pdf</t>
+          <t>PMC5627928_fullText.xml</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -39772,35 +39812,35 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R03161</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>R07238.supplementary.0b7925ad1ed9c793</t>
+          <t>R03161.transport_archive.0ef4d4796c84feff</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>supplementary</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0b7925ad1ed9c7939a79ba6294d17abc4b23fca77e52ec50df5463d050940d1e</t>
+          <t>0ef4d4796c84fefff7b8450bc56400f8c59f4bdcf074fc51404edff5e4e217f6</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>49526</v>
+        <v>726772</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/supplementaryFiles</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>mmc1.docx</t>
+          <t>PMC5627928_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -39812,35 +39852,35 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R04092</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>R07238.supplementary.f346f9bdcc964013</t>
+          <t>R04092.evidence_xml.0fb90085e30680fa</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>supplementary</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>f346f9bdcc964013ecb7c4282d6b30f1ab334e035d98adcc653de1447fbe9a9a</t>
+          <t>0fb90085e30680fa8a9896b80afb9da4f9466ba0051ea2ffb89a13e06a5013a3</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>14286928</v>
+        <v>77995</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6288047/fullTextXML</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>mmc2.zip</t>
+          <t>PMC6288047_fullText.xml</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -39852,35 +39892,35 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R05839</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>R07238.derived.49b84e369d4bb31b</t>
+          <t>R05839.evidence_xml.18ffd43dee955086</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>49b84e369d4bb31b4ebdcd25265be3174105c3433e6fbb865f34a445775516a1</t>
+          <t>18ffd43dee955086eae0947027dc85e1d765e181357143650e9fef0b0dfbef74</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>34855493</v>
+        <v>75205</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC7566014/fullTextXML</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>g a.skp</t>
+          <t>PMC7566014_fullText.xml</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -39892,35 +39932,35 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R08646</t>
+          <t>R08877</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>R08646.supplementary.cfda7e29b12b9784</t>
+          <t>R08877.evidence_xml.e8712e4198baab4c</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>supplementary</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>cfda7e29b12b97846343963f9f3b64e784bc79644fb1ee1ca31170be78d75327</t>
+          <t>e8712e4198baab4c79ee53c54ea30b4d96721e2d47e08b657a6b19b4bf41891a</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>42279</v>
+        <v>111864</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/fullTextXML</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>mmc1.docx</t>
+          <t>PMC10714394_fullText.xml</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -39932,35 +39972,35 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R03161</t>
+          <t>R08877</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>R03161.evidence_xml.466f3a1e78e8b0f1</t>
+          <t>R08877.transport_archive.ed8e864a3225e9c4</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>466f3a1e78e8b0f148b1f28f97b61f7134c61488c837c5c5a26ef7316cebc1e9</t>
+          <t>ed8e864a3225e9c4cecf84e5f4670c985de4c6d453d0b7b459ad5870e6627f97</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>59018</v>
+        <v>704921</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/supplementaryFiles</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>PMC5627928_fullText.xml</t>
+          <t>PMC10714394_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -39972,35 +40012,35 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R03161</t>
+          <t>R09236</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>R03161.transport_archive.0ef4d4796c84feff</t>
+          <t>R09236.evidence_xml.72064fe9276d8309</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>0ef4d4796c84fefff7b8450bc56400f8c59f4bdcf074fc51404edff5e4e217f6</t>
+          <t>72064fe9276d830984364e82e4567877578408565c650d856c531204a17ded89</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>726772</v>
+        <v>193052</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/fullTextXML</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>PMC5627928_supplementaryFiles.zip</t>
+          <t>PMC10535533_fullText.xml</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -40012,35 +40052,35 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R04092</t>
+          <t>R09236</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>R04092.evidence_xml.0fb90085e30680fa</t>
+          <t>R09236.transport_archive.f3c6856282b7e8d6</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>0fb90085e30680fa8a9896b80afb9da4f9466ba0051ea2ffb89a13e06a5013a3</t>
+          <t>f3c6856282b7e8d694d35a87eae016d8e66aa902189c7c3311a1153ea24752e0</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>77995</v>
+        <v>483405</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6288047/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/supplementaryFiles</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>PMC6288047_fullText.xml</t>
+          <t>PMC10535533_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -40052,12 +40092,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>R05839</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>R05839.evidence_xml.18ffd43dee955086</t>
+          <t>R10086.evidence_xml.074f3cb8a39355a5</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -40067,20 +40107,20 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>18ffd43dee955086eae0947027dc85e1d765e181357143650e9fef0b0dfbef74</t>
+          <t>074f3cb8a39355a5d7cfb8af0139c674b72aec8e5d08bcd20b8f0e46d0d88fbe</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>75205</v>
+        <v>118002</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC7566014/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/fullTextXML</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>PMC7566014_fullText.xml</t>
+          <t>PMC10837232_fullText.xml</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -40092,35 +40132,35 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>R08877</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>R08877.evidence_xml.e8712e4198baab4c</t>
+          <t>R10086.transport_archive.4d9eddf454b786ed</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>e8712e4198baab4c79ee53c54ea30b4d96721e2d47e08b657a6b19b4bf41891a</t>
+          <t>4d9eddf454b786eddece423a320b28d7f96959a935334ddc7c7e2fe32d39bc9b</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>111864</v>
+        <v>641038</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/supplementaryFiles</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>PMC10714394_fullText.xml</t>
+          <t>PMC10837232_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -40132,35 +40172,35 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>R08877</t>
+          <t>R12985</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>R08877.transport_archive.ed8e864a3225e9c4</t>
+          <t>R12985.evidence_xml.f1a80564a8a1fa4b</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ed8e864a3225e9c4cecf84e5f4670c985de4c6d453d0b7b459ad5870e6627f97</t>
+          <t>f1a80564a8a1fa4b638bb6097c75cb3709b4c7487b6c8012474fd4e1865576cc</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>704921</v>
+        <v>173586</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/fullTextXML</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>PMC10714394_supplementaryFiles.zip</t>
+          <t>PMC12937426_fullText.xml</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -40172,35 +40212,35 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>R09236</t>
+          <t>R12985</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>R09236.evidence_xml.72064fe9276d8309</t>
+          <t>R12985.transport_archive.418d45f1ca296020</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>72064fe9276d830984364e82e4567877578408565c650d856c531204a17ded89</t>
+          <t>418d45f1ca2960209df0bfc1c3d44069413edc213239570a3d71d08d01f3e3e0</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>193052</v>
+        <v>672244</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/supplementaryFiles</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>PMC10535533_fullText.xml</t>
+          <t>PMC12937426_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -40212,35 +40252,35 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>R09236</t>
+          <t>R05542</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>R09236.transport_archive.f3c6856282b7e8d6</t>
+          <t>R05542.evidence_xml.9ee6c9217e7c01e1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>f3c6856282b7e8d694d35a87eae016d8e66aa902189c7c3311a1153ea24752e0</t>
+          <t>9ee6c9217e7c01e1604e3170e0041677e5b9d0f14b59ee1e9717c1082d9d193a</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>483405</v>
+        <v>100215</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC9056904/fullTextXML</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>PMC10535533_supplementaryFiles.zip</t>
+          <t>PMC9056904_fullText.xml</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -40252,12 +40292,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>R10086</t>
+          <t>R06325</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>R10086.evidence_xml.074f3cb8a39355a5</t>
+          <t>R06325.evidence_xml.645deb707d3790b5</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -40267,20 +40307,20 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>074f3cb8a39355a5d7cfb8af0139c674b72aec8e5d08bcd20b8f0e46d0d88fbe</t>
+          <t>645deb707d3790b518690b7413885823461bb57a3dfa5bb587202d8f16dda296</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>118002</v>
+        <v>160509</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/fullTextXML</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>PMC10837232_fullText.xml</t>
+          <t>PMC8290346_fullText.xml</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -40292,12 +40332,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>R10086</t>
+          <t>R06325</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>R10086.transport_archive.4d9eddf454b786ed</t>
+          <t>R06325.transport_archive.6eb4ef126661714a</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -40307,20 +40347,20 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>4d9eddf454b786eddece423a320b28d7f96959a935334ddc7c7e2fe32d39bc9b</t>
+          <t>6eb4ef126661714ae89bde97acdddac2c2a582864ca26ff9af569cfe609a4226</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>641038</v>
+        <v>1730580</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/supplementaryFiles</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>PMC10837232_supplementaryFiles.zip</t>
+          <t>PMC8290346_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -40332,12 +40372,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>R12985</t>
+          <t>R07238</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>R12985.evidence_xml.f1a80564a8a1fa4b</t>
+          <t>R07238.evidence_xml.6c93b117d7bd5886</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -40347,20 +40387,20 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>f1a80564a8a1fa4b638bb6097c75cb3709b4c7487b6c8012474fd4e1865576cc</t>
+          <t>6c93b117d7bd588658aabfd8b7ec679110899d8f556eb6b90b071e6057ddd2cd</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>173586</v>
+        <v>151458</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/fullTextXML</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>PMC12937426_fullText.xml</t>
+          <t>PMC8044681_fullText.xml</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -40372,12 +40412,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>R12985</t>
+          <t>R07238</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>R12985.transport_archive.418d45f1ca296020</t>
+          <t>R07238.transport_archive.3785c23cb2f4ab50</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -40387,20 +40427,20 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>418d45f1ca2960209df0bfc1c3d44069413edc213239570a3d71d08d01f3e3e0</t>
+          <t>3785c23cb2f4ab50f5b2b5cbb581da63ced9f8d1e69a91e6faca839b6b57587d</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>672244</v>
+        <v>14596266</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>PMC12937426_supplementaryFiles.zip</t>
+          <t>PMC8044681_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -40412,12 +40452,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>R05542</t>
+          <t>R03477</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>R05542.evidence_xml.9ee6c9217e7c01e1</t>
+          <t>R03477.evidence_xml.c127b68ddfdcfec8</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -40427,20 +40467,20 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>9ee6c9217e7c01e1604e3170e0041677e5b9d0f14b59ee1e9717c1082d9d193a</t>
+          <t>c127b68ddfdcfec8d98508723d4d7a4b250ec3f82c4c75756cb539406519a8f7</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>100215</v>
+        <v>121650</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC9056904/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5371168/fullTextXML</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>PMC9056904_fullText.xml</t>
+          <t>PMC5371168_fullText.xml</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -40452,12 +40492,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>R06325</t>
+          <t>R08646</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>R06325.evidence_xml.645deb707d3790b5</t>
+          <t>R08646.evidence_xml.c7b723e8020f6582</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -40467,20 +40507,20 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>645deb707d3790b518690b7413885823461bb57a3dfa5bb587202d8f16dda296</t>
+          <t>c7b723e8020f65823eaf8b08c6b56c36aab85784bbef3b10c9a85a820b960d3a</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>160509</v>
+        <v>304277</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/fullTextXML</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>PMC8290346_fullText.xml</t>
+          <t>PMC10559078_fullText.xml</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -40492,12 +40532,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>R06325</t>
+          <t>R08646</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>R06325.transport_archive.6eb4ef126661714a</t>
+          <t>R08646.transport_archive.ecda9ea461a3deb3</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -40507,20 +40547,20 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>6eb4ef126661714ae89bde97acdddac2c2a582864ca26ff9af569cfe609a4226</t>
+          <t>ecda9ea461a3deb361931eb51186e88488c4d6ae284899e1feb1d611de42550a</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1730580</v>
+        <v>1539133</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>PMC8290346_supplementaryFiles.zip</t>
+          <t>PMC10559078_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -40532,12 +40572,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R09804</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>R07238.evidence_xml.6c93b117d7bd5886</t>
+          <t>R09804.evidence_xml.2ca7af24c486ae9e</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -40547,20 +40587,20 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>6c93b117d7bd588658aabfd8b7ec679110899d8f556eb6b90b071e6057ddd2cd</t>
+          <t>2ca7af24c486ae9eb9c65682356964011c985b22a4a36f4ee07ea3a705c38951</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>151458</v>
+        <v>211630</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC11076452/fullTextXML</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>PMC8044681_fullText.xml</t>
+          <t>PMC11076452_fullText.xml</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -40572,35 +40612,35 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R11503</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>R07238.transport_archive.3785c23cb2f4ab50</t>
+          <t>R11503.evidence_xml.4002d57be59c215c</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>3785c23cb2f4ab50f5b2b5cbb581da63ced9f8d1e69a91e6faca839b6b57587d</t>
+          <t>4002d57be59c215cea8477a4b667f20f9ffb09680e70af377a81ffae74b99801</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>14596266</v>
+        <v>258637</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12561102/fullTextXML</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>PMC8044681_supplementaryFiles.zip</t>
+          <t>PMC12561102_fullText.xml</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -40612,12 +40652,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>R03477</t>
+          <t>R11844</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>R03477.evidence_xml.c127b68ddfdcfec8</t>
+          <t>R11844.evidence_xml.9c39d5f64ac01253</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -40627,20 +40667,20 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>c127b68ddfdcfec8d98508723d4d7a4b250ec3f82c4c75756cb539406519a8f7</t>
+          <t>9c39d5f64ac01253c8bb4866ce3974997765b2d47e37641f3717e99e0d7f1f61</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>121650</v>
+        <v>256247</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5371168/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/fullTextXML</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>PMC5371168_fullText.xml</t>
+          <t>PMC12125087_fullText.xml</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -40652,35 +40692,35 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>R08646</t>
+          <t>R11844</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>R08646.evidence_xml.c7b723e8020f6582</t>
+          <t>R11844.transport_archive.60ef29cf0a557bf4</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>c7b723e8020f65823eaf8b08c6b56c36aab85784bbef3b10c9a85a820b960d3a</t>
+          <t>60ef29cf0a557bf44838f4a3f45e2dbf1b1a2001547f5c0b976b48cc64c1b6d9</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>304277</v>
+        <v>521862</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/supplementaryFiles</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>PMC10559078_fullText.xml</t>
+          <t>PMC12125087_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -40692,35 +40732,35 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>R08646</t>
+          <t>R05213</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>R08646.transport_archive.ecda9ea461a3deb3</t>
+          <t>R05213.evidence_xml.17894ab410001846</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ecda9ea461a3deb361931eb51186e88488c4d6ae284899e1feb1d611de42550a</t>
+          <t>17894ab41000184655d2f9f9a0daa796981ab3658678c6b123eb9f3deb1bf45a</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>1539133</v>
+        <v>130954</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/fullTextXML</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>PMC10559078_supplementaryFiles.zip</t>
+          <t>PMC6858683_fullText.xml</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -40732,35 +40772,35 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>R09804</t>
+          <t>R05213</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>R09804.evidence_xml.2ca7af24c486ae9e</t>
+          <t>R05213.transport_archive.c61c88cf9fd489be</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2ca7af24c486ae9eb9c65682356964011c985b22a4a36f4ee07ea3a705c38951</t>
+          <t>c61c88cf9fd489beab88c1b72bbfe5f13167f32c984b6dba6e48ba97c6136b7b</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>211630</v>
+        <v>1960371</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC11076452/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/supplementaryFiles</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>PMC11076452_fullText.xml</t>
+          <t>PMC6858683_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -40772,12 +40812,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>R11503</t>
+          <t>R09585</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>R11503.evidence_xml.4002d57be59c215c</t>
+          <t>R09585.evidence_xml.a3430f38fa1652de</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -40787,20 +40827,20 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4002d57be59c215cea8477a4b667f20f9ffb09680e70af377a81ffae74b99801</t>
+          <t>a3430f38fa1652de3145ffc47f0da514ee41e12ef8e95acc30330d6b3a01efd2</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>258637</v>
+        <v>100534</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12561102/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10609292/fullTextXML</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>PMC12561102_fullText.xml</t>
+          <t>PMC10609292_fullText.xml</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -40812,238 +40852,38 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>R11844</t>
+          <t>R11596</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>R11844.evidence_xml.9c39d5f64ac01253</t>
+          <t>R11596.main.0b2e2d98dffd5449</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>9c39d5f64ac01253c8bb4866ce3974997765b2d47e37641f3717e99e0d7f1f61</t>
+          <t>0b2e2d98dffd544958b06cc2229d310e4b7d529bd3914c47f20d6a66789a28be</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>256247</v>
+        <v>1659399</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/fullTextXML</t>
+          <t>https://repositorium.uminho.pt/server/api/core/bitstreams/7262c516-6b14-4001-a173-517d1187c8d9/content</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>PMC12125087_fullText.xml</t>
+          <t>R11596_2025_Facultative_anaerobic_bacteria_enable_syntrophic_fatty_acids_degradation_under_0b2e2d98dffd.pdf</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>R11844</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>R11844.transport_archive.60ef29cf0a557bf4</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>transport_archive</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>60ef29cf0a557bf44838f4a3f45e2dbf1b1a2001547f5c0b976b48cc64c1b6d9</t>
-        </is>
-      </c>
-      <c r="E70" t="n">
-        <v>521862</v>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/supplementaryFiles</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>PMC12125087_supplementaryFiles.zip</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>R05213</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>R05213.evidence_xml.17894ab410001846</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>evidence_xml</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>17894ab41000184655d2f9f9a0daa796981ab3658678c6b123eb9f3deb1bf45a</t>
-        </is>
-      </c>
-      <c r="E71" t="n">
-        <v>130954</v>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/fullTextXML</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>PMC6858683_fullText.xml</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>R05213</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>R05213.transport_archive.c61c88cf9fd489be</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>transport_archive</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>c61c88cf9fd489beab88c1b72bbfe5f13167f32c984b6dba6e48ba97c6136b7b</t>
-        </is>
-      </c>
-      <c r="E72" t="n">
-        <v>1960371</v>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/supplementaryFiles</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>PMC6858683_supplementaryFiles.zip</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>R09585</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>R09585.evidence_xml.a3430f38fa1652de</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>evidence_xml</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>a3430f38fa1652de3145ffc47f0da514ee41e12ef8e95acc30330d6b3a01efd2</t>
-        </is>
-      </c>
-      <c r="E73" t="n">
-        <v>100534</v>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10609292/fullTextXML</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>PMC10609292_fullText.xml</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>R11596</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>R11596.main.0b2e2d98dffd5449</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>0b2e2d98dffd544958b06cc2229d310e4b7d529bd3914c47f20d6a66789a28be</t>
-        </is>
-      </c>
-      <c r="E74" t="n">
-        <v>1659399</v>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>https://repositorium.uminho.pt/server/api/core/bitstreams/7262c516-6b14-4001-a173-517d1187c8d9/content</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>R11596_2025_Facultative_anaerobic_bacteria_enable_syntrophic_fatty_acids_degradation_under_0b2e2d98dffd.pdf</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
         <is>
           <t>历史已获取，当前原件未恢复</t>
         </is>

</xml_diff>

<commit_message>
Persist recovered historical originals and manually verified thesis version
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -1181,7 +1181,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6471,14 +6471,14 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="H141" t="b">
         <v>0</v>
       </c>
       <c r="I141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -9881,7 +9881,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -11499,7 +11499,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -12097,7 +12097,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -14231,7 +14231,7 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>historical_acquired_current_original_not_restored</t>
         </is>
       </c>
       <c r="G482" t="inlineStr">
@@ -23342,7 +23342,7 @@
       </c>
       <c r="F537" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G537" t="inlineStr">
@@ -24118,7 +24118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X136"/>
+  <dimension ref="A1:X148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.063474+00:00</t>
+          <t>2026-10-17T08:41:26.347549+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.064520+00:00</t>
+          <t>2026-10-17T08:41:26.348430+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.064547+00:00</t>
+          <t>2026-10-17T08:41:26.348449+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.064855+00:00</t>
+          <t>2026-10-17T08:41:26.348663+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.066256+00:00</t>
+          <t>2026-10-17T08:41:26.349868+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.066787+00:00</t>
+          <t>2026-10-17T08:41:26.350359+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.072610+00:00</t>
+          <t>2026-10-17T08:41:26.355666+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.075260+00:00</t>
+          <t>2026-10-17T08:41:26.357985+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.076350+00:00</t>
+          <t>2026-10-17T08:41:26.359052+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.076686+00:00</t>
+          <t>2026-10-17T08:41:26.359415+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.077674+00:00</t>
+          <t>2026-10-17T08:41:26.360113+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.078358+00:00</t>
+          <t>2026-10-17T08:41:26.360772+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.079359+00:00</t>
+          <t>2026-10-17T08:41:26.361748+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.079614+00:00</t>
+          <t>2026-10-17T08:41:26.362194+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.080474+00:00</t>
+          <t>2026-10-17T08:41:26.363386+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.088624+00:00</t>
+          <t>2026-10-17T08:41:26.372425+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.089384+00:00</t>
+          <t>2026-10-17T08:41:26.373227+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.090592+00:00</t>
+          <t>2026-10-17T08:41:26.374560+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.093199+00:00</t>
+          <t>2026-10-17T08:41:26.377155+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.094323+00:00</t>
+          <t>2026-10-17T08:41:26.378277+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.095591+00:00</t>
+          <t>2026-10-17T08:41:26.379520+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.100766+00:00</t>
+          <t>2026-10-17T08:41:26.383696+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.103231+00:00</t>
+          <t>2026-10-17T08:41:26.385865+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.105032+00:00</t>
+          <t>2026-10-17T08:41:26.387656+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.105721+00:00</t>
+          <t>2026-10-17T08:41:26.388360+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.106094+00:00</t>
+          <t>2026-10-17T08:41:26.388717+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.108162+00:00</t>
+          <t>2026-10-17T08:41:26.390754+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.109513+00:00</t>
+          <t>2026-10-17T08:41:26.391984+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.111550+00:00</t>
+          <t>2026-10-17T08:41:26.394173+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.113562+00:00</t>
+          <t>2026-10-17T08:41:26.396198+00:00</t>
         </is>
       </c>
     </row>
@@ -27571,7 +27571,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.113585+00:00</t>
+          <t>2026-10-17T08:41:26.396223+00:00</t>
         </is>
       </c>
     </row>
@@ -27679,7 +27679,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.114164+00:00</t>
+          <t>2026-10-17T08:41:26.396798+00:00</t>
         </is>
       </c>
     </row>
@@ -27787,7 +27787,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.115802+00:00</t>
+          <t>2026-10-17T08:41:26.398655+00:00</t>
         </is>
       </c>
     </row>
@@ -27895,7 +27895,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.118694+00:00</t>
+          <t>2026-10-17T08:41:26.401497+00:00</t>
         </is>
       </c>
     </row>
@@ -28003,7 +28003,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.121076+00:00</t>
+          <t>2026-10-17T08:41:26.403628+00:00</t>
         </is>
       </c>
     </row>
@@ -28111,7 +28111,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.122437+00:00</t>
+          <t>2026-10-17T08:41:26.404796+00:00</t>
         </is>
       </c>
     </row>
@@ -28219,7 +28219,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.125376+00:00</t>
+          <t>2026-10-17T08:41:26.407614+00:00</t>
         </is>
       </c>
     </row>
@@ -28327,7 +28327,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.126131+00:00</t>
+          <t>2026-10-17T08:41:26.408280+00:00</t>
         </is>
       </c>
     </row>
@@ -28435,7 +28435,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.127706+00:00</t>
+          <t>2026-10-17T08:41:26.409854+00:00</t>
         </is>
       </c>
     </row>
@@ -28543,7 +28543,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.127959+00:00</t>
+          <t>2026-10-17T08:41:26.410087+00:00</t>
         </is>
       </c>
     </row>
@@ -28651,7 +28651,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.130052+00:00</t>
+          <t>2026-10-17T08:41:26.412406+00:00</t>
         </is>
       </c>
     </row>
@@ -28759,7 +28759,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.133038+00:00</t>
+          <t>2026-10-17T08:41:26.415377+00:00</t>
         </is>
       </c>
     </row>
@@ -28867,7 +28867,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.135048+00:00</t>
+          <t>2026-10-17T08:41:26.416672+00:00</t>
         </is>
       </c>
     </row>
@@ -28975,7 +28975,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.135888+00:00</t>
+          <t>2026-10-17T08:41:26.417239+00:00</t>
         </is>
       </c>
     </row>
@@ -29083,7 +29083,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.138727+00:00</t>
+          <t>2026-10-17T08:41:26.420095+00:00</t>
         </is>
       </c>
     </row>
@@ -29191,7 +29191,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.140001+00:00</t>
+          <t>2026-10-17T08:41:26.423131+00:00</t>
         </is>
       </c>
     </row>
@@ -29299,7 +29299,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.143888+00:00</t>
+          <t>2026-10-17T08:41:26.427088+00:00</t>
         </is>
       </c>
     </row>
@@ -29407,7 +29407,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.145829+00:00</t>
+          <t>2026-10-17T08:41:26.428750+00:00</t>
         </is>
       </c>
     </row>
@@ -29515,7 +29515,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.148342+00:00</t>
+          <t>2026-10-17T08:41:26.430950+00:00</t>
         </is>
       </c>
     </row>
@@ -29623,7 +29623,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.149670+00:00</t>
+          <t>2026-10-17T08:41:26.432009+00:00</t>
         </is>
       </c>
     </row>
@@ -29731,7 +29731,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.150250+00:00</t>
+          <t>2026-10-17T08:41:26.432842+00:00</t>
         </is>
       </c>
     </row>
@@ -29839,7 +29839,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.150665+00:00</t>
+          <t>2026-10-17T08:41:26.433238+00:00</t>
         </is>
       </c>
     </row>
@@ -29947,7 +29947,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.152240+00:00</t>
+          <t>2026-10-17T08:41:26.434747+00:00</t>
         </is>
       </c>
     </row>
@@ -30055,7 +30055,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.153614+00:00</t>
+          <t>2026-10-17T08:41:26.436053+00:00</t>
         </is>
       </c>
     </row>
@@ -30163,7 +30163,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.155168+00:00</t>
+          <t>2026-10-17T08:41:26.437725+00:00</t>
         </is>
       </c>
     </row>
@@ -30271,7 +30271,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.155522+00:00</t>
+          <t>2026-10-17T08:41:26.438065+00:00</t>
         </is>
       </c>
     </row>
@@ -30379,7 +30379,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.156734+00:00</t>
+          <t>2026-10-17T08:41:26.439341+00:00</t>
         </is>
       </c>
     </row>
@@ -30487,7 +30487,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.158428+00:00</t>
+          <t>2026-10-17T08:41:26.440835+00:00</t>
         </is>
       </c>
     </row>
@@ -30595,7 +30595,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.159050+00:00</t>
+          <t>2026-10-17T08:41:26.441462+00:00</t>
         </is>
       </c>
     </row>
@@ -30703,7 +30703,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.160059+00:00</t>
+          <t>2026-10-17T08:41:26.442440+00:00</t>
         </is>
       </c>
     </row>
@@ -30811,7 +30811,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.160429+00:00</t>
+          <t>2026-10-17T08:41:26.442744+00:00</t>
         </is>
       </c>
     </row>
@@ -30919,7 +30919,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.165936+00:00</t>
+          <t>2026-10-17T08:41:26.447955+00:00</t>
         </is>
       </c>
     </row>
@@ -31019,7 +31019,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.165969+00:00</t>
+          <t>2026-10-17T08:41:26.447997+00:00</t>
         </is>
       </c>
     </row>
@@ -31127,7 +31127,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.166603+00:00</t>
+          <t>2026-10-17T08:41:26.448579+00:00</t>
         </is>
       </c>
     </row>
@@ -31235,7 +31235,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.167125+00:00</t>
+          <t>2026-10-17T08:41:26.449417+00:00</t>
         </is>
       </c>
     </row>
@@ -31343,7 +31343,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.168258+00:00</t>
+          <t>2026-10-17T08:41:26.450583+00:00</t>
         </is>
       </c>
     </row>
@@ -31451,7 +31451,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.171604+00:00</t>
+          <t>2026-10-17T08:41:26.453562+00:00</t>
         </is>
       </c>
     </row>
@@ -31559,7 +31559,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.171873+00:00</t>
+          <t>2026-10-17T08:41:26.453806+00:00</t>
         </is>
       </c>
     </row>
@@ -31667,7 +31667,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.177827+00:00</t>
+          <t>2026-10-17T08:41:26.457976+00:00</t>
         </is>
       </c>
     </row>
@@ -31775,7 +31775,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.178794+00:00</t>
+          <t>2026-10-17T08:41:26.458752+00:00</t>
         </is>
       </c>
     </row>
@@ -31883,7 +31883,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.181058+00:00</t>
+          <t>2026-10-17T08:41:26.461083+00:00</t>
         </is>
       </c>
     </row>
@@ -31991,7 +31991,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.182976+00:00</t>
+          <t>2026-10-17T08:41:26.463378+00:00</t>
         </is>
       </c>
     </row>
@@ -32091,7 +32091,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.183000+00:00</t>
+          <t>2026-10-17T08:41:26.463415+00:00</t>
         </is>
       </c>
     </row>
@@ -32199,7 +32199,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.185032+00:00</t>
+          <t>2026-10-17T08:41:26.465152+00:00</t>
         </is>
       </c>
     </row>
@@ -32307,7 +32307,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.187465+00:00</t>
+          <t>2026-10-17T08:41:26.467911+00:00</t>
         </is>
       </c>
     </row>
@@ -32415,7 +32415,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.196702+00:00</t>
+          <t>2026-10-17T08:41:26.475797+00:00</t>
         </is>
       </c>
     </row>
@@ -32523,7 +32523,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.198462+00:00</t>
+          <t>2026-10-17T08:41:26.477151+00:00</t>
         </is>
       </c>
     </row>
@@ -32631,7 +32631,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.198639+00:00</t>
+          <t>2026-10-17T08:41:26.477342+00:00</t>
         </is>
       </c>
     </row>
@@ -32731,7 +32731,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.198655+00:00</t>
+          <t>2026-10-17T08:41:26.477358+00:00</t>
         </is>
       </c>
     </row>
@@ -32839,7 +32839,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.204636+00:00</t>
+          <t>2026-10-17T08:41:26.482258+00:00</t>
         </is>
       </c>
     </row>
@@ -32943,7 +32943,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.205046+00:00</t>
+          <t>2026-10-17T08:41:26.482661+00:00</t>
         </is>
       </c>
     </row>
@@ -33047,7 +33047,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.205497+00:00</t>
+          <t>2026-10-17T08:41:26.483085+00:00</t>
         </is>
       </c>
     </row>
@@ -33151,7 +33151,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.205940+00:00</t>
+          <t>2026-10-17T08:41:26.483530+00:00</t>
         </is>
       </c>
     </row>
@@ -33255,7 +33255,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.206739+00:00</t>
+          <t>2026-10-17T08:41:26.484216+00:00</t>
         </is>
       </c>
     </row>
@@ -33359,7 +33359,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.208101+00:00</t>
+          <t>2026-10-17T08:41:26.485608+00:00</t>
         </is>
       </c>
     </row>
@@ -33463,7 +33463,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.208918+00:00</t>
+          <t>2026-10-17T08:41:26.486423+00:00</t>
         </is>
       </c>
     </row>
@@ -33567,7 +33567,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.209217+00:00</t>
+          <t>2026-10-17T08:41:26.486729+00:00</t>
         </is>
       </c>
     </row>
@@ -33675,13 +33675,13 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.209977+00:00</t>
+          <t>2026-10-17T08:41:26.487747+00:00</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -33775,7 +33775,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.210001+00:00</t>
+          <t>2026-10-17T08:41:26.487778+00:00</t>
         </is>
       </c>
     </row>
@@ -33883,7 +33883,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.210062+00:00</t>
+          <t>2026-10-17T08:41:26.487838+00:00</t>
         </is>
       </c>
     </row>
@@ -33991,7 +33991,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.210327+00:00</t>
+          <t>2026-10-17T08:41:26.488055+00:00</t>
         </is>
       </c>
     </row>
@@ -34099,7 +34099,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.210543+00:00</t>
+          <t>2026-10-17T08:41:26.488170+00:00</t>
         </is>
       </c>
     </row>
@@ -34211,7 +34211,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.210684+00:00</t>
+          <t>2026-10-17T08:41:26.488285+00:00</t>
         </is>
       </c>
     </row>
@@ -34319,7 +34319,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.211058+00:00</t>
+          <t>2026-10-17T08:41:26.488690+00:00</t>
         </is>
       </c>
     </row>
@@ -34427,7 +34427,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.211246+00:00</t>
+          <t>2026-10-17T08:41:26.488874+00:00</t>
         </is>
       </c>
     </row>
@@ -34539,7 +34539,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.211380+00:00</t>
+          <t>2026-10-17T08:41:26.488922+00:00</t>
         </is>
       </c>
     </row>
@@ -34651,7 +34651,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.211458+00:00</t>
+          <t>2026-10-17T08:41:26.488979+00:00</t>
         </is>
       </c>
     </row>
@@ -34763,7 +34763,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.211607+00:00</t>
+          <t>2026-10-17T08:41:26.489115+00:00</t>
         </is>
       </c>
     </row>
@@ -34875,7 +34875,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.211653+00:00</t>
+          <t>2026-10-17T08:41:26.489159+00:00</t>
         </is>
       </c>
     </row>
@@ -34983,7 +34983,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.212108+00:00</t>
+          <t>2026-10-17T08:41:26.489642+00:00</t>
         </is>
       </c>
     </row>
@@ -35091,7 +35091,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.212161+00:00</t>
+          <t>2026-10-17T08:41:26.489690+00:00</t>
         </is>
       </c>
     </row>
@@ -35191,7 +35191,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.212171+00:00</t>
+          <t>2026-10-17T08:41:26.489700+00:00</t>
         </is>
       </c>
     </row>
@@ -35227,13 +35227,21 @@
           <t>papers/R07238/supplementary/f346f9bdcc96_mmc2.zip</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>original_files/supplementary/R07238/mmc2.zip</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-supplements/R07238/official/mmc2.zip</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/supplementary/R07238/mmc2.zip</t>
+        </is>
+      </c>
       <c r="K104" t="inlineStr">
         <is>
           <t>zip</t>
@@ -35249,12 +35257,12 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
@@ -35291,7 +35299,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.212176+00:00</t>
+          <t>2026-10-17T08:41:26.499634+00:00</t>
         </is>
       </c>
     </row>
@@ -35395,7 +35403,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.212180+00:00</t>
+          <t>2026-10-17T08:41:26.499697+00:00</t>
         </is>
       </c>
     </row>
@@ -35495,7 +35503,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.212184+00:00</t>
+          <t>2026-10-17T08:41:26.499702+00:00</t>
         </is>
       </c>
     </row>
@@ -35603,7 +35611,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.212422+00:00</t>
+          <t>2026-10-17T08:41:26.499961+00:00</t>
         </is>
       </c>
     </row>
@@ -35711,7 +35719,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213837+00:00</t>
+          <t>2026-10-17T08:41:26.501055+00:00</t>
         </is>
       </c>
     </row>
@@ -35805,7 +35813,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213865+00:00</t>
+          <t>2026-10-17T08:41:26.501080+00:00</t>
         </is>
       </c>
     </row>
@@ -35899,7 +35907,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213870+00:00</t>
+          <t>2026-10-17T08:41:26.501084+00:00</t>
         </is>
       </c>
     </row>
@@ -35993,7 +36001,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213873+00:00</t>
+          <t>2026-10-17T08:41:26.501087+00:00</t>
         </is>
       </c>
     </row>
@@ -36087,7 +36095,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213876+00:00</t>
+          <t>2026-10-17T08:41:26.501090+00:00</t>
         </is>
       </c>
     </row>
@@ -36181,7 +36189,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213880+00:00</t>
+          <t>2026-10-17T08:41:26.501092+00:00</t>
         </is>
       </c>
     </row>
@@ -36275,7 +36283,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213884+00:00</t>
+          <t>2026-10-17T08:41:26.501095+00:00</t>
         </is>
       </c>
     </row>
@@ -36369,7 +36377,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213887+00:00</t>
+          <t>2026-10-17T08:41:26.501097+00:00</t>
         </is>
       </c>
     </row>
@@ -36463,7 +36471,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213891+00:00</t>
+          <t>2026-10-17T08:41:26.501100+00:00</t>
         </is>
       </c>
     </row>
@@ -36557,7 +36565,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213895+00:00</t>
+          <t>2026-10-17T08:41:26.501103+00:00</t>
         </is>
       </c>
     </row>
@@ -36651,7 +36659,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213898+00:00</t>
+          <t>2026-10-17T08:41:26.501106+00:00</t>
         </is>
       </c>
     </row>
@@ -36745,7 +36753,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213901+00:00</t>
+          <t>2026-10-17T08:41:26.501108+00:00</t>
         </is>
       </c>
     </row>
@@ -36839,7 +36847,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213905+00:00</t>
+          <t>2026-10-17T08:41:26.501111+00:00</t>
         </is>
       </c>
     </row>
@@ -36933,7 +36941,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213908+00:00</t>
+          <t>2026-10-17T08:41:26.501113+00:00</t>
         </is>
       </c>
     </row>
@@ -37027,7 +37035,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213911+00:00</t>
+          <t>2026-10-17T08:41:26.501117+00:00</t>
         </is>
       </c>
     </row>
@@ -37121,7 +37129,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213914+00:00</t>
+          <t>2026-10-17T08:41:26.501120+00:00</t>
         </is>
       </c>
     </row>
@@ -37215,7 +37223,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213918+00:00</t>
+          <t>2026-10-17T08:41:26.501123+00:00</t>
         </is>
       </c>
     </row>
@@ -37309,7 +37317,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213921+00:00</t>
+          <t>2026-10-17T08:41:26.501132+00:00</t>
         </is>
       </c>
     </row>
@@ -37403,7 +37411,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213924+00:00</t>
+          <t>2026-10-17T08:41:26.501137+00:00</t>
         </is>
       </c>
     </row>
@@ -37497,7 +37505,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213927+00:00</t>
+          <t>2026-10-17T08:41:26.501140+00:00</t>
         </is>
       </c>
     </row>
@@ -37591,7 +37599,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213929+00:00</t>
+          <t>2026-10-17T08:41:26.501142+00:00</t>
         </is>
       </c>
     </row>
@@ -37685,7 +37693,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213933+00:00</t>
+          <t>2026-10-17T08:41:26.501145+00:00</t>
         </is>
       </c>
     </row>
@@ -37779,7 +37787,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213936+00:00</t>
+          <t>2026-10-17T08:41:26.501148+00:00</t>
         </is>
       </c>
     </row>
@@ -37873,7 +37881,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213939+00:00</t>
+          <t>2026-10-17T08:41:26.501151+00:00</t>
         </is>
       </c>
     </row>
@@ -37967,7 +37975,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213943+00:00</t>
+          <t>2026-10-17T08:41:26.501154+00:00</t>
         </is>
       </c>
     </row>
@@ -38061,7 +38069,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213946+00:00</t>
+          <t>2026-10-17T08:41:26.501157+00:00</t>
         </is>
       </c>
     </row>
@@ -38155,7 +38163,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213949+00:00</t>
+          <t>2026-10-17T08:41:26.501159+00:00</t>
         </is>
       </c>
     </row>
@@ -38249,7 +38257,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213952+00:00</t>
+          <t>2026-10-17T08:41:26.501162+00:00</t>
         </is>
       </c>
     </row>
@@ -38285,13 +38293,21 @@
           <t>papers/R11596/main/0b2e2d98dffd_R11596_2025_Facultative_anaerobic_bacteria_enable_syntrophic_fatty_acids_degradation_under_0b2e2d98dffd.pdf</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R11596_2025_Facultative_anaerobic_bacteria_enable_syntrophic_fatty_acids_degradation_under_0b2e2d98dffd.pdf</t>
+        </is>
+      </c>
       <c r="I136" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-current-run/candidates/R11596_2025_Facultative_anaerobic_bacteria_enable_syntrophic_fatty_acids_degradation_under_0b2e2d98dffd.pdf</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R11596_2025_Facultative_anaerobic_bacteria_enable_syntrophic_fatty_acids_degradation_under_0b2e2d98dffd.pdf</t>
+        </is>
+      </c>
       <c r="K136" t="inlineStr">
         <is>
           <t>pdf</t>
@@ -38307,12 +38323,12 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
@@ -38349,7 +38365,1095 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T08:38:06.213955+00:00</t>
+          <t>2026-10-17T08:41:26.502323+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="b">
+        <v>1</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>R13955</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>R13955.main.82d3dd4c7af3e63a</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E137" t="b">
+        <v>0</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion_7549e1025985.pdf</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion_7549e1025985.pdf</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion_7549e1025985.pdf</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L137" t="n">
+        <v>14662119</v>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>82d3dd4c7af3e63a708ab83da8c0b4011affe749fea236491c93f91ec4cd59c9</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr"/>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>University-published doctoral thesis / publisher PDF (repository cover explicitly states Version of Record)</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr"/>
+      <c r="U137" t="inlineStr"/>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W137" t="inlineStr"/>
+      <c r="X137" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512014+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="b">
+        <v>1</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>R02274</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>R02274.main.4c7da8384f1f6e3d</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E138" t="b">
+        <v>0</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L138" t="n">
+        <v>471480</v>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>4c7da8384f1f6e3d8bd2681eab23bdb95e3057009cf4c7ec7aacc7cdb9eaf43d</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr"/>
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>4c7da8384f1f6e3d8bd2681eab23bdb95e3057009cf4c7ec7aacc7cdb9eaf43d</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr"/>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W138" t="inlineStr"/>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512105+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="b">
+        <v>0</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>R10086</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>R10086.main.84777bfb7a2cd42f</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E139" t="b">
+        <v>0</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L139" t="n">
+        <v>984310</v>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr"/>
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr"/>
+      <c r="V139" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W139" t="inlineStr"/>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512113+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="b">
+        <v>1</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>R03477</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>R03477.main.79583f4a64fb2fbb</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E140" t="b">
+        <v>0</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>R03477_2017_Pretreatment_methods_of_lignocellulosic_biomass_for_anaerobic_digestion.pdf</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R03477_2017_Pretreatment_methods_of_lignocellulosic_biomass_for_anaerobic_digestion.pdf</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L140" t="n">
+        <v>1714874</v>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>79583f4a64fb2fbb4a1f4f471fe6001b159213acb1f3bbd19d6dc0be5c714fa5</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1186/s13568-017-0375-4.pdf</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr"/>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>79583f4a64fb2fbb4a1f4f471fe6001b159213acb1f3bbd19d6dc0be5c714fa5</t>
+        </is>
+      </c>
+      <c r="U140" t="inlineStr"/>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W140" t="inlineStr"/>
+      <c r="X140" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512116+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="b">
+        <v>1</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>R09804</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>R09804.main.b3cc83d613ad3c36</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E141" t="b">
+        <v>0</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>R09804_2024_Anaerobic_digestion_of_process_water_from_hydrothermal_treatment_processes.pdf</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R09804_2024_Anaerobic_digestion_of_process_water_from_hydrothermal_treatment_processes.pdf</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L141" t="n">
+        <v>5135812</v>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>b3cc83d613ad3c36f93b78eace000ebc5a603966523ee71c2e6a0bd85a8ede3e</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1186/s40643-024-00756-6.pdf</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>b3cc83d613ad3c36f93b78eace000ebc5a603966523ee71c2e6a0bd85a8ede3e</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr"/>
+      <c r="V141" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W141" t="inlineStr"/>
+      <c r="X141" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512119+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="b">
+        <v>1</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>R11844</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>R11844.main.c41816bf825167dc</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E142" t="b">
+        <v>0</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>R11844_2025_Micro-aeration_for_improving_anaerobic_treatment_and_biogas_production_from.pdf</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R11844_2025_Micro-aeration_for_improving_anaerobic_treatment_and_biogas_production_from.pdf</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L142" t="n">
+        <v>1333380</v>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>c41816bf825167dcb78ff5eb81c8d0dab0d8d8110cd2a23a04cd1109acb34919</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1007/s00253-025-13519-w.pdf</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>c41816bf825167dcb78ff5eb81c8d0dab0d8d8110cd2a23a04cd1109acb34919</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr"/>
+      <c r="V142" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W142" t="inlineStr"/>
+      <c r="X142" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512122+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="b">
+        <v>1</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>R03155</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>R03155.main.2875ce0c137df622</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E143" t="b">
+        <v>0</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L143" t="n">
+        <v>5745828</v>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>学位/机构存档原稿</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr"/>
+      <c r="V143" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W143" t="inlineStr"/>
+      <c r="X143" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512126+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="b">
+        <v>1</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>R05213</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>R05213.main.bcab84a15ce93062</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E144" t="b">
+        <v>0</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>R05213_2019_The_use_of_lytic_polysaccharide_monooxygenases_in_anaerobic_digestion.pdf</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R05213_2019_The_use_of_lytic_polysaccharide_monooxygenases_in_anaerobic_digestion.pdf</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L144" t="n">
+        <v>1022660</v>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr"/>
+      <c r="V144" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W144" t="inlineStr"/>
+      <c r="X144" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512129+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="b">
+        <v>1</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>R06036</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>R06036.main.0bdc7b19fdb70091</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E145" t="b">
+        <v>0</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L145" t="n">
+        <v>927168</v>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr"/>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr"/>
+      <c r="V145" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W145" t="inlineStr"/>
+      <c r="X145" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512132+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="b">
+        <v>1</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>R09240</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>R09240.main.da8dbeb874b19b59</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E146" t="b">
+        <v>0</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L146" t="n">
+        <v>1315227</v>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>da8dbeb874b19b59dbea53c11766a209aaa0b0bc319e2128c94340ae78cecfaf</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>https://technology.matthey.com/docserver/fulltext/jmtr/67/4/Zimmerman_16a_Imp.pdf?expires=1791804248&amp;id=id&amp;accname=guest&amp;checksum=934385598F9DDA2349B917F1B50C4858</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr"/>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>da8dbeb874b19b59dbea53c11766a209aaa0b0bc319e2128c94340ae78cecfaf</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr"/>
+      <c r="V146" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W146" t="inlineStr"/>
+      <c r="X146" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512135+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="b">
+        <v>1</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>R13899</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>R13899.main.19143e56fa77ce99</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E147" t="b">
+        <v>0</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L147" t="n">
+        <v>479092</v>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr"/>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>出版版本（原页出版信息）</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr"/>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W147" t="inlineStr"/>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512149+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="b">
+        <v>0</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>R13955</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>R13955.main.6714f79deccd703d</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E148" t="b">
+        <v>0</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>/workspace/library-files/ad-oxygen-fulltexts/R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L148" t="n">
+        <v>14662119</v>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>historical_acquired_current_original_not_restored</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>historical_only_original_missing</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr"/>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>学位/机构存档原稿</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>Historical record; source rights not reassessed</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr"/>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>historical_only_current_original_missing</t>
+        </is>
+      </c>
+      <c r="W148" t="inlineStr"/>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>2026-10-17T08:41:26.512152+00:00</t>
         </is>
       </c>
     </row>
@@ -38364,7 +39468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38697,21 +39801,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>R07238.supplementary.f346f9bdcc964013</t>
+          <t>R07238.derived.49b84e369d4bb31b</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>supplementary</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>f346f9bdcc964013ecb7c4282d6b30f1ab334e035d98adcc653de1447fbe9a9a</t>
+          <t>49b84e369d4bb31b4ebdcd25265be3174105c3433e6fbb865f34a445775516a1</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>14286928</v>
+        <v>34855493</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -38720,7 +39824,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>mmc2.zip</t>
+          <t>g a.skp</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -38732,35 +39836,35 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R08646</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>R07238.derived.49b84e369d4bb31b</t>
+          <t>R08646.supplementary.cfda7e29b12b9784</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>supplementary</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>49b84e369d4bb31b4ebdcd25265be3174105c3433e6fbb865f34a445775516a1</t>
+          <t>cfda7e29b12b97846343963f9f3b64e784bc79644fb1ee1ca31170be78d75327</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>34855493</v>
+        <v>42279</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>g a.skp</t>
+          <t>mmc1.docx</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -38772,35 +39876,35 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>R08646</t>
+          <t>R03161</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>R08646.supplementary.cfda7e29b12b9784</t>
+          <t>R03161.evidence_xml.466f3a1e78e8b0f1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>supplementary</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>cfda7e29b12b97846343963f9f3b64e784bc79644fb1ee1ca31170be78d75327</t>
+          <t>466f3a1e78e8b0f148b1f28f97b61f7134c61488c837c5c5a26ef7316cebc1e9</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>42279</v>
+        <v>59018</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/fullTextXML</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>mmc1.docx</t>
+          <t>PMC5627928_fullText.xml</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -38817,30 +39921,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>R03161.evidence_xml.466f3a1e78e8b0f1</t>
+          <t>R03161.transport_archive.0ef4d4796c84feff</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>466f3a1e78e8b0f148b1f28f97b61f7134c61488c837c5c5a26ef7316cebc1e9</t>
+          <t>0ef4d4796c84fefff7b8450bc56400f8c59f4bdcf074fc51404edff5e4e217f6</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>59018</v>
+        <v>726772</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/supplementaryFiles</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>PMC5627928_fullText.xml</t>
+          <t>PMC5627928_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -38852,35 +39956,35 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>R03161</t>
+          <t>R04092</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>R03161.transport_archive.0ef4d4796c84feff</t>
+          <t>R04092.evidence_xml.0fb90085e30680fa</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0ef4d4796c84fefff7b8450bc56400f8c59f4bdcf074fc51404edff5e4e217f6</t>
+          <t>0fb90085e30680fa8a9896b80afb9da4f9466ba0051ea2ffb89a13e06a5013a3</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>726772</v>
+        <v>77995</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6288047/fullTextXML</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>PMC5627928_supplementaryFiles.zip</t>
+          <t>PMC6288047_fullText.xml</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -38892,12 +39996,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>R04092</t>
+          <t>R05839</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>R04092.evidence_xml.0fb90085e30680fa</t>
+          <t>R05839.evidence_xml.18ffd43dee955086</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -38907,20 +40011,20 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0fb90085e30680fa8a9896b80afb9da4f9466ba0051ea2ffb89a13e06a5013a3</t>
+          <t>18ffd43dee955086eae0947027dc85e1d765e181357143650e9fef0b0dfbef74</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>77995</v>
+        <v>75205</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6288047/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC7566014/fullTextXML</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>PMC6288047_fullText.xml</t>
+          <t>PMC7566014_fullText.xml</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -38932,12 +40036,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>R05839</t>
+          <t>R08877</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>R05839.evidence_xml.18ffd43dee955086</t>
+          <t>R08877.evidence_xml.e8712e4198baab4c</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -38947,20 +40051,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>18ffd43dee955086eae0947027dc85e1d765e181357143650e9fef0b0dfbef74</t>
+          <t>e8712e4198baab4c79ee53c54ea30b4d96721e2d47e08b657a6b19b4bf41891a</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>75205</v>
+        <v>111864</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC7566014/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/fullTextXML</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>PMC7566014_fullText.xml</t>
+          <t>PMC10714394_fullText.xml</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -38977,30 +40081,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R08877.evidence_xml.e8712e4198baab4c</t>
+          <t>R08877.transport_archive.ed8e864a3225e9c4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>e8712e4198baab4c79ee53c54ea30b4d96721e2d47e08b657a6b19b4bf41891a</t>
+          <t>ed8e864a3225e9c4cecf84e5f4670c985de4c6d453d0b7b459ad5870e6627f97</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>111864</v>
+        <v>704921</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/supplementaryFiles</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>PMC10714394_fullText.xml</t>
+          <t>PMC10714394_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -39012,35 +40116,35 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>R08877</t>
+          <t>R09236</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R08877.transport_archive.ed8e864a3225e9c4</t>
+          <t>R09236.evidence_xml.72064fe9276d8309</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ed8e864a3225e9c4cecf84e5f4670c985de4c6d453d0b7b459ad5870e6627f97</t>
+          <t>72064fe9276d830984364e82e4567877578408565c650d856c531204a17ded89</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>704921</v>
+        <v>193052</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/fullTextXML</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>PMC10714394_supplementaryFiles.zip</t>
+          <t>PMC10535533_fullText.xml</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -39057,30 +40161,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R09236.evidence_xml.72064fe9276d8309</t>
+          <t>R09236.transport_archive.f3c6856282b7e8d6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>72064fe9276d830984364e82e4567877578408565c650d856c531204a17ded89</t>
+          <t>f3c6856282b7e8d694d35a87eae016d8e66aa902189c7c3311a1153ea24752e0</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>193052</v>
+        <v>483405</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/supplementaryFiles</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>PMC10535533_fullText.xml</t>
+          <t>PMC10535533_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -39092,35 +40196,35 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>R09236</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R09236.transport_archive.f3c6856282b7e8d6</t>
+          <t>R10086.evidence_xml.074f3cb8a39355a5</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>f3c6856282b7e8d694d35a87eae016d8e66aa902189c7c3311a1153ea24752e0</t>
+          <t>074f3cb8a39355a5d7cfb8af0139c674b72aec8e5d08bcd20b8f0e46d0d88fbe</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>483405</v>
+        <v>118002</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/fullTextXML</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>PMC10535533_supplementaryFiles.zip</t>
+          <t>PMC10837232_fullText.xml</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -39137,30 +40241,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R10086.evidence_xml.074f3cb8a39355a5</t>
+          <t>R10086.transport_archive.4d9eddf454b786ed</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>074f3cb8a39355a5d7cfb8af0139c674b72aec8e5d08bcd20b8f0e46d0d88fbe</t>
+          <t>4d9eddf454b786eddece423a320b28d7f96959a935334ddc7c7e2fe32d39bc9b</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>118002</v>
+        <v>641038</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/supplementaryFiles</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>PMC10837232_fullText.xml</t>
+          <t>PMC10837232_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -39172,35 +40276,35 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>R10086</t>
+          <t>R12985</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R10086.transport_archive.4d9eddf454b786ed</t>
+          <t>R12985.evidence_xml.f1a80564a8a1fa4b</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>4d9eddf454b786eddece423a320b28d7f96959a935334ddc7c7e2fe32d39bc9b</t>
+          <t>f1a80564a8a1fa4b638bb6097c75cb3709b4c7487b6c8012474fd4e1865576cc</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>641038</v>
+        <v>173586</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/fullTextXML</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>PMC10837232_supplementaryFiles.zip</t>
+          <t>PMC12937426_fullText.xml</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -39217,30 +40321,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R12985.evidence_xml.f1a80564a8a1fa4b</t>
+          <t>R12985.transport_archive.418d45f1ca296020</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>f1a80564a8a1fa4b638bb6097c75cb3709b4c7487b6c8012474fd4e1865576cc</t>
+          <t>418d45f1ca2960209df0bfc1c3d44069413edc213239570a3d71d08d01f3e3e0</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>173586</v>
+        <v>672244</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/supplementaryFiles</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>PMC12937426_fullText.xml</t>
+          <t>PMC12937426_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -39252,35 +40356,35 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>R12985</t>
+          <t>R05542</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R12985.transport_archive.418d45f1ca296020</t>
+          <t>R05542.evidence_xml.9ee6c9217e7c01e1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>418d45f1ca2960209df0bfc1c3d44069413edc213239570a3d71d08d01f3e3e0</t>
+          <t>9ee6c9217e7c01e1604e3170e0041677e5b9d0f14b59ee1e9717c1082d9d193a</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>672244</v>
+        <v>100215</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC9056904/fullTextXML</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>PMC12937426_supplementaryFiles.zip</t>
+          <t>PMC9056904_fullText.xml</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -39292,12 +40396,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>R05542</t>
+          <t>R06325</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R05542.evidence_xml.9ee6c9217e7c01e1</t>
+          <t>R06325.evidence_xml.645deb707d3790b5</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -39307,20 +40411,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>9ee6c9217e7c01e1604e3170e0041677e5b9d0f14b59ee1e9717c1082d9d193a</t>
+          <t>645deb707d3790b518690b7413885823461bb57a3dfa5bb587202d8f16dda296</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>100215</v>
+        <v>160509</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC9056904/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/fullTextXML</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>PMC9056904_fullText.xml</t>
+          <t>PMC8290346_fullText.xml</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -39337,30 +40441,30 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R06325.evidence_xml.645deb707d3790b5</t>
+          <t>R06325.transport_archive.6eb4ef126661714a</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>645deb707d3790b518690b7413885823461bb57a3dfa5bb587202d8f16dda296</t>
+          <t>6eb4ef126661714ae89bde97acdddac2c2a582864ca26ff9af569cfe609a4226</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>160509</v>
+        <v>1730580</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/supplementaryFiles</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>PMC8290346_fullText.xml</t>
+          <t>PMC8290346_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -39372,35 +40476,35 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R06325</t>
+          <t>R07238</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R06325.transport_archive.6eb4ef126661714a</t>
+          <t>R07238.evidence_xml.6c93b117d7bd5886</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>6eb4ef126661714ae89bde97acdddac2c2a582864ca26ff9af569cfe609a4226</t>
+          <t>6c93b117d7bd588658aabfd8b7ec679110899d8f556eb6b90b071e6057ddd2cd</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1730580</v>
+        <v>151458</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/fullTextXML</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>PMC8290346_supplementaryFiles.zip</t>
+          <t>PMC8044681_fullText.xml</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -39417,30 +40521,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R07238.evidence_xml.6c93b117d7bd5886</t>
+          <t>R07238.transport_archive.3785c23cb2f4ab50</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>6c93b117d7bd588658aabfd8b7ec679110899d8f556eb6b90b071e6057ddd2cd</t>
+          <t>3785c23cb2f4ab50f5b2b5cbb581da63ced9f8d1e69a91e6faca839b6b57587d</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>151458</v>
+        <v>14596266</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>PMC8044681_fullText.xml</t>
+          <t>PMC8044681_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -39452,35 +40556,35 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R03477</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>R07238.transport_archive.3785c23cb2f4ab50</t>
+          <t>R03477.evidence_xml.c127b68ddfdcfec8</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3785c23cb2f4ab50f5b2b5cbb581da63ced9f8d1e69a91e6faca839b6b57587d</t>
+          <t>c127b68ddfdcfec8d98508723d4d7a4b250ec3f82c4c75756cb539406519a8f7</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>14596266</v>
+        <v>121650</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5371168/fullTextXML</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>PMC8044681_supplementaryFiles.zip</t>
+          <t>PMC5371168_fullText.xml</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -39492,12 +40596,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>R03477</t>
+          <t>R08646</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>R03477.evidence_xml.c127b68ddfdcfec8</t>
+          <t>R08646.evidence_xml.c7b723e8020f6582</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -39507,20 +40611,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>c127b68ddfdcfec8d98508723d4d7a4b250ec3f82c4c75756cb539406519a8f7</t>
+          <t>c7b723e8020f65823eaf8b08c6b56c36aab85784bbef3b10c9a85a820b960d3a</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>121650</v>
+        <v>304277</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5371168/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/fullTextXML</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>PMC5371168_fullText.xml</t>
+          <t>PMC10559078_fullText.xml</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -39537,30 +40641,30 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>R08646.evidence_xml.c7b723e8020f6582</t>
+          <t>R08646.transport_archive.ecda9ea461a3deb3</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>c7b723e8020f65823eaf8b08c6b56c36aab85784bbef3b10c9a85a820b960d3a</t>
+          <t>ecda9ea461a3deb361931eb51186e88488c4d6ae284899e1feb1d611de42550a</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>304277</v>
+        <v>1539133</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>PMC10559078_fullText.xml</t>
+          <t>PMC10559078_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -39572,35 +40676,35 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>R08646</t>
+          <t>R09804</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>R08646.transport_archive.ecda9ea461a3deb3</t>
+          <t>R09804.evidence_xml.2ca7af24c486ae9e</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ecda9ea461a3deb361931eb51186e88488c4d6ae284899e1feb1d611de42550a</t>
+          <t>2ca7af24c486ae9eb9c65682356964011c985b22a4a36f4ee07ea3a705c38951</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1539133</v>
+        <v>211630</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC11076452/fullTextXML</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>PMC10559078_supplementaryFiles.zip</t>
+          <t>PMC11076452_fullText.xml</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -39612,12 +40716,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R09804</t>
+          <t>R11503</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>R09804.evidence_xml.2ca7af24c486ae9e</t>
+          <t>R11503.evidence_xml.4002d57be59c215c</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -39627,20 +40731,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2ca7af24c486ae9eb9c65682356964011c985b22a4a36f4ee07ea3a705c38951</t>
+          <t>4002d57be59c215cea8477a4b667f20f9ffb09680e70af377a81ffae74b99801</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>211630</v>
+        <v>258637</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC11076452/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12561102/fullTextXML</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>PMC11076452_fullText.xml</t>
+          <t>PMC12561102_fullText.xml</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -39652,12 +40756,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R11503</t>
+          <t>R11844</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>R11503.evidence_xml.4002d57be59c215c</t>
+          <t>R11844.evidence_xml.9c39d5f64ac01253</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -39667,20 +40771,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4002d57be59c215cea8477a4b667f20f9ffb09680e70af377a81ffae74b99801</t>
+          <t>9c39d5f64ac01253c8bb4866ce3974997765b2d47e37641f3717e99e0d7f1f61</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>258637</v>
+        <v>256247</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12561102/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/fullTextXML</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>PMC12561102_fullText.xml</t>
+          <t>PMC12125087_fullText.xml</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -39697,30 +40801,30 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>R11844.evidence_xml.9c39d5f64ac01253</t>
+          <t>R11844.transport_archive.60ef29cf0a557bf4</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>9c39d5f64ac01253c8bb4866ce3974997765b2d47e37641f3717e99e0d7f1f61</t>
+          <t>60ef29cf0a557bf44838f4a3f45e2dbf1b1a2001547f5c0b976b48cc64c1b6d9</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>256247</v>
+        <v>521862</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/supplementaryFiles</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>PMC12125087_fullText.xml</t>
+          <t>PMC12125087_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -39732,35 +40836,35 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R11844</t>
+          <t>R05213</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>R11844.transport_archive.60ef29cf0a557bf4</t>
+          <t>R05213.evidence_xml.17894ab410001846</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>60ef29cf0a557bf44838f4a3f45e2dbf1b1a2001547f5c0b976b48cc64c1b6d9</t>
+          <t>17894ab41000184655d2f9f9a0daa796981ab3658678c6b123eb9f3deb1bf45a</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>521862</v>
+        <v>130954</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/fullTextXML</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>PMC12125087_supplementaryFiles.zip</t>
+          <t>PMC6858683_fullText.xml</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -39777,30 +40881,30 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>R05213.evidence_xml.17894ab410001846</t>
+          <t>R05213.transport_archive.c61c88cf9fd489be</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>17894ab41000184655d2f9f9a0daa796981ab3658678c6b123eb9f3deb1bf45a</t>
+          <t>c61c88cf9fd489beab88c1b72bbfe5f13167f32c984b6dba6e48ba97c6136b7b</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>130954</v>
+        <v>1960371</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/fullTextXML</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/supplementaryFiles</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>PMC6858683_fullText.xml</t>
+          <t>PMC6858683_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -39812,35 +40916,35 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R05213</t>
+          <t>R09585</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>R05213.transport_archive.c61c88cf9fd489be</t>
+          <t>R09585.evidence_xml.a3430f38fa1652de</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>evidence_xml</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>c61c88cf9fd489beab88c1b72bbfe5f13167f32c984b6dba6e48ba97c6136b7b</t>
+          <t>a3430f38fa1652de3145ffc47f0da514ee41e12ef8e95acc30330d6b3a01efd2</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1960371</v>
+        <v>100534</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10609292/fullTextXML</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>PMC6858683_supplementaryFiles.zip</t>
+          <t>PMC10609292_fullText.xml</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -39852,35 +40956,31 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R09585</t>
+          <t>R02274</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>R09585.evidence_xml.a3430f38fa1652de</t>
+          <t>R02274.main.4c7da8384f1f6e3d</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>a3430f38fa1652de3145ffc47f0da514ee41e12ef8e95acc30330d6b3a01efd2</t>
+          <t>4c7da8384f1f6e3d8bd2681eab23bdb95e3057009cf4c7ec7aacc7cdb9eaf43d</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>100534</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10609292/fullTextXML</t>
-        </is>
-      </c>
+        <v>471480</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>PMC10609292_fullText.xml</t>
+          <t>R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -39892,12 +40992,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R11596</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>R11596.main.0b2e2d98dffd5449</t>
+          <t>R10086.main.84777bfb7a2cd42f</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -39907,23 +41007,371 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>0b2e2d98dffd544958b06cc2229d310e4b7d529bd3914c47f20d6a66789a28be</t>
+          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1659399</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>https://repositorium.uminho.pt/server/api/core/bitstreams/7262c516-6b14-4001-a173-517d1187c8d9/content</t>
-        </is>
-      </c>
+        <v>984310</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>R11596_2025_Facultative_anaerobic_bacteria_enable_syntrophic_fatty_acids_degradation_under_0b2e2d98dffd.pdf</t>
+          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>R03477</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>R03477.main.79583f4a64fb2fbb</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>79583f4a64fb2fbb4a1f4f471fe6001b159213acb1f3bbd19d6dc0be5c714fa5</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1714874</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1186/s13568-017-0375-4.pdf</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>R03477_2017_Pretreatment_methods_of_lignocellulosic_biomass_for_anaerobic_digestion.pdf</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>R09804</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>R09804.main.b3cc83d613ad3c36</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>b3cc83d613ad3c36f93b78eace000ebc5a603966523ee71c2e6a0bd85a8ede3e</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>5135812</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1186/s40643-024-00756-6.pdf</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>R09804_2024_Anaerobic_digestion_of_process_water_from_hydrothermal_treatment_processes.pdf</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>R11844</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>R11844.main.c41816bf825167dc</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>c41816bf825167dcb78ff5eb81c8d0dab0d8d8110cd2a23a04cd1109acb34919</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1333380</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1007/s00253-025-13519-w.pdf</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>R11844_2025_Micro-aeration_for_improving_anaerobic_treatment_and_biogas_production_from.pdf</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>R03155</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>R03155.main.2875ce0c137df622</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>5745828</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>R05213</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>R05213.main.bcab84a15ce93062</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1022660</v>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>R05213_2019_The_use_of_lytic_polysaccharide_monooxygenases_in_anaerobic_digestion.pdf</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>R06036</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>R06036.main.0bdc7b19fdb70091</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>927168</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>R09240</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>R09240.main.da8dbeb874b19b59</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>da8dbeb874b19b59dbea53c11766a209aaa0b0bc319e2128c94340ae78cecfaf</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1315227</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://technology.matthey.com/docserver/fulltext/jmtr/67/4/Zimmerman_16a_Imp.pdf?expires=1791804248&amp;id=id&amp;accname=guest&amp;checksum=934385598F9DDA2349B917F1B50C4858</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>R13899</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>R13899.main.19143e56fa77ce99</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>479092</v>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>历史已获取，当前原件未恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>R13955</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>R13955.main.6714f79deccd703d</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>14662119</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>历史已获取，当前原件未恢复</t>
         </is>

</xml_diff>

<commit_message>
Finish historical recovery pass and persist all acquired originals
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.904273+00:00</t>
+          <t>2026-10-17T08:48:34.414866+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.905189+00:00</t>
+          <t>2026-10-17T08:48:34.415826+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.905206+00:00</t>
+          <t>2026-10-17T08:48:34.415848+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.905435+00:00</t>
+          <t>2026-10-17T08:48:34.416068+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.906557+00:00</t>
+          <t>2026-10-17T08:48:34.417185+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.907155+00:00</t>
+          <t>2026-10-17T08:48:34.417701+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.912766+00:00</t>
+          <t>2026-10-17T08:48:34.423229+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.915129+00:00</t>
+          <t>2026-10-17T08:48:34.425700+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.916063+00:00</t>
+          <t>2026-10-17T08:48:34.426638+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.916401+00:00</t>
+          <t>2026-10-17T08:48:34.426969+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.917160+00:00</t>
+          <t>2026-10-17T08:48:34.427726+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.917831+00:00</t>
+          <t>2026-10-17T08:48:34.428415+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.918829+00:00</t>
+          <t>2026-10-17T08:48:34.429377+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.919137+00:00</t>
+          <t>2026-10-17T08:48:34.429633+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.920004+00:00</t>
+          <t>2026-10-17T08:48:34.430500+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.927635+00:00</t>
+          <t>2026-10-17T08:48:34.438320+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.928369+00:00</t>
+          <t>2026-10-17T08:48:34.439036+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.929842+00:00</t>
+          <t>2026-10-17T08:48:34.440353+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.932436+00:00</t>
+          <t>2026-10-17T08:48:34.442916+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.933531+00:00</t>
+          <t>2026-10-17T08:48:34.444073+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.934703+00:00</t>
+          <t>2026-10-17T08:48:34.445378+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.939437+00:00</t>
+          <t>2026-10-17T08:48:34.449469+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.941604+00:00</t>
+          <t>2026-10-17T08:48:34.451649+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.943391+00:00</t>
+          <t>2026-10-17T08:48:34.453524+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.944061+00:00</t>
+          <t>2026-10-17T08:48:34.454218+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.944434+00:00</t>
+          <t>2026-10-17T08:48:34.454627+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.946420+00:00</t>
+          <t>2026-10-17T08:48:34.456619+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.947791+00:00</t>
+          <t>2026-10-17T08:48:34.457877+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.949851+00:00</t>
+          <t>2026-10-17T08:48:34.460092+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.951799+00:00</t>
+          <t>2026-10-17T08:48:34.462188+00:00</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.952358+00:00</t>
+          <t>2026-10-17T08:48:34.462778+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.952900+00:00</t>
+          <t>2026-10-17T08:48:34.463360+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.954641+00:00</t>
+          <t>2026-10-17T08:48:34.464957+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.957651+00:00</t>
+          <t>2026-10-17T08:48:34.467972+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.959806+00:00</t>
+          <t>2026-10-17T08:48:34.470166+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.960997+00:00</t>
+          <t>2026-10-17T08:48:34.471690+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.963934+00:00</t>
+          <t>2026-10-17T08:48:34.474676+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.964748+00:00</t>
+          <t>2026-10-17T08:48:34.475380+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.966479+00:00</t>
+          <t>2026-10-17T08:48:34.477020+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.966802+00:00</t>
+          <t>2026-10-17T08:48:34.477279+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.968728+00:00</t>
+          <t>2026-10-17T08:48:34.479228+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.971648+00:00</t>
+          <t>2026-10-17T08:48:34.482113+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.972944+00:00</t>
+          <t>2026-10-17T08:48:34.483686+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.973514+00:00</t>
+          <t>2026-10-17T08:48:34.484226+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.976168+00:00</t>
+          <t>2026-10-17T08:48:34.486927+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.977366+00:00</t>
+          <t>2026-10-17T08:48:34.488074+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.981029+00:00</t>
+          <t>2026-10-17T08:48:34.491491+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.982778+00:00</t>
+          <t>2026-10-17T08:48:34.493124+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.984771+00:00</t>
+          <t>2026-10-17T08:48:34.494971+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.985843+00:00</t>
+          <t>2026-10-17T08:48:34.496068+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.986284+00:00</t>
+          <t>2026-10-17T08:48:34.496533+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.986664+00:00</t>
+          <t>2026-10-17T08:48:34.498029+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.988158+00:00</t>
+          <t>2026-10-17T08:48:34.499591+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.989444+00:00</t>
+          <t>2026-10-17T08:48:34.500972+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.990928+00:00</t>
+          <t>2026-10-17T08:48:34.502676+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.991256+00:00</t>
+          <t>2026-10-17T08:48:34.503027+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.992500+00:00</t>
+          <t>2026-10-17T08:48:34.504169+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.993959+00:00</t>
+          <t>2026-10-17T08:48:34.505592+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.994589+00:00</t>
+          <t>2026-10-17T08:48:34.506246+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.995547+00:00</t>
+          <t>2026-10-17T08:48:34.507262+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:55.995849+00:00</t>
+          <t>2026-10-17T08:48:34.507614+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.001013+00:00</t>
+          <t>2026-10-17T08:48:34.512772+00:00</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.001406+00:00</t>
+          <t>2026-10-17T08:48:34.513182+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.001994+00:00</t>
+          <t>2026-10-17T08:48:34.513808+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.002443+00:00</t>
+          <t>2026-10-17T08:48:34.514255+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.003493+00:00</t>
+          <t>2026-10-17T08:48:34.515453+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.006401+00:00</t>
+          <t>2026-10-17T08:48:34.518479+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.006633+00:00</t>
+          <t>2026-10-17T08:48:34.518729+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.010697+00:00</t>
+          <t>2026-10-17T08:48:34.523058+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.011473+00:00</t>
+          <t>2026-10-17T08:48:34.523855+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.013531+00:00</t>
+          <t>2026-10-17T08:48:34.526042+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.015354+00:00</t>
+          <t>2026-10-17T08:48:34.528362+00:00</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.016245+00:00</t>
+          <t>2026-10-17T08:48:34.529282+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.017666+00:00</t>
+          <t>2026-10-17T08:48:34.530725+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.019949+00:00</t>
+          <t>2026-10-17T08:48:34.533011+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.027962+00:00</t>
+          <t>2026-10-17T08:48:34.540949+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.029286+00:00</t>
+          <t>2026-10-17T08:48:34.542264+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.029496+00:00</t>
+          <t>2026-10-17T08:48:34.542426+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.029513+00:00</t>
+          <t>2026-10-17T08:48:34.542439+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.034484+00:00</t>
+          <t>2026-10-17T08:48:34.547286+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.035055+00:00</t>
+          <t>2026-10-17T08:48:34.547660+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.035512+00:00</t>
+          <t>2026-10-17T08:48:34.548019+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.035944+00:00</t>
+          <t>2026-10-17T08:48:34.548447+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.038194+00:00</t>
+          <t>2026-10-17T08:48:34.549132+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.039618+00:00</t>
+          <t>2026-10-17T08:48:34.550533+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.040679+00:00</t>
+          <t>2026-10-17T08:48:34.551393+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.041019+00:00</t>
+          <t>2026-10-17T08:48:34.551702+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.042397+00:00</t>
+          <t>2026-10-17T08:48:34.552347+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.042428+00:00</t>
+          <t>2026-10-17T08:48:34.552361+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.042502+00:00</t>
+          <t>2026-10-17T08:48:34.552413+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.042728+00:00</t>
+          <t>2026-10-17T08:48:34.552629+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.042851+00:00</t>
+          <t>2026-10-17T08:48:34.552744+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.043169+00:00</t>
+          <t>2026-10-17T08:48:34.552857+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.043604+00:00</t>
+          <t>2026-10-17T08:48:34.553234+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.043810+00:00</t>
+          <t>2026-10-17T08:48:34.553446+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.043867+00:00</t>
+          <t>2026-10-17T08:48:34.553532+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.043928+00:00</t>
+          <t>2026-10-17T08:48:34.553595+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.044068+00:00</t>
+          <t>2026-10-17T08:48:34.553741+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.044115+00:00</t>
+          <t>2026-10-17T08:48:34.553791+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.044617+00:00</t>
+          <t>2026-10-17T08:48:34.554245+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.044676+00:00</t>
+          <t>2026-10-17T08:48:34.554329+00:00</t>
         </is>
       </c>
     </row>
@@ -35215,7 +35215,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.044687+00:00</t>
+          <t>2026-10-17T08:48:34.554341+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35323,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.058032+00:00</t>
+          <t>2026-10-17T08:48:34.564175+00:00</t>
         </is>
       </c>
     </row>
@@ -35427,7 +35427,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.058127+00:00</t>
+          <t>2026-10-17T08:48:34.564239+00:00</t>
         </is>
       </c>
     </row>
@@ -35535,7 +35535,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.058434+00:00</t>
+          <t>2026-10-17T08:48:34.564367+00:00</t>
         </is>
       </c>
     </row>
@@ -35643,7 +35643,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.058709+00:00</t>
+          <t>2026-10-17T08:48:34.564600+00:00</t>
         </is>
       </c>
     </row>
@@ -35751,7 +35751,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060089+00:00</t>
+          <t>2026-10-17T08:48:34.565688+00:00</t>
         </is>
       </c>
     </row>
@@ -35853,7 +35853,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060207+00:00</t>
+          <t>2026-10-17T08:48:34.565772+00:00</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35947,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060222+00:00</t>
+          <t>2026-10-17T08:48:34.565783+00:00</t>
         </is>
       </c>
     </row>
@@ -36049,7 +36049,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060308+00:00</t>
+          <t>2026-10-17T08:48:34.565861+00:00</t>
         </is>
       </c>
     </row>
@@ -36151,7 +36151,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060430+00:00</t>
+          <t>2026-10-17T08:48:34.565943+00:00</t>
         </is>
       </c>
     </row>
@@ -36253,7 +36253,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060544+00:00</t>
+          <t>2026-10-17T08:48:34.566050+00:00</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36347,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060555+00:00</t>
+          <t>2026-10-17T08:48:34.566061+00:00</t>
         </is>
       </c>
     </row>
@@ -36449,7 +36449,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060706+00:00</t>
+          <t>2026-10-17T08:48:34.566213+00:00</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36543,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060717+00:00</t>
+          <t>2026-10-17T08:48:34.566224+00:00</t>
         </is>
       </c>
     </row>
@@ -36645,7 +36645,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060820+00:00</t>
+          <t>2026-10-17T08:48:34.566346+00:00</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060831+00:00</t>
+          <t>2026-10-17T08:48:34.566358+00:00</t>
         </is>
       </c>
     </row>
@@ -36841,7 +36841,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060968+00:00</t>
+          <t>2026-10-17T08:48:34.566495+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36935,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.060982+00:00</t>
+          <t>2026-10-17T08:48:34.566507+00:00</t>
         </is>
       </c>
     </row>
@@ -37037,7 +37037,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.061074+00:00</t>
+          <t>2026-10-17T08:48:34.566598+00:00</t>
         </is>
       </c>
     </row>
@@ -37139,7 +37139,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.061217+00:00</t>
+          <t>2026-10-17T08:48:34.566735+00:00</t>
         </is>
       </c>
     </row>
@@ -37233,7 +37233,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.061230+00:00</t>
+          <t>2026-10-17T08:48:34.566747+00:00</t>
         </is>
       </c>
     </row>
@@ -37335,7 +37335,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.061444+00:00</t>
+          <t>2026-10-17T08:48:34.566871+00:00</t>
         </is>
       </c>
     </row>
@@ -37429,7 +37429,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.061462+00:00</t>
+          <t>2026-10-17T08:48:34.566882+00:00</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37531,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.061629+00:00</t>
+          <t>2026-10-17T08:48:34.566983+00:00</t>
         </is>
       </c>
     </row>
@@ -37633,7 +37633,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.061873+00:00</t>
+          <t>2026-10-17T08:48:34.567221+00:00</t>
         </is>
       </c>
     </row>
@@ -37727,7 +37727,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.061886+00:00</t>
+          <t>2026-10-17T08:48:34.567233+00:00</t>
         </is>
       </c>
     </row>
@@ -37829,7 +37829,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.062047+00:00</t>
+          <t>2026-10-17T08:48:34.567413+00:00</t>
         </is>
       </c>
     </row>
@@ -37931,7 +37931,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.062307+00:00</t>
+          <t>2026-10-17T08:48:34.567618+00:00</t>
         </is>
       </c>
     </row>
@@ -38033,7 +38033,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.062564+00:00</t>
+          <t>2026-10-17T08:48:34.567809+00:00</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.062577+00:00</t>
+          <t>2026-10-17T08:48:34.567820+00:00</t>
         </is>
       </c>
     </row>
@@ -38229,7 +38229,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.062688+00:00</t>
+          <t>2026-10-17T08:48:34.567928+00:00</t>
         </is>
       </c>
     </row>
@@ -38323,7 +38323,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.062699+00:00</t>
+          <t>2026-10-17T08:48:34.567938+00:00</t>
         </is>
       </c>
     </row>
@@ -38357,13 +38357,21 @@
           <t>papers/R09585/evidence/a3430f38fa16_PMC10609292_fullText.xml</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>original_files/source_evidence/R09585/PMC10609292_fullText.xml</t>
+        </is>
+      </c>
       <c r="I135" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-supplements/R09585/evidence/PMC10609292_fullText.xml</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr"/>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/source_evidence/R09585/PMC10609292_fullText.xml</t>
+        </is>
+      </c>
       <c r="K135" t="inlineStr">
         <is>
           <t>xml</t>
@@ -38379,12 +38387,12 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
@@ -38417,7 +38425,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.062704+00:00</t>
+          <t>2026-10-17T08:48:34.568038+00:00</t>
         </is>
       </c>
     </row>
@@ -38525,7 +38533,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.063910+00:00</t>
+          <t>2026-10-17T08:48:34.569082+00:00</t>
         </is>
       </c>
     </row>
@@ -38617,7 +38625,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075431+00:00</t>
+          <t>2026-10-17T08:48:34.578938+00:00</t>
         </is>
       </c>
     </row>
@@ -38705,7 +38713,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075521+00:00</t>
+          <t>2026-10-17T08:48:34.579000+00:00</t>
         </is>
       </c>
     </row>
@@ -38793,7 +38801,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075529+00:00</t>
+          <t>2026-10-17T08:48:34.579006+00:00</t>
         </is>
       </c>
     </row>
@@ -38885,7 +38893,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075533+00:00</t>
+          <t>2026-10-17T08:48:34.579011+00:00</t>
         </is>
       </c>
     </row>
@@ -38977,7 +38985,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075536+00:00</t>
+          <t>2026-10-17T08:48:34.579014+00:00</t>
         </is>
       </c>
     </row>
@@ -39069,7 +39077,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075540+00:00</t>
+          <t>2026-10-17T08:48:34.579018+00:00</t>
         </is>
       </c>
     </row>
@@ -39161,7 +39169,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075544+00:00</t>
+          <t>2026-10-17T08:48:34.579022+00:00</t>
         </is>
       </c>
     </row>
@@ -39249,7 +39257,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075548+00:00</t>
+          <t>2026-10-17T08:48:34.579025+00:00</t>
         </is>
       </c>
     </row>
@@ -39341,7 +39349,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075552+00:00</t>
+          <t>2026-10-17T08:48:34.579029+00:00</t>
         </is>
       </c>
     </row>
@@ -39433,7 +39441,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075555+00:00</t>
+          <t>2026-10-17T08:48:34.579033+00:00</t>
         </is>
       </c>
     </row>
@@ -39521,7 +39529,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075559+00:00</t>
+          <t>2026-10-17T08:48:34.579036+00:00</t>
         </is>
       </c>
     </row>
@@ -39613,7 +39621,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T08:47:56.075562+00:00</t>
+          <t>2026-10-17T08:48:34.579041+00:00</t>
         </is>
       </c>
     </row>
@@ -39628,7 +39636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40276,35 +40284,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>R09585</t>
+          <t>R02274</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R09585.evidence_xml.a3430f38fa1652de</t>
+          <t>R02274.main.4c7da8384f1f6e3d</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>evidence_xml</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>a3430f38fa1652de3145ffc47f0da514ee41e12ef8e95acc30330d6b3a01efd2</t>
+          <t>4c7da8384f1f6e3d8bd2681eab23bdb95e3057009cf4c7ec7aacc7cdb9eaf43d</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>100534</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10609292/fullTextXML</t>
-        </is>
-      </c>
+        <v>471480</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>PMC10609292_fullText.xml</t>
+          <t>R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -40316,12 +40320,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>R02274</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R02274.main.4c7da8384f1f6e3d</t>
+          <t>R10086.main.84777bfb7a2cd42f</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -40331,16 +40335,16 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4c7da8384f1f6e3d8bd2681eab23bdb95e3057009cf4c7ec7aacc7cdb9eaf43d</t>
+          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>471480</v>
+        <v>984310</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
+          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -40352,12 +40356,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>R10086</t>
+          <t>R03477</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R10086.main.84777bfb7a2cd42f</t>
+          <t>R03477.main.79583f4a64fb2fbb</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -40367,16 +40371,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
+          <t>79583f4a64fb2fbb4a1f4f471fe6001b159213acb1f3bbd19d6dc0be5c714fa5</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>984310</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
+        <v>1714874</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1186/s13568-017-0375-4.pdf</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
+          <t>R03477_2017_Pretreatment_methods_of_lignocellulosic_biomass_for_anaerobic_digestion.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -40388,12 +40396,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>R03477</t>
+          <t>R09804</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R03477.main.79583f4a64fb2fbb</t>
+          <t>R09804.main.b3cc83d613ad3c36</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -40403,20 +40411,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>79583f4a64fb2fbb4a1f4f471fe6001b159213acb1f3bbd19d6dc0be5c714fa5</t>
+          <t>b3cc83d613ad3c36f93b78eace000ebc5a603966523ee71c2e6a0bd85a8ede3e</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1714874</v>
+        <v>5135812</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://link.springer.com/content/pdf/10.1186/s13568-017-0375-4.pdf</t>
+          <t>https://link.springer.com/content/pdf/10.1186/s40643-024-00756-6.pdf</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>R03477_2017_Pretreatment_methods_of_lignocellulosic_biomass_for_anaerobic_digestion.pdf</t>
+          <t>R09804_2024_Anaerobic_digestion_of_process_water_from_hydrothermal_treatment_processes.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -40428,12 +40436,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>R09804</t>
+          <t>R11844</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R09804.main.b3cc83d613ad3c36</t>
+          <t>R11844.main.c41816bf825167dc</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -40443,20 +40451,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>b3cc83d613ad3c36f93b78eace000ebc5a603966523ee71c2e6a0bd85a8ede3e</t>
+          <t>c41816bf825167dcb78ff5eb81c8d0dab0d8d8110cd2a23a04cd1109acb34919</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>5135812</v>
+        <v>1333380</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://link.springer.com/content/pdf/10.1186/s40643-024-00756-6.pdf</t>
+          <t>https://link.springer.com/content/pdf/10.1007/s00253-025-13519-w.pdf</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>R09804_2024_Anaerobic_digestion_of_process_water_from_hydrothermal_treatment_processes.pdf</t>
+          <t>R11844_2025_Micro-aeration_for_improving_anaerobic_treatment_and_biogas_production_from.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -40468,12 +40476,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>R11844</t>
+          <t>R03155</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R11844.main.c41816bf825167dc</t>
+          <t>R03155.main.2875ce0c137df622</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -40483,20 +40491,20 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>c41816bf825167dcb78ff5eb81c8d0dab0d8d8110cd2a23a04cd1109acb34919</t>
+          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1333380</v>
+        <v>5745828</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://link.springer.com/content/pdf/10.1007/s00253-025-13519-w.pdf</t>
+          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>R11844_2025_Micro-aeration_for_improving_anaerobic_treatment_and_biogas_production_from.pdf</t>
+          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -40508,12 +40516,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>R03155</t>
+          <t>R05213</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R03155.main.2875ce0c137df622</t>
+          <t>R05213.main.bcab84a15ce93062</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -40523,20 +40531,16 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
+          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>5745828</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
-        </is>
-      </c>
+        <v>1022660</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
+          <t>R05213_2019_The_use_of_lytic_polysaccharide_monooxygenases_in_anaerobic_digestion.pdf</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -40548,12 +40552,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>R05213</t>
+          <t>R06036</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R05213.main.bcab84a15ce93062</t>
+          <t>R06036.main.0bdc7b19fdb70091</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -40563,16 +40567,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
+          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1022660</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
+        <v>927168</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>R05213_2019_The_use_of_lytic_polysaccharide_monooxygenases_in_anaerobic_digestion.pdf</t>
+          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -40584,12 +40592,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>R06036</t>
+          <t>R09240</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R06036.main.0bdc7b19fdb70091</t>
+          <t>R09240.main.da8dbeb874b19b59</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -40599,20 +40607,20 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
+          <t>da8dbeb874b19b59dbea53c11766a209aaa0b0bc319e2128c94340ae78cecfaf</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>927168</v>
+        <v>1315227</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
+          <t>https://technology.matthey.com/docserver/fulltext/jmtr/67/4/Zimmerman_16a_Imp.pdf?expires=1791804248&amp;id=id&amp;accname=guest&amp;checksum=934385598F9DDA2349B917F1B50C4858</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
+          <t>R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -40624,12 +40632,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R09240</t>
+          <t>R13899</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R09240.main.da8dbeb874b19b59</t>
+          <t>R13899.main.19143e56fa77ce99</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -40639,20 +40647,16 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>da8dbeb874b19b59dbea53c11766a209aaa0b0bc319e2128c94340ae78cecfaf</t>
+          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1315227</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>https://technology.matthey.com/docserver/fulltext/jmtr/67/4/Zimmerman_16a_Imp.pdf?expires=1791804248&amp;id=id&amp;accname=guest&amp;checksum=934385598F9DDA2349B917F1B50C4858</t>
-        </is>
-      </c>
+        <v>479092</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -40664,12 +40668,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>R13899</t>
+          <t>R13955</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>R13899.main.19143e56fa77ce99</t>
+          <t>R13955.main.6714f79deccd703d</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -40679,59 +40683,23 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
+          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>479092</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
+        <v>14662119</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>R13955</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>R13955.main.6714f79deccd703d</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>14662119</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
         <is>
           <t>历史已获取，当前原件未恢复</t>
         </is>

</xml_diff>

<commit_message>
Persist checked official supplementary materials and full-text evidence
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="H22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
         <v>1</v>
@@ -1616,11 +1616,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>explicit_no_attachments_in_complete_JATS</t>
         </is>
       </c>
       <c r="H28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -2218,11 +2218,11 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>explicit_no_attachments_in_complete_JATS</t>
         </is>
       </c>
       <c r="H42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="H61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I61" t="n">
         <v>1</v>
@@ -3168,7 +3168,7 @@
         </is>
       </c>
       <c r="H64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I64" t="n">
         <v>1</v>
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.414866+00:00</t>
+          <t>2026-10-17T08:49:38.773058+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.415826+00:00</t>
+          <t>2026-10-17T08:49:38.773987+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.415848+00:00</t>
+          <t>2026-10-17T08:49:38.774012+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.416068+00:00</t>
+          <t>2026-10-17T08:49:38.774282+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.417185+00:00</t>
+          <t>2026-10-17T08:49:38.775405+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.417701+00:00</t>
+          <t>2026-10-17T08:49:38.775847+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.423229+00:00</t>
+          <t>2026-10-17T08:49:38.780860+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.425700+00:00</t>
+          <t>2026-10-17T08:49:38.783071+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.426638+00:00</t>
+          <t>2026-10-17T08:49:38.783936+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.426969+00:00</t>
+          <t>2026-10-17T08:49:38.784244+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.427726+00:00</t>
+          <t>2026-10-17T08:49:38.785018+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.428415+00:00</t>
+          <t>2026-10-17T08:49:38.785738+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.429377+00:00</t>
+          <t>2026-10-17T08:49:38.786652+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.429633+00:00</t>
+          <t>2026-10-17T08:49:38.786886+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.430500+00:00</t>
+          <t>2026-10-17T08:49:38.787746+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.438320+00:00</t>
+          <t>2026-10-17T08:49:38.795817+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.439036+00:00</t>
+          <t>2026-10-17T08:49:38.796540+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.440353+00:00</t>
+          <t>2026-10-17T08:49:38.797745+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.442916+00:00</t>
+          <t>2026-10-17T08:49:38.800301+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.444073+00:00</t>
+          <t>2026-10-17T08:49:38.801379+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.445378+00:00</t>
+          <t>2026-10-17T08:49:38.802577+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.449469+00:00</t>
+          <t>2026-10-17T08:49:38.806712+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.451649+00:00</t>
+          <t>2026-10-17T08:49:38.808860+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.453524+00:00</t>
+          <t>2026-10-17T08:49:38.810686+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.454218+00:00</t>
+          <t>2026-10-17T08:49:38.811335+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.454627+00:00</t>
+          <t>2026-10-17T08:49:38.811683+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.456619+00:00</t>
+          <t>2026-10-17T08:49:38.813757+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.457877+00:00</t>
+          <t>2026-10-17T08:49:38.814984+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.460092+00:00</t>
+          <t>2026-10-17T08:49:38.817017+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.462188+00:00</t>
+          <t>2026-10-17T08:49:38.818973+00:00</t>
         </is>
       </c>
     </row>
@@ -27542,7 +27542,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.462778+00:00</t>
+          <t>2026-10-17T08:49:38.819681+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.463360+00:00</t>
+          <t>2026-10-17T08:49:38.820250+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.464957+00:00</t>
+          <t>2026-10-17T08:49:38.821884+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.467972+00:00</t>
+          <t>2026-10-17T08:49:38.824676+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.470166+00:00</t>
+          <t>2026-10-17T08:49:38.826766+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.471690+00:00</t>
+          <t>2026-10-17T08:49:38.827952+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.474676+00:00</t>
+          <t>2026-10-17T08:49:38.830825+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.475380+00:00</t>
+          <t>2026-10-17T08:49:38.831526+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.477020+00:00</t>
+          <t>2026-10-17T08:49:38.833417+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.477279+00:00</t>
+          <t>2026-10-17T08:49:38.833701+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.479228+00:00</t>
+          <t>2026-10-17T08:49:38.835570+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.482113+00:00</t>
+          <t>2026-10-17T08:49:38.838376+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.483686+00:00</t>
+          <t>2026-10-17T08:49:38.839805+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.484226+00:00</t>
+          <t>2026-10-17T08:49:38.840363+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.486927+00:00</t>
+          <t>2026-10-17T08:49:38.843205+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.488074+00:00</t>
+          <t>2026-10-17T08:49:38.844425+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.491491+00:00</t>
+          <t>2026-10-17T08:49:38.847816+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.493124+00:00</t>
+          <t>2026-10-17T08:49:38.849521+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.494971+00:00</t>
+          <t>2026-10-17T08:49:38.851333+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.496068+00:00</t>
+          <t>2026-10-17T08:49:38.852320+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.496533+00:00</t>
+          <t>2026-10-17T08:49:38.852755+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.498029+00:00</t>
+          <t>2026-10-17T08:49:38.853110+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.499591+00:00</t>
+          <t>2026-10-17T08:49:38.854589+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.500972+00:00</t>
+          <t>2026-10-17T08:49:38.856074+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.502676+00:00</t>
+          <t>2026-10-17T08:49:38.857795+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.503027+00:00</t>
+          <t>2026-10-17T08:49:38.858149+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.504169+00:00</t>
+          <t>2026-10-17T08:49:38.859628+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.505592+00:00</t>
+          <t>2026-10-17T08:49:38.861002+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.506246+00:00</t>
+          <t>2026-10-17T08:49:38.861595+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.507262+00:00</t>
+          <t>2026-10-17T08:49:38.862579+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.507614+00:00</t>
+          <t>2026-10-17T08:49:38.862894+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.512772+00:00</t>
+          <t>2026-10-17T08:49:38.868252+00:00</t>
         </is>
       </c>
     </row>
@@ -30998,7 +30998,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.513182+00:00</t>
+          <t>2026-10-17T08:49:38.868680+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.513808+00:00</t>
+          <t>2026-10-17T08:49:38.869227+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.514255+00:00</t>
+          <t>2026-10-17T08:49:38.869752+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.515453+00:00</t>
+          <t>2026-10-17T08:49:38.870837+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.518479+00:00</t>
+          <t>2026-10-17T08:49:38.873844+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.518729+00:00</t>
+          <t>2026-10-17T08:49:38.874092+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.523058+00:00</t>
+          <t>2026-10-17T08:49:38.878273+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.523855+00:00</t>
+          <t>2026-10-17T08:49:38.879027+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.526042+00:00</t>
+          <t>2026-10-17T08:49:38.881082+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.528362+00:00</t>
+          <t>2026-10-17T08:49:38.883006+00:00</t>
         </is>
       </c>
     </row>
@@ -32078,7 +32078,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.529282+00:00</t>
+          <t>2026-10-17T08:49:38.883883+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.530725+00:00</t>
+          <t>2026-10-17T08:49:38.885610+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.533011+00:00</t>
+          <t>2026-10-17T08:49:38.887841+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.540949+00:00</t>
+          <t>2026-10-17T08:49:38.897928+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.542264+00:00</t>
+          <t>2026-10-17T08:49:38.899277+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.542426+00:00</t>
+          <t>2026-10-17T08:49:38.899467+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.542439+00:00</t>
+          <t>2026-10-17T08:49:38.899483+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.547286+00:00</t>
+          <t>2026-10-17T08:49:38.904401+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.547660+00:00</t>
+          <t>2026-10-17T08:49:38.904782+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.548019+00:00</t>
+          <t>2026-10-17T08:49:38.905566+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.548447+00:00</t>
+          <t>2026-10-17T08:49:38.905986+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.549132+00:00</t>
+          <t>2026-10-17T08:49:38.906686+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.550533+00:00</t>
+          <t>2026-10-17T08:49:38.908042+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.551393+00:00</t>
+          <t>2026-10-17T08:49:38.908853+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.551702+00:00</t>
+          <t>2026-10-17T08:49:38.909146+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.552347+00:00</t>
+          <t>2026-10-17T08:49:38.909819+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.552361+00:00</t>
+          <t>2026-10-17T08:49:38.909835+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.552413+00:00</t>
+          <t>2026-10-17T08:49:38.909881+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.552629+00:00</t>
+          <t>2026-10-17T08:49:38.910096+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.552744+00:00</t>
+          <t>2026-10-17T08:49:38.910210+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.552857+00:00</t>
+          <t>2026-10-17T08:49:38.910338+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.553234+00:00</t>
+          <t>2026-10-17T08:49:38.910707+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.553446+00:00</t>
+          <t>2026-10-17T08:49:38.910889+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.553532+00:00</t>
+          <t>2026-10-17T08:49:38.910940+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.553595+00:00</t>
+          <t>2026-10-17T08:49:38.910998+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.553741+00:00</t>
+          <t>2026-10-17T08:49:38.911137+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.553791+00:00</t>
+          <t>2026-10-17T08:49:38.911182+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.554245+00:00</t>
+          <t>2026-10-17T08:49:38.911644+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.554329+00:00</t>
+          <t>2026-10-17T08:49:38.911690+00:00</t>
         </is>
       </c>
     </row>
@@ -35215,7 +35215,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.554341+00:00</t>
+          <t>2026-10-17T08:49:38.911700+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35323,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.564175+00:00</t>
+          <t>2026-10-17T08:49:38.921260+00:00</t>
         </is>
       </c>
     </row>
@@ -35427,7 +35427,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.564239+00:00</t>
+          <t>2026-10-17T08:49:38.921333+00:00</t>
         </is>
       </c>
     </row>
@@ -35498,7 +35498,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P106" t="inlineStr">
@@ -35535,7 +35535,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.564367+00:00</t>
+          <t>2026-10-17T08:49:38.921429+00:00</t>
         </is>
       </c>
     </row>
@@ -35643,7 +35643,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.564600+00:00</t>
+          <t>2026-10-17T08:49:38.921688+00:00</t>
         </is>
       </c>
     </row>
@@ -35751,7 +35751,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.565688+00:00</t>
+          <t>2026-10-17T08:49:38.922660+00:00</t>
         </is>
       </c>
     </row>
@@ -35820,7 +35820,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P109" t="inlineStr">
@@ -35853,7 +35853,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.565772+00:00</t>
+          <t>2026-10-17T08:49:38.922741+00:00</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35947,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.565783+00:00</t>
+          <t>2026-10-17T08:49:38.922752+00:00</t>
         </is>
       </c>
     </row>
@@ -36016,7 +36016,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
@@ -36049,7 +36049,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.565861+00:00</t>
+          <t>2026-10-17T08:49:38.922829+00:00</t>
         </is>
       </c>
     </row>
@@ -36118,7 +36118,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
@@ -36151,7 +36151,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.565943+00:00</t>
+          <t>2026-10-17T08:49:38.922907+00:00</t>
         </is>
       </c>
     </row>
@@ -36220,7 +36220,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P113" t="inlineStr">
@@ -36253,7 +36253,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566050+00:00</t>
+          <t>2026-10-17T08:49:38.923010+00:00</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36347,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566061+00:00</t>
+          <t>2026-10-17T08:49:38.923021+00:00</t>
         </is>
       </c>
     </row>
@@ -36416,7 +36416,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
@@ -36449,7 +36449,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566213+00:00</t>
+          <t>2026-10-17T08:49:38.923166+00:00</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36543,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566224+00:00</t>
+          <t>2026-10-17T08:49:38.923177+00:00</t>
         </is>
       </c>
     </row>
@@ -36612,7 +36612,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -36645,7 +36645,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566346+00:00</t>
+          <t>2026-10-17T08:49:38.923274+00:00</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566358+00:00</t>
+          <t>2026-10-17T08:49:38.923285+00:00</t>
         </is>
       </c>
     </row>
@@ -36808,7 +36808,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -36841,7 +36841,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566495+00:00</t>
+          <t>2026-10-17T08:49:38.923434+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36935,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566507+00:00</t>
+          <t>2026-10-17T08:49:38.923445+00:00</t>
         </is>
       </c>
     </row>
@@ -37004,7 +37004,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
@@ -37037,7 +37037,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566598+00:00</t>
+          <t>2026-10-17T08:49:38.923531+00:00</t>
         </is>
       </c>
     </row>
@@ -37106,7 +37106,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
@@ -37139,7 +37139,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566735+00:00</t>
+          <t>2026-10-17T08:49:38.923659+00:00</t>
         </is>
       </c>
     </row>
@@ -37233,7 +37233,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566747+00:00</t>
+          <t>2026-10-17T08:49:38.923670+00:00</t>
         </is>
       </c>
     </row>
@@ -37302,7 +37302,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
@@ -37335,7 +37335,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566871+00:00</t>
+          <t>2026-10-17T08:49:38.923787+00:00</t>
         </is>
       </c>
     </row>
@@ -37429,7 +37429,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566882+00:00</t>
+          <t>2026-10-17T08:49:38.923796+00:00</t>
         </is>
       </c>
     </row>
@@ -37498,7 +37498,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -37531,7 +37531,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.566983+00:00</t>
+          <t>2026-10-17T08:49:38.923913+00:00</t>
         </is>
       </c>
     </row>
@@ -37600,7 +37600,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
@@ -37633,7 +37633,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.567221+00:00</t>
+          <t>2026-10-17T08:49:38.924129+00:00</t>
         </is>
       </c>
     </row>
@@ -37727,7 +37727,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.567233+00:00</t>
+          <t>2026-10-17T08:49:38.924140+00:00</t>
         </is>
       </c>
     </row>
@@ -37796,7 +37796,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
@@ -37829,7 +37829,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.567413+00:00</t>
+          <t>2026-10-17T08:49:38.924310+00:00</t>
         </is>
       </c>
     </row>
@@ -37898,7 +37898,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
@@ -37931,7 +37931,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.567618+00:00</t>
+          <t>2026-10-17T08:49:38.924503+00:00</t>
         </is>
       </c>
     </row>
@@ -38000,7 +38000,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
@@ -38033,7 +38033,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.567809+00:00</t>
+          <t>2026-10-17T08:49:38.924694+00:00</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.567820+00:00</t>
+          <t>2026-10-17T08:49:38.924705+00:00</t>
         </is>
       </c>
     </row>
@@ -38196,7 +38196,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
@@ -38229,7 +38229,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.567928+00:00</t>
+          <t>2026-10-17T08:49:38.924813+00:00</t>
         </is>
       </c>
     </row>
@@ -38323,7 +38323,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.567938+00:00</t>
+          <t>2026-10-17T08:49:38.924824+00:00</t>
         </is>
       </c>
     </row>
@@ -38392,7 +38392,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
@@ -38425,7 +38425,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.568038+00:00</t>
+          <t>2026-10-17T08:49:38.924911+00:00</t>
         </is>
       </c>
     </row>
@@ -38533,7 +38533,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.569082+00:00</t>
+          <t>2026-10-17T08:49:38.925981+00:00</t>
         </is>
       </c>
     </row>
@@ -38625,7 +38625,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.578938+00:00</t>
+          <t>2026-10-17T08:49:38.935211+00:00</t>
         </is>
       </c>
     </row>
@@ -38713,7 +38713,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579000+00:00</t>
+          <t>2026-10-17T08:49:38.935268+00:00</t>
         </is>
       </c>
     </row>
@@ -38801,7 +38801,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579006+00:00</t>
+          <t>2026-10-17T08:49:38.935274+00:00</t>
         </is>
       </c>
     </row>
@@ -38893,7 +38893,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579011+00:00</t>
+          <t>2026-10-17T08:49:38.935278+00:00</t>
         </is>
       </c>
     </row>
@@ -38985,7 +38985,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579014+00:00</t>
+          <t>2026-10-17T08:49:38.935281+00:00</t>
         </is>
       </c>
     </row>
@@ -39077,7 +39077,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579018+00:00</t>
+          <t>2026-10-17T08:49:38.935284+00:00</t>
         </is>
       </c>
     </row>
@@ -39169,7 +39169,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579022+00:00</t>
+          <t>2026-10-17T08:49:38.935300+00:00</t>
         </is>
       </c>
     </row>
@@ -39257,7 +39257,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579025+00:00</t>
+          <t>2026-10-17T08:49:38.935303+00:00</t>
         </is>
       </c>
     </row>
@@ -39349,7 +39349,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579029+00:00</t>
+          <t>2026-10-17T08:49:38.935306+00:00</t>
         </is>
       </c>
     </row>
@@ -39441,7 +39441,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579033+00:00</t>
+          <t>2026-10-17T08:49:38.935309+00:00</t>
         </is>
       </c>
     </row>
@@ -39529,7 +39529,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579036+00:00</t>
+          <t>2026-10-17T08:49:38.935313+00:00</t>
         </is>
       </c>
     </row>
@@ -39621,7 +39621,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T08:48:34.579041+00:00</t>
+          <t>2026-10-17T08:49:38.935317+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete existing PMC supplementary review with original-format files
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -10613,7 +10613,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>access_failed</t>
         </is>
       </c>
       <c r="H239" t="b">
@@ -11508,7 +11508,7 @@
         </is>
       </c>
       <c r="H260" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I260" t="n">
         <v>1</v>
@@ -14490,11 +14490,11 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>explicit_no_attachments_in_complete_JATS</t>
         </is>
       </c>
       <c r="H330" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I330" t="n">
         <v>0</v>
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.716531+00:00</t>
+          <t>2026-10-17T08:53:27.689130+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.717428+00:00</t>
+          <t>2026-10-17T08:53:27.690136+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.717445+00:00</t>
+          <t>2026-10-17T08:53:27.690161+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.717694+00:00</t>
+          <t>2026-10-17T08:53:27.690440+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.718864+00:00</t>
+          <t>2026-10-17T08:53:27.691576+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.719488+00:00</t>
+          <t>2026-10-17T08:53:27.692049+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.724821+00:00</t>
+          <t>2026-10-17T08:53:27.697241+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.727114+00:00</t>
+          <t>2026-10-17T08:53:27.699490+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.728141+00:00</t>
+          <t>2026-10-17T08:53:27.700845+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.728645+00:00</t>
+          <t>2026-10-17T08:53:27.701576+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.729402+00:00</t>
+          <t>2026-10-17T08:53:27.702459+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.730074+00:00</t>
+          <t>2026-10-17T08:53:27.703113+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.730983+00:00</t>
+          <t>2026-10-17T08:53:27.704007+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.731230+00:00</t>
+          <t>2026-10-17T08:53:27.704240+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.732088+00:00</t>
+          <t>2026-10-17T08:53:27.705409+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.739642+00:00</t>
+          <t>2026-10-17T08:53:27.713660+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.740488+00:00</t>
+          <t>2026-10-17T08:53:27.714537+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.741731+00:00</t>
+          <t>2026-10-17T08:53:27.716095+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.744380+00:00</t>
+          <t>2026-10-17T08:53:27.719570+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.745493+00:00</t>
+          <t>2026-10-17T08:53:27.720771+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.746674+00:00</t>
+          <t>2026-10-17T08:53:27.722433+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.750938+00:00</t>
+          <t>2026-10-17T08:53:27.727375+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.753168+00:00</t>
+          <t>2026-10-17T08:53:27.729978+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.755033+00:00</t>
+          <t>2026-10-17T08:53:27.732186+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.755897+00:00</t>
+          <t>2026-10-17T08:53:27.733155+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.756269+00:00</t>
+          <t>2026-10-17T08:53:27.733633+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.758424+00:00</t>
+          <t>2026-10-17T08:53:27.735711+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.759661+00:00</t>
+          <t>2026-10-17T08:53:27.737380+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.761699+00:00</t>
+          <t>2026-10-17T08:53:27.740520+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.763645+00:00</t>
+          <t>2026-10-17T08:53:27.743134+00:00</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.764185+00:00</t>
+          <t>2026-10-17T08:53:27.743970+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.764747+00:00</t>
+          <t>2026-10-17T08:53:27.744940+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.766385+00:00</t>
+          <t>2026-10-17T08:53:27.746646+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.769143+00:00</t>
+          <t>2026-10-17T08:53:27.749667+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.771471+00:00</t>
+          <t>2026-10-17T08:53:27.752446+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.772773+00:00</t>
+          <t>2026-10-17T08:53:27.754560+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.775623+00:00</t>
+          <t>2026-10-17T08:53:27.758372+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.776326+00:00</t>
+          <t>2026-10-17T08:53:27.759134+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.777944+00:00</t>
+          <t>2026-10-17T08:53:27.760848+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.778215+00:00</t>
+          <t>2026-10-17T08:53:27.761116+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.780202+00:00</t>
+          <t>2026-10-17T08:53:27.763255+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.783148+00:00</t>
+          <t>2026-10-17T08:53:27.767281+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.784471+00:00</t>
+          <t>2026-10-17T08:53:27.768794+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.785085+00:00</t>
+          <t>2026-10-17T08:53:27.769872+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.787687+00:00</t>
+          <t>2026-10-17T08:53:27.772880+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.788870+00:00</t>
+          <t>2026-10-17T08:53:27.774339+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.792431+00:00</t>
+          <t>2026-10-17T08:53:27.777843+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.794232+00:00</t>
+          <t>2026-10-17T08:53:27.779569+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.796072+00:00</t>
+          <t>2026-10-17T08:53:27.781387+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.797127+00:00</t>
+          <t>2026-10-17T08:53:27.782356+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.797623+00:00</t>
+          <t>2026-10-17T08:53:27.782820+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.797987+00:00</t>
+          <t>2026-10-17T08:53:27.783193+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.799620+00:00</t>
+          <t>2026-10-17T08:53:27.784814+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.800955+00:00</t>
+          <t>2026-10-17T08:53:27.786369+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.802602+00:00</t>
+          <t>2026-10-17T08:53:27.787860+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.802958+00:00</t>
+          <t>2026-10-17T08:53:27.788189+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.804236+00:00</t>
+          <t>2026-10-17T08:53:27.789506+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.805661+00:00</t>
+          <t>2026-10-17T08:53:27.790976+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.806286+00:00</t>
+          <t>2026-10-17T08:53:27.791627+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.807260+00:00</t>
+          <t>2026-10-17T08:53:27.792595+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.807700+00:00</t>
+          <t>2026-10-17T08:53:27.792978+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.812888+00:00</t>
+          <t>2026-10-17T08:53:27.799128+00:00</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.813323+00:00</t>
+          <t>2026-10-17T08:53:27.800097+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.813908+00:00</t>
+          <t>2026-10-17T08:53:27.800904+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.814372+00:00</t>
+          <t>2026-10-17T08:53:27.801406+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.815422+00:00</t>
+          <t>2026-10-17T08:53:27.802611+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.818309+00:00</t>
+          <t>2026-10-17T08:53:27.806184+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.818553+00:00</t>
+          <t>2026-10-17T08:53:27.806504+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.823036+00:00</t>
+          <t>2026-10-17T08:53:27.811210+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.823888+00:00</t>
+          <t>2026-10-17T08:53:27.812067+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.826458+00:00</t>
+          <t>2026-10-17T08:53:27.814429+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.828338+00:00</t>
+          <t>2026-10-17T08:53:27.816266+00:00</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.829330+00:00</t>
+          <t>2026-10-17T08:53:27.817224+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.830879+00:00</t>
+          <t>2026-10-17T08:53:27.818682+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.833145+00:00</t>
+          <t>2026-10-17T08:53:27.821071+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.840888+00:00</t>
+          <t>2026-10-17T08:53:27.830303+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.842290+00:00</t>
+          <t>2026-10-17T08:53:27.831875+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.842484+00:00</t>
+          <t>2026-10-17T08:53:27.832061+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.842497+00:00</t>
+          <t>2026-10-17T08:53:27.832077+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.847593+00:00</t>
+          <t>2026-10-17T08:53:27.837404+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.847978+00:00</t>
+          <t>2026-10-17T08:53:27.837841+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.848408+00:00</t>
+          <t>2026-10-17T08:53:27.838198+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.848814+00:00</t>
+          <t>2026-10-17T08:53:27.838625+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.849601+00:00</t>
+          <t>2026-10-17T08:53:27.839559+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.850997+00:00</t>
+          <t>2026-10-17T08:53:27.840999+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.851871+00:00</t>
+          <t>2026-10-17T08:53:27.841857+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.852181+00:00</t>
+          <t>2026-10-17T08:53:27.842175+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.852828+00:00</t>
+          <t>2026-10-17T08:53:27.842938+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.852842+00:00</t>
+          <t>2026-10-17T08:53:27.842961+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.852892+00:00</t>
+          <t>2026-10-17T08:53:27.843016+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.853127+00:00</t>
+          <t>2026-10-17T08:53:27.843250+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.853247+00:00</t>
+          <t>2026-10-17T08:53:27.843423+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.853376+00:00</t>
+          <t>2026-10-17T08:53:27.843543+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.853765+00:00</t>
+          <t>2026-10-17T08:53:27.843923+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.853948+00:00</t>
+          <t>2026-10-17T08:53:27.844121+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.854002+00:00</t>
+          <t>2026-10-17T08:53:27.844179+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.854065+00:00</t>
+          <t>2026-10-17T08:53:27.844243+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.854214+00:00</t>
+          <t>2026-10-17T08:53:27.844407+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.854261+00:00</t>
+          <t>2026-10-17T08:53:27.844457+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.854757+00:00</t>
+          <t>2026-10-17T08:53:27.845103+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.854814+00:00</t>
+          <t>2026-10-17T08:53:27.845188+00:00</t>
         </is>
       </c>
     </row>
@@ -35215,7 +35215,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.854824+00:00</t>
+          <t>2026-10-17T08:53:27.845200+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35323,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.863783+00:00</t>
+          <t>2026-10-17T08:53:27.855402+00:00</t>
         </is>
       </c>
     </row>
@@ -35427,7 +35427,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.863830+00:00</t>
+          <t>2026-10-17T08:53:27.855478+00:00</t>
         </is>
       </c>
     </row>
@@ -35535,7 +35535,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.863917+00:00</t>
+          <t>2026-10-17T08:53:27.855598+00:00</t>
         </is>
       </c>
     </row>
@@ -35643,7 +35643,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.864147+00:00</t>
+          <t>2026-10-17T08:53:27.855895+00:00</t>
         </is>
       </c>
     </row>
@@ -35751,7 +35751,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865250+00:00</t>
+          <t>2026-10-17T08:53:27.857171+00:00</t>
         </is>
       </c>
     </row>
@@ -35853,7 +35853,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865368+00:00</t>
+          <t>2026-10-17T08:53:27.857282+00:00</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35947,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865381+00:00</t>
+          <t>2026-10-17T08:53:27.857325+00:00</t>
         </is>
       </c>
     </row>
@@ -36049,7 +36049,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865464+00:00</t>
+          <t>2026-10-17T08:53:27.857507+00:00</t>
         </is>
       </c>
     </row>
@@ -36151,7 +36151,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865566+00:00</t>
+          <t>2026-10-17T08:53:27.857875+00:00</t>
         </is>
       </c>
     </row>
@@ -36253,7 +36253,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865674+00:00</t>
+          <t>2026-10-17T08:53:27.858003+00:00</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36347,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865685+00:00</t>
+          <t>2026-10-17T08:53:27.858016+00:00</t>
         </is>
       </c>
     </row>
@@ -36449,7 +36449,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865837+00:00</t>
+          <t>2026-10-17T08:53:27.858172+00:00</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36543,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865849+00:00</t>
+          <t>2026-10-17T08:53:27.858184+00:00</t>
         </is>
       </c>
     </row>
@@ -36645,7 +36645,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865946+00:00</t>
+          <t>2026-10-17T08:53:27.858285+00:00</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.865957+00:00</t>
+          <t>2026-10-17T08:53:27.858325+00:00</t>
         </is>
       </c>
     </row>
@@ -36841,7 +36841,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866089+00:00</t>
+          <t>2026-10-17T08:53:27.858465+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36935,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866101+00:00</t>
+          <t>2026-10-17T08:53:27.858478+00:00</t>
         </is>
       </c>
     </row>
@@ -37037,7 +37037,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866190+00:00</t>
+          <t>2026-10-17T08:53:27.858570+00:00</t>
         </is>
       </c>
     </row>
@@ -37139,7 +37139,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866349+00:00</t>
+          <t>2026-10-17T08:53:27.858702+00:00</t>
         </is>
       </c>
     </row>
@@ -37233,7 +37233,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866361+00:00</t>
+          <t>2026-10-17T08:53:27.858713+00:00</t>
         </is>
       </c>
     </row>
@@ -37335,7 +37335,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866480+00:00</t>
+          <t>2026-10-17T08:53:27.858928+00:00</t>
         </is>
       </c>
     </row>
@@ -37429,7 +37429,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866492+00:00</t>
+          <t>2026-10-17T08:53:27.859016+00:00</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37531,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866594+00:00</t>
+          <t>2026-10-17T08:53:27.859132+00:00</t>
         </is>
       </c>
     </row>
@@ -37633,7 +37633,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866813+00:00</t>
+          <t>2026-10-17T08:53:27.859386+00:00</t>
         </is>
       </c>
     </row>
@@ -37727,7 +37727,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866824+00:00</t>
+          <t>2026-10-17T08:53:27.859402+00:00</t>
         </is>
       </c>
     </row>
@@ -37829,7 +37829,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.866982+00:00</t>
+          <t>2026-10-17T08:53:27.859570+00:00</t>
         </is>
       </c>
     </row>
@@ -37931,7 +37931,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.867192+00:00</t>
+          <t>2026-10-17T08:53:27.859858+00:00</t>
         </is>
       </c>
     </row>
@@ -38033,7 +38033,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.867408+00:00</t>
+          <t>2026-10-17T08:53:27.860078+00:00</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.867421+00:00</t>
+          <t>2026-10-17T08:53:27.860092+00:00</t>
         </is>
       </c>
     </row>
@@ -38229,7 +38229,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.867528+00:00</t>
+          <t>2026-10-17T08:53:27.860200+00:00</t>
         </is>
       </c>
     </row>
@@ -38323,7 +38323,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.867538+00:00</t>
+          <t>2026-10-17T08:53:27.860212+00:00</t>
         </is>
       </c>
     </row>
@@ -38425,7 +38425,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.867625+00:00</t>
+          <t>2026-10-17T08:53:27.860324+00:00</t>
         </is>
       </c>
     </row>
@@ -38533,7 +38533,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.868698+00:00</t>
+          <t>2026-10-17T08:53:27.861550+00:00</t>
         </is>
       </c>
     </row>
@@ -38625,7 +38625,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.877931+00:00</t>
+          <t>2026-10-17T08:53:27.871932+00:00</t>
         </is>
       </c>
     </row>
@@ -38713,7 +38713,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.877985+00:00</t>
+          <t>2026-10-17T08:53:27.872016+00:00</t>
         </is>
       </c>
     </row>
@@ -38801,7 +38801,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.877990+00:00</t>
+          <t>2026-10-17T08:53:27.872024+00:00</t>
         </is>
       </c>
     </row>
@@ -38893,7 +38893,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.877994+00:00</t>
+          <t>2026-10-17T08:53:27.872028+00:00</t>
         </is>
       </c>
     </row>
@@ -38985,7 +38985,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.877997+00:00</t>
+          <t>2026-10-17T08:53:27.872032+00:00</t>
         </is>
       </c>
     </row>
@@ -39077,7 +39077,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.878000+00:00</t>
+          <t>2026-10-17T08:53:27.872036+00:00</t>
         </is>
       </c>
     </row>
@@ -39169,7 +39169,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.878003+00:00</t>
+          <t>2026-10-17T08:53:27.872038+00:00</t>
         </is>
       </c>
     </row>
@@ -39257,7 +39257,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.878007+00:00</t>
+          <t>2026-10-17T08:53:27.872042+00:00</t>
         </is>
       </c>
     </row>
@@ -39349,7 +39349,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.878010+00:00</t>
+          <t>2026-10-17T08:53:27.872045+00:00</t>
         </is>
       </c>
     </row>
@@ -39441,7 +39441,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.878013+00:00</t>
+          <t>2026-10-17T08:53:27.872048+00:00</t>
         </is>
       </c>
     </row>
@@ -39529,7 +39529,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.878016+00:00</t>
+          <t>2026-10-17T08:53:27.872052+00:00</t>
         </is>
       </c>
     </row>
@@ -39621,7 +39621,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T08:52:38.878020+00:00</t>
+          <t>2026-10-17T08:53:27.872056+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Continue existing literature records and persist all acquired candidates
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -1181,7 +1181,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.689130+00:00</t>
+          <t>2026-10-17T08:56:30.799244+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.690136+00:00</t>
+          <t>2026-10-17T08:56:30.800160+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.690161+00:00</t>
+          <t>2026-10-17T08:56:30.800178+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.690440+00:00</t>
+          <t>2026-10-17T08:56:30.800416+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.691576+00:00</t>
+          <t>2026-10-17T08:56:30.801602+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.692049+00:00</t>
+          <t>2026-10-17T08:56:30.802059+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.697241+00:00</t>
+          <t>2026-10-17T08:56:30.807348+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.699490+00:00</t>
+          <t>2026-10-17T08:56:30.809749+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.700845+00:00</t>
+          <t>2026-10-17T08:56:30.810691+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.701576+00:00</t>
+          <t>2026-10-17T08:56:30.811017+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.702459+00:00</t>
+          <t>2026-10-17T08:56:30.811723+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.703113+00:00</t>
+          <t>2026-10-17T08:56:30.812445+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.704007+00:00</t>
+          <t>2026-10-17T08:56:30.813349+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.704240+00:00</t>
+          <t>2026-10-17T08:56:30.813638+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.705409+00:00</t>
+          <t>2026-10-17T08:56:30.814495+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.713660+00:00</t>
+          <t>2026-10-17T08:56:30.821922+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.714537+00:00</t>
+          <t>2026-10-17T08:56:30.822928+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.716095+00:00</t>
+          <t>2026-10-17T08:56:30.824223+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.719570+00:00</t>
+          <t>2026-10-17T08:56:30.826907+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.720771+00:00</t>
+          <t>2026-10-17T08:56:30.828064+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.722433+00:00</t>
+          <t>2026-10-17T08:56:30.829681+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.727375+00:00</t>
+          <t>2026-10-17T08:56:30.834250+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.729978+00:00</t>
+          <t>2026-10-17T08:56:30.836758+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.732186+00:00</t>
+          <t>2026-10-17T08:56:30.838828+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.733155+00:00</t>
+          <t>2026-10-17T08:56:30.839621+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.733633+00:00</t>
+          <t>2026-10-17T08:56:30.839984+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.735711+00:00</t>
+          <t>2026-10-17T08:56:30.842205+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.737380+00:00</t>
+          <t>2026-10-17T08:56:30.843576+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.740520+00:00</t>
+          <t>2026-10-17T08:56:30.846174+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.743134+00:00</t>
+          <t>2026-10-17T08:56:30.848229+00:00</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.743970+00:00</t>
+          <t>2026-10-17T08:56:30.848812+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.744940+00:00</t>
+          <t>2026-10-17T08:56:30.849376+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.746646+00:00</t>
+          <t>2026-10-17T08:56:30.851004+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.749667+00:00</t>
+          <t>2026-10-17T08:56:30.853754+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.752446+00:00</t>
+          <t>2026-10-17T08:56:30.855843+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.754560+00:00</t>
+          <t>2026-10-17T08:56:30.857273+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.758372+00:00</t>
+          <t>2026-10-17T08:56:30.860558+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.759134+00:00</t>
+          <t>2026-10-17T08:56:30.861685+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.760848+00:00</t>
+          <t>2026-10-17T08:56:30.863542+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.761116+00:00</t>
+          <t>2026-10-17T08:56:30.863831+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.763255+00:00</t>
+          <t>2026-10-17T08:56:30.865744+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.767281+00:00</t>
+          <t>2026-10-17T08:56:30.869036+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.768794+00:00</t>
+          <t>2026-10-17T08:56:30.870479+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.769872+00:00</t>
+          <t>2026-10-17T08:56:30.871035+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.772880+00:00</t>
+          <t>2026-10-17T08:56:30.873770+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.774339+00:00</t>
+          <t>2026-10-17T08:56:30.874954+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.777843+00:00</t>
+          <t>2026-10-17T08:56:30.878589+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.779569+00:00</t>
+          <t>2026-10-17T08:56:30.880216+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.781387+00:00</t>
+          <t>2026-10-17T08:56:30.882129+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.782356+00:00</t>
+          <t>2026-10-17T08:56:30.883090+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.782820+00:00</t>
+          <t>2026-10-17T08:56:30.883575+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.783193+00:00</t>
+          <t>2026-10-17T08:56:30.883957+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.784814+00:00</t>
+          <t>2026-10-17T08:56:30.885569+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.786369+00:00</t>
+          <t>2026-10-17T08:56:30.887246+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.787860+00:00</t>
+          <t>2026-10-17T08:56:30.888775+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.788189+00:00</t>
+          <t>2026-10-17T08:56:30.889115+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.789506+00:00</t>
+          <t>2026-10-17T08:56:30.890618+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.790976+00:00</t>
+          <t>2026-10-17T08:56:30.893276+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.791627+00:00</t>
+          <t>2026-10-17T08:56:30.894536+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.792595+00:00</t>
+          <t>2026-10-17T08:56:30.895991+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.792978+00:00</t>
+          <t>2026-10-17T08:56:30.896469+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.799128+00:00</t>
+          <t>2026-10-17T08:56:30.902352+00:00</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.800097+00:00</t>
+          <t>2026-10-17T08:56:30.903092+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.800904+00:00</t>
+          <t>2026-10-17T08:56:30.903810+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.801406+00:00</t>
+          <t>2026-10-17T08:56:30.904742+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.802611+00:00</t>
+          <t>2026-10-17T08:56:30.906926+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.806184+00:00</t>
+          <t>2026-10-17T08:56:30.911982+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.806504+00:00</t>
+          <t>2026-10-17T08:56:30.912517+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.811210+00:00</t>
+          <t>2026-10-17T08:56:30.917042+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.812067+00:00</t>
+          <t>2026-10-17T08:56:30.918118+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.814429+00:00</t>
+          <t>2026-10-17T08:56:30.920324+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.816266+00:00</t>
+          <t>2026-10-17T08:56:30.922193+00:00</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.817224+00:00</t>
+          <t>2026-10-17T08:56:30.923487+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.818682+00:00</t>
+          <t>2026-10-17T08:56:30.925228+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.821071+00:00</t>
+          <t>2026-10-17T08:56:30.927813+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.830303+00:00</t>
+          <t>2026-10-17T08:56:30.936077+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.831875+00:00</t>
+          <t>2026-10-17T08:56:30.937459+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.832061+00:00</t>
+          <t>2026-10-17T08:56:30.937638+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.832077+00:00</t>
+          <t>2026-10-17T08:56:30.937652+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.837404+00:00</t>
+          <t>2026-10-17T08:56:30.943248+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.837841+00:00</t>
+          <t>2026-10-17T08:56:30.943744+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.838198+00:00</t>
+          <t>2026-10-17T08:56:30.944104+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.838625+00:00</t>
+          <t>2026-10-17T08:56:30.944517+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.839559+00:00</t>
+          <t>2026-10-17T08:56:30.945366+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.840999+00:00</t>
+          <t>2026-10-17T08:56:30.947281+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.841857+00:00</t>
+          <t>2026-10-17T08:56:30.948208+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.842175+00:00</t>
+          <t>2026-10-17T08:56:30.948540+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.842938+00:00</t>
+          <t>2026-10-17T08:56:30.949180+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.842961+00:00</t>
+          <t>2026-10-17T08:56:30.949195+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.843016+00:00</t>
+          <t>2026-10-17T08:56:30.949242+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.843250+00:00</t>
+          <t>2026-10-17T08:56:30.949514+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.843423+00:00</t>
+          <t>2026-10-17T08:56:30.949641+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.843543+00:00</t>
+          <t>2026-10-17T08:56:30.949839+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.843923+00:00</t>
+          <t>2026-10-17T08:56:30.950228+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.844121+00:00</t>
+          <t>2026-10-17T08:56:30.950449+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.844179+00:00</t>
+          <t>2026-10-17T08:56:30.950512+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.844243+00:00</t>
+          <t>2026-10-17T08:56:30.950575+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.844407+00:00</t>
+          <t>2026-10-17T08:56:30.950719+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.844457+00:00</t>
+          <t>2026-10-17T08:56:30.950848+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.845103+00:00</t>
+          <t>2026-10-17T08:56:30.951327+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.845188+00:00</t>
+          <t>2026-10-17T08:56:30.951384+00:00</t>
         </is>
       </c>
     </row>
@@ -35215,7 +35215,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.845200+00:00</t>
+          <t>2026-10-17T08:56:30.951395+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35323,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.855402+00:00</t>
+          <t>2026-10-17T08:56:30.961746+00:00</t>
         </is>
       </c>
     </row>
@@ -35427,7 +35427,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.855478+00:00</t>
+          <t>2026-10-17T08:56:30.961828+00:00</t>
         </is>
       </c>
     </row>
@@ -35535,7 +35535,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.855598+00:00</t>
+          <t>2026-10-17T08:56:30.961948+00:00</t>
         </is>
       </c>
     </row>
@@ -35643,7 +35643,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.855895+00:00</t>
+          <t>2026-10-17T08:56:30.962190+00:00</t>
         </is>
       </c>
     </row>
@@ -35751,7 +35751,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.857171+00:00</t>
+          <t>2026-10-17T08:56:30.963316+00:00</t>
         </is>
       </c>
     </row>
@@ -35853,7 +35853,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.857282+00:00</t>
+          <t>2026-10-17T08:56:30.963424+00:00</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35947,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.857325+00:00</t>
+          <t>2026-10-17T08:56:30.963437+00:00</t>
         </is>
       </c>
     </row>
@@ -36049,7 +36049,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.857507+00:00</t>
+          <t>2026-10-17T08:56:30.963516+00:00</t>
         </is>
       </c>
     </row>
@@ -36151,7 +36151,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.857875+00:00</t>
+          <t>2026-10-17T08:56:30.963597+00:00</t>
         </is>
       </c>
     </row>
@@ -36253,7 +36253,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858003+00:00</t>
+          <t>2026-10-17T08:56:30.963706+00:00</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36347,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858016+00:00</t>
+          <t>2026-10-17T08:56:30.963718+00:00</t>
         </is>
       </c>
     </row>
@@ -36449,7 +36449,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858172+00:00</t>
+          <t>2026-10-17T08:56:30.963872+00:00</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36543,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858184+00:00</t>
+          <t>2026-10-17T08:56:30.963884+00:00</t>
         </is>
       </c>
     </row>
@@ -36645,7 +36645,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858285+00:00</t>
+          <t>2026-10-17T08:56:30.963984+00:00</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858325+00:00</t>
+          <t>2026-10-17T08:56:30.963994+00:00</t>
         </is>
       </c>
     </row>
@@ -36841,7 +36841,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858465+00:00</t>
+          <t>2026-10-17T08:56:30.964125+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36935,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858478+00:00</t>
+          <t>2026-10-17T08:56:30.964136+00:00</t>
         </is>
       </c>
     </row>
@@ -37037,7 +37037,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858570+00:00</t>
+          <t>2026-10-17T08:56:30.964224+00:00</t>
         </is>
       </c>
     </row>
@@ -37139,7 +37139,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858702+00:00</t>
+          <t>2026-10-17T08:56:30.964371+00:00</t>
         </is>
       </c>
     </row>
@@ -37233,7 +37233,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858713+00:00</t>
+          <t>2026-10-17T08:56:30.964385+00:00</t>
         </is>
       </c>
     </row>
@@ -37335,7 +37335,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.858928+00:00</t>
+          <t>2026-10-17T08:56:30.964503+00:00</t>
         </is>
       </c>
     </row>
@@ -37429,7 +37429,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.859016+00:00</t>
+          <t>2026-10-17T08:56:30.964514+00:00</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37531,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.859132+00:00</t>
+          <t>2026-10-17T08:56:30.964615+00:00</t>
         </is>
       </c>
     </row>
@@ -37633,7 +37633,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.859386+00:00</t>
+          <t>2026-10-17T08:56:30.964838+00:00</t>
         </is>
       </c>
     </row>
@@ -37727,7 +37727,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.859402+00:00</t>
+          <t>2026-10-17T08:56:30.964849+00:00</t>
         </is>
       </c>
     </row>
@@ -37829,7 +37829,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.859570+00:00</t>
+          <t>2026-10-17T08:56:30.965006+00:00</t>
         </is>
       </c>
     </row>
@@ -37931,7 +37931,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.859858+00:00</t>
+          <t>2026-10-17T08:56:30.965196+00:00</t>
         </is>
       </c>
     </row>
@@ -38033,7 +38033,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.860078+00:00</t>
+          <t>2026-10-17T08:56:30.965458+00:00</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.860092+00:00</t>
+          <t>2026-10-17T08:56:30.965500+00:00</t>
         </is>
       </c>
     </row>
@@ -38229,7 +38229,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.860200+00:00</t>
+          <t>2026-10-17T08:56:30.965632+00:00</t>
         </is>
       </c>
     </row>
@@ -38323,7 +38323,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.860212+00:00</t>
+          <t>2026-10-17T08:56:30.965644+00:00</t>
         </is>
       </c>
     </row>
@@ -38425,7 +38425,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.860324+00:00</t>
+          <t>2026-10-17T08:56:30.965732+00:00</t>
         </is>
       </c>
     </row>
@@ -38533,7 +38533,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.861550+00:00</t>
+          <t>2026-10-17T08:56:30.966804+00:00</t>
         </is>
       </c>
     </row>
@@ -38625,7 +38625,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.871932+00:00</t>
+          <t>2026-10-17T08:56:30.976947+00:00</t>
         </is>
       </c>
     </row>
@@ -38657,13 +38657,21 @@
         </is>
       </c>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" t="inlineStr"/>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
+        </is>
+      </c>
       <c r="I138" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-fulltexts/R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr"/>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
+        </is>
+      </c>
       <c r="K138" t="inlineStr">
         <is>
           <t>pdf</t>
@@ -38679,15 +38687,19 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
-        </is>
-      </c>
-      <c r="P138" t="inlineStr"/>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>https://www.scielo.br/j/bjce/a/Fsb5BG69HCqpVRTqkxS4stm/?lang=en&amp;format=pdf</t>
+        </is>
+      </c>
       <c r="Q138" t="inlineStr"/>
       <c r="R138" t="inlineStr">
         <is>
@@ -38713,7 +38725,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872016+00:00</t>
+          <t>2026-10-17T08:56:30.977437+00:00</t>
         </is>
       </c>
     </row>
@@ -38801,7 +38813,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872024+00:00</t>
+          <t>2026-10-17T08:56:30.977455+00:00</t>
         </is>
       </c>
     </row>
@@ -38893,7 +38905,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872028+00:00</t>
+          <t>2026-10-17T08:56:30.977459+00:00</t>
         </is>
       </c>
     </row>
@@ -38985,7 +38997,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872032+00:00</t>
+          <t>2026-10-17T08:56:30.977463+00:00</t>
         </is>
       </c>
     </row>
@@ -39077,7 +39089,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872036+00:00</t>
+          <t>2026-10-17T08:56:30.977466+00:00</t>
         </is>
       </c>
     </row>
@@ -39169,7 +39181,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872038+00:00</t>
+          <t>2026-10-17T08:56:30.977469+00:00</t>
         </is>
       </c>
     </row>
@@ -39257,7 +39269,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872042+00:00</t>
+          <t>2026-10-17T08:56:30.977472+00:00</t>
         </is>
       </c>
     </row>
@@ -39349,7 +39361,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872045+00:00</t>
+          <t>2026-10-17T08:56:30.977495+00:00</t>
         </is>
       </c>
     </row>
@@ -39441,7 +39453,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872048+00:00</t>
+          <t>2026-10-17T08:56:30.977498+00:00</t>
         </is>
       </c>
     </row>
@@ -39529,7 +39541,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872052+00:00</t>
+          <t>2026-10-17T08:56:30.977502+00:00</t>
         </is>
       </c>
     </row>
@@ -39621,7 +39633,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T08:53:27.872056+00:00</t>
+          <t>2026-10-17T08:56:30.977505+00:00</t>
         </is>
       </c>
     </row>
@@ -39636,7 +39648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40284,12 +40296,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>R02274</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R02274.main.4c7da8384f1f6e3d</t>
+          <t>R10086.main.84777bfb7a2cd42f</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -40299,16 +40311,16 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4c7da8384f1f6e3d8bd2681eab23bdb95e3057009cf4c7ec7aacc7cdb9eaf43d</t>
+          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>471480</v>
+        <v>984310</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>R02274_2016_ANAEROBIC_DIGESTION_OF_WASTEWATER_WITH_HIGH_SULFATE_CONCENTRATION_USING.pdf</t>
+          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -40320,12 +40332,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>R10086</t>
+          <t>R03477</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R10086.main.84777bfb7a2cd42f</t>
+          <t>R03477.main.79583f4a64fb2fbb</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -40335,16 +40347,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
+          <t>79583f4a64fb2fbb4a1f4f471fe6001b159213acb1f3bbd19d6dc0be5c714fa5</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>984310</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
+        <v>1714874</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1186/s13568-017-0375-4.pdf</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
+          <t>R03477_2017_Pretreatment_methods_of_lignocellulosic_biomass_for_anaerobic_digestion.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -40356,12 +40372,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>R03477</t>
+          <t>R09804</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R03477.main.79583f4a64fb2fbb</t>
+          <t>R09804.main.b3cc83d613ad3c36</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -40371,20 +40387,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>79583f4a64fb2fbb4a1f4f471fe6001b159213acb1f3bbd19d6dc0be5c714fa5</t>
+          <t>b3cc83d613ad3c36f93b78eace000ebc5a603966523ee71c2e6a0bd85a8ede3e</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1714874</v>
+        <v>5135812</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://link.springer.com/content/pdf/10.1186/s13568-017-0375-4.pdf</t>
+          <t>https://link.springer.com/content/pdf/10.1186/s40643-024-00756-6.pdf</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>R03477_2017_Pretreatment_methods_of_lignocellulosic_biomass_for_anaerobic_digestion.pdf</t>
+          <t>R09804_2024_Anaerobic_digestion_of_process_water_from_hydrothermal_treatment_processes.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -40396,12 +40412,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>R09804</t>
+          <t>R11844</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R09804.main.b3cc83d613ad3c36</t>
+          <t>R11844.main.c41816bf825167dc</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -40411,20 +40427,20 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>b3cc83d613ad3c36f93b78eace000ebc5a603966523ee71c2e6a0bd85a8ede3e</t>
+          <t>c41816bf825167dcb78ff5eb81c8d0dab0d8d8110cd2a23a04cd1109acb34919</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>5135812</v>
+        <v>1333380</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://link.springer.com/content/pdf/10.1186/s40643-024-00756-6.pdf</t>
+          <t>https://link.springer.com/content/pdf/10.1007/s00253-025-13519-w.pdf</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>R09804_2024_Anaerobic_digestion_of_process_water_from_hydrothermal_treatment_processes.pdf</t>
+          <t>R11844_2025_Micro-aeration_for_improving_anaerobic_treatment_and_biogas_production_from.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -40436,12 +40452,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>R11844</t>
+          <t>R03155</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R11844.main.c41816bf825167dc</t>
+          <t>R03155.main.2875ce0c137df622</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -40451,20 +40467,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>c41816bf825167dcb78ff5eb81c8d0dab0d8d8110cd2a23a04cd1109acb34919</t>
+          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1333380</v>
+        <v>5745828</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://link.springer.com/content/pdf/10.1007/s00253-025-13519-w.pdf</t>
+          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>R11844_2025_Micro-aeration_for_improving_anaerobic_treatment_and_biogas_production_from.pdf</t>
+          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -40476,12 +40492,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>R03155</t>
+          <t>R05213</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R03155.main.2875ce0c137df622</t>
+          <t>R05213.main.bcab84a15ce93062</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -40491,20 +40507,16 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
+          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>5745828</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
-        </is>
-      </c>
+        <v>1022660</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
+          <t>R05213_2019_The_use_of_lytic_polysaccharide_monooxygenases_in_anaerobic_digestion.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -40516,12 +40528,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>R05213</t>
+          <t>R06036</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R05213.main.bcab84a15ce93062</t>
+          <t>R06036.main.0bdc7b19fdb70091</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -40531,16 +40543,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>bcab84a15ce930626c5a8f88083f5a7bb857b403c5e0ba13af2f6aaed379f051</t>
+          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1022660</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
+        <v>927168</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>R05213_2019_The_use_of_lytic_polysaccharide_monooxygenases_in_anaerobic_digestion.pdf</t>
+          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -40552,12 +40568,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>R06036</t>
+          <t>R09240</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R06036.main.0bdc7b19fdb70091</t>
+          <t>R09240.main.da8dbeb874b19b59</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -40567,20 +40583,20 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
+          <t>da8dbeb874b19b59dbea53c11766a209aaa0b0bc319e2128c94340ae78cecfaf</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>927168</v>
+        <v>1315227</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
+          <t>https://technology.matthey.com/docserver/fulltext/jmtr/67/4/Zimmerman_16a_Imp.pdf?expires=1791804248&amp;id=id&amp;accname=guest&amp;checksum=934385598F9DDA2349B917F1B50C4858</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
+          <t>R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -40592,12 +40608,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>R09240</t>
+          <t>R13899</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>R09240.main.da8dbeb874b19b59</t>
+          <t>R13899.main.19143e56fa77ce99</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -40607,20 +40623,16 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>da8dbeb874b19b59dbea53c11766a209aaa0b0bc319e2128c94340ae78cecfaf</t>
+          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1315227</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>https://technology.matthey.com/docserver/fulltext/jmtr/67/4/Zimmerman_16a_Imp.pdf?expires=1791804248&amp;id=id&amp;accname=guest&amp;checksum=934385598F9DDA2349B917F1B50C4858</t>
-        </is>
-      </c>
+        <v>479092</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -40632,12 +40644,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R13899</t>
+          <t>R13955</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>R13899.main.19143e56fa77ce99</t>
+          <t>R13955.main.6714f79deccd703d</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -40647,59 +40659,23 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
+          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>479092</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
+        <v>14662119</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>R13955</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>R13955.main.6714f79deccd703d</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>14662119</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
         <is>
           <t>历史已获取，当前原件未恢复</t>
         </is>

</xml_diff>

<commit_message>
Persist publisher supplementary checks and acquired original attachments
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>access_failed</t>
         </is>
       </c>
       <c r="H2" t="b">
@@ -541,7 +541,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>access_failed</t>
         </is>
       </c>
       <c r="H3" t="b">
@@ -584,7 +584,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>access_failed</t>
         </is>
       </c>
       <c r="H4" t="b">
@@ -627,7 +627,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>access_failed</t>
         </is>
       </c>
       <c r="H5" t="b">
@@ -670,7 +670,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>not_checked</t>
+          <t>checked_no_file_links_found_coverage_unconfirmed</t>
         </is>
       </c>
       <c r="H6" t="b">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -24118,7 +24118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X148"/>
+  <dimension ref="A1:X153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.397990+00:00</t>
+          <t>2026-10-17T09:22:30.796820+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.398928+00:00</t>
+          <t>2026-10-17T09:22:30.797808+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.398946+00:00</t>
+          <t>2026-10-17T09:22:30.797834+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.399165+00:00</t>
+          <t>2026-10-17T09:22:30.798075+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.400322+00:00</t>
+          <t>2026-10-17T09:22:30.799161+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.400788+00:00</t>
+          <t>2026-10-17T09:22:30.799657+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.405740+00:00</t>
+          <t>2026-10-17T09:22:30.806684+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.408011+00:00</t>
+          <t>2026-10-17T09:22:30.809068+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.408983+00:00</t>
+          <t>2026-10-17T09:22:30.810077+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.409344+00:00</t>
+          <t>2026-10-17T09:22:30.810447+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.410087+00:00</t>
+          <t>2026-10-17T09:22:30.811231+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.410793+00:00</t>
+          <t>2026-10-17T09:22:30.811895+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.411771+00:00</t>
+          <t>2026-10-17T09:22:30.813125+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.412008+00:00</t>
+          <t>2026-10-17T09:22:30.813546+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.412923+00:00</t>
+          <t>2026-10-17T09:22:30.815065+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.420701+00:00</t>
+          <t>2026-10-17T09:22:30.827603+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.421469+00:00</t>
+          <t>2026-10-17T09:22:30.828480+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.422725+00:00</t>
+          <t>2026-10-17T09:22:30.829715+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.425155+00:00</t>
+          <t>2026-10-17T09:22:30.832179+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.426397+00:00</t>
+          <t>2026-10-17T09:22:30.833261+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.427604+00:00</t>
+          <t>2026-10-17T09:22:30.836519+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.431773+00:00</t>
+          <t>2026-10-17T09:22:30.840897+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.434006+00:00</t>
+          <t>2026-10-17T09:22:30.843206+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.435857+00:00</t>
+          <t>2026-10-17T09:22:30.845025+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.436585+00:00</t>
+          <t>2026-10-17T09:22:30.845844+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.436962+00:00</t>
+          <t>2026-10-17T09:22:30.846404+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.439020+00:00</t>
+          <t>2026-10-17T09:22:30.849761+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.440276+00:00</t>
+          <t>2026-10-17T09:22:30.851231+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.442335+00:00</t>
+          <t>2026-10-17T09:22:30.853569+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.444563+00:00</t>
+          <t>2026-10-17T09:22:30.855568+00:00</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.445134+00:00</t>
+          <t>2026-10-17T09:22:30.856223+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.445745+00:00</t>
+          <t>2026-10-17T09:22:30.857027+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.447361+00:00</t>
+          <t>2026-10-17T09:22:30.858685+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.450499+00:00</t>
+          <t>2026-10-17T09:22:30.861565+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.452702+00:00</t>
+          <t>2026-10-17T09:22:30.863686+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.454237+00:00</t>
+          <t>2026-10-17T09:22:30.864982+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.457383+00:00</t>
+          <t>2026-10-17T09:22:30.868329+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.458212+00:00</t>
+          <t>2026-10-17T09:22:30.869095+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.459932+00:00</t>
+          <t>2026-10-17T09:22:30.870786+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.460193+00:00</t>
+          <t>2026-10-17T09:22:30.871077+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.462100+00:00</t>
+          <t>2026-10-17T09:22:30.873193+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.464912+00:00</t>
+          <t>2026-10-17T09:22:30.876224+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.466239+00:00</t>
+          <t>2026-10-17T09:22:30.877886+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.466805+00:00</t>
+          <t>2026-10-17T09:22:30.878568+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.469366+00:00</t>
+          <t>2026-10-17T09:22:30.881156+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.470556+00:00</t>
+          <t>2026-10-17T09:22:30.882410+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.474195+00:00</t>
+          <t>2026-10-17T09:22:30.885911+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.476001+00:00</t>
+          <t>2026-10-17T09:22:30.887548+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.478136+00:00</t>
+          <t>2026-10-17T09:22:30.889373+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.479178+00:00</t>
+          <t>2026-10-17T09:22:30.890430+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.479647+00:00</t>
+          <t>2026-10-17T09:22:30.890895+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.480032+00:00</t>
+          <t>2026-10-17T09:22:30.891311+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.481515+00:00</t>
+          <t>2026-10-17T09:22:30.892760+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.482780+00:00</t>
+          <t>2026-10-17T09:22:30.894044+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.484329+00:00</t>
+          <t>2026-10-17T09:22:30.895535+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.484676+00:00</t>
+          <t>2026-10-17T09:22:30.895879+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.486184+00:00</t>
+          <t>2026-10-17T09:22:30.897140+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.487589+00:00</t>
+          <t>2026-10-17T09:22:30.898728+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.488190+00:00</t>
+          <t>2026-10-17T09:22:30.899486+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.489160+00:00</t>
+          <t>2026-10-17T09:22:30.900846+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.489506+00:00</t>
+          <t>2026-10-17T09:22:30.901456+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.494459+00:00</t>
+          <t>2026-10-17T09:22:30.909196+00:00</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.494848+00:00</t>
+          <t>2026-10-17T09:22:30.909830+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.495477+00:00</t>
+          <t>2026-10-17T09:22:30.910534+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.495935+00:00</t>
+          <t>2026-10-17T09:22:30.911314+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.497029+00:00</t>
+          <t>2026-10-17T09:22:30.913496+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.500034+00:00</t>
+          <t>2026-10-17T09:22:30.919978+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.500313+00:00</t>
+          <t>2026-10-17T09:22:30.920430+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.504480+00:00</t>
+          <t>2026-10-17T09:22:30.925021+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.505361+00:00</t>
+          <t>2026-10-17T09:22:30.926206+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.507744+00:00</t>
+          <t>2026-10-17T09:22:30.929279+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.509557+00:00</t>
+          <t>2026-10-17T09:22:30.931353+00:00</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.510485+00:00</t>
+          <t>2026-10-17T09:22:30.932351+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.511881+00:00</t>
+          <t>2026-10-17T09:22:30.933806+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.514082+00:00</t>
+          <t>2026-10-17T09:22:30.936305+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.522272+00:00</t>
+          <t>2026-10-17T09:22:30.946091+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.523881+00:00</t>
+          <t>2026-10-17T09:22:30.947882+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.524056+00:00</t>
+          <t>2026-10-17T09:22:30.948160+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.524069+00:00</t>
+          <t>2026-10-17T09:22:30.948183+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.529202+00:00</t>
+          <t>2026-10-17T09:22:30.953807+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.529732+00:00</t>
+          <t>2026-10-17T09:22:30.954420+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.530106+00:00</t>
+          <t>2026-10-17T09:22:30.954933+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.530548+00:00</t>
+          <t>2026-10-17T09:22:30.955388+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.531514+00:00</t>
+          <t>2026-10-17T09:22:30.956198+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.532936+00:00</t>
+          <t>2026-10-17T09:22:30.957844+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.533848+00:00</t>
+          <t>2026-10-17T09:22:30.959001+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.534151+00:00</t>
+          <t>2026-10-17T09:22:30.959548+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.534842+00:00</t>
+          <t>2026-10-17T09:22:30.960282+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.534856+00:00</t>
+          <t>2026-10-17T09:22:30.960325+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.534909+00:00</t>
+          <t>2026-10-17T09:22:30.960392+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.535129+00:00</t>
+          <t>2026-10-17T09:22:30.960629+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.535250+00:00</t>
+          <t>2026-10-17T09:22:30.960751+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.535381+00:00</t>
+          <t>2026-10-17T09:22:30.960998+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.535758+00:00</t>
+          <t>2026-10-17T09:22:30.961531+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.535954+00:00</t>
+          <t>2026-10-17T09:22:30.961830+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.536010+00:00</t>
+          <t>2026-10-17T09:22:30.961902+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.536071+00:00</t>
+          <t>2026-10-17T09:22:30.961966+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.536211+00:00</t>
+          <t>2026-10-17T09:22:30.962108+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.536255+00:00</t>
+          <t>2026-10-17T09:22:30.962153+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.536742+00:00</t>
+          <t>2026-10-17T09:22:30.962836+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.536803+00:00</t>
+          <t>2026-10-17T09:22:30.962910+00:00</t>
         </is>
       </c>
     </row>
@@ -35215,7 +35215,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.536814+00:00</t>
+          <t>2026-10-17T09:22:30.962922+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35323,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.546506+00:00</t>
+          <t>2026-10-17T09:22:30.974519+00:00</t>
         </is>
       </c>
     </row>
@@ -35427,7 +35427,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.546569+00:00</t>
+          <t>2026-10-17T09:22:30.974611+00:00</t>
         </is>
       </c>
     </row>
@@ -35535,7 +35535,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.546672+00:00</t>
+          <t>2026-10-17T09:22:30.974739+00:00</t>
         </is>
       </c>
     </row>
@@ -35643,7 +35643,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.546907+00:00</t>
+          <t>2026-10-17T09:22:30.974998+00:00</t>
         </is>
       </c>
     </row>
@@ -35751,7 +35751,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.547910+00:00</t>
+          <t>2026-10-17T09:22:30.976314+00:00</t>
         </is>
       </c>
     </row>
@@ -35853,7 +35853,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548129+00:00</t>
+          <t>2026-10-17T09:22:30.976449+00:00</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35947,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548152+00:00</t>
+          <t>2026-10-17T09:22:30.976464+00:00</t>
         </is>
       </c>
     </row>
@@ -36049,7 +36049,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548246+00:00</t>
+          <t>2026-10-17T09:22:30.976553+00:00</t>
         </is>
       </c>
     </row>
@@ -36151,7 +36151,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548355+00:00</t>
+          <t>2026-10-17T09:22:30.976641+00:00</t>
         </is>
       </c>
     </row>
@@ -36253,7 +36253,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548469+00:00</t>
+          <t>2026-10-17T09:22:30.976751+00:00</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36347,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548481+00:00</t>
+          <t>2026-10-17T09:22:30.976763+00:00</t>
         </is>
       </c>
     </row>
@@ -36449,7 +36449,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548637+00:00</t>
+          <t>2026-10-17T09:22:30.976944+00:00</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36543,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548648+00:00</t>
+          <t>2026-10-17T09:22:30.976957+00:00</t>
         </is>
       </c>
     </row>
@@ -36645,7 +36645,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548748+00:00</t>
+          <t>2026-10-17T09:22:30.977067+00:00</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548759+00:00</t>
+          <t>2026-10-17T09:22:30.977077+00:00</t>
         </is>
       </c>
     </row>
@@ -36841,7 +36841,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548900+00:00</t>
+          <t>2026-10-17T09:22:30.977214+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36935,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.548911+00:00</t>
+          <t>2026-10-17T09:22:30.977225+00:00</t>
         </is>
       </c>
     </row>
@@ -37037,7 +37037,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549000+00:00</t>
+          <t>2026-10-17T09:22:30.977336+00:00</t>
         </is>
       </c>
     </row>
@@ -37139,7 +37139,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549131+00:00</t>
+          <t>2026-10-17T09:22:30.977471+00:00</t>
         </is>
       </c>
     </row>
@@ -37233,7 +37233,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549143+00:00</t>
+          <t>2026-10-17T09:22:30.977504+00:00</t>
         </is>
       </c>
     </row>
@@ -37335,7 +37335,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549262+00:00</t>
+          <t>2026-10-17T09:22:30.977626+00:00</t>
         </is>
       </c>
     </row>
@@ -37429,7 +37429,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549273+00:00</t>
+          <t>2026-10-17T09:22:30.977636+00:00</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37531,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549393+00:00</t>
+          <t>2026-10-17T09:22:30.977743+00:00</t>
         </is>
       </c>
     </row>
@@ -37633,7 +37633,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549645+00:00</t>
+          <t>2026-10-17T09:22:30.977967+00:00</t>
         </is>
       </c>
     </row>
@@ -37727,7 +37727,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549661+00:00</t>
+          <t>2026-10-17T09:22:30.977979+00:00</t>
         </is>
       </c>
     </row>
@@ -37829,7 +37829,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.549970+00:00</t>
+          <t>2026-10-17T09:22:30.978141+00:00</t>
         </is>
       </c>
     </row>
@@ -37931,7 +37931,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.550184+00:00</t>
+          <t>2026-10-17T09:22:30.978372+00:00</t>
         </is>
       </c>
     </row>
@@ -38033,7 +38033,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.550411+00:00</t>
+          <t>2026-10-17T09:22:30.978571+00:00</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.550425+00:00</t>
+          <t>2026-10-17T09:22:30.978583+00:00</t>
         </is>
       </c>
     </row>
@@ -38229,7 +38229,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.550538+00:00</t>
+          <t>2026-10-17T09:22:30.978693+00:00</t>
         </is>
       </c>
     </row>
@@ -38323,7 +38323,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.550549+00:00</t>
+          <t>2026-10-17T09:22:30.978704+00:00</t>
         </is>
       </c>
     </row>
@@ -38425,7 +38425,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.550637+00:00</t>
+          <t>2026-10-17T09:22:30.978794+00:00</t>
         </is>
       </c>
     </row>
@@ -38533,13 +38533,13 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.551804+00:00</t>
+          <t>2026-10-17T09:22:30.979941+00:00</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -38625,7 +38625,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.561397+00:00</t>
+          <t>2026-10-17T09:22:30.989797+00:00</t>
         </is>
       </c>
     </row>
@@ -38725,7 +38725,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.561907+00:00</t>
+          <t>2026-10-17T09:22:30.990309+00:00</t>
         </is>
       </c>
     </row>
@@ -38813,7 +38813,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.561923+00:00</t>
+          <t>2026-10-17T09:22:30.990325+00:00</t>
         </is>
       </c>
     </row>
@@ -38913,7 +38913,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.563075+00:00</t>
+          <t>2026-10-17T09:22:30.991480+00:00</t>
         </is>
       </c>
     </row>
@@ -39013,7 +39013,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.566559+00:00</t>
+          <t>2026-10-17T09:22:30.994900+00:00</t>
         </is>
       </c>
     </row>
@@ -39113,7 +39113,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.567542+00:00</t>
+          <t>2026-10-17T09:22:30.995850+00:00</t>
         </is>
       </c>
     </row>
@@ -39205,7 +39205,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.567560+00:00</t>
+          <t>2026-10-17T09:22:30.995866+00:00</t>
         </is>
       </c>
     </row>
@@ -39272,7 +39272,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P144" t="inlineStr">
@@ -39305,7 +39305,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.568262+00:00</t>
+          <t>2026-10-17T09:22:30.996571+00:00</t>
         </is>
       </c>
     </row>
@@ -39397,7 +39397,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.568276+00:00</t>
+          <t>2026-10-17T09:22:30.996586+00:00</t>
         </is>
       </c>
     </row>
@@ -39489,7 +39489,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.568280+00:00</t>
+          <t>2026-10-17T09:22:30.996589+00:00</t>
         </is>
       </c>
     </row>
@@ -39577,7 +39577,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.568284+00:00</t>
+          <t>2026-10-17T09:22:30.996592+00:00</t>
         </is>
       </c>
     </row>
@@ -39669,7 +39669,487 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T09:09:29.568302+00:00</t>
+          <t>2026-10-17T09:22:30.996595+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="b">
+        <v>1</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>R06588</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>R06588.main.a69e903d7886bcd0</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E149" t="b">
+        <v>0</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>R06588_2021_Effect_of_Rotten_Butter_Shock_Load_on_Anaerobic_Digestion_of_Chicken_Manure_a69e903d7886.pdf</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R06588_2021_Effect_of_Rotten_Butter_Shock_Load_on_Anaerobic_Digestion_of_Chicken_Manure_a69e903d7886.pdf</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R06588_2021_Effect_of_Rotten_Butter_Shock_Load_on_Anaerobic_Digestion_of_Chicken_Manure_a69e903d7886.pdf</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R06588_2021_Effect_of_Rotten_Butter_Shock_Load_on_Anaerobic_Digestion_of_Chicken_Manure_a69e903d7886.pdf</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L149" t="n">
+        <v>1226404</v>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>a69e903d7886bcd01cf3b4d34bb10798d152945594161598f6eb01c877a7c074</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>https://journal.ugm.ac.id/agritech/article/download/56792/32685</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr"/>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>出版版（agriTECH 41(4),2021,362–375；自身题名作者及DOI页首核验）</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr"/>
+      <c r="U149" t="inlineStr"/>
+      <c r="V149" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W149" t="inlineStr"/>
+      <c r="X149" t="inlineStr">
+        <is>
+          <t>2026-10-17T09:22:30.997493+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="b">
+        <v>1</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>R10492</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>R10492.main.3e5bb123d9d9d4ad</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E150" t="b">
+        <v>0</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>R10492_2024_Metagenomic_analysis_reveals_metabolic_mechanism_of_enhancing_lignocellulosic_anaerobic_digestion_me_3e5bb123d9d9.pdf</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R10492_2024_Metagenomic_analysis_reveals_metabolic_mechanism_of_enhancing_lignocellulosic_anaerobic_digestion_me_3e5bb123d9d9.pdf</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R10492_2024_Metagenomic_analysis_reveals_metabolic_mechanism_of_enhancing_lignocellulosic_anaerobic_digestion_me_3e5bb123d9d9.pdf</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R10492_2024_Metagenomic_analysis_reveals_metabolic_mechanism_of_enhancing_lignocellulosic_anaerobic_digestion_me_3e5bb123d9d9.pdf</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L150" t="n">
+        <v>1587578</v>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>3e5bb123d9d9d4add19c728f272d23055ccb980cf99cb60f516f7c2567ccee11</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>https://dspace.lib.cranfield.ac.uk/server/api/core/bitstreams/6052bc57-8e4b-48b8-aca7-00399ad7eace/content</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr"/>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>作者接受稿（PDF第一页明确Author Accepted Manuscript及正式DOI；不是预印本）</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr"/>
+      <c r="U150" t="inlineStr"/>
+      <c r="V150" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W150" t="inlineStr"/>
+      <c r="X150" t="inlineStr">
+        <is>
+          <t>2026-10-17T09:22:30.998716+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="b">
+        <v>1</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>R04928</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>R04928.main.9d47028c02204ac0</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E151" t="b">
+        <v>0</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>R04928_2019_MATHEMATICAL_MODEL_FOR_QUANTITATIVE_ANALYSIS_OF_ACIDOGENIC_PERFORMANCE_UNDER_MICROAERATION_CONDITION_9d47028c0220.pdf</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R04928_2019_MATHEMATICAL_MODEL_FOR_QUANTITATIVE_ANALYSIS_OF_ACIDOGENIC_PERFORMANCE_UNDER_MICROAERATION_CONDITION_9d47028c0220.pdf</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R04928_2019_MATHEMATICAL_MODEL_FOR_QUANTITATIVE_ANALYSIS_OF_ACIDOGENIC_PERFORMANCE_UNDER_MICROAERATION_CONDITION_9d47028c0220.pdf</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R04928_2019_MATHEMATICAL_MODEL_FOR_QUANTITATIVE_ANALYSIS_OF_ACIDOGENIC_PERFORMANCE_UNDER_MICROAERATION_CONDITION_9d47028c0220.pdf</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L151" t="n">
+        <v>614108</v>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>9d47028c02204ac08f73849bdf73af55c1e235aa3593b2b281d139b85d58607f</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>https://jrtppi.id/index.php/jrtppi/article/download/31/24</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr"/>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>期刊正式文章页提供的出版PDF（10(1):12–21）；PDF DOI栏为占位符，DOI由同一期刊文章页的citation_doi独立核对</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr"/>
+      <c r="U151" t="inlineStr"/>
+      <c r="V151" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W151" t="inlineStr"/>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>2026-10-17T09:22:30.999166+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="b">
+        <v>1</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>R13955</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>R13955.main.536763265cdc087f</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E152" t="b">
+        <v>0</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>R13955_2017_Biogas_Production_Thesis__20261017_variant_536763265cdc.pdf</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13955_2017_Biogas_Production_Thesis__20261017_variant_536763265cdc.pdf</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13955_2017_Biogas_Production_Thesis__20261017_variant_536763265cdc.pdf</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13955_2017_Biogas_Production_Thesis__20261017_variant_536763265cdc.pdf</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>14662119</v>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>536763265cdc087f2b0941e5305f33d2b98cc70ec29c58af4e238d1801b5fdce</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr"/>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>大学出版学位论文/仓储明确标注Publisher PDF；本轮另一字节副本，143页提取文字与已核验副本逐页相同</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr"/>
+      <c r="U152" t="inlineStr"/>
+      <c r="V152" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W152" t="inlineStr"/>
+      <c r="X152" t="inlineStr">
+        <is>
+          <t>2026-10-17T09:22:31.008715+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="b">
+        <v>0</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>R00735</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>R00735.evidence_html.fbe84942b58dfb81</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>evidence_html</t>
+        </is>
+      </c>
+      <c r="E153" t="b">
+        <v>0</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>publisher_article_page_20261017.html</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>original_files/source_evidence/R00735/publisher_article_page_20261017.html</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>original_files/source_evidence/R00735/publisher_article_page_20261017.html</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/source_evidence/R00735/publisher_article_page_20261017.html</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>18604</v>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>fbe84942b58dfb81b99138bd5095557649cf00b707c88f4a366d3346941335db</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>https://elibrary.asabe.org/abstract.asp?aid=44112&amp;t=3&amp;dabs=Y&amp;redir=&amp;redirType=</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr"/>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Article HTML with anonymous server session identifiers removed</t>
+        </is>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr"/>
+      <c r="U153" t="inlineStr"/>
+      <c r="V153" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W153" t="inlineStr"/>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>2026-10-17T09:22:31.008898+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Persist exact-item repository follow-ups and publisher download controls
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="H22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
         <v>1</v>
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="H61" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I61" t="n">
         <v>1</v>
@@ -3168,7 +3168,7 @@
         </is>
       </c>
       <c r="H64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
         <v>1</v>
@@ -3254,7 +3254,7 @@
         </is>
       </c>
       <c r="H66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
@@ -4028,7 +4028,7 @@
         </is>
       </c>
       <c r="H84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I84" t="n">
         <v>1</v>
@@ -6303,7 +6303,7 @@
         </is>
       </c>
       <c r="H137" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I137" t="n">
         <v>2</v>
@@ -7292,7 +7292,7 @@
         </is>
       </c>
       <c r="H160" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I160" t="n">
         <v>1</v>
@@ -7851,7 +7851,7 @@
         </is>
       </c>
       <c r="H173" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I173" t="n">
         <v>1</v>
@@ -11508,7 +11508,7 @@
         </is>
       </c>
       <c r="H260" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I260" t="n">
         <v>1</v>
@@ -14231,7 +14231,7 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.751670+00:00</t>
+          <t>2026-10-17T11:35:14.018757+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.752624+00:00</t>
+          <t>2026-10-17T11:35:14.019632+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.752645+00:00</t>
+          <t>2026-10-17T11:35:14.019651+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.752875+00:00</t>
+          <t>2026-10-17T11:35:14.019889+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.754222+00:00</t>
+          <t>2026-10-17T11:35:14.021061+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.754835+00:00</t>
+          <t>2026-10-17T11:35:14.021656+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.761392+00:00</t>
+          <t>2026-10-17T11:35:14.030091+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.764188+00:00</t>
+          <t>2026-10-17T11:35:14.032794+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.765166+00:00</t>
+          <t>2026-10-17T11:35:14.033763+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.765549+00:00</t>
+          <t>2026-10-17T11:35:14.034124+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.766311+00:00</t>
+          <t>2026-10-17T11:35:14.034962+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.767162+00:00</t>
+          <t>2026-10-17T11:35:14.035806+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.768395+00:00</t>
+          <t>2026-10-17T11:35:14.036746+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.768681+00:00</t>
+          <t>2026-10-17T11:35:14.037006+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.769582+00:00</t>
+          <t>2026-10-17T11:35:14.038213+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.779734+00:00</t>
+          <t>2026-10-17T11:35:14.051652+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.781079+00:00</t>
+          <t>2026-10-17T11:35:14.052513+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.783372+00:00</t>
+          <t>2026-10-17T11:35:14.053955+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.787143+00:00</t>
+          <t>2026-10-17T11:35:14.056695+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.788441+00:00</t>
+          <t>2026-10-17T11:35:14.057801+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.789692+00:00</t>
+          <t>2026-10-17T11:35:14.059133+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.796142+00:00</t>
+          <t>2026-10-17T11:35:14.064527+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.798941+00:00</t>
+          <t>2026-10-17T11:35:14.066989+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.800817+00:00</t>
+          <t>2026-10-17T11:35:14.068896+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.801592+00:00</t>
+          <t>2026-10-17T11:35:14.069627+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.801983+00:00</t>
+          <t>2026-10-17T11:35:14.070019+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.804439+00:00</t>
+          <t>2026-10-17T11:35:14.072241+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.806000+00:00</t>
+          <t>2026-10-17T11:35:14.073784+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.808507+00:00</t>
+          <t>2026-10-17T11:35:14.076357+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.810676+00:00</t>
+          <t>2026-10-17T11:35:14.078638+00:00</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.811242+00:00</t>
+          <t>2026-10-17T11:35:14.079355+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.811964+00:00</t>
+          <t>2026-10-17T11:35:14.079923+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.813925+00:00</t>
+          <t>2026-10-17T11:35:14.081675+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.817390+00:00</t>
+          <t>2026-10-17T11:35:14.084683+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.819921+00:00</t>
+          <t>2026-10-17T11:35:14.086961+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.821426+00:00</t>
+          <t>2026-10-17T11:35:14.089042+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.825250+00:00</t>
+          <t>2026-10-17T11:35:14.091975+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.826352+00:00</t>
+          <t>2026-10-17T11:35:14.092667+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.828097+00:00</t>
+          <t>2026-10-17T11:35:14.094232+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.828377+00:00</t>
+          <t>2026-10-17T11:35:14.094516+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.830584+00:00</t>
+          <t>2026-10-17T11:35:14.096422+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.834044+00:00</t>
+          <t>2026-10-17T11:35:14.099714+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.835586+00:00</t>
+          <t>2026-10-17T11:35:14.101117+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.836610+00:00</t>
+          <t>2026-10-17T11:35:14.102230+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.840104+00:00</t>
+          <t>2026-10-17T11:35:14.105080+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.841361+00:00</t>
+          <t>2026-10-17T11:35:14.106491+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.845669+00:00</t>
+          <t>2026-10-17T11:35:14.110249+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.847758+00:00</t>
+          <t>2026-10-17T11:35:14.111896+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.851150+00:00</t>
+          <t>2026-10-17T11:35:14.113778+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.852431+00:00</t>
+          <t>2026-10-17T11:35:14.114715+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.852933+00:00</t>
+          <t>2026-10-17T11:35:14.115147+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.853436+00:00</t>
+          <t>2026-10-17T11:35:14.115557+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.855272+00:00</t>
+          <t>2026-10-17T11:35:14.117005+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.856667+00:00</t>
+          <t>2026-10-17T11:35:14.118280+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.858413+00:00</t>
+          <t>2026-10-17T11:35:14.119763+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.858785+00:00</t>
+          <t>2026-10-17T11:35:14.120098+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.860464+00:00</t>
+          <t>2026-10-17T11:35:14.121256+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.862140+00:00</t>
+          <t>2026-10-17T11:35:14.122663+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.862916+00:00</t>
+          <t>2026-10-17T11:35:14.123231+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.863921+00:00</t>
+          <t>2026-10-17T11:35:14.124155+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.864275+00:00</t>
+          <t>2026-10-17T11:35:14.124573+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.870545+00:00</t>
+          <t>2026-10-17T11:35:14.130456+00:00</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.871098+00:00</t>
+          <t>2026-10-17T11:35:14.130885+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.871758+00:00</t>
+          <t>2026-10-17T11:35:14.131453+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.872342+00:00</t>
+          <t>2026-10-17T11:35:14.131877+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.874070+00:00</t>
+          <t>2026-10-17T11:35:14.133033+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.878062+00:00</t>
+          <t>2026-10-17T11:35:14.136659+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.878692+00:00</t>
+          <t>2026-10-17T11:35:14.136967+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.883985+00:00</t>
+          <t>2026-10-17T11:35:14.142054+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.884874+00:00</t>
+          <t>2026-10-17T11:35:14.142892+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.887125+00:00</t>
+          <t>2026-10-17T11:35:14.145095+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.888937+00:00</t>
+          <t>2026-10-17T11:35:14.147003+00:00</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.889875+00:00</t>
+          <t>2026-10-17T11:35:14.148103+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.891436+00:00</t>
+          <t>2026-10-17T11:35:14.149825+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.893929+00:00</t>
+          <t>2026-10-17T11:35:14.152405+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.903998+00:00</t>
+          <t>2026-10-17T11:35:14.165927+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.905761+00:00</t>
+          <t>2026-10-17T11:35:14.167614+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.905981+00:00</t>
+          <t>2026-10-17T11:35:14.167793+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.905997+00:00</t>
+          <t>2026-10-17T11:35:14.167808+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.913923+00:00</t>
+          <t>2026-10-17T11:35:14.173246+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.914535+00:00</t>
+          <t>2026-10-17T11:35:14.173989+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.914913+00:00</t>
+          <t>2026-10-17T11:35:14.174418+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.915354+00:00</t>
+          <t>2026-10-17T11:35:14.174816+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.916100+00:00</t>
+          <t>2026-10-17T11:35:14.175527+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.917738+00:00</t>
+          <t>2026-10-17T11:35:14.176893+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.918624+00:00</t>
+          <t>2026-10-17T11:35:14.177733+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.919156+00:00</t>
+          <t>2026-10-17T11:35:14.178065+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.919919+00:00</t>
+          <t>2026-10-17T11:35:14.178753+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.919937+00:00</t>
+          <t>2026-10-17T11:35:14.178766+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.919992+00:00</t>
+          <t>2026-10-17T11:35:14.178814+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.920219+00:00</t>
+          <t>2026-10-17T11:35:14.179049+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.920366+00:00</t>
+          <t>2026-10-17T11:35:14.179167+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.920494+00:00</t>
+          <t>2026-10-17T11:35:14.179282+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.920873+00:00</t>
+          <t>2026-10-17T11:35:14.179980+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.921087+00:00</t>
+          <t>2026-10-17T11:35:14.180239+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.921145+00:00</t>
+          <t>2026-10-17T11:35:14.180345+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.921213+00:00</t>
+          <t>2026-10-17T11:35:14.180413+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.921777+00:00</t>
+          <t>2026-10-17T11:35:14.180563+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.925374+00:00</t>
+          <t>2026-10-17T11:35:14.180608+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.925994+00:00</t>
+          <t>2026-10-17T11:35:14.181156+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.926075+00:00</t>
+          <t>2026-10-17T11:35:14.181219+00:00</t>
         </is>
       </c>
     </row>
@@ -35215,7 +35215,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.926088+00:00</t>
+          <t>2026-10-17T11:35:14.181231+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35323,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.936629+00:00</t>
+          <t>2026-10-17T11:35:14.195987+00:00</t>
         </is>
       </c>
     </row>
@@ -35427,7 +35427,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.936812+00:00</t>
+          <t>2026-10-17T11:35:14.196091+00:00</t>
         </is>
       </c>
     </row>
@@ -35535,7 +35535,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.937009+00:00</t>
+          <t>2026-10-17T11:35:14.196232+00:00</t>
         </is>
       </c>
     </row>
@@ -35643,7 +35643,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.937278+00:00</t>
+          <t>2026-10-17T11:35:14.196552+00:00</t>
         </is>
       </c>
     </row>
@@ -35751,7 +35751,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.938650+00:00</t>
+          <t>2026-10-17T11:35:14.197741+00:00</t>
         </is>
       </c>
     </row>
@@ -35853,7 +35853,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.938766+00:00</t>
+          <t>2026-10-17T11:35:14.197840+00:00</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35947,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.938779+00:00</t>
+          <t>2026-10-17T11:35:14.197853+00:00</t>
         </is>
       </c>
     </row>
@@ -36049,7 +36049,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.938877+00:00</t>
+          <t>2026-10-17T11:35:14.197934+00:00</t>
         </is>
       </c>
     </row>
@@ -36151,7 +36151,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.938970+00:00</t>
+          <t>2026-10-17T11:35:14.198016+00:00</t>
         </is>
       </c>
     </row>
@@ -36253,7 +36253,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.939087+00:00</t>
+          <t>2026-10-17T11:35:14.198121+00:00</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36347,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.939097+00:00</t>
+          <t>2026-10-17T11:35:14.198131+00:00</t>
         </is>
       </c>
     </row>
@@ -36449,7 +36449,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.939916+00:00</t>
+          <t>2026-10-17T11:35:14.198308+00:00</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36543,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.939951+00:00</t>
+          <t>2026-10-17T11:35:14.198321+00:00</t>
         </is>
       </c>
     </row>
@@ -36645,7 +36645,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940092+00:00</t>
+          <t>2026-10-17T11:35:14.198424+00:00</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940107+00:00</t>
+          <t>2026-10-17T11:35:14.198435+00:00</t>
         </is>
       </c>
     </row>
@@ -36841,7 +36841,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940406+00:00</t>
+          <t>2026-10-17T11:35:14.198579+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36935,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940431+00:00</t>
+          <t>2026-10-17T11:35:14.198589+00:00</t>
         </is>
       </c>
     </row>
@@ -37037,7 +37037,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940541+00:00</t>
+          <t>2026-10-17T11:35:14.198676+00:00</t>
         </is>
       </c>
     </row>
@@ -37139,7 +37139,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940685+00:00</t>
+          <t>2026-10-17T11:35:14.198992+00:00</t>
         </is>
       </c>
     </row>
@@ -37233,7 +37233,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940698+00:00</t>
+          <t>2026-10-17T11:35:14.199017+00:00</t>
         </is>
       </c>
     </row>
@@ -37335,7 +37335,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940828+00:00</t>
+          <t>2026-10-17T11:35:14.199151+00:00</t>
         </is>
       </c>
     </row>
@@ -37429,7 +37429,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940839+00:00</t>
+          <t>2026-10-17T11:35:14.199163+00:00</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37531,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.940951+00:00</t>
+          <t>2026-10-17T11:35:14.199279+00:00</t>
         </is>
       </c>
     </row>
@@ -37633,7 +37633,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.941190+00:00</t>
+          <t>2026-10-17T11:35:14.199533+00:00</t>
         </is>
       </c>
     </row>
@@ -37727,7 +37727,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.941202+00:00</t>
+          <t>2026-10-17T11:35:14.199546+00:00</t>
         </is>
       </c>
     </row>
@@ -37829,7 +37829,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.941413+00:00</t>
+          <t>2026-10-17T11:35:14.199713+00:00</t>
         </is>
       </c>
     </row>
@@ -37931,7 +37931,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.941760+00:00</t>
+          <t>2026-10-17T11:35:14.199907+00:00</t>
         </is>
       </c>
     </row>
@@ -38033,7 +38033,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.941985+00:00</t>
+          <t>2026-10-17T11:35:14.200099+00:00</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.942000+00:00</t>
+          <t>2026-10-17T11:35:14.200111+00:00</t>
         </is>
       </c>
     </row>
@@ -38229,7 +38229,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.942116+00:00</t>
+          <t>2026-10-17T11:35:14.200219+00:00</t>
         </is>
       </c>
     </row>
@@ -38323,7 +38323,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.942127+00:00</t>
+          <t>2026-10-17T11:35:14.200229+00:00</t>
         </is>
       </c>
     </row>
@@ -38425,7 +38425,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.942273+00:00</t>
+          <t>2026-10-17T11:35:14.200334+00:00</t>
         </is>
       </c>
     </row>
@@ -38533,7 +38533,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.943473+00:00</t>
+          <t>2026-10-17T11:35:14.201468+00:00</t>
         </is>
       </c>
     </row>
@@ -38625,7 +38625,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.957014+00:00</t>
+          <t>2026-10-17T11:35:14.216859+00:00</t>
         </is>
       </c>
     </row>
@@ -38725,7 +38725,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.957697+00:00</t>
+          <t>2026-10-17T11:35:14.217364+00:00</t>
         </is>
       </c>
     </row>
@@ -38813,7 +38813,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.957723+00:00</t>
+          <t>2026-10-17T11:35:14.217382+00:00</t>
         </is>
       </c>
     </row>
@@ -38913,7 +38913,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.958921+00:00</t>
+          <t>2026-10-17T11:35:14.218605+00:00</t>
         </is>
       </c>
     </row>
@@ -39013,7 +39013,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.962728+00:00</t>
+          <t>2026-10-17T11:35:14.222010+00:00</t>
         </is>
       </c>
     </row>
@@ -39113,7 +39113,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.963766+00:00</t>
+          <t>2026-10-17T11:35:14.222894+00:00</t>
         </is>
       </c>
     </row>
@@ -39205,7 +39205,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.963792+00:00</t>
+          <t>2026-10-17T11:35:14.222910+00:00</t>
         </is>
       </c>
     </row>
@@ -39305,7 +39305,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.964829+00:00</t>
+          <t>2026-10-17T11:35:14.223576+00:00</t>
         </is>
       </c>
     </row>
@@ -39397,7 +39397,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.964856+00:00</t>
+          <t>2026-10-17T11:35:14.223590+00:00</t>
         </is>
       </c>
     </row>
@@ -39428,14 +39428,26 @@
           <t>R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr"/>
-      <c r="H146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+        </is>
+      </c>
       <c r="I146" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-fulltexts/R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+        </is>
+      </c>
       <c r="K146" t="inlineStr">
         <is>
           <t>pdf</t>
@@ -39451,23 +39463,23 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>https://technology.matthey.com/docserver/fulltext/jmtr/67/4/Zimmerman_16a_Imp.pdf?expires=1791804248&amp;id=id&amp;accname=guest&amp;checksum=934385598F9DDA2349B917F1B50C4858</t>
+          <t>https://technology.matthey.com/content/journals/10.1595/205651323X16778518231554</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr"/>
       <c r="R146" t="inlineStr">
         <is>
-          <t>出版版本（原页出版信息）</t>
+          <t>Version of record; Johnson Matthey Technology Review 67(4), 2023, pp371–401</t>
         </is>
       </c>
       <c r="S146" t="inlineStr">
@@ -39489,7 +39501,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.964859+00:00</t>
+          <t>2026-10-17T11:35:14.224421+00:00</t>
         </is>
       </c>
     </row>
@@ -39577,7 +39589,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.964863+00:00</t>
+          <t>2026-10-17T11:35:14.224435+00:00</t>
         </is>
       </c>
     </row>
@@ -39669,7 +39681,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.964866+00:00</t>
+          <t>2026-10-17T11:35:14.224439+00:00</t>
         </is>
       </c>
     </row>
@@ -39765,7 +39777,7 @@
       <c r="W149" t="inlineStr"/>
       <c r="X149" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.965774+00:00</t>
+          <t>2026-10-17T11:35:14.225200+00:00</t>
         </is>
       </c>
     </row>
@@ -39861,7 +39873,7 @@
       <c r="W150" t="inlineStr"/>
       <c r="X150" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.966849+00:00</t>
+          <t>2026-10-17T11:35:14.226235+00:00</t>
         </is>
       </c>
     </row>
@@ -39957,7 +39969,7 @@
       <c r="W151" t="inlineStr"/>
       <c r="X151" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.967395+00:00</t>
+          <t>2026-10-17T11:35:14.226693+00:00</t>
         </is>
       </c>
     </row>
@@ -40053,7 +40065,7 @@
       <c r="W152" t="inlineStr"/>
       <c r="X152" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.978374+00:00</t>
+          <t>2026-10-17T11:35:14.240034+00:00</t>
         </is>
       </c>
     </row>
@@ -40149,7 +40161,7 @@
       <c r="W153" t="inlineStr"/>
       <c r="X153" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.978607+00:00</t>
+          <t>2026-10-17T11:35:14.240270+00:00</t>
         </is>
       </c>
     </row>
@@ -40245,7 +40257,7 @@
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.978789+00:00</t>
+          <t>2026-10-17T11:35:14.240483+00:00</t>
         </is>
       </c>
     </row>
@@ -40341,7 +40353,7 @@
       <c r="W155" t="inlineStr"/>
       <c r="X155" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.979256+00:00</t>
+          <t>2026-10-17T11:35:14.240923+00:00</t>
         </is>
       </c>
     </row>
@@ -40437,7 +40449,7 @@
       <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.979666+00:00</t>
+          <t>2026-10-17T11:35:14.241199+00:00</t>
         </is>
       </c>
     </row>
@@ -40533,7 +40545,7 @@
       <c r="W157" t="inlineStr"/>
       <c r="X157" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.980044+00:00</t>
+          <t>2026-10-17T11:35:14.241696+00:00</t>
         </is>
       </c>
     </row>
@@ -40629,7 +40641,7 @@
       <c r="W158" t="inlineStr"/>
       <c r="X158" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.981284+00:00</t>
+          <t>2026-10-17T11:35:14.243009+00:00</t>
         </is>
       </c>
     </row>
@@ -40725,7 +40737,7 @@
       <c r="W159" t="inlineStr"/>
       <c r="X159" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.983167+00:00</t>
+          <t>2026-10-17T11:35:14.244939+00:00</t>
         </is>
       </c>
     </row>
@@ -40821,7 +40833,7 @@
       <c r="W160" t="inlineStr"/>
       <c r="X160" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.983819+00:00</t>
+          <t>2026-10-17T11:35:14.245709+00:00</t>
         </is>
       </c>
     </row>
@@ -40917,7 +40929,7 @@
       <c r="W161" t="inlineStr"/>
       <c r="X161" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.984113+00:00</t>
+          <t>2026-10-17T11:35:14.246016+00:00</t>
         </is>
       </c>
     </row>
@@ -41013,7 +41025,7 @@
       <c r="W162" t="inlineStr"/>
       <c r="X162" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.984178+00:00</t>
+          <t>2026-10-17T11:35:14.246073+00:00</t>
         </is>
       </c>
     </row>
@@ -41109,7 +41121,7 @@
       <c r="W163" t="inlineStr"/>
       <c r="X163" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.984257+00:00</t>
+          <t>2026-10-17T11:35:14.246141+00:00</t>
         </is>
       </c>
     </row>
@@ -41205,7 +41217,7 @@
       <c r="W164" t="inlineStr"/>
       <c r="X164" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.984593+00:00</t>
+          <t>2026-10-17T11:35:14.246806+00:00</t>
         </is>
       </c>
     </row>
@@ -41301,7 +41313,7 @@
       <c r="W165" t="inlineStr"/>
       <c r="X165" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.985036+00:00</t>
+          <t>2026-10-17T11:35:14.247624+00:00</t>
         </is>
       </c>
     </row>
@@ -41397,7 +41409,7 @@
       <c r="W166" t="inlineStr"/>
       <c r="X166" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.985412+00:00</t>
+          <t>2026-10-17T11:35:14.248464+00:00</t>
         </is>
       </c>
     </row>
@@ -41493,7 +41505,7 @@
       <c r="W167" t="inlineStr"/>
       <c r="X167" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.986247+00:00</t>
+          <t>2026-10-17T11:35:14.250105+00:00</t>
         </is>
       </c>
     </row>
@@ -41589,7 +41601,7 @@
       <c r="W168" t="inlineStr"/>
       <c r="X168" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.986691+00:00</t>
+          <t>2026-10-17T11:35:14.250869+00:00</t>
         </is>
       </c>
     </row>
@@ -41685,7 +41697,7 @@
       <c r="W169" t="inlineStr"/>
       <c r="X169" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.986858+00:00</t>
+          <t>2026-10-17T11:35:14.251055+00:00</t>
         </is>
       </c>
     </row>
@@ -41781,7 +41793,7 @@
       <c r="W170" t="inlineStr"/>
       <c r="X170" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.987011+00:00</t>
+          <t>2026-10-17T11:35:14.251223+00:00</t>
         </is>
       </c>
     </row>
@@ -41877,7 +41889,7 @@
       <c r="W171" t="inlineStr"/>
       <c r="X171" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.987148+00:00</t>
+          <t>2026-10-17T11:35:14.251749+00:00</t>
         </is>
       </c>
     </row>
@@ -41973,7 +41985,7 @@
       <c r="W172" t="inlineStr"/>
       <c r="X172" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.987208+00:00</t>
+          <t>2026-10-17T11:35:14.252004+00:00</t>
         </is>
       </c>
     </row>
@@ -42069,7 +42081,7 @@
       <c r="W173" t="inlineStr"/>
       <c r="X173" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.987277+00:00</t>
+          <t>2026-10-17T11:35:14.252081+00:00</t>
         </is>
       </c>
     </row>
@@ -42165,7 +42177,7 @@
       <c r="W174" t="inlineStr"/>
       <c r="X174" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.987689+00:00</t>
+          <t>2026-10-17T11:35:14.252470+00:00</t>
         </is>
       </c>
     </row>
@@ -42261,7 +42273,7 @@
       <c r="W175" t="inlineStr"/>
       <c r="X175" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.988072+00:00</t>
+          <t>2026-10-17T11:35:14.252842+00:00</t>
         </is>
       </c>
     </row>
@@ -42357,7 +42369,7 @@
       <c r="W176" t="inlineStr"/>
       <c r="X176" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.988404+00:00</t>
+          <t>2026-10-17T11:35:14.253139+00:00</t>
         </is>
       </c>
     </row>
@@ -42453,7 +42465,7 @@
       <c r="W177" t="inlineStr"/>
       <c r="X177" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.988748+00:00</t>
+          <t>2026-10-17T11:35:14.253566+00:00</t>
         </is>
       </c>
     </row>
@@ -42549,7 +42561,7 @@
       <c r="W178" t="inlineStr"/>
       <c r="X178" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.988878+00:00</t>
+          <t>2026-10-17T11:35:14.253811+00:00</t>
         </is>
       </c>
     </row>
@@ -42645,7 +42657,7 @@
       <c r="W179" t="inlineStr"/>
       <c r="X179" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.989778+00:00</t>
+          <t>2026-10-17T11:35:14.254663+00:00</t>
         </is>
       </c>
     </row>
@@ -42741,7 +42753,7 @@
       <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.990493+00:00</t>
+          <t>2026-10-17T11:35:14.255415+00:00</t>
         </is>
       </c>
     </row>
@@ -42837,7 +42849,7 @@
       <c r="W181" t="inlineStr"/>
       <c r="X181" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.990624+00:00</t>
+          <t>2026-10-17T11:35:14.255538+00:00</t>
         </is>
       </c>
     </row>
@@ -42933,7 +42945,7 @@
       <c r="W182" t="inlineStr"/>
       <c r="X182" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.991122+00:00</t>
+          <t>2026-10-17T11:35:14.256032+00:00</t>
         </is>
       </c>
     </row>
@@ -43029,7 +43041,7 @@
       <c r="W183" t="inlineStr"/>
       <c r="X183" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.991312+00:00</t>
+          <t>2026-10-17T11:35:14.256099+00:00</t>
         </is>
       </c>
     </row>
@@ -43125,7 +43137,7 @@
       <c r="W184" t="inlineStr"/>
       <c r="X184" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.991391+00:00</t>
+          <t>2026-10-17T11:35:14.256153+00:00</t>
         </is>
       </c>
     </row>
@@ -43221,7 +43233,7 @@
       <c r="W185" t="inlineStr"/>
       <c r="X185" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.991746+00:00</t>
+          <t>2026-10-17T11:35:14.256461+00:00</t>
         </is>
       </c>
     </row>
@@ -43317,7 +43329,7 @@
       <c r="W186" t="inlineStr"/>
       <c r="X186" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.991813+00:00</t>
+          <t>2026-10-17T11:35:14.256514+00:00</t>
         </is>
       </c>
     </row>
@@ -43413,7 +43425,7 @@
       <c r="W187" t="inlineStr"/>
       <c r="X187" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.991982+00:00</t>
+          <t>2026-10-17T11:35:14.256676+00:00</t>
         </is>
       </c>
     </row>
@@ -43509,7 +43521,7 @@
       <c r="W188" t="inlineStr"/>
       <c r="X188" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.992038+00:00</t>
+          <t>2026-10-17T11:35:14.256727+00:00</t>
         </is>
       </c>
     </row>
@@ -43605,7 +43617,7 @@
       <c r="W189" t="inlineStr"/>
       <c r="X189" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.992397+00:00</t>
+          <t>2026-10-17T11:35:14.257060+00:00</t>
         </is>
       </c>
     </row>
@@ -43701,7 +43713,7 @@
       <c r="W190" t="inlineStr"/>
       <c r="X190" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.992467+00:00</t>
+          <t>2026-10-17T11:35:14.257120+00:00</t>
         </is>
       </c>
     </row>
@@ -43797,7 +43809,7 @@
       <c r="W191" t="inlineStr"/>
       <c r="X191" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.993143+00:00</t>
+          <t>2026-10-17T11:35:14.257738+00:00</t>
         </is>
       </c>
     </row>
@@ -43893,7 +43905,7 @@
       <c r="W192" t="inlineStr"/>
       <c r="X192" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.993251+00:00</t>
+          <t>2026-10-17T11:35:14.257822+00:00</t>
         </is>
       </c>
     </row>
@@ -43989,7 +44001,7 @@
       <c r="W193" t="inlineStr"/>
       <c r="X193" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.993756+00:00</t>
+          <t>2026-10-17T11:35:14.258161+00:00</t>
         </is>
       </c>
     </row>
@@ -44085,7 +44097,7 @@
       <c r="W194" t="inlineStr"/>
       <c r="X194" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.994053+00:00</t>
+          <t>2026-10-17T11:35:14.258393+00:00</t>
         </is>
       </c>
     </row>
@@ -44181,7 +44193,7 @@
       <c r="W195" t="inlineStr"/>
       <c r="X195" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.994371+00:00</t>
+          <t>2026-10-17T11:35:14.258672+00:00</t>
         </is>
       </c>
     </row>
@@ -44277,7 +44289,7 @@
       <c r="W196" t="inlineStr"/>
       <c r="X196" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.994512+00:00</t>
+          <t>2026-10-17T11:35:14.258730+00:00</t>
         </is>
       </c>
     </row>
@@ -44373,7 +44385,7 @@
       <c r="W197" t="inlineStr"/>
       <c r="X197" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.994652+00:00</t>
+          <t>2026-10-17T11:35:14.258926+00:00</t>
         </is>
       </c>
     </row>
@@ -44469,7 +44481,7 @@
       <c r="W198" t="inlineStr"/>
       <c r="X198" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.994991+00:00</t>
+          <t>2026-10-17T11:35:14.259282+00:00</t>
         </is>
       </c>
     </row>
@@ -44565,7 +44577,7 @@
       <c r="W199" t="inlineStr"/>
       <c r="X199" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.995355+00:00</t>
+          <t>2026-10-17T11:35:14.259733+00:00</t>
         </is>
       </c>
     </row>
@@ -44661,7 +44673,7 @@
       <c r="W200" t="inlineStr"/>
       <c r="X200" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.995432+00:00</t>
+          <t>2026-10-17T11:35:14.259821+00:00</t>
         </is>
       </c>
     </row>
@@ -44757,7 +44769,7 @@
       <c r="W201" t="inlineStr"/>
       <c r="X201" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.995951+00:00</t>
+          <t>2026-10-17T11:35:14.260400+00:00</t>
         </is>
       </c>
     </row>
@@ -44853,7 +44865,7 @@
       <c r="W202" t="inlineStr"/>
       <c r="X202" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.996275+00:00</t>
+          <t>2026-10-17T11:35:14.260814+00:00</t>
         </is>
       </c>
     </row>
@@ -44949,7 +44961,7 @@
       <c r="W203" t="inlineStr"/>
       <c r="X203" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.996417+00:00</t>
+          <t>2026-10-17T11:35:14.260887+00:00</t>
         </is>
       </c>
     </row>
@@ -45045,7 +45057,7 @@
       <c r="W204" t="inlineStr"/>
       <c r="X204" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.996732+00:00</t>
+          <t>2026-10-17T11:35:14.261183+00:00</t>
         </is>
       </c>
     </row>
@@ -45141,7 +45153,7 @@
       <c r="W205" t="inlineStr"/>
       <c r="X205" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.996796+00:00</t>
+          <t>2026-10-17T11:35:14.261247+00:00</t>
         </is>
       </c>
     </row>
@@ -45237,7 +45249,7 @@
       <c r="W206" t="inlineStr"/>
       <c r="X206" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.996874+00:00</t>
+          <t>2026-10-17T11:35:14.261346+00:00</t>
         </is>
       </c>
     </row>
@@ -45333,7 +45345,7 @@
       <c r="W207" t="inlineStr"/>
       <c r="X207" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.996938+00:00</t>
+          <t>2026-10-17T11:35:14.261416+00:00</t>
         </is>
       </c>
     </row>
@@ -45429,7 +45441,7 @@
       <c r="W208" t="inlineStr"/>
       <c r="X208" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.996994+00:00</t>
+          <t>2026-10-17T11:35:14.261548+00:00</t>
         </is>
       </c>
     </row>
@@ -45525,7 +45537,7 @@
       <c r="W209" t="inlineStr"/>
       <c r="X209" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.997048+00:00</t>
+          <t>2026-10-17T11:35:14.261604+00:00</t>
         </is>
       </c>
     </row>
@@ -45621,7 +45633,7 @@
       <c r="W210" t="inlineStr"/>
       <c r="X210" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.997423+00:00</t>
+          <t>2026-10-17T11:35:14.261918+00:00</t>
         </is>
       </c>
     </row>
@@ -45717,7 +45729,7 @@
       <c r="W211" t="inlineStr"/>
       <c r="X211" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.997579+00:00</t>
+          <t>2026-10-17T11:35:14.262045+00:00</t>
         </is>
       </c>
     </row>
@@ -45813,7 +45825,7 @@
       <c r="W212" t="inlineStr"/>
       <c r="X212" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.997886+00:00</t>
+          <t>2026-10-17T11:35:14.262204+00:00</t>
         </is>
       </c>
     </row>
@@ -45880,7 +45892,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P213" t="inlineStr">
@@ -45909,7 +45921,7 @@
       <c r="W213" t="inlineStr"/>
       <c r="X213" t="inlineStr">
         <is>
-          <t>2026-10-17T09:57:00.998123+00:00</t>
+          <t>2026-10-17T11:35:14.262406+00:00</t>
         </is>
       </c>
     </row>
@@ -45924,7 +45936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46688,12 +46700,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>R09240</t>
+          <t>R13899</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R09240.main.da8dbeb874b19b59</t>
+          <t>R13899.main.19143e56fa77ce99</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -46703,20 +46715,16 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>da8dbeb874b19b59dbea53c11766a209aaa0b0bc319e2128c94340ae78cecfaf</t>
+          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1315227</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://technology.matthey.com/docserver/fulltext/jmtr/67/4/Zimmerman_16a_Imp.pdf?expires=1791804248&amp;id=id&amp;accname=guest&amp;checksum=934385598F9DDA2349B917F1B50C4858</t>
-        </is>
-      </c>
+        <v>479092</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>R09240_2023_Microbubble_Intensification_of_Bioprocessing.pdf</t>
+          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -46728,12 +46736,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>R13899</t>
+          <t>R13955</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R13899.main.19143e56fa77ce99</t>
+          <t>R13955.main.6714f79deccd703d</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -46743,59 +46751,23 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
+          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>479092</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
+        <v>14662119</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>R13955</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>R13955.main.6714f79deccd703d</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>14662119</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
         <is>
           <t>历史已获取，当前原件未恢复</t>
         </is>

</xml_diff>

<commit_message>
Register complete university thesis PDF sets and reconcile SI partial success
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="H22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
         <v>1</v>
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="H61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I61" t="n">
         <v>1</v>
@@ -3168,7 +3168,7 @@
         </is>
       </c>
       <c r="H64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I64" t="n">
         <v>1</v>
@@ -3254,7 +3254,7 @@
         </is>
       </c>
       <c r="H66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
@@ -4028,7 +4028,7 @@
         </is>
       </c>
       <c r="H84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I84" t="n">
         <v>1</v>
@@ -6303,7 +6303,7 @@
         </is>
       </c>
       <c r="H137" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I137" t="n">
         <v>2</v>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>access_failed</t>
+          <t>partial_or_access_failed</t>
         </is>
       </c>
       <c r="H141" t="b">
@@ -7292,7 +7292,7 @@
         </is>
       </c>
       <c r="H160" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I160" t="n">
         <v>1</v>
@@ -7851,7 +7851,7 @@
         </is>
       </c>
       <c r="H173" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I173" t="n">
         <v>1</v>
@@ -11508,7 +11508,7 @@
         </is>
       </c>
       <c r="H260" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I260" t="n">
         <v>1</v>
@@ -23885,7 +23885,7 @@
       </c>
       <c r="F550" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G550" t="inlineStr">
@@ -23928,7 +23928,7 @@
       </c>
       <c r="F551" t="inlineStr">
         <is>
-          <t>not_downloaded</t>
+          <t>downloaded_verified</t>
         </is>
       </c>
       <c r="G551" t="inlineStr">
@@ -24118,7 +24118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X213"/>
+  <dimension ref="A1:X227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.018757+00:00</t>
+          <t>2026-10-17T11:36:14.465524+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.019632+00:00</t>
+          <t>2026-10-17T11:36:14.466490+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.019651+00:00</t>
+          <t>2026-10-17T11:36:14.466518+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.019889+00:00</t>
+          <t>2026-10-17T11:36:14.466816+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.021061+00:00</t>
+          <t>2026-10-17T11:36:14.468030+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.021656+00:00</t>
+          <t>2026-10-17T11:36:14.468576+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.030091+00:00</t>
+          <t>2026-10-17T11:36:14.474688+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.032794+00:00</t>
+          <t>2026-10-17T11:36:14.477536+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.033763+00:00</t>
+          <t>2026-10-17T11:36:14.479122+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.034124+00:00</t>
+          <t>2026-10-17T11:36:14.479537+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.034962+00:00</t>
+          <t>2026-10-17T11:36:14.480424+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.035806+00:00</t>
+          <t>2026-10-17T11:36:14.481286+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.036746+00:00</t>
+          <t>2026-10-17T11:36:14.482579+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.037006+00:00</t>
+          <t>2026-10-17T11:36:14.482849+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.038213+00:00</t>
+          <t>2026-10-17T11:36:14.483863+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.051652+00:00</t>
+          <t>2026-10-17T11:36:14.493591+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.052513+00:00</t>
+          <t>2026-10-17T11:36:14.494479+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.053955+00:00</t>
+          <t>2026-10-17T11:36:14.495966+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.056695+00:00</t>
+          <t>2026-10-17T11:36:14.498481+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.057801+00:00</t>
+          <t>2026-10-17T11:36:14.499740+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.059133+00:00</t>
+          <t>2026-10-17T11:36:14.501177+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.064527+00:00</t>
+          <t>2026-10-17T11:36:14.505575+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.066989+00:00</t>
+          <t>2026-10-17T11:36:14.507982+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.068896+00:00</t>
+          <t>2026-10-17T11:36:14.509983+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.069627+00:00</t>
+          <t>2026-10-17T11:36:14.510921+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.070019+00:00</t>
+          <t>2026-10-17T11:36:14.511386+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.072241+00:00</t>
+          <t>2026-10-17T11:36:14.513444+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.073784+00:00</t>
+          <t>2026-10-17T11:36:14.514784+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.076357+00:00</t>
+          <t>2026-10-17T11:36:14.516827+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.078638+00:00</t>
+          <t>2026-10-17T11:36:14.519113+00:00</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.079355+00:00</t>
+          <t>2026-10-17T11:36:14.519817+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.079923+00:00</t>
+          <t>2026-10-17T11:36:14.520406+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.081675+00:00</t>
+          <t>2026-10-17T11:36:14.522372+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.084683+00:00</t>
+          <t>2026-10-17T11:36:14.525241+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.086961+00:00</t>
+          <t>2026-10-17T11:36:14.527771+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.089042+00:00</t>
+          <t>2026-10-17T11:36:14.529045+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.091975+00:00</t>
+          <t>2026-10-17T11:36:14.532351+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.092667+00:00</t>
+          <t>2026-10-17T11:36:14.533225+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.094232+00:00</t>
+          <t>2026-10-17T11:36:14.535079+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.094516+00:00</t>
+          <t>2026-10-17T11:36:14.535389+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.096422+00:00</t>
+          <t>2026-10-17T11:36:14.537394+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.099714+00:00</t>
+          <t>2026-10-17T11:36:14.540573+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.101117+00:00</t>
+          <t>2026-10-17T11:36:14.542368+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.102230+00:00</t>
+          <t>2026-10-17T11:36:14.543044+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.105080+00:00</t>
+          <t>2026-10-17T11:36:14.545728+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.106491+00:00</t>
+          <t>2026-10-17T11:36:14.546859+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.110249+00:00</t>
+          <t>2026-10-17T11:36:14.550406+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.111896+00:00</t>
+          <t>2026-10-17T11:36:14.552080+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.113778+00:00</t>
+          <t>2026-10-17T11:36:14.554373+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.114715+00:00</t>
+          <t>2026-10-17T11:36:14.555551+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.115147+00:00</t>
+          <t>2026-10-17T11:36:14.556051+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.115557+00:00</t>
+          <t>2026-10-17T11:36:14.556553+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.117005+00:00</t>
+          <t>2026-10-17T11:36:14.558371+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.118280+00:00</t>
+          <t>2026-10-17T11:36:14.559673+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.119763+00:00</t>
+          <t>2026-10-17T11:36:14.561285+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.120098+00:00</t>
+          <t>2026-10-17T11:36:14.561721+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.121256+00:00</t>
+          <t>2026-10-17T11:36:14.562928+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.122663+00:00</t>
+          <t>2026-10-17T11:36:14.564502+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.123231+00:00</t>
+          <t>2026-10-17T11:36:14.565160+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.124155+00:00</t>
+          <t>2026-10-17T11:36:14.566363+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.124573+00:00</t>
+          <t>2026-10-17T11:36:14.566789+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.130456+00:00</t>
+          <t>2026-10-17T11:36:14.572494+00:00</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.130885+00:00</t>
+          <t>2026-10-17T11:36:14.572954+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.131453+00:00</t>
+          <t>2026-10-17T11:36:14.573592+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.131877+00:00</t>
+          <t>2026-10-17T11:36:14.574027+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.133033+00:00</t>
+          <t>2026-10-17T11:36:14.575107+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.136659+00:00</t>
+          <t>2026-10-17T11:36:14.578176+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.136967+00:00</t>
+          <t>2026-10-17T11:36:14.578465+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.142054+00:00</t>
+          <t>2026-10-17T11:36:14.582641+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.142892+00:00</t>
+          <t>2026-10-17T11:36:14.583386+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.145095+00:00</t>
+          <t>2026-10-17T11:36:14.585584+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.147003+00:00</t>
+          <t>2026-10-17T11:36:14.587478+00:00</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.148103+00:00</t>
+          <t>2026-10-17T11:36:14.588430+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.149825+00:00</t>
+          <t>2026-10-17T11:36:14.590122+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.152405+00:00</t>
+          <t>2026-10-17T11:36:14.592871+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.165927+00:00</t>
+          <t>2026-10-17T11:36:14.602777+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.167614+00:00</t>
+          <t>2026-10-17T11:36:14.604230+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.167793+00:00</t>
+          <t>2026-10-17T11:36:14.604441+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.167808+00:00</t>
+          <t>2026-10-17T11:36:14.604457+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.173246+00:00</t>
+          <t>2026-10-17T11:36:14.610623+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.173989+00:00</t>
+          <t>2026-10-17T11:36:14.611106+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.174418+00:00</t>
+          <t>2026-10-17T11:36:14.611500+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.174816+00:00</t>
+          <t>2026-10-17T11:36:14.611957+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.175527+00:00</t>
+          <t>2026-10-17T11:36:14.612754+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.176893+00:00</t>
+          <t>2026-10-17T11:36:14.614415+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.177733+00:00</t>
+          <t>2026-10-17T11:36:14.615246+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.178065+00:00</t>
+          <t>2026-10-17T11:36:14.615604+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.178753+00:00</t>
+          <t>2026-10-17T11:36:14.616476+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.178766+00:00</t>
+          <t>2026-10-17T11:36:14.616503+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.178814+00:00</t>
+          <t>2026-10-17T11:36:14.616567+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.179049+00:00</t>
+          <t>2026-10-17T11:36:14.616797+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.179167+00:00</t>
+          <t>2026-10-17T11:36:14.616922+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.179282+00:00</t>
+          <t>2026-10-17T11:36:14.617038+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.179980+00:00</t>
+          <t>2026-10-17T11:36:14.617446+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.180239+00:00</t>
+          <t>2026-10-17T11:36:14.617683+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.180345+00:00</t>
+          <t>2026-10-17T11:36:14.617739+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.180413+00:00</t>
+          <t>2026-10-17T11:36:14.617799+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.180563+00:00</t>
+          <t>2026-10-17T11:36:14.617954+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.180608+00:00</t>
+          <t>2026-10-17T11:36:14.617998+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.181156+00:00</t>
+          <t>2026-10-17T11:36:14.618662+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.181219+00:00</t>
+          <t>2026-10-17T11:36:14.618738+00:00</t>
         </is>
       </c>
     </row>
@@ -35215,7 +35215,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.181231+00:00</t>
+          <t>2026-10-17T11:36:14.618751+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35323,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.195987+00:00</t>
+          <t>2026-10-17T11:36:14.630430+00:00</t>
         </is>
       </c>
     </row>
@@ -35427,7 +35427,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.196091+00:00</t>
+          <t>2026-10-17T11:36:14.630538+00:00</t>
         </is>
       </c>
     </row>
@@ -35535,7 +35535,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.196232+00:00</t>
+          <t>2026-10-17T11:36:14.630688+00:00</t>
         </is>
       </c>
     </row>
@@ -35643,7 +35643,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.196552+00:00</t>
+          <t>2026-10-17T11:36:14.630932+00:00</t>
         </is>
       </c>
     </row>
@@ -35751,7 +35751,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.197741+00:00</t>
+          <t>2026-10-17T11:36:14.631987+00:00</t>
         </is>
       </c>
     </row>
@@ -35853,7 +35853,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.197840+00:00</t>
+          <t>2026-10-17T11:36:14.632079+00:00</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35947,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.197853+00:00</t>
+          <t>2026-10-17T11:36:14.632091+00:00</t>
         </is>
       </c>
     </row>
@@ -36049,7 +36049,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.197934+00:00</t>
+          <t>2026-10-17T11:36:14.632173+00:00</t>
         </is>
       </c>
     </row>
@@ -36151,7 +36151,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198016+00:00</t>
+          <t>2026-10-17T11:36:14.632255+00:00</t>
         </is>
       </c>
     </row>
@@ -36253,7 +36253,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198121+00:00</t>
+          <t>2026-10-17T11:36:14.632378+00:00</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36347,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198131+00:00</t>
+          <t>2026-10-17T11:36:14.632391+00:00</t>
         </is>
       </c>
     </row>
@@ -36449,7 +36449,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198308+00:00</t>
+          <t>2026-10-17T11:36:14.632548+00:00</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36543,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198321+00:00</t>
+          <t>2026-10-17T11:36:14.632559+00:00</t>
         </is>
       </c>
     </row>
@@ -36645,7 +36645,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198424+00:00</t>
+          <t>2026-10-17T11:36:14.632660+00:00</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36739,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198435+00:00</t>
+          <t>2026-10-17T11:36:14.632671+00:00</t>
         </is>
       </c>
     </row>
@@ -36841,7 +36841,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198579+00:00</t>
+          <t>2026-10-17T11:36:14.632820+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36935,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198589+00:00</t>
+          <t>2026-10-17T11:36:14.632830+00:00</t>
         </is>
       </c>
     </row>
@@ -37037,7 +37037,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198676+00:00</t>
+          <t>2026-10-17T11:36:14.632923+00:00</t>
         </is>
       </c>
     </row>
@@ -37139,7 +37139,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.198992+00:00</t>
+          <t>2026-10-17T11:36:14.633056+00:00</t>
         </is>
       </c>
     </row>
@@ -37233,7 +37233,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.199017+00:00</t>
+          <t>2026-10-17T11:36:14.633067+00:00</t>
         </is>
       </c>
     </row>
@@ -37335,7 +37335,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.199151+00:00</t>
+          <t>2026-10-17T11:36:14.633200+00:00</t>
         </is>
       </c>
     </row>
@@ -37429,7 +37429,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.199163+00:00</t>
+          <t>2026-10-17T11:36:14.633211+00:00</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37531,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.199279+00:00</t>
+          <t>2026-10-17T11:36:14.633331+00:00</t>
         </is>
       </c>
     </row>
@@ -37633,7 +37633,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.199533+00:00</t>
+          <t>2026-10-17T11:36:14.633578+00:00</t>
         </is>
       </c>
     </row>
@@ -37727,7 +37727,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.199546+00:00</t>
+          <t>2026-10-17T11:36:14.633592+00:00</t>
         </is>
       </c>
     </row>
@@ -37829,7 +37829,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.199713+00:00</t>
+          <t>2026-10-17T11:36:14.633754+00:00</t>
         </is>
       </c>
     </row>
@@ -37931,7 +37931,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.199907+00:00</t>
+          <t>2026-10-17T11:36:14.633972+00:00</t>
         </is>
       </c>
     </row>
@@ -38033,7 +38033,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.200099+00:00</t>
+          <t>2026-10-17T11:36:14.634171+00:00</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.200111+00:00</t>
+          <t>2026-10-17T11:36:14.634182+00:00</t>
         </is>
       </c>
     </row>
@@ -38229,7 +38229,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.200219+00:00</t>
+          <t>2026-10-17T11:36:14.634319+00:00</t>
         </is>
       </c>
     </row>
@@ -38323,7 +38323,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.200229+00:00</t>
+          <t>2026-10-17T11:36:14.634331+00:00</t>
         </is>
       </c>
     </row>
@@ -38425,7 +38425,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.200334+00:00</t>
+          <t>2026-10-17T11:36:14.634424+00:00</t>
         </is>
       </c>
     </row>
@@ -38533,7 +38533,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.201468+00:00</t>
+          <t>2026-10-17T11:36:14.635500+00:00</t>
         </is>
       </c>
     </row>
@@ -38625,7 +38625,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.216859+00:00</t>
+          <t>2026-10-17T11:36:14.650789+00:00</t>
         </is>
       </c>
     </row>
@@ -38725,7 +38725,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.217364+00:00</t>
+          <t>2026-10-17T11:36:14.651345+00:00</t>
         </is>
       </c>
     </row>
@@ -38813,7 +38813,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.217382+00:00</t>
+          <t>2026-10-17T11:36:14.651365+00:00</t>
         </is>
       </c>
     </row>
@@ -38913,7 +38913,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.218605+00:00</t>
+          <t>2026-10-17T11:36:14.652619+00:00</t>
         </is>
       </c>
     </row>
@@ -39013,7 +39013,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.222010+00:00</t>
+          <t>2026-10-17T11:36:14.656085+00:00</t>
         </is>
       </c>
     </row>
@@ -39113,7 +39113,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.222894+00:00</t>
+          <t>2026-10-17T11:36:14.656996+00:00</t>
         </is>
       </c>
     </row>
@@ -39205,7 +39205,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.222910+00:00</t>
+          <t>2026-10-17T11:36:14.657014+00:00</t>
         </is>
       </c>
     </row>
@@ -39305,7 +39305,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.223576+00:00</t>
+          <t>2026-10-17T11:36:14.657805+00:00</t>
         </is>
       </c>
     </row>
@@ -39397,7 +39397,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.223590+00:00</t>
+          <t>2026-10-17T11:36:14.657828+00:00</t>
         </is>
       </c>
     </row>
@@ -39468,7 +39468,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P146" t="inlineStr">
@@ -39501,7 +39501,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.224421+00:00</t>
+          <t>2026-10-17T11:36:14.658693+00:00</t>
         </is>
       </c>
     </row>
@@ -39589,7 +39589,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.224435+00:00</t>
+          <t>2026-10-17T11:36:14.658710+00:00</t>
         </is>
       </c>
     </row>
@@ -39681,7 +39681,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.224439+00:00</t>
+          <t>2026-10-17T11:36:14.658713+00:00</t>
         </is>
       </c>
     </row>
@@ -39777,7 +39777,7 @@
       <c r="W149" t="inlineStr"/>
       <c r="X149" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.225200+00:00</t>
+          <t>2026-10-17T11:36:14.659505+00:00</t>
         </is>
       </c>
     </row>
@@ -39873,7 +39873,7 @@
       <c r="W150" t="inlineStr"/>
       <c r="X150" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.226235+00:00</t>
+          <t>2026-10-17T11:36:14.660617+00:00</t>
         </is>
       </c>
     </row>
@@ -39969,7 +39969,7 @@
       <c r="W151" t="inlineStr"/>
       <c r="X151" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.226693+00:00</t>
+          <t>2026-10-17T11:36:14.661069+00:00</t>
         </is>
       </c>
     </row>
@@ -40065,7 +40065,7 @@
       <c r="W152" t="inlineStr"/>
       <c r="X152" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.240034+00:00</t>
+          <t>2026-10-17T11:36:14.671952+00:00</t>
         </is>
       </c>
     </row>
@@ -40161,7 +40161,7 @@
       <c r="W153" t="inlineStr"/>
       <c r="X153" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.240270+00:00</t>
+          <t>2026-10-17T11:36:14.672158+00:00</t>
         </is>
       </c>
     </row>
@@ -40257,7 +40257,7 @@
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.240483+00:00</t>
+          <t>2026-10-17T11:36:14.672345+00:00</t>
         </is>
       </c>
     </row>
@@ -40353,7 +40353,7 @@
       <c r="W155" t="inlineStr"/>
       <c r="X155" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.240923+00:00</t>
+          <t>2026-10-17T11:36:14.672815+00:00</t>
         </is>
       </c>
     </row>
@@ -40449,7 +40449,7 @@
       <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.241199+00:00</t>
+          <t>2026-10-17T11:36:14.673100+00:00</t>
         </is>
       </c>
     </row>
@@ -40545,7 +40545,7 @@
       <c r="W157" t="inlineStr"/>
       <c r="X157" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.241696+00:00</t>
+          <t>2026-10-17T11:36:14.673526+00:00</t>
         </is>
       </c>
     </row>
@@ -40641,7 +40641,7 @@
       <c r="W158" t="inlineStr"/>
       <c r="X158" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.243009+00:00</t>
+          <t>2026-10-17T11:36:14.674751+00:00</t>
         </is>
       </c>
     </row>
@@ -40737,7 +40737,7 @@
       <c r="W159" t="inlineStr"/>
       <c r="X159" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.244939+00:00</t>
+          <t>2026-10-17T11:36:14.676697+00:00</t>
         </is>
       </c>
     </row>
@@ -40833,7 +40833,7 @@
       <c r="W160" t="inlineStr"/>
       <c r="X160" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.245709+00:00</t>
+          <t>2026-10-17T11:36:14.677458+00:00</t>
         </is>
       </c>
     </row>
@@ -40929,7 +40929,7 @@
       <c r="W161" t="inlineStr"/>
       <c r="X161" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.246016+00:00</t>
+          <t>2026-10-17T11:36:14.677877+00:00</t>
         </is>
       </c>
     </row>
@@ -41025,7 +41025,7 @@
       <c r="W162" t="inlineStr"/>
       <c r="X162" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.246073+00:00</t>
+          <t>2026-10-17T11:36:14.677957+00:00</t>
         </is>
       </c>
     </row>
@@ -41121,7 +41121,7 @@
       <c r="W163" t="inlineStr"/>
       <c r="X163" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.246141+00:00</t>
+          <t>2026-10-17T11:36:14.678026+00:00</t>
         </is>
       </c>
     </row>
@@ -41217,7 +41217,7 @@
       <c r="W164" t="inlineStr"/>
       <c r="X164" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.246806+00:00</t>
+          <t>2026-10-17T11:36:14.678449+00:00</t>
         </is>
       </c>
     </row>
@@ -41313,7 +41313,7 @@
       <c r="W165" t="inlineStr"/>
       <c r="X165" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.247624+00:00</t>
+          <t>2026-10-17T11:36:14.679109+00:00</t>
         </is>
       </c>
     </row>
@@ -41409,7 +41409,7 @@
       <c r="W166" t="inlineStr"/>
       <c r="X166" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.248464+00:00</t>
+          <t>2026-10-17T11:36:14.679528+00:00</t>
         </is>
       </c>
     </row>
@@ -41505,7 +41505,7 @@
       <c r="W167" t="inlineStr"/>
       <c r="X167" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.250105+00:00</t>
+          <t>2026-10-17T11:36:14.680269+00:00</t>
         </is>
       </c>
     </row>
@@ -41601,7 +41601,7 @@
       <c r="W168" t="inlineStr"/>
       <c r="X168" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.250869+00:00</t>
+          <t>2026-10-17T11:36:14.680779+00:00</t>
         </is>
       </c>
     </row>
@@ -41697,7 +41697,7 @@
       <c r="W169" t="inlineStr"/>
       <c r="X169" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.251055+00:00</t>
+          <t>2026-10-17T11:36:14.680957+00:00</t>
         </is>
       </c>
     </row>
@@ -41793,7 +41793,7 @@
       <c r="W170" t="inlineStr"/>
       <c r="X170" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.251223+00:00</t>
+          <t>2026-10-17T11:36:14.681107+00:00</t>
         </is>
       </c>
     </row>
@@ -41889,7 +41889,7 @@
       <c r="W171" t="inlineStr"/>
       <c r="X171" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.251749+00:00</t>
+          <t>2026-10-17T11:36:14.681247+00:00</t>
         </is>
       </c>
     </row>
@@ -41985,7 +41985,7 @@
       <c r="W172" t="inlineStr"/>
       <c r="X172" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.252004+00:00</t>
+          <t>2026-10-17T11:36:14.681341+00:00</t>
         </is>
       </c>
     </row>
@@ -42081,7 +42081,7 @@
       <c r="W173" t="inlineStr"/>
       <c r="X173" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.252081+00:00</t>
+          <t>2026-10-17T11:36:14.681414+00:00</t>
         </is>
       </c>
     </row>
@@ -42177,7 +42177,7 @@
       <c r="W174" t="inlineStr"/>
       <c r="X174" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.252470+00:00</t>
+          <t>2026-10-17T11:36:14.681786+00:00</t>
         </is>
       </c>
     </row>
@@ -42273,7 +42273,7 @@
       <c r="W175" t="inlineStr"/>
       <c r="X175" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.252842+00:00</t>
+          <t>2026-10-17T11:36:14.682157+00:00</t>
         </is>
       </c>
     </row>
@@ -42369,7 +42369,7 @@
       <c r="W176" t="inlineStr"/>
       <c r="X176" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.253139+00:00</t>
+          <t>2026-10-17T11:36:14.682456+00:00</t>
         </is>
       </c>
     </row>
@@ -42465,7 +42465,7 @@
       <c r="W177" t="inlineStr"/>
       <c r="X177" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.253566+00:00</t>
+          <t>2026-10-17T11:36:14.682800+00:00</t>
         </is>
       </c>
     </row>
@@ -42561,7 +42561,7 @@
       <c r="W178" t="inlineStr"/>
       <c r="X178" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.253811+00:00</t>
+          <t>2026-10-17T11:36:14.682930+00:00</t>
         </is>
       </c>
     </row>
@@ -42657,7 +42657,7 @@
       <c r="W179" t="inlineStr"/>
       <c r="X179" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.254663+00:00</t>
+          <t>2026-10-17T11:36:14.683616+00:00</t>
         </is>
       </c>
     </row>
@@ -42753,7 +42753,7 @@
       <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.255415+00:00</t>
+          <t>2026-10-17T11:36:14.684231+00:00</t>
         </is>
       </c>
     </row>
@@ -42849,7 +42849,7 @@
       <c r="W181" t="inlineStr"/>
       <c r="X181" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.255538+00:00</t>
+          <t>2026-10-17T11:36:14.684363+00:00</t>
         </is>
       </c>
     </row>
@@ -42945,7 +42945,7 @@
       <c r="W182" t="inlineStr"/>
       <c r="X182" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.256032+00:00</t>
+          <t>2026-10-17T11:36:14.684854+00:00</t>
         </is>
       </c>
     </row>
@@ -43041,7 +43041,7 @@
       <c r="W183" t="inlineStr"/>
       <c r="X183" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.256099+00:00</t>
+          <t>2026-10-17T11:36:14.684922+00:00</t>
         </is>
       </c>
     </row>
@@ -43137,7 +43137,7 @@
       <c r="W184" t="inlineStr"/>
       <c r="X184" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.256153+00:00</t>
+          <t>2026-10-17T11:36:14.685095+00:00</t>
         </is>
       </c>
     </row>
@@ -43233,7 +43233,7 @@
       <c r="W185" t="inlineStr"/>
       <c r="X185" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.256461+00:00</t>
+          <t>2026-10-17T11:36:14.685416+00:00</t>
         </is>
       </c>
     </row>
@@ -43329,7 +43329,7 @@
       <c r="W186" t="inlineStr"/>
       <c r="X186" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.256514+00:00</t>
+          <t>2026-10-17T11:36:14.685493+00:00</t>
         </is>
       </c>
     </row>
@@ -43425,7 +43425,7 @@
       <c r="W187" t="inlineStr"/>
       <c r="X187" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.256676+00:00</t>
+          <t>2026-10-17T11:36:14.685661+00:00</t>
         </is>
       </c>
     </row>
@@ -43521,7 +43521,7 @@
       <c r="W188" t="inlineStr"/>
       <c r="X188" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.256727+00:00</t>
+          <t>2026-10-17T11:36:14.685714+00:00</t>
         </is>
       </c>
     </row>
@@ -43617,7 +43617,7 @@
       <c r="W189" t="inlineStr"/>
       <c r="X189" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.257060+00:00</t>
+          <t>2026-10-17T11:36:14.686121+00:00</t>
         </is>
       </c>
     </row>
@@ -43713,7 +43713,7 @@
       <c r="W190" t="inlineStr"/>
       <c r="X190" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.257120+00:00</t>
+          <t>2026-10-17T11:36:14.686203+00:00</t>
         </is>
       </c>
     </row>
@@ -43809,7 +43809,7 @@
       <c r="W191" t="inlineStr"/>
       <c r="X191" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.257738+00:00</t>
+          <t>2026-10-17T11:36:14.686863+00:00</t>
         </is>
       </c>
     </row>
@@ -43905,7 +43905,7 @@
       <c r="W192" t="inlineStr"/>
       <c r="X192" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.257822+00:00</t>
+          <t>2026-10-17T11:36:14.686960+00:00</t>
         </is>
       </c>
     </row>
@@ -44001,7 +44001,7 @@
       <c r="W193" t="inlineStr"/>
       <c r="X193" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.258161+00:00</t>
+          <t>2026-10-17T11:36:14.687325+00:00</t>
         </is>
       </c>
     </row>
@@ -44097,7 +44097,7 @@
       <c r="W194" t="inlineStr"/>
       <c r="X194" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.258393+00:00</t>
+          <t>2026-10-17T11:36:14.687481+00:00</t>
         </is>
       </c>
     </row>
@@ -44193,7 +44193,7 @@
       <c r="W195" t="inlineStr"/>
       <c r="X195" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.258672+00:00</t>
+          <t>2026-10-17T11:36:14.687783+00:00</t>
         </is>
       </c>
     </row>
@@ -44289,7 +44289,7 @@
       <c r="W196" t="inlineStr"/>
       <c r="X196" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.258730+00:00</t>
+          <t>2026-10-17T11:36:14.687859+00:00</t>
         </is>
       </c>
     </row>
@@ -44385,7 +44385,7 @@
       <c r="W197" t="inlineStr"/>
       <c r="X197" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.258926+00:00</t>
+          <t>2026-10-17T11:36:14.687984+00:00</t>
         </is>
       </c>
     </row>
@@ -44481,7 +44481,7 @@
       <c r="W198" t="inlineStr"/>
       <c r="X198" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.259282+00:00</t>
+          <t>2026-10-17T11:36:14.688402+00:00</t>
         </is>
       </c>
     </row>
@@ -44577,7 +44577,7 @@
       <c r="W199" t="inlineStr"/>
       <c r="X199" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.259733+00:00</t>
+          <t>2026-10-17T11:36:14.688823+00:00</t>
         </is>
       </c>
     </row>
@@ -44673,7 +44673,7 @@
       <c r="W200" t="inlineStr"/>
       <c r="X200" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.259821+00:00</t>
+          <t>2026-10-17T11:36:14.688907+00:00</t>
         </is>
       </c>
     </row>
@@ -44769,7 +44769,7 @@
       <c r="W201" t="inlineStr"/>
       <c r="X201" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.260400+00:00</t>
+          <t>2026-10-17T11:36:14.689395+00:00</t>
         </is>
       </c>
     </row>
@@ -44865,7 +44865,7 @@
       <c r="W202" t="inlineStr"/>
       <c r="X202" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.260814+00:00</t>
+          <t>2026-10-17T11:36:14.689729+00:00</t>
         </is>
       </c>
     </row>
@@ -44961,7 +44961,7 @@
       <c r="W203" t="inlineStr"/>
       <c r="X203" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.260887+00:00</t>
+          <t>2026-10-17T11:36:14.689781+00:00</t>
         </is>
       </c>
     </row>
@@ -45057,7 +45057,7 @@
       <c r="W204" t="inlineStr"/>
       <c r="X204" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.261183+00:00</t>
+          <t>2026-10-17T11:36:14.690077+00:00</t>
         </is>
       </c>
     </row>
@@ -45153,7 +45153,7 @@
       <c r="W205" t="inlineStr"/>
       <c r="X205" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.261247+00:00</t>
+          <t>2026-10-17T11:36:14.690271+00:00</t>
         </is>
       </c>
     </row>
@@ -45249,7 +45249,7 @@
       <c r="W206" t="inlineStr"/>
       <c r="X206" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.261346+00:00</t>
+          <t>2026-10-17T11:36:14.690397+00:00</t>
         </is>
       </c>
     </row>
@@ -45345,7 +45345,7 @@
       <c r="W207" t="inlineStr"/>
       <c r="X207" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.261416+00:00</t>
+          <t>2026-10-17T11:36:14.690462+00:00</t>
         </is>
       </c>
     </row>
@@ -45441,7 +45441,7 @@
       <c r="W208" t="inlineStr"/>
       <c r="X208" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.261548+00:00</t>
+          <t>2026-10-17T11:36:14.690515+00:00</t>
         </is>
       </c>
     </row>
@@ -45537,7 +45537,7 @@
       <c r="W209" t="inlineStr"/>
       <c r="X209" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.261604+00:00</t>
+          <t>2026-10-17T11:36:14.690566+00:00</t>
         </is>
       </c>
     </row>
@@ -45633,7 +45633,7 @@
       <c r="W210" t="inlineStr"/>
       <c r="X210" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.261918+00:00</t>
+          <t>2026-10-17T11:36:14.691066+00:00</t>
         </is>
       </c>
     </row>
@@ -45729,7 +45729,7 @@
       <c r="W211" t="inlineStr"/>
       <c r="X211" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.262045+00:00</t>
+          <t>2026-10-17T11:36:14.691225+00:00</t>
         </is>
       </c>
     </row>
@@ -45825,7 +45825,7 @@
       <c r="W212" t="inlineStr"/>
       <c r="X212" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.262204+00:00</t>
+          <t>2026-10-17T11:36:14.691423+00:00</t>
         </is>
       </c>
     </row>
@@ -45921,7 +45921,1351 @@
       <c r="W213" t="inlineStr"/>
       <c r="X213" t="inlineStr">
         <is>
-          <t>2026-10-17T11:35:14.262406+00:00</t>
+          <t>2026-10-17T11:36:14.691807+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="b">
+        <v>1</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>R13968</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>R13968.main.a98ded9fe4a3b73c</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E214" t="b">
+        <v>0</v>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Nhatthaphon_sr_front_p.pdf</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_front_p.pdf</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_front_p.pdf</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr"/>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13968_Nhatthaphon_sr_front_p.pdf</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L214" t="n">
+        <v>1147423</v>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>a98ded9fe4a3b73cc9408cef83da94bef7ee46dac09a1a9ab5b014070070ac7a</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452208</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr"/>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr"/>
+      <c r="U214" t="inlineStr"/>
+      <c r="V214" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W214" t="inlineStr"/>
+      <c r="X214" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.692795+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="b">
+        <v>0</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>R13968</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>R13968.main.ed6af2c70fa34cca</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E215" t="b">
+        <v>0</v>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Nhatthaphon_sr_ch1_p.pdf</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch1_p.pdf</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch1_p.pdf</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr"/>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13968_Nhatthaphon_sr_ch1_p.pdf</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L215" t="n">
+        <v>657184</v>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>ed6af2c70fa34ccadfc217ee28e24971d899d99a19d6933f0e377e371c70e59e</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452209</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr"/>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T215" t="inlineStr"/>
+      <c r="U215" t="inlineStr"/>
+      <c r="V215" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W215" t="inlineStr"/>
+      <c r="X215" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.693259+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="b">
+        <v>0</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>R13968</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>R13968.main.db164a7cb44673e9</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E216" t="b">
+        <v>0</v>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Nhatthaphon_sr_ch2_p.pdf</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch2_p.pdf</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch2_p.pdf</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr"/>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13968_Nhatthaphon_sr_ch2_p.pdf</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L216" t="n">
+        <v>2222750</v>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>db164a7cb44673e94b3023ccb7d02eb60ee91282cc7e6fcd89e31ae859b8ad75</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452210</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr"/>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T216" t="inlineStr"/>
+      <c r="U216" t="inlineStr"/>
+      <c r="V216" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W216" t="inlineStr"/>
+      <c r="X216" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.694843+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="b">
+        <v>0</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>R13968</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>R13968.main.a58d9c0c6dccab4f</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E217" t="b">
+        <v>0</v>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Nhatthaphon_sr_ch3_p.pdf</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch3_p.pdf</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch3_p.pdf</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr"/>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13968_Nhatthaphon_sr_ch3_p.pdf</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L217" t="n">
+        <v>1230431</v>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>a58d9c0c6dccab4f535d87b9f82f45309f2b33bdfec9db5f198589f650c48f00</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452211</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr"/>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr"/>
+      <c r="U217" t="inlineStr"/>
+      <c r="V217" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W217" t="inlineStr"/>
+      <c r="X217" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.695784+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="b">
+        <v>0</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>R13968</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>R13968.main.31fee06cf27de2a2</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E218" t="b">
+        <v>0</v>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Nhatthaphon_sr_ch4_p.pdf</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch4_p.pdf</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch4_p.pdf</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr"/>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13968_Nhatthaphon_sr_ch4_p.pdf</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L218" t="n">
+        <v>1571765</v>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>31fee06cf27de2a2a708bd14a09a8bc73303ebcd67efe353efcc01fc79b20cfd</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452212</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr"/>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T218" t="inlineStr"/>
+      <c r="U218" t="inlineStr"/>
+      <c r="V218" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W218" t="inlineStr"/>
+      <c r="X218" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.697122+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="b">
+        <v>0</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>R13968</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>R13968.main.a97b06850912d4a8</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E219" t="b">
+        <v>0</v>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Nhatthaphon_sr_ch5_p.pdf</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch5_p.pdf</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_ch5_p.pdf</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr"/>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13968_Nhatthaphon_sr_ch5_p.pdf</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L219" t="n">
+        <v>661960</v>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>a97b06850912d4a801036181f1999825b65250e340cdc1295395aa9670b107cf</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452213</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr"/>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr"/>
+      <c r="U219" t="inlineStr"/>
+      <c r="V219" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W219" t="inlineStr"/>
+      <c r="X219" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.697881+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="b">
+        <v>0</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>R13968</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>R13968.main.1eeabd66eb09e704</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E220" t="b">
+        <v>0</v>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Nhatthaphon_sr_back_p.pdf</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_back_p.pdf</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13968_Nhatthaphon_sr_back_p.pdf</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr"/>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13968_Nhatthaphon_sr_back_p.pdf</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L220" t="n">
+        <v>1492934</v>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>1eeabd66eb09e7047569c92f557035bd252ce64d3d8a5cf08cc1dd8d56d27c31</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452214</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr"/>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr"/>
+      <c r="U220" t="inlineStr"/>
+      <c r="V220" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W220" t="inlineStr"/>
+      <c r="X220" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.698870+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="b">
+        <v>1</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>R13969</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>R13969.main.82240174e4cc091f</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E221" t="b">
+        <v>0</v>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Pairin_tu_front_p.pdf</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_front_p.pdf</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_front_p.pdf</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr"/>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13969_Pairin_tu_front_p.pdf</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L221" t="n">
+        <v>1130768</v>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>82240174e4cc091f5f38a7251df829ad9fe6d768ac10914b2cfd27bb6ae8ebc1</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452176</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr"/>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr"/>
+      <c r="U221" t="inlineStr"/>
+      <c r="V221" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W221" t="inlineStr"/>
+      <c r="X221" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.699610+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="b">
+        <v>0</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>R13969</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>R13969.main.239995a5c23d7580</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E222" t="b">
+        <v>0</v>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Pairin_tu_ch1_p.pdf</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch1_p.pdf</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch1_p.pdf</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr"/>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13969_Pairin_tu_ch1_p.pdf</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L222" t="n">
+        <v>649972</v>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>239995a5c23d758049b99db0ca8aa1752790e940bee916370a0b9ad22becc3ea</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452177</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr"/>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T222" t="inlineStr"/>
+      <c r="U222" t="inlineStr"/>
+      <c r="V222" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W222" t="inlineStr"/>
+      <c r="X222" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.700214+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="b">
+        <v>0</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>R13969</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>R13969.main.e243a1071df26efb</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E223" t="b">
+        <v>0</v>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Pairin_tu_ch2_p.pdf</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch2_p.pdf</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch2_p.pdf</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr"/>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13969_Pairin_tu_ch2_p.pdf</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L223" t="n">
+        <v>1666115</v>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>e243a1071df26efb7b0f26c3399c69d9312dd4c1be4278790cdab042b6ee13ed</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452178</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr"/>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T223" t="inlineStr"/>
+      <c r="U223" t="inlineStr"/>
+      <c r="V223" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W223" t="inlineStr"/>
+      <c r="X223" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.701321+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="b">
+        <v>0</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>R13969</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>R13969.main.32ca8cbb364b193d</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E224" t="b">
+        <v>0</v>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Pairin_tu_ch3_p.pdf</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch3_p.pdf</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch3_p.pdf</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr"/>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13969_Pairin_tu_ch3_p.pdf</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L224" t="n">
+        <v>1017982</v>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>32ca8cbb364b193de87f882ae894fcbc5fef9f26ed5e6f97de81c52c3faf4e30</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452179</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr"/>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T224" t="inlineStr"/>
+      <c r="U224" t="inlineStr"/>
+      <c r="V224" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W224" t="inlineStr"/>
+      <c r="X224" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.702029+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="b">
+        <v>0</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>R13969</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>R13969.main.61359ef0b77b9afe</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E225" t="b">
+        <v>0</v>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Pairin_tu_ch4_p.pdf</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch4_p.pdf</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch4_p.pdf</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr"/>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13969_Pairin_tu_ch4_p.pdf</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L225" t="n">
+        <v>1935008</v>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>61359ef0b77b9afe3705e5fef209f4c11dabf953e463ece6b7edff0b5d787ad1</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452180</t>
+        </is>
+      </c>
+      <c r="Q225" t="inlineStr"/>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T225" t="inlineStr"/>
+      <c r="U225" t="inlineStr"/>
+      <c r="V225" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W225" t="inlineStr"/>
+      <c r="X225" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.703254+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="b">
+        <v>0</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>R13969</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>R13969.main.546cae968d98e8de</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E226" t="b">
+        <v>0</v>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Pairin_tu_ch5_p.pdf</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch5_p.pdf</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_ch5_p.pdf</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr"/>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13969_Pairin_tu_ch5_p.pdf</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L226" t="n">
+        <v>637595</v>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>546cae968d98e8de6bc8531eb6157f426feb10dd51c5b00ecfeca016b79f69c8</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452181</t>
+        </is>
+      </c>
+      <c r="Q226" t="inlineStr"/>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T226" t="inlineStr"/>
+      <c r="U226" t="inlineStr"/>
+      <c r="V226" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W226" t="inlineStr"/>
+      <c r="X226" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.704361+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="b">
+        <v>0</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>R13969</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>R13969.main.cd34536c2889613d</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E227" t="b">
+        <v>0</v>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Pairin_tu_back_p.pdf</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_back_p.pdf</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>original_files/fulltext/R13969_Pairin_tu_back_p.pdf</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr"/>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/fulltext/R13969_Pairin_tu_back_p.pdf</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>pdf</t>
+        </is>
+      </c>
+      <c r="L227" t="n">
+        <v>1314955</v>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>cd34536c2889613d83052b35c5557bc57988c12cf3c36642ceb2df5752712ce8</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>present_sha_verified</t>
+        </is>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>local_acquired_pending_remote_readback</t>
+        </is>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>https://digiverse.chula.ac.th/digital/api/DownloadDigitalFile/dowload/452182</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr"/>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>University archived 2015 MSc thesis; complete set of 7 original PDF parts; use together in listed order</t>
+        </is>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>Private authorized research backup; source license not inferred</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr"/>
+      <c r="U227" t="inlineStr"/>
+      <c r="V227" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="W227" t="inlineStr"/>
+      <c r="X227" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:36:14.705233+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Persist declared attachment CDN recovery and exact historical-byte check
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -6475,10 +6475,10 @@
         </is>
       </c>
       <c r="H141" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I141" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="142">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.465524+00:00</t>
+          <t>2026-10-17T11:37:12.303087+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.466490+00:00</t>
+          <t>2026-10-17T11:37:12.303983+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.466518+00:00</t>
+          <t>2026-10-17T11:37:12.304004+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.466816+00:00</t>
+          <t>2026-10-17T11:37:12.304222+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.468030+00:00</t>
+          <t>2026-10-17T11:37:12.308146+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.468576+00:00</t>
+          <t>2026-10-17T11:37:12.308648+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.474688+00:00</t>
+          <t>2026-10-17T11:37:12.314349+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.477536+00:00</t>
+          <t>2026-10-17T11:37:12.316609+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.479122+00:00</t>
+          <t>2026-10-17T11:37:12.317523+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.479537+00:00</t>
+          <t>2026-10-17T11:37:12.317844+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.480424+00:00</t>
+          <t>2026-10-17T11:37:12.318560+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.481286+00:00</t>
+          <t>2026-10-17T11:37:12.319203+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.482579+00:00</t>
+          <t>2026-10-17T11:37:12.320097+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.482849+00:00</t>
+          <t>2026-10-17T11:37:12.320346+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.483863+00:00</t>
+          <t>2026-10-17T11:37:12.321201+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.493591+00:00</t>
+          <t>2026-10-17T11:37:12.331059+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.494479+00:00</t>
+          <t>2026-10-17T11:37:12.331918+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.495966+00:00</t>
+          <t>2026-10-17T11:37:12.334746+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.498481+00:00</t>
+          <t>2026-10-17T11:37:12.341748+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.499740+00:00</t>
+          <t>2026-10-17T11:37:12.342975+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.501177+00:00</t>
+          <t>2026-10-17T11:37:12.344179+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.505575+00:00</t>
+          <t>2026-10-17T11:37:12.348763+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.507982+00:00</t>
+          <t>2026-10-17T11:37:12.351038+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.509983+00:00</t>
+          <t>2026-10-17T11:37:12.352832+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.510921+00:00</t>
+          <t>2026-10-17T11:37:12.353508+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.511386+00:00</t>
+          <t>2026-10-17T11:37:12.353864+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.513444+00:00</t>
+          <t>2026-10-17T11:37:12.356011+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.514784+00:00</t>
+          <t>2026-10-17T11:37:12.357278+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.516827+00:00</t>
+          <t>2026-10-17T11:37:12.359391+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.519113+00:00</t>
+          <t>2026-10-17T11:37:12.361444+00:00</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.519817+00:00</t>
+          <t>2026-10-17T11:37:12.362021+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.520406+00:00</t>
+          <t>2026-10-17T11:37:12.362589+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.522372+00:00</t>
+          <t>2026-10-17T11:37:12.364197+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.525241+00:00</t>
+          <t>2026-10-17T11:37:12.366977+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.527771+00:00</t>
+          <t>2026-10-17T11:37:12.369091+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.529045+00:00</t>
+          <t>2026-10-17T11:37:12.370281+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.532351+00:00</t>
+          <t>2026-10-17T11:37:12.373128+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.533225+00:00</t>
+          <t>2026-10-17T11:37:12.373845+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.535079+00:00</t>
+          <t>2026-10-17T11:37:12.375431+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.535389+00:00</t>
+          <t>2026-10-17T11:37:12.375690+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.537394+00:00</t>
+          <t>2026-10-17T11:37:12.377585+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.540573+00:00</t>
+          <t>2026-10-17T11:37:12.380411+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.542368+00:00</t>
+          <t>2026-10-17T11:37:12.381730+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.543044+00:00</t>
+          <t>2026-10-17T11:37:12.382253+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.545728+00:00</t>
+          <t>2026-10-17T11:37:12.384837+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.546859+00:00</t>
+          <t>2026-10-17T11:37:12.385966+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.550406+00:00</t>
+          <t>2026-10-17T11:37:12.389538+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.552080+00:00</t>
+          <t>2026-10-17T11:37:12.391235+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.554373+00:00</t>
+          <t>2026-10-17T11:37:12.393076+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.555551+00:00</t>
+          <t>2026-10-17T11:37:12.394033+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.556051+00:00</t>
+          <t>2026-10-17T11:37:12.394474+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.556553+00:00</t>
+          <t>2026-10-17T11:37:12.394836+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.558371+00:00</t>
+          <t>2026-10-17T11:37:12.396307+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.559673+00:00</t>
+          <t>2026-10-17T11:37:12.397612+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.561285+00:00</t>
+          <t>2026-10-17T11:37:12.399101+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.561721+00:00</t>
+          <t>2026-10-17T11:37:12.399440+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.562928+00:00</t>
+          <t>2026-10-17T11:37:12.400597+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.564502+00:00</t>
+          <t>2026-10-17T11:37:12.401971+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.565160+00:00</t>
+          <t>2026-10-17T11:37:12.402574+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.566363+00:00</t>
+          <t>2026-10-17T11:37:12.403514+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.566789+00:00</t>
+          <t>2026-10-17T11:37:12.403818+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.572494+00:00</t>
+          <t>2026-10-17T11:37:12.408981+00:00</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.572954+00:00</t>
+          <t>2026-10-17T11:37:12.409417+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.573592+00:00</t>
+          <t>2026-10-17T11:37:12.409986+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.574027+00:00</t>
+          <t>2026-10-17T11:37:12.410432+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.575107+00:00</t>
+          <t>2026-10-17T11:37:12.411495+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.578176+00:00</t>
+          <t>2026-10-17T11:37:12.414438+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.578465+00:00</t>
+          <t>2026-10-17T11:37:12.414679+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.582641+00:00</t>
+          <t>2026-10-17T11:37:12.419070+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.583386+00:00</t>
+          <t>2026-10-17T11:37:12.419910+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.585584+00:00</t>
+          <t>2026-10-17T11:37:12.422040+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.587478+00:00</t>
+          <t>2026-10-17T11:37:12.423783+00:00</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.588430+00:00</t>
+          <t>2026-10-17T11:37:12.424655+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.590122+00:00</t>
+          <t>2026-10-17T11:37:12.426067+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.592871+00:00</t>
+          <t>2026-10-17T11:37:12.428245+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.602777+00:00</t>
+          <t>2026-10-17T11:37:12.436161+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.604230+00:00</t>
+          <t>2026-10-17T11:37:12.437512+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.604441+00:00</t>
+          <t>2026-10-17T11:37:12.437668+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.604457+00:00</t>
+          <t>2026-10-17T11:37:12.437680+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.610623+00:00</t>
+          <t>2026-10-17T11:37:12.442625+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.611106+00:00</t>
+          <t>2026-10-17T11:37:12.443005+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.611500+00:00</t>
+          <t>2026-10-17T11:37:12.443381+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.611957+00:00</t>
+          <t>2026-10-17T11:37:12.443776+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.612754+00:00</t>
+          <t>2026-10-17T11:37:12.444473+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.614415+00:00</t>
+          <t>2026-10-17T11:37:12.445862+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.615246+00:00</t>
+          <t>2026-10-17T11:37:12.446685+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.615604+00:00</t>
+          <t>2026-10-17T11:37:12.446982+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.616476+00:00</t>
+          <t>2026-10-17T11:37:12.447632+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.616503+00:00</t>
+          <t>2026-10-17T11:37:12.447645+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.616567+00:00</t>
+          <t>2026-10-17T11:37:12.447692+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.616797+00:00</t>
+          <t>2026-10-17T11:37:12.447905+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.616922+00:00</t>
+          <t>2026-10-17T11:37:12.448021+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.617038+00:00</t>
+          <t>2026-10-17T11:37:12.448135+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.617446+00:00</t>
+          <t>2026-10-17T11:37:12.448520+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.617683+00:00</t>
+          <t>2026-10-17T11:37:12.448705+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.617739+00:00</t>
+          <t>2026-10-17T11:37:12.448759+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.617799+00:00</t>
+          <t>2026-10-17T11:37:12.448820+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.617954+00:00</t>
+          <t>2026-10-17T11:37:12.448959+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.617998+00:00</t>
+          <t>2026-10-17T11:37:12.449003+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.618662+00:00</t>
+          <t>2026-10-17T11:37:12.449492+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.618738+00:00</t>
+          <t>2026-10-17T11:37:12.449544+00:00</t>
         </is>
       </c>
     </row>
@@ -35151,13 +35151,21 @@
           <t>papers/R07238/supplementary/0b7925ad1ed9_mmc1.docx</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>original_files/supplementary/R07238/mmc1.docx</t>
+        </is>
+      </c>
       <c r="I103" t="inlineStr">
         <is>
           <t>/workspace/library-files/ad-oxygen-supplements/R07238/official/mmc1.docx</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>/workspace/FirstCodex/results/ad-oxygen-literature-20261006/original_files/supplementary/R07238/mmc1.docx</t>
+        </is>
+      </c>
       <c r="K103" t="inlineStr">
         <is>
           <t>docx</t>
@@ -35173,17 +35181,17 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>present_sha_verified</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>local_acquired_pending_remote_readback</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://ars.els-cdn.com/content/image/1-s2.0-S1350417721000730-mmc1.docx</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -35193,7 +35201,7 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>original_supplementary_attachment</t>
+          <t>Official publisher supplementary Word document; exact historical SHA256</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
@@ -35215,7 +35223,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.618751+00:00</t>
+          <t>2026-10-17T11:37:12.449614+00:00</t>
         </is>
       </c>
     </row>
@@ -35323,7 +35331,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.630430+00:00</t>
+          <t>2026-10-17T11:37:12.459410+00:00</t>
         </is>
       </c>
     </row>
@@ -35427,7 +35435,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.630538+00:00</t>
+          <t>2026-10-17T11:37:12.459480+00:00</t>
         </is>
       </c>
     </row>
@@ -35535,7 +35543,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.630688+00:00</t>
+          <t>2026-10-17T11:37:12.459579+00:00</t>
         </is>
       </c>
     </row>
@@ -35643,7 +35651,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.630932+00:00</t>
+          <t>2026-10-17T11:37:12.459808+00:00</t>
         </is>
       </c>
     </row>
@@ -35751,7 +35759,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.631987+00:00</t>
+          <t>2026-10-17T11:37:12.460799+00:00</t>
         </is>
       </c>
     </row>
@@ -35853,7 +35861,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632079+00:00</t>
+          <t>2026-10-17T11:37:12.460885+00:00</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35955,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632091+00:00</t>
+          <t>2026-10-17T11:37:12.460895+00:00</t>
         </is>
       </c>
     </row>
@@ -36049,7 +36057,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632173+00:00</t>
+          <t>2026-10-17T11:37:12.460973+00:00</t>
         </is>
       </c>
     </row>
@@ -36151,7 +36159,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632255+00:00</t>
+          <t>2026-10-17T11:37:12.461056+00:00</t>
         </is>
       </c>
     </row>
@@ -36253,7 +36261,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632378+00:00</t>
+          <t>2026-10-17T11:37:12.461161+00:00</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36355,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632391+00:00</t>
+          <t>2026-10-17T11:37:12.461172+00:00</t>
         </is>
       </c>
     </row>
@@ -36449,7 +36457,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632548+00:00</t>
+          <t>2026-10-17T11:37:12.461341+00:00</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36551,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632559+00:00</t>
+          <t>2026-10-17T11:37:12.461355+00:00</t>
         </is>
       </c>
     </row>
@@ -36645,7 +36653,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632660+00:00</t>
+          <t>2026-10-17T11:37:12.461457+00:00</t>
         </is>
       </c>
     </row>
@@ -36739,7 +36747,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632671+00:00</t>
+          <t>2026-10-17T11:37:12.461468+00:00</t>
         </is>
       </c>
     </row>
@@ -36841,7 +36849,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632820+00:00</t>
+          <t>2026-10-17T11:37:12.461627+00:00</t>
         </is>
       </c>
     </row>
@@ -36935,7 +36943,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632830+00:00</t>
+          <t>2026-10-17T11:37:12.461639+00:00</t>
         </is>
       </c>
     </row>
@@ -37037,7 +37045,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.632923+00:00</t>
+          <t>2026-10-17T11:37:12.461730+00:00</t>
         </is>
       </c>
     </row>
@@ -37139,7 +37147,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633056+00:00</t>
+          <t>2026-10-17T11:37:12.461865+00:00</t>
         </is>
       </c>
     </row>
@@ -37233,7 +37241,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633067+00:00</t>
+          <t>2026-10-17T11:37:12.461876+00:00</t>
         </is>
       </c>
     </row>
@@ -37335,7 +37343,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633200+00:00</t>
+          <t>2026-10-17T11:37:12.462007+00:00</t>
         </is>
       </c>
     </row>
@@ -37429,7 +37437,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633211+00:00</t>
+          <t>2026-10-17T11:37:12.462018+00:00</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37539,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633331+00:00</t>
+          <t>2026-10-17T11:37:12.462124+00:00</t>
         </is>
       </c>
     </row>
@@ -37633,7 +37641,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633578+00:00</t>
+          <t>2026-10-17T11:37:12.462412+00:00</t>
         </is>
       </c>
     </row>
@@ -37727,7 +37735,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633592+00:00</t>
+          <t>2026-10-17T11:37:12.462434+00:00</t>
         </is>
       </c>
     </row>
@@ -37829,7 +37837,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633754+00:00</t>
+          <t>2026-10-17T11:37:12.462603+00:00</t>
         </is>
       </c>
     </row>
@@ -37931,7 +37939,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.633972+00:00</t>
+          <t>2026-10-17T11:37:12.462803+00:00</t>
         </is>
       </c>
     </row>
@@ -38033,7 +38041,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.634171+00:00</t>
+          <t>2026-10-17T11:37:12.462997+00:00</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38135,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.634182+00:00</t>
+          <t>2026-10-17T11:37:12.463009+00:00</t>
         </is>
       </c>
     </row>
@@ -38229,7 +38237,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.634319+00:00</t>
+          <t>2026-10-17T11:37:12.463120+00:00</t>
         </is>
       </c>
     </row>
@@ -38323,7 +38331,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.634331+00:00</t>
+          <t>2026-10-17T11:37:12.463131+00:00</t>
         </is>
       </c>
     </row>
@@ -38425,7 +38433,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.634424+00:00</t>
+          <t>2026-10-17T11:37:12.463223+00:00</t>
         </is>
       </c>
     </row>
@@ -38533,7 +38541,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.635500+00:00</t>
+          <t>2026-10-17T11:37:12.464321+00:00</t>
         </is>
       </c>
     </row>
@@ -38625,7 +38633,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.650789+00:00</t>
+          <t>2026-10-17T11:37:12.479223+00:00</t>
         </is>
       </c>
     </row>
@@ -38725,7 +38733,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.651345+00:00</t>
+          <t>2026-10-17T11:37:12.479671+00:00</t>
         </is>
       </c>
     </row>
@@ -38813,7 +38821,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.651365+00:00</t>
+          <t>2026-10-17T11:37:12.479685+00:00</t>
         </is>
       </c>
     </row>
@@ -38913,7 +38921,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.652619+00:00</t>
+          <t>2026-10-17T11:37:12.480801+00:00</t>
         </is>
       </c>
     </row>
@@ -39013,7 +39021,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.656085+00:00</t>
+          <t>2026-10-17T11:37:12.484207+00:00</t>
         </is>
       </c>
     </row>
@@ -39113,7 +39121,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.656996+00:00</t>
+          <t>2026-10-17T11:37:12.485123+00:00</t>
         </is>
       </c>
     </row>
@@ -39205,7 +39213,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.657014+00:00</t>
+          <t>2026-10-17T11:37:12.485141+00:00</t>
         </is>
       </c>
     </row>
@@ -39305,7 +39313,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.657805+00:00</t>
+          <t>2026-10-17T11:37:12.485858+00:00</t>
         </is>
       </c>
     </row>
@@ -39397,7 +39405,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.657828+00:00</t>
+          <t>2026-10-17T11:37:12.485873+00:00</t>
         </is>
       </c>
     </row>
@@ -39501,7 +39509,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.658693+00:00</t>
+          <t>2026-10-17T11:37:12.486712+00:00</t>
         </is>
       </c>
     </row>
@@ -39589,7 +39597,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.658710+00:00</t>
+          <t>2026-10-17T11:37:12.486727+00:00</t>
         </is>
       </c>
     </row>
@@ -39681,7 +39689,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.658713+00:00</t>
+          <t>2026-10-17T11:37:12.486730+00:00</t>
         </is>
       </c>
     </row>
@@ -39777,7 +39785,7 @@
       <c r="W149" t="inlineStr"/>
       <c r="X149" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.659505+00:00</t>
+          <t>2026-10-17T11:37:12.487515+00:00</t>
         </is>
       </c>
     </row>
@@ -39873,7 +39881,7 @@
       <c r="W150" t="inlineStr"/>
       <c r="X150" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.660617+00:00</t>
+          <t>2026-10-17T11:37:12.488596+00:00</t>
         </is>
       </c>
     </row>
@@ -39969,7 +39977,7 @@
       <c r="W151" t="inlineStr"/>
       <c r="X151" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.661069+00:00</t>
+          <t>2026-10-17T11:37:12.489035+00:00</t>
         </is>
       </c>
     </row>
@@ -40065,7 +40073,7 @@
       <c r="W152" t="inlineStr"/>
       <c r="X152" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.671952+00:00</t>
+          <t>2026-10-17T11:37:12.498819+00:00</t>
         </is>
       </c>
     </row>
@@ -40161,7 +40169,7 @@
       <c r="W153" t="inlineStr"/>
       <c r="X153" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.672158+00:00</t>
+          <t>2026-10-17T11:37:12.498976+00:00</t>
         </is>
       </c>
     </row>
@@ -40257,7 +40265,7 @@
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.672345+00:00</t>
+          <t>2026-10-17T11:37:12.499137+00:00</t>
         </is>
       </c>
     </row>
@@ -40353,7 +40361,7 @@
       <c r="W155" t="inlineStr"/>
       <c r="X155" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.672815+00:00</t>
+          <t>2026-10-17T11:37:12.499585+00:00</t>
         </is>
       </c>
     </row>
@@ -40449,7 +40457,7 @@
       <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.673100+00:00</t>
+          <t>2026-10-17T11:37:12.499843+00:00</t>
         </is>
       </c>
     </row>
@@ -40545,7 +40553,7 @@
       <c r="W157" t="inlineStr"/>
       <c r="X157" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.673526+00:00</t>
+          <t>2026-10-17T11:37:12.500173+00:00</t>
         </is>
       </c>
     </row>
@@ -40641,7 +40649,7 @@
       <c r="W158" t="inlineStr"/>
       <c r="X158" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.674751+00:00</t>
+          <t>2026-10-17T11:37:12.501322+00:00</t>
         </is>
       </c>
     </row>
@@ -40737,7 +40745,7 @@
       <c r="W159" t="inlineStr"/>
       <c r="X159" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.676697+00:00</t>
+          <t>2026-10-17T11:37:12.503087+00:00</t>
         </is>
       </c>
     </row>
@@ -40833,7 +40841,7 @@
       <c r="W160" t="inlineStr"/>
       <c r="X160" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.677458+00:00</t>
+          <t>2026-10-17T11:37:12.503692+00:00</t>
         </is>
       </c>
     </row>
@@ -40929,7 +40937,7 @@
       <c r="W161" t="inlineStr"/>
       <c r="X161" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.677877+00:00</t>
+          <t>2026-10-17T11:37:12.503954+00:00</t>
         </is>
       </c>
     </row>
@@ -41025,7 +41033,7 @@
       <c r="W162" t="inlineStr"/>
       <c r="X162" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.677957+00:00</t>
+          <t>2026-10-17T11:37:12.504006+00:00</t>
         </is>
       </c>
     </row>
@@ -41121,7 +41129,7 @@
       <c r="W163" t="inlineStr"/>
       <c r="X163" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.678026+00:00</t>
+          <t>2026-10-17T11:37:12.504068+00:00</t>
         </is>
       </c>
     </row>
@@ -41217,7 +41225,7 @@
       <c r="W164" t="inlineStr"/>
       <c r="X164" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.678449+00:00</t>
+          <t>2026-10-17T11:37:12.504369+00:00</t>
         </is>
       </c>
     </row>
@@ -41313,7 +41321,7 @@
       <c r="W165" t="inlineStr"/>
       <c r="X165" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.679109+00:00</t>
+          <t>2026-10-17T11:37:12.504792+00:00</t>
         </is>
       </c>
     </row>
@@ -41409,7 +41417,7 @@
       <c r="W166" t="inlineStr"/>
       <c r="X166" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.679528+00:00</t>
+          <t>2026-10-17T11:37:12.505128+00:00</t>
         </is>
       </c>
     </row>
@@ -41505,7 +41513,7 @@
       <c r="W167" t="inlineStr"/>
       <c r="X167" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.680269+00:00</t>
+          <t>2026-10-17T11:37:12.505841+00:00</t>
         </is>
       </c>
     </row>
@@ -41601,7 +41609,7 @@
       <c r="W168" t="inlineStr"/>
       <c r="X168" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.680779+00:00</t>
+          <t>2026-10-17T11:37:12.506219+00:00</t>
         </is>
       </c>
     </row>
@@ -41697,7 +41705,7 @@
       <c r="W169" t="inlineStr"/>
       <c r="X169" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.680957+00:00</t>
+          <t>2026-10-17T11:37:12.506386+00:00</t>
         </is>
       </c>
     </row>
@@ -41793,7 +41801,7 @@
       <c r="W170" t="inlineStr"/>
       <c r="X170" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.681107+00:00</t>
+          <t>2026-10-17T11:37:12.506532+00:00</t>
         </is>
       </c>
     </row>
@@ -41889,7 +41897,7 @@
       <c r="W171" t="inlineStr"/>
       <c r="X171" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.681247+00:00</t>
+          <t>2026-10-17T11:37:12.506660+00:00</t>
         </is>
       </c>
     </row>
@@ -41985,7 +41993,7 @@
       <c r="W172" t="inlineStr"/>
       <c r="X172" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.681341+00:00</t>
+          <t>2026-10-17T11:37:12.506718+00:00</t>
         </is>
       </c>
     </row>
@@ -42081,7 +42089,7 @@
       <c r="W173" t="inlineStr"/>
       <c r="X173" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.681414+00:00</t>
+          <t>2026-10-17T11:37:12.506780+00:00</t>
         </is>
       </c>
     </row>
@@ -42177,7 +42185,7 @@
       <c r="W174" t="inlineStr"/>
       <c r="X174" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.681786+00:00</t>
+          <t>2026-10-17T11:37:12.507131+00:00</t>
         </is>
       </c>
     </row>
@@ -42273,7 +42281,7 @@
       <c r="W175" t="inlineStr"/>
       <c r="X175" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.682157+00:00</t>
+          <t>2026-10-17T11:37:12.507516+00:00</t>
         </is>
       </c>
     </row>
@@ -42369,7 +42377,7 @@
       <c r="W176" t="inlineStr"/>
       <c r="X176" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.682456+00:00</t>
+          <t>2026-10-17T11:37:12.507796+00:00</t>
         </is>
       </c>
     </row>
@@ -42465,7 +42473,7 @@
       <c r="W177" t="inlineStr"/>
       <c r="X177" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.682800+00:00</t>
+          <t>2026-10-17T11:37:12.508135+00:00</t>
         </is>
       </c>
     </row>
@@ -42561,7 +42569,7 @@
       <c r="W178" t="inlineStr"/>
       <c r="X178" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.682930+00:00</t>
+          <t>2026-10-17T11:37:12.508261+00:00</t>
         </is>
       </c>
     </row>
@@ -42657,7 +42665,7 @@
       <c r="W179" t="inlineStr"/>
       <c r="X179" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.683616+00:00</t>
+          <t>2026-10-17T11:37:12.508950+00:00</t>
         </is>
       </c>
     </row>
@@ -42753,7 +42761,7 @@
       <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.684231+00:00</t>
+          <t>2026-10-17T11:37:12.509578+00:00</t>
         </is>
       </c>
     </row>
@@ -42849,7 +42857,7 @@
       <c r="W181" t="inlineStr"/>
       <c r="X181" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.684363+00:00</t>
+          <t>2026-10-17T11:37:12.509677+00:00</t>
         </is>
       </c>
     </row>
@@ -42945,7 +42953,7 @@
       <c r="W182" t="inlineStr"/>
       <c r="X182" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.684854+00:00</t>
+          <t>2026-10-17T11:37:12.510167+00:00</t>
         </is>
       </c>
     </row>
@@ -43041,7 +43049,7 @@
       <c r="W183" t="inlineStr"/>
       <c r="X183" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.684922+00:00</t>
+          <t>2026-10-17T11:37:12.510232+00:00</t>
         </is>
       </c>
     </row>
@@ -43137,7 +43145,7 @@
       <c r="W184" t="inlineStr"/>
       <c r="X184" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.685095+00:00</t>
+          <t>2026-10-17T11:37:12.510285+00:00</t>
         </is>
       </c>
     </row>
@@ -43233,7 +43241,7 @@
       <c r="W185" t="inlineStr"/>
       <c r="X185" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.685416+00:00</t>
+          <t>2026-10-17T11:37:12.510582+00:00</t>
         </is>
       </c>
     </row>
@@ -43329,7 +43337,7 @@
       <c r="W186" t="inlineStr"/>
       <c r="X186" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.685493+00:00</t>
+          <t>2026-10-17T11:37:12.510630+00:00</t>
         </is>
       </c>
     </row>
@@ -43425,7 +43433,7 @@
       <c r="W187" t="inlineStr"/>
       <c r="X187" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.685661+00:00</t>
+          <t>2026-10-17T11:37:12.510784+00:00</t>
         </is>
       </c>
     </row>
@@ -43521,7 +43529,7 @@
       <c r="W188" t="inlineStr"/>
       <c r="X188" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.685714+00:00</t>
+          <t>2026-10-17T11:37:12.510835+00:00</t>
         </is>
       </c>
     </row>
@@ -43617,7 +43625,7 @@
       <c r="W189" t="inlineStr"/>
       <c r="X189" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.686121+00:00</t>
+          <t>2026-10-17T11:37:12.511162+00:00</t>
         </is>
       </c>
     </row>
@@ -43713,7 +43721,7 @@
       <c r="W190" t="inlineStr"/>
       <c r="X190" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.686203+00:00</t>
+          <t>2026-10-17T11:37:12.511226+00:00</t>
         </is>
       </c>
     </row>
@@ -43809,7 +43817,7 @@
       <c r="W191" t="inlineStr"/>
       <c r="X191" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.686863+00:00</t>
+          <t>2026-10-17T11:37:12.511823+00:00</t>
         </is>
       </c>
     </row>
@@ -43905,7 +43913,7 @@
       <c r="W192" t="inlineStr"/>
       <c r="X192" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.686960+00:00</t>
+          <t>2026-10-17T11:37:12.511906+00:00</t>
         </is>
       </c>
     </row>
@@ -44001,7 +44009,7 @@
       <c r="W193" t="inlineStr"/>
       <c r="X193" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.687325+00:00</t>
+          <t>2026-10-17T11:37:12.512244+00:00</t>
         </is>
       </c>
     </row>
@@ -44097,7 +44105,7 @@
       <c r="W194" t="inlineStr"/>
       <c r="X194" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.687481+00:00</t>
+          <t>2026-10-17T11:37:12.512400+00:00</t>
         </is>
       </c>
     </row>
@@ -44193,7 +44201,7 @@
       <c r="W195" t="inlineStr"/>
       <c r="X195" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.687783+00:00</t>
+          <t>2026-10-17T11:37:12.512648+00:00</t>
         </is>
       </c>
     </row>
@@ -44289,7 +44297,7 @@
       <c r="W196" t="inlineStr"/>
       <c r="X196" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.687859+00:00</t>
+          <t>2026-10-17T11:37:12.512703+00:00</t>
         </is>
       </c>
     </row>
@@ -44385,7 +44393,7 @@
       <c r="W197" t="inlineStr"/>
       <c r="X197" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.687984+00:00</t>
+          <t>2026-10-17T11:37:12.512826+00:00</t>
         </is>
       </c>
     </row>
@@ -44481,7 +44489,7 @@
       <c r="W198" t="inlineStr"/>
       <c r="X198" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.688402+00:00</t>
+          <t>2026-10-17T11:37:12.513164+00:00</t>
         </is>
       </c>
     </row>
@@ -44577,7 +44585,7 @@
       <c r="W199" t="inlineStr"/>
       <c r="X199" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.688823+00:00</t>
+          <t>2026-10-17T11:37:12.513539+00:00</t>
         </is>
       </c>
     </row>
@@ -44673,7 +44681,7 @@
       <c r="W200" t="inlineStr"/>
       <c r="X200" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.688907+00:00</t>
+          <t>2026-10-17T11:37:12.513611+00:00</t>
         </is>
       </c>
     </row>
@@ -44769,7 +44777,7 @@
       <c r="W201" t="inlineStr"/>
       <c r="X201" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.689395+00:00</t>
+          <t>2026-10-17T11:37:12.514068+00:00</t>
         </is>
       </c>
     </row>
@@ -44865,7 +44873,7 @@
       <c r="W202" t="inlineStr"/>
       <c r="X202" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.689729+00:00</t>
+          <t>2026-10-17T11:37:12.514383+00:00</t>
         </is>
       </c>
     </row>
@@ -44961,7 +44969,7 @@
       <c r="W203" t="inlineStr"/>
       <c r="X203" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.689781+00:00</t>
+          <t>2026-10-17T11:37:12.514434+00:00</t>
         </is>
       </c>
     </row>
@@ -45057,7 +45065,7 @@
       <c r="W204" t="inlineStr"/>
       <c r="X204" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.690077+00:00</t>
+          <t>2026-10-17T11:37:12.514730+00:00</t>
         </is>
       </c>
     </row>
@@ -45153,7 +45161,7 @@
       <c r="W205" t="inlineStr"/>
       <c r="X205" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.690271+00:00</t>
+          <t>2026-10-17T11:37:12.514792+00:00</t>
         </is>
       </c>
     </row>
@@ -45249,7 +45257,7 @@
       <c r="W206" t="inlineStr"/>
       <c r="X206" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.690397+00:00</t>
+          <t>2026-10-17T11:37:12.514864+00:00</t>
         </is>
       </c>
     </row>
@@ -45345,7 +45353,7 @@
       <c r="W207" t="inlineStr"/>
       <c r="X207" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.690462+00:00</t>
+          <t>2026-10-17T11:37:12.514927+00:00</t>
         </is>
       </c>
     </row>
@@ -45441,7 +45449,7 @@
       <c r="W208" t="inlineStr"/>
       <c r="X208" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.690515+00:00</t>
+          <t>2026-10-17T11:37:12.514979+00:00</t>
         </is>
       </c>
     </row>
@@ -45537,7 +45545,7 @@
       <c r="W209" t="inlineStr"/>
       <c r="X209" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.690566+00:00</t>
+          <t>2026-10-17T11:37:12.515028+00:00</t>
         </is>
       </c>
     </row>
@@ -45633,7 +45641,7 @@
       <c r="W210" t="inlineStr"/>
       <c r="X210" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.691066+00:00</t>
+          <t>2026-10-17T11:37:12.515357+00:00</t>
         </is>
       </c>
     </row>
@@ -45729,7 +45737,7 @@
       <c r="W211" t="inlineStr"/>
       <c r="X211" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.691225+00:00</t>
+          <t>2026-10-17T11:37:12.515487+00:00</t>
         </is>
       </c>
     </row>
@@ -45825,7 +45833,7 @@
       <c r="W212" t="inlineStr"/>
       <c r="X212" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.691423+00:00</t>
+          <t>2026-10-17T11:37:12.515634+00:00</t>
         </is>
       </c>
     </row>
@@ -45921,7 +45929,7 @@
       <c r="W213" t="inlineStr"/>
       <c r="X213" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.691807+00:00</t>
+          <t>2026-10-17T11:37:12.515784+00:00</t>
         </is>
       </c>
     </row>
@@ -45988,7 +45996,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P214" t="inlineStr">
@@ -46017,7 +46025,7 @@
       <c r="W214" t="inlineStr"/>
       <c r="X214" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.692795+00:00</t>
+          <t>2026-10-17T11:37:12.516527+00:00</t>
         </is>
       </c>
     </row>
@@ -46084,7 +46092,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P215" t="inlineStr">
@@ -46113,7 +46121,7 @@
       <c r="W215" t="inlineStr"/>
       <c r="X215" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.693259+00:00</t>
+          <t>2026-10-17T11:37:12.517135+00:00</t>
         </is>
       </c>
     </row>
@@ -46180,7 +46188,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P216" t="inlineStr">
@@ -46209,7 +46217,7 @@
       <c r="W216" t="inlineStr"/>
       <c r="X216" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.694843+00:00</t>
+          <t>2026-10-17T11:37:12.518618+00:00</t>
         </is>
       </c>
     </row>
@@ -46276,7 +46284,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P217" t="inlineStr">
@@ -46305,7 +46313,7 @@
       <c r="W217" t="inlineStr"/>
       <c r="X217" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.695784+00:00</t>
+          <t>2026-10-17T11:37:12.519422+00:00</t>
         </is>
       </c>
     </row>
@@ -46372,7 +46380,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P218" t="inlineStr">
@@ -46401,7 +46409,7 @@
       <c r="W218" t="inlineStr"/>
       <c r="X218" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.697122+00:00</t>
+          <t>2026-10-17T11:37:12.520503+00:00</t>
         </is>
       </c>
     </row>
@@ -46468,7 +46476,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P219" t="inlineStr">
@@ -46497,7 +46505,7 @@
       <c r="W219" t="inlineStr"/>
       <c r="X219" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.697881+00:00</t>
+          <t>2026-10-17T11:37:12.520958+00:00</t>
         </is>
       </c>
     </row>
@@ -46564,7 +46572,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P220" t="inlineStr">
@@ -46593,7 +46601,7 @@
       <c r="W220" t="inlineStr"/>
       <c r="X220" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.698870+00:00</t>
+          <t>2026-10-17T11:37:12.521930+00:00</t>
         </is>
       </c>
     </row>
@@ -46660,7 +46668,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P221" t="inlineStr">
@@ -46689,7 +46697,7 @@
       <c r="W221" t="inlineStr"/>
       <c r="X221" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.699610+00:00</t>
+          <t>2026-10-17T11:37:12.522673+00:00</t>
         </is>
       </c>
     </row>
@@ -46756,7 +46764,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P222" t="inlineStr">
@@ -46785,7 +46793,7 @@
       <c r="W222" t="inlineStr"/>
       <c r="X222" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.700214+00:00</t>
+          <t>2026-10-17T11:37:12.523107+00:00</t>
         </is>
       </c>
     </row>
@@ -46852,7 +46860,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P223" t="inlineStr">
@@ -46881,7 +46889,7 @@
       <c r="W223" t="inlineStr"/>
       <c r="X223" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.701321+00:00</t>
+          <t>2026-10-17T11:37:12.524168+00:00</t>
         </is>
       </c>
     </row>
@@ -46948,7 +46956,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P224" t="inlineStr">
@@ -46977,7 +46985,7 @@
       <c r="W224" t="inlineStr"/>
       <c r="X224" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.702029+00:00</t>
+          <t>2026-10-17T11:37:12.524832+00:00</t>
         </is>
       </c>
     </row>
@@ -47044,7 +47052,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P225" t="inlineStr">
@@ -47073,7 +47081,7 @@
       <c r="W225" t="inlineStr"/>
       <c r="X225" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.703254+00:00</t>
+          <t>2026-10-17T11:37:12.526067+00:00</t>
         </is>
       </c>
     </row>
@@ -47140,7 +47148,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P226" t="inlineStr">
@@ -47169,7 +47177,7 @@
       <c r="W226" t="inlineStr"/>
       <c r="X226" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.704361+00:00</t>
+          <t>2026-10-17T11:37:12.526515+00:00</t>
         </is>
       </c>
     </row>
@@ -47236,7 +47244,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P227" t="inlineStr">
@@ -47265,7 +47273,7 @@
       <c r="W227" t="inlineStr"/>
       <c r="X227" t="inlineStr">
         <is>
-          <t>2026-10-17T11:36:14.705233+00:00</t>
+          <t>2026-10-17T11:37:12.527360+00:00</t>
         </is>
       </c>
     </row>
@@ -47280,7 +47288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47453,21 +47461,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R07238.supplementary.0b7925ad1ed9c793</t>
+          <t>R07238.derived.49b84e369d4bb31b</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>supplementary</t>
+          <t>derived</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0b7925ad1ed9c7939a79ba6294d17abc4b23fca77e52ec50df5463d050940d1e</t>
+          <t>49b84e369d4bb31b4ebdcd25265be3174105c3433e6fbb865f34a445775516a1</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>49526</v>
+        <v>34855493</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -47476,7 +47484,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>mmc1.docx</t>
+          <t>g a.skp</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -47488,35 +47496,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R03161</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R07238.derived.49b84e369d4bb31b</t>
+          <t>R03161.transport_archive.0ef4d4796c84feff</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>transport_archive</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>49b84e369d4bb31b4ebdcd25265be3174105c3433e6fbb865f34a445775516a1</t>
+          <t>0ef4d4796c84fefff7b8450bc56400f8c59f4bdcf074fc51404edff5e4e217f6</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>34855493</v>
+        <v>726772</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/supplementaryFiles</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>g a.skp</t>
+          <t>PMC5627928_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -47528,12 +47536,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>R03161</t>
+          <t>R08877</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>R03161.transport_archive.0ef4d4796c84feff</t>
+          <t>R08877.transport_archive.ed8e864a3225e9c4</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -47543,20 +47551,20 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0ef4d4796c84fefff7b8450bc56400f8c59f4bdcf074fc51404edff5e4e217f6</t>
+          <t>ed8e864a3225e9c4cecf84e5f4670c985de4c6d453d0b7b459ad5870e6627f97</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>726772</v>
+        <v>704921</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/supplementaryFiles</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>PMC5627928_supplementaryFiles.zip</t>
+          <t>PMC10714394_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -47568,12 +47576,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>R08877</t>
+          <t>R09236</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R08877.transport_archive.ed8e864a3225e9c4</t>
+          <t>R09236.transport_archive.f3c6856282b7e8d6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -47583,20 +47591,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ed8e864a3225e9c4cecf84e5f4670c985de4c6d453d0b7b459ad5870e6627f97</t>
+          <t>f3c6856282b7e8d694d35a87eae016d8e66aa902189c7c3311a1153ea24752e0</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>704921</v>
+        <v>483405</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/supplementaryFiles</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PMC10714394_supplementaryFiles.zip</t>
+          <t>PMC10535533_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -47608,12 +47616,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R09236</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>R09236.transport_archive.f3c6856282b7e8d6</t>
+          <t>R10086.transport_archive.4d9eddf454b786ed</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -47623,20 +47631,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>f3c6856282b7e8d694d35a87eae016d8e66aa902189c7c3311a1153ea24752e0</t>
+          <t>4d9eddf454b786eddece423a320b28d7f96959a935334ddc7c7e2fe32d39bc9b</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>483405</v>
+        <v>641038</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/supplementaryFiles</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>PMC10535533_supplementaryFiles.zip</t>
+          <t>PMC10837232_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -47648,12 +47656,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>R10086</t>
+          <t>R12985</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>R10086.transport_archive.4d9eddf454b786ed</t>
+          <t>R12985.transport_archive.418d45f1ca296020</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -47663,20 +47671,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4d9eddf454b786eddece423a320b28d7f96959a935334ddc7c7e2fe32d39bc9b</t>
+          <t>418d45f1ca2960209df0bfc1c3d44069413edc213239570a3d71d08d01f3e3e0</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>641038</v>
+        <v>672244</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/supplementaryFiles</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>PMC10837232_supplementaryFiles.zip</t>
+          <t>PMC12937426_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -47688,12 +47696,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>R12985</t>
+          <t>R06325</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>R12985.transport_archive.418d45f1ca296020</t>
+          <t>R06325.transport_archive.6eb4ef126661714a</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -47703,20 +47711,20 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>418d45f1ca2960209df0bfc1c3d44069413edc213239570a3d71d08d01f3e3e0</t>
+          <t>6eb4ef126661714ae89bde97acdddac2c2a582864ca26ff9af569cfe609a4226</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>672244</v>
+        <v>1730580</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/supplementaryFiles</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>PMC12937426_supplementaryFiles.zip</t>
+          <t>PMC8290346_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -47728,12 +47736,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>R06325</t>
+          <t>R07238</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>R06325.transport_archive.6eb4ef126661714a</t>
+          <t>R07238.transport_archive.3785c23cb2f4ab50</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -47743,20 +47751,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6eb4ef126661714ae89bde97acdddac2c2a582864ca26ff9af569cfe609a4226</t>
+          <t>3785c23cb2f4ab50f5b2b5cbb581da63ced9f8d1e69a91e6faca839b6b57587d</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1730580</v>
+        <v>14596266</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>PMC8290346_supplementaryFiles.zip</t>
+          <t>PMC8044681_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -47768,12 +47776,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R08646</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>R07238.transport_archive.3785c23cb2f4ab50</t>
+          <t>R08646.transport_archive.ecda9ea461a3deb3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -47783,20 +47791,20 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3785c23cb2f4ab50f5b2b5cbb581da63ced9f8d1e69a91e6faca839b6b57587d</t>
+          <t>ecda9ea461a3deb361931eb51186e88488c4d6ae284899e1feb1d611de42550a</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>14596266</v>
+        <v>1539133</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>PMC8044681_supplementaryFiles.zip</t>
+          <t>PMC10559078_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -47808,12 +47816,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>R08646</t>
+          <t>R11844</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>R08646.transport_archive.ecda9ea461a3deb3</t>
+          <t>R11844.transport_archive.60ef29cf0a557bf4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -47823,20 +47831,20 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ecda9ea461a3deb361931eb51186e88488c4d6ae284899e1feb1d611de42550a</t>
+          <t>60ef29cf0a557bf44838f4a3f45e2dbf1b1a2001547f5c0b976b48cc64c1b6d9</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1539133</v>
+        <v>521862</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/supplementaryFiles</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>PMC10559078_supplementaryFiles.zip</t>
+          <t>PMC12125087_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -47848,12 +47856,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>R11844</t>
+          <t>R05213</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>R11844.transport_archive.60ef29cf0a557bf4</t>
+          <t>R05213.transport_archive.c61c88cf9fd489be</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -47863,20 +47871,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>60ef29cf0a557bf44838f4a3f45e2dbf1b1a2001547f5c0b976b48cc64c1b6d9</t>
+          <t>c61c88cf9fd489beab88c1b72bbfe5f13167f32c984b6dba6e48ba97c6136b7b</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>521862</v>
+        <v>1960371</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/supplementaryFiles</t>
+          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/supplementaryFiles</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>PMC12125087_supplementaryFiles.zip</t>
+          <t>PMC6858683_supplementaryFiles.zip</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -47888,35 +47896,31 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>R05213</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R05213.transport_archive.c61c88cf9fd489be</t>
+          <t>R10086.main.84777bfb7a2cd42f</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>c61c88cf9fd489beab88c1b72bbfe5f13167f32c984b6dba6e48ba97c6136b7b</t>
+          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1960371</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/supplementaryFiles</t>
-        </is>
-      </c>
+        <v>984310</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>PMC6858683_supplementaryFiles.zip</t>
+          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -47928,12 +47932,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>R10086</t>
+          <t>R03155</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R10086.main.84777bfb7a2cd42f</t>
+          <t>R03155.main.2875ce0c137df622</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -47943,16 +47947,20 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
+          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>984310</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
+        <v>5745828</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
+          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -47964,12 +47972,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>R03155</t>
+          <t>R06036</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R03155.main.2875ce0c137df622</t>
+          <t>R06036.main.0bdc7b19fdb70091</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -47979,20 +47987,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
+          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>5745828</v>
+        <v>927168</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
+          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
+          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -48004,12 +48012,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>R06036</t>
+          <t>R13899</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R06036.main.0bdc7b19fdb70091</t>
+          <t>R13899.main.19143e56fa77ce99</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -48019,20 +48027,16 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
+          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>927168</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
-        </is>
-      </c>
+        <v>479092</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
+          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -48044,12 +48048,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>R13899</t>
+          <t>R13955</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R13899.main.19143e56fa77ce99</t>
+          <t>R13955.main.6714f79deccd703d</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -48059,59 +48063,23 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
+          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>479092</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
+        <v>14662119</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>R13955</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>R13955.main.6714f79deccd703d</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>14662119</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
         <is>
           <t>历史已获取，当前原件未恢复</t>
         </is>

</xml_diff>

<commit_message>
Preserve corrected supplementary evidence and external database size metadata
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -6471,7 +6471,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>partial_or_access_failed</t>
+          <t>downloaded</t>
         </is>
       </c>
       <c r="H141" t="b">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.303087+00:00</t>
+          <t>2026-10-17T11:42:59.362587+00:00</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24455,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.303983+00:00</t>
+          <t>2026-10-17T11:42:59.363566+00:00</t>
         </is>
       </c>
     </row>
@@ -24555,7 +24555,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.304004+00:00</t>
+          <t>2026-10-17T11:42:59.363595+00:00</t>
         </is>
       </c>
     </row>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.304222+00:00</t>
+          <t>2026-10-17T11:42:59.363833+00:00</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24771,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.308146+00:00</t>
+          <t>2026-10-17T11:42:59.364965+00:00</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24879,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.308648+00:00</t>
+          <t>2026-10-17T11:42:59.365568+00:00</t>
         </is>
       </c>
     </row>
@@ -24987,7 +24987,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.314349+00:00</t>
+          <t>2026-10-17T11:42:59.371124+00:00</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.316609+00:00</t>
+          <t>2026-10-17T11:42:59.373557+00:00</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.317523+00:00</t>
+          <t>2026-10-17T11:42:59.374457+00:00</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25311,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.317844+00:00</t>
+          <t>2026-10-17T11:42:59.374852+00:00</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.318560+00:00</t>
+          <t>2026-10-17T11:42:59.375581+00:00</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25527,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.319203+00:00</t>
+          <t>2026-10-17T11:42:59.376216+00:00</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25635,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.320097+00:00</t>
+          <t>2026-10-17T11:42:59.377100+00:00</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.320346+00:00</t>
+          <t>2026-10-17T11:42:59.377359+00:00</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25851,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.321201+00:00</t>
+          <t>2026-10-17T11:42:59.378216+00:00</t>
         </is>
       </c>
     </row>
@@ -25959,7 +25959,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.331059+00:00</t>
+          <t>2026-10-17T11:42:59.386871+00:00</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26067,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.331918+00:00</t>
+          <t>2026-10-17T11:42:59.387809+00:00</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26175,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.334746+00:00</t>
+          <t>2026-10-17T11:42:59.389095+00:00</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26283,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.341748+00:00</t>
+          <t>2026-10-17T11:42:59.391663+00:00</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26391,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.342975+00:00</t>
+          <t>2026-10-17T11:42:59.392860+00:00</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26499,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.344179+00:00</t>
+          <t>2026-10-17T11:42:59.394174+00:00</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26607,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.348763+00:00</t>
+          <t>2026-10-17T11:42:59.398752+00:00</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.351038+00:00</t>
+          <t>2026-10-17T11:42:59.401000+00:00</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.352832+00:00</t>
+          <t>2026-10-17T11:42:59.402895+00:00</t>
         </is>
       </c>
     </row>
@@ -26931,7 +26931,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.353508+00:00</t>
+          <t>2026-10-17T11:42:59.403565+00:00</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.353864+00:00</t>
+          <t>2026-10-17T11:42:59.403947+00:00</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27147,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.356011+00:00</t>
+          <t>2026-10-17T11:42:59.406172+00:00</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.357278+00:00</t>
+          <t>2026-10-17T11:42:59.407521+00:00</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27363,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.359391+00:00</t>
+          <t>2026-10-17T11:42:59.409662+00:00</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.361444+00:00</t>
+          <t>2026-10-17T11:42:59.411756+00:00</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27579,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.362021+00:00</t>
+          <t>2026-10-17T11:42:59.412358+00:00</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27687,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.362589+00:00</t>
+          <t>2026-10-17T11:42:59.412911+00:00</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27795,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.364197+00:00</t>
+          <t>2026-10-17T11:42:59.414879+00:00</t>
         </is>
       </c>
     </row>
@@ -27903,7 +27903,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.366977+00:00</t>
+          <t>2026-10-17T11:42:59.417946+00:00</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28011,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.369091+00:00</t>
+          <t>2026-10-17T11:42:59.420136+00:00</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28119,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.370281+00:00</t>
+          <t>2026-10-17T11:42:59.421413+00:00</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28227,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.373128+00:00</t>
+          <t>2026-10-17T11:42:59.424313+00:00</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28335,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.373845+00:00</t>
+          <t>2026-10-17T11:42:59.424994+00:00</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28443,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.375431+00:00</t>
+          <t>2026-10-17T11:42:59.426709+00:00</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28551,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.375690+00:00</t>
+          <t>2026-10-17T11:42:59.426989+00:00</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28659,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.377585+00:00</t>
+          <t>2026-10-17T11:42:59.428841+00:00</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28767,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.380411+00:00</t>
+          <t>2026-10-17T11:42:59.431699+00:00</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.381730+00:00</t>
+          <t>2026-10-17T11:42:59.433089+00:00</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28983,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.382253+00:00</t>
+          <t>2026-10-17T11:42:59.433648+00:00</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29091,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.384837+00:00</t>
+          <t>2026-10-17T11:42:59.436352+00:00</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.385966+00:00</t>
+          <t>2026-10-17T11:42:59.437768+00:00</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29307,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.389538+00:00</t>
+          <t>2026-10-17T11:42:59.441198+00:00</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29415,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.391235+00:00</t>
+          <t>2026-10-17T11:42:59.442875+00:00</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.393076+00:00</t>
+          <t>2026-10-17T11:42:59.444700+00:00</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29631,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.394033+00:00</t>
+          <t>2026-10-17T11:42:59.445765+00:00</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29739,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.394474+00:00</t>
+          <t>2026-10-17T11:42:59.446209+00:00</t>
         </is>
       </c>
     </row>
@@ -29847,7 +29847,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.394836+00:00</t>
+          <t>2026-10-17T11:42:59.446633+00:00</t>
         </is>
       </c>
     </row>
@@ -29955,7 +29955,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.396307+00:00</t>
+          <t>2026-10-17T11:42:59.448235+00:00</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.397612+00:00</t>
+          <t>2026-10-17T11:42:59.449734+00:00</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30171,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.399101+00:00</t>
+          <t>2026-10-17T11:42:59.451341+00:00</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30279,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.399440+00:00</t>
+          <t>2026-10-17T11:42:59.451692+00:00</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30387,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.400597+00:00</t>
+          <t>2026-10-17T11:42:59.452849+00:00</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30495,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.401971+00:00</t>
+          <t>2026-10-17T11:42:59.454360+00:00</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.402574+00:00</t>
+          <t>2026-10-17T11:42:59.454934+00:00</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.403514+00:00</t>
+          <t>2026-10-17T11:42:59.455862+00:00</t>
         </is>
       </c>
     </row>
@@ -30819,7 +30819,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.403818+00:00</t>
+          <t>2026-10-17T11:42:59.456176+00:00</t>
         </is>
       </c>
     </row>
@@ -30927,7 +30927,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.408981+00:00</t>
+          <t>2026-10-17T11:42:59.461923+00:00</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31035,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.409417+00:00</t>
+          <t>2026-10-17T11:42:59.462418+00:00</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31143,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.409986+00:00</t>
+          <t>2026-10-17T11:42:59.462977+00:00</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31251,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.410432+00:00</t>
+          <t>2026-10-17T11:42:59.463416+00:00</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31359,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.411495+00:00</t>
+          <t>2026-10-17T11:42:59.464466+00:00</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31467,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.414438+00:00</t>
+          <t>2026-10-17T11:42:59.467638+00:00</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31575,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.414679+00:00</t>
+          <t>2026-10-17T11:42:59.467917+00:00</t>
         </is>
       </c>
     </row>
@@ -31683,7 +31683,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.419070+00:00</t>
+          <t>2026-10-17T11:42:59.472358+00:00</t>
         </is>
       </c>
     </row>
@@ -31791,7 +31791,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.419910+00:00</t>
+          <t>2026-10-17T11:42:59.473135+00:00</t>
         </is>
       </c>
     </row>
@@ -31899,7 +31899,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.422040+00:00</t>
+          <t>2026-10-17T11:42:59.475382+00:00</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32007,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.423783+00:00</t>
+          <t>2026-10-17T11:42:59.477168+00:00</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32115,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.424655+00:00</t>
+          <t>2026-10-17T11:42:59.478100+00:00</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32223,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.426067+00:00</t>
+          <t>2026-10-17T11:42:59.479514+00:00</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.428245+00:00</t>
+          <t>2026-10-17T11:42:59.481729+00:00</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32439,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.436161+00:00</t>
+          <t>2026-10-17T11:42:59.491521+00:00</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32547,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.437512+00:00</t>
+          <t>2026-10-17T11:42:59.492995+00:00</t>
         </is>
       </c>
     </row>
@@ -32655,7 +32655,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.437668+00:00</t>
+          <t>2026-10-17T11:42:59.493241+00:00</t>
         </is>
       </c>
     </row>
@@ -32755,7 +32755,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.437680+00:00</t>
+          <t>2026-10-17T11:42:59.493263+00:00</t>
         </is>
       </c>
     </row>
@@ -32863,7 +32863,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.442625+00:00</t>
+          <t>2026-10-17T11:42:59.498723+00:00</t>
         </is>
       </c>
     </row>
@@ -32967,7 +32967,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.443005+00:00</t>
+          <t>2026-10-17T11:42:59.499148+00:00</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33071,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.443381+00:00</t>
+          <t>2026-10-17T11:42:59.499525+00:00</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33175,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.443776+00:00</t>
+          <t>2026-10-17T11:42:59.499919+00:00</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33279,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.444473+00:00</t>
+          <t>2026-10-17T11:42:59.500631+00:00</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33383,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.445862+00:00</t>
+          <t>2026-10-17T11:42:59.502000+00:00</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33487,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.446685+00:00</t>
+          <t>2026-10-17T11:42:59.502806+00:00</t>
         </is>
       </c>
     </row>
@@ -33591,7 +33591,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.446982+00:00</t>
+          <t>2026-10-17T11:42:59.503108+00:00</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33699,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.447632+00:00</t>
+          <t>2026-10-17T11:42:59.503743+00:00</t>
         </is>
       </c>
     </row>
@@ -33799,7 +33799,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.447645+00:00</t>
+          <t>2026-10-17T11:42:59.503757+00:00</t>
         </is>
       </c>
     </row>
@@ -33907,7 +33907,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.447692+00:00</t>
+          <t>2026-10-17T11:42:59.503811+00:00</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.447905+00:00</t>
+          <t>2026-10-17T11:42:59.504036+00:00</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34123,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.448021+00:00</t>
+          <t>2026-10-17T11:42:59.504169+00:00</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34235,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.448135+00:00</t>
+          <t>2026-10-17T11:42:59.504283+00:00</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34343,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.448520+00:00</t>
+          <t>2026-10-17T11:42:59.504743+00:00</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34451,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.448705+00:00</t>
+          <t>2026-10-17T11:42:59.504962+00:00</t>
         </is>
       </c>
     </row>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.448759+00:00</t>
+          <t>2026-10-17T11:42:59.505020+00:00</t>
         </is>
       </c>
     </row>
@@ -34675,7 +34675,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.448820+00:00</t>
+          <t>2026-10-17T11:42:59.505104+00:00</t>
         </is>
       </c>
     </row>
@@ -34787,7 +34787,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.448959+00:00</t>
+          <t>2026-10-17T11:42:59.505257+00:00</t>
         </is>
       </c>
     </row>
@@ -34899,7 +34899,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.449003+00:00</t>
+          <t>2026-10-17T11:42:59.505330+00:00</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.449492+00:00</t>
+          <t>2026-10-17T11:42:59.506011+00:00</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35115,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.449544+00:00</t>
+          <t>2026-10-17T11:42:59.506091+00:00</t>
         </is>
       </c>
     </row>
@@ -35186,7 +35186,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>local_acquired_pending_remote_readback</t>
+          <t>git_remote_verified_20261017</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
@@ -35223,7 +35223,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.449614+00:00</t>
+          <t>2026-10-17T11:42:59.506166+00:00</t>
         </is>
       </c>
     </row>
@@ -35331,7 +35331,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.459410+00:00</t>
+          <t>2026-10-17T11:42:59.516379+00:00</t>
         </is>
       </c>
     </row>
@@ -35389,12 +35389,12 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>available_as_verified_original_archive_member</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>available_via_canonical_original_archive</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
@@ -35435,7 +35435,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.459480+00:00</t>
+          <t>2026-10-17T11:42:59.516457+00:00</t>
         </is>
       </c>
     </row>
@@ -35543,7 +35543,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.459579+00:00</t>
+          <t>2026-10-17T11:42:59.664314+00:00</t>
         </is>
       </c>
     </row>
@@ -35651,7 +35651,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.459808+00:00</t>
+          <t>2026-10-17T11:42:59.664603+00:00</t>
         </is>
       </c>
     </row>
@@ -35759,7 +35759,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.460799+00:00</t>
+          <t>2026-10-17T11:42:59.665853+00:00</t>
         </is>
       </c>
     </row>
@@ -35861,7 +35861,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.460885+00:00</t>
+          <t>2026-10-17T11:42:59.665972+00:00</t>
         </is>
       </c>
     </row>
@@ -35917,12 +35917,12 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
@@ -35955,7 +35955,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.460895+00:00</t>
+          <t>2026-10-17T11:42:59.665988+00:00</t>
         </is>
       </c>
     </row>
@@ -36057,7 +36057,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.460973+00:00</t>
+          <t>2026-10-17T11:42:59.666219+00:00</t>
         </is>
       </c>
     </row>
@@ -36159,7 +36159,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461056+00:00</t>
+          <t>2026-10-17T11:42:59.666329+00:00</t>
         </is>
       </c>
     </row>
@@ -36261,7 +36261,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461161+00:00</t>
+          <t>2026-10-17T11:42:59.666449+00:00</t>
         </is>
       </c>
     </row>
@@ -36317,12 +36317,12 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P114" t="inlineStr">
@@ -36355,7 +36355,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461172+00:00</t>
+          <t>2026-10-17T11:42:59.666461+00:00</t>
         </is>
       </c>
     </row>
@@ -36457,7 +36457,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461341+00:00</t>
+          <t>2026-10-17T11:42:59.666932+00:00</t>
         </is>
       </c>
     </row>
@@ -36513,12 +36513,12 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -36551,7 +36551,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461355+00:00</t>
+          <t>2026-10-17T11:42:59.666949+00:00</t>
         </is>
       </c>
     </row>
@@ -36653,7 +36653,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461457+00:00</t>
+          <t>2026-10-17T11:42:59.667173+00:00</t>
         </is>
       </c>
     </row>
@@ -36709,12 +36709,12 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -36747,7 +36747,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461468+00:00</t>
+          <t>2026-10-17T11:42:59.667184+00:00</t>
         </is>
       </c>
     </row>
@@ -36849,7 +36849,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461627+00:00</t>
+          <t>2026-10-17T11:42:59.667733+00:00</t>
         </is>
       </c>
     </row>
@@ -36905,12 +36905,12 @@
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -36943,7 +36943,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461639+00:00</t>
+          <t>2026-10-17T11:42:59.667747+00:00</t>
         </is>
       </c>
     </row>
@@ -37045,7 +37045,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461730+00:00</t>
+          <t>2026-10-17T11:42:59.668023+00:00</t>
         </is>
       </c>
     </row>
@@ -37147,7 +37147,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461865+00:00</t>
+          <t>2026-10-17T11:42:59.668155+00:00</t>
         </is>
       </c>
     </row>
@@ -37203,12 +37203,12 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
@@ -37241,7 +37241,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.461876+00:00</t>
+          <t>2026-10-17T11:42:59.668166+00:00</t>
         </is>
       </c>
     </row>
@@ -37343,7 +37343,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.462007+00:00</t>
+          <t>2026-10-17T11:42:59.668786+00:00</t>
         </is>
       </c>
     </row>
@@ -37399,12 +37399,12 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -37437,7 +37437,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.462018+00:00</t>
+          <t>2026-10-17T11:42:59.668798+00:00</t>
         </is>
       </c>
     </row>
@@ -37539,7 +37539,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.462124+00:00</t>
+          <t>2026-10-17T11:42:59.679117+00:00</t>
         </is>
       </c>
     </row>
@@ -37641,7 +37641,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.462412+00:00</t>
+          <t>2026-10-17T11:42:59.679386+00:00</t>
         </is>
       </c>
     </row>
@@ -37697,12 +37697,12 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
@@ -37735,7 +37735,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.462434+00:00</t>
+          <t>2026-10-17T11:42:59.679403+00:00</t>
         </is>
       </c>
     </row>
@@ -37837,7 +37837,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.462603+00:00</t>
+          <t>2026-10-17T11:42:59.679720+00:00</t>
         </is>
       </c>
     </row>
@@ -37939,7 +37939,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.462803+00:00</t>
+          <t>2026-10-17T11:42:59.679923+00:00</t>
         </is>
       </c>
     </row>
@@ -38041,7 +38041,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.462997+00:00</t>
+          <t>2026-10-17T11:42:59.680120+00:00</t>
         </is>
       </c>
     </row>
@@ -38097,12 +38097,12 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
@@ -38135,7 +38135,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.463009+00:00</t>
+          <t>2026-10-17T11:42:59.680138+00:00</t>
         </is>
       </c>
     </row>
@@ -38237,7 +38237,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.463120+00:00</t>
+          <t>2026-10-17T11:42:59.680497+00:00</t>
         </is>
       </c>
     </row>
@@ -38293,12 +38293,12 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>historical_acquired_current_original_not_restored</t>
+          <t>redundant_transport_archive_not_retained</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>historical_only_original_missing</t>
+          <t>canonical_original_attachments_available</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.463131+00:00</t>
+          <t>2026-10-17T11:42:59.680510+00:00</t>
         </is>
       </c>
     </row>
@@ -38433,7 +38433,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.463223+00:00</t>
+          <t>2026-10-17T11:42:59.681648+00:00</t>
         </is>
       </c>
     </row>
@@ -38541,7 +38541,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.464321+00:00</t>
+          <t>2026-10-17T11:42:59.682701+00:00</t>
         </is>
       </c>
     </row>
@@ -38633,7 +38633,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.479223+00:00</t>
+          <t>2026-10-17T11:42:59.693667+00:00</t>
         </is>
       </c>
     </row>
@@ -38733,7 +38733,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.479671+00:00</t>
+          <t>2026-10-17T11:42:59.694193+00:00</t>
         </is>
       </c>
     </row>
@@ -38821,7 +38821,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.479685+00:00</t>
+          <t>2026-10-17T11:42:59.694217+00:00</t>
         </is>
       </c>
     </row>
@@ -38921,7 +38921,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.480801+00:00</t>
+          <t>2026-10-17T11:42:59.695527+00:00</t>
         </is>
       </c>
     </row>
@@ -39021,7 +39021,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.484207+00:00</t>
+          <t>2026-10-17T11:42:59.699793+00:00</t>
         </is>
       </c>
     </row>
@@ -39121,7 +39121,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.485123+00:00</t>
+          <t>2026-10-17T11:42:59.700865+00:00</t>
         </is>
       </c>
     </row>
@@ -39213,7 +39213,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.485141+00:00</t>
+          <t>2026-10-17T11:42:59.700896+00:00</t>
         </is>
       </c>
     </row>
@@ -39313,7 +39313,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.485858+00:00</t>
+          <t>2026-10-17T11:42:59.701616+00:00</t>
         </is>
       </c>
     </row>
@@ -39405,7 +39405,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.485873+00:00</t>
+          <t>2026-10-17T11:42:59.701637+00:00</t>
         </is>
       </c>
     </row>
@@ -39509,7 +39509,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.486712+00:00</t>
+          <t>2026-10-17T11:42:59.702476+00:00</t>
         </is>
       </c>
     </row>
@@ -39597,7 +39597,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.486727+00:00</t>
+          <t>2026-10-17T11:42:59.702493+00:00</t>
         </is>
       </c>
     </row>
@@ -39689,7 +39689,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.486730+00:00</t>
+          <t>2026-10-17T11:42:59.702497+00:00</t>
         </is>
       </c>
     </row>
@@ -39785,7 +39785,7 @@
       <c r="W149" t="inlineStr"/>
       <c r="X149" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.487515+00:00</t>
+          <t>2026-10-17T11:42:59.703262+00:00</t>
         </is>
       </c>
     </row>
@@ -39881,7 +39881,7 @@
       <c r="W150" t="inlineStr"/>
       <c r="X150" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.488596+00:00</t>
+          <t>2026-10-17T11:42:59.704338+00:00</t>
         </is>
       </c>
     </row>
@@ -39977,7 +39977,7 @@
       <c r="W151" t="inlineStr"/>
       <c r="X151" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.489035+00:00</t>
+          <t>2026-10-17T11:42:59.704752+00:00</t>
         </is>
       </c>
     </row>
@@ -40073,7 +40073,7 @@
       <c r="W152" t="inlineStr"/>
       <c r="X152" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.498819+00:00</t>
+          <t>2026-10-17T11:42:59.715101+00:00</t>
         </is>
       </c>
     </row>
@@ -40169,7 +40169,7 @@
       <c r="W153" t="inlineStr"/>
       <c r="X153" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.498976+00:00</t>
+          <t>2026-10-17T11:42:59.715277+00:00</t>
         </is>
       </c>
     </row>
@@ -40265,7 +40265,7 @@
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.499137+00:00</t>
+          <t>2026-10-17T11:42:59.715597+00:00</t>
         </is>
       </c>
     </row>
@@ -40361,7 +40361,7 @@
       <c r="W155" t="inlineStr"/>
       <c r="X155" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.499585+00:00</t>
+          <t>2026-10-17T11:42:59.716108+00:00</t>
         </is>
       </c>
     </row>
@@ -40457,7 +40457,7 @@
       <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.499843+00:00</t>
+          <t>2026-10-17T11:42:59.716418+00:00</t>
         </is>
       </c>
     </row>
@@ -40553,7 +40553,7 @@
       <c r="W157" t="inlineStr"/>
       <c r="X157" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.500173+00:00</t>
+          <t>2026-10-17T11:42:59.716761+00:00</t>
         </is>
       </c>
     </row>
@@ -40649,7 +40649,7 @@
       <c r="W158" t="inlineStr"/>
       <c r="X158" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.501322+00:00</t>
+          <t>2026-10-17T11:42:59.717914+00:00</t>
         </is>
       </c>
     </row>
@@ -40745,7 +40745,7 @@
       <c r="W159" t="inlineStr"/>
       <c r="X159" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.503087+00:00</t>
+          <t>2026-10-17T11:42:59.719750+00:00</t>
         </is>
       </c>
     </row>
@@ -40841,7 +40841,7 @@
       <c r="W160" t="inlineStr"/>
       <c r="X160" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.503692+00:00</t>
+          <t>2026-10-17T11:42:59.720424+00:00</t>
         </is>
       </c>
     </row>
@@ -40937,7 +40937,7 @@
       <c r="W161" t="inlineStr"/>
       <c r="X161" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.503954+00:00</t>
+          <t>2026-10-17T11:42:59.720758+00:00</t>
         </is>
       </c>
     </row>
@@ -41033,7 +41033,7 @@
       <c r="W162" t="inlineStr"/>
       <c r="X162" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.504006+00:00</t>
+          <t>2026-10-17T11:42:59.720827+00:00</t>
         </is>
       </c>
     </row>
@@ -41129,7 +41129,7 @@
       <c r="W163" t="inlineStr"/>
       <c r="X163" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.504068+00:00</t>
+          <t>2026-10-17T11:42:59.720897+00:00</t>
         </is>
       </c>
     </row>
@@ -41225,7 +41225,7 @@
       <c r="W164" t="inlineStr"/>
       <c r="X164" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.504369+00:00</t>
+          <t>2026-10-17T11:42:59.721180+00:00</t>
         </is>
       </c>
     </row>
@@ -41321,7 +41321,7 @@
       <c r="W165" t="inlineStr"/>
       <c r="X165" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.504792+00:00</t>
+          <t>2026-10-17T11:42:59.721711+00:00</t>
         </is>
       </c>
     </row>
@@ -41417,7 +41417,7 @@
       <c r="W166" t="inlineStr"/>
       <c r="X166" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.505128+00:00</t>
+          <t>2026-10-17T11:42:59.722069+00:00</t>
         </is>
       </c>
     </row>
@@ -41513,7 +41513,7 @@
       <c r="W167" t="inlineStr"/>
       <c r="X167" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.505841+00:00</t>
+          <t>2026-10-17T11:42:59.722763+00:00</t>
         </is>
       </c>
     </row>
@@ -41609,7 +41609,7 @@
       <c r="W168" t="inlineStr"/>
       <c r="X168" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.506219+00:00</t>
+          <t>2026-10-17T11:42:59.723366+00:00</t>
         </is>
       </c>
     </row>
@@ -41705,7 +41705,7 @@
       <c r="W169" t="inlineStr"/>
       <c r="X169" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.506386+00:00</t>
+          <t>2026-10-17T11:42:59.723649+00:00</t>
         </is>
       </c>
     </row>
@@ -41801,7 +41801,7 @@
       <c r="W170" t="inlineStr"/>
       <c r="X170" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.506532+00:00</t>
+          <t>2026-10-17T11:42:59.723808+00:00</t>
         </is>
       </c>
     </row>
@@ -41897,7 +41897,7 @@
       <c r="W171" t="inlineStr"/>
       <c r="X171" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.506660+00:00</t>
+          <t>2026-10-17T11:42:59.723941+00:00</t>
         </is>
       </c>
     </row>
@@ -41993,7 +41993,7 @@
       <c r="W172" t="inlineStr"/>
       <c r="X172" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.506718+00:00</t>
+          <t>2026-10-17T11:42:59.724000+00:00</t>
         </is>
       </c>
     </row>
@@ -42089,7 +42089,7 @@
       <c r="W173" t="inlineStr"/>
       <c r="X173" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.506780+00:00</t>
+          <t>2026-10-17T11:42:59.724069+00:00</t>
         </is>
       </c>
     </row>
@@ -42185,7 +42185,7 @@
       <c r="W174" t="inlineStr"/>
       <c r="X174" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.507131+00:00</t>
+          <t>2026-10-17T11:42:59.724467+00:00</t>
         </is>
       </c>
     </row>
@@ -42281,7 +42281,7 @@
       <c r="W175" t="inlineStr"/>
       <c r="X175" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.507516+00:00</t>
+          <t>2026-10-17T11:42:59.727394+00:00</t>
         </is>
       </c>
     </row>
@@ -42377,7 +42377,7 @@
       <c r="W176" t="inlineStr"/>
       <c r="X176" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.507796+00:00</t>
+          <t>2026-10-17T11:42:59.727742+00:00</t>
         </is>
       </c>
     </row>
@@ -42473,7 +42473,7 @@
       <c r="W177" t="inlineStr"/>
       <c r="X177" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.508135+00:00</t>
+          <t>2026-10-17T11:42:59.728091+00:00</t>
         </is>
       </c>
     </row>
@@ -42569,7 +42569,7 @@
       <c r="W178" t="inlineStr"/>
       <c r="X178" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.508261+00:00</t>
+          <t>2026-10-17T11:42:59.728229+00:00</t>
         </is>
       </c>
     </row>
@@ -42665,7 +42665,7 @@
       <c r="W179" t="inlineStr"/>
       <c r="X179" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.508950+00:00</t>
+          <t>2026-10-17T11:42:59.728970+00:00</t>
         </is>
       </c>
     </row>
@@ -42761,7 +42761,7 @@
       <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.509578+00:00</t>
+          <t>2026-10-17T11:42:59.730102+00:00</t>
         </is>
       </c>
     </row>
@@ -42857,7 +42857,7 @@
       <c r="W181" t="inlineStr"/>
       <c r="X181" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.509677+00:00</t>
+          <t>2026-10-17T11:42:59.730254+00:00</t>
         </is>
       </c>
     </row>
@@ -42953,7 +42953,7 @@
       <c r="W182" t="inlineStr"/>
       <c r="X182" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.510167+00:00</t>
+          <t>2026-10-17T11:42:59.730911+00:00</t>
         </is>
       </c>
     </row>
@@ -43049,7 +43049,7 @@
       <c r="W183" t="inlineStr"/>
       <c r="X183" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.510232+00:00</t>
+          <t>2026-10-17T11:42:59.731127+00:00</t>
         </is>
       </c>
     </row>
@@ -43145,7 +43145,7 @@
       <c r="W184" t="inlineStr"/>
       <c r="X184" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.510285+00:00</t>
+          <t>2026-10-17T11:42:59.731746+00:00</t>
         </is>
       </c>
     </row>
@@ -43241,7 +43241,7 @@
       <c r="W185" t="inlineStr"/>
       <c r="X185" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.510582+00:00</t>
+          <t>2026-10-17T11:42:59.732360+00:00</t>
         </is>
       </c>
     </row>
@@ -43337,7 +43337,7 @@
       <c r="W186" t="inlineStr"/>
       <c r="X186" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.510630+00:00</t>
+          <t>2026-10-17T11:42:59.732424+00:00</t>
         </is>
       </c>
     </row>
@@ -43433,7 +43433,7 @@
       <c r="W187" t="inlineStr"/>
       <c r="X187" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.510784+00:00</t>
+          <t>2026-10-17T11:42:59.732826+00:00</t>
         </is>
       </c>
     </row>
@@ -43529,7 +43529,7 @@
       <c r="W188" t="inlineStr"/>
       <c r="X188" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.510835+00:00</t>
+          <t>2026-10-17T11:42:59.732901+00:00</t>
         </is>
       </c>
     </row>
@@ -43625,7 +43625,7 @@
       <c r="W189" t="inlineStr"/>
       <c r="X189" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.511162+00:00</t>
+          <t>2026-10-17T11:42:59.733232+00:00</t>
         </is>
       </c>
     </row>
@@ -43721,7 +43721,7 @@
       <c r="W190" t="inlineStr"/>
       <c r="X190" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.511226+00:00</t>
+          <t>2026-10-17T11:42:59.733323+00:00</t>
         </is>
       </c>
     </row>
@@ -43817,7 +43817,7 @@
       <c r="W191" t="inlineStr"/>
       <c r="X191" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.511823+00:00</t>
+          <t>2026-10-17T11:42:59.734023+00:00</t>
         </is>
       </c>
     </row>
@@ -43913,7 +43913,7 @@
       <c r="W192" t="inlineStr"/>
       <c r="X192" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.511906+00:00</t>
+          <t>2026-10-17T11:42:59.734127+00:00</t>
         </is>
       </c>
     </row>
@@ -44009,7 +44009,7 @@
       <c r="W193" t="inlineStr"/>
       <c r="X193" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.512244+00:00</t>
+          <t>2026-10-17T11:42:59.734681+00:00</t>
         </is>
       </c>
     </row>
@@ -44105,7 +44105,7 @@
       <c r="W194" t="inlineStr"/>
       <c r="X194" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.512400+00:00</t>
+          <t>2026-10-17T11:42:59.734858+00:00</t>
         </is>
       </c>
     </row>
@@ -44201,7 +44201,7 @@
       <c r="W195" t="inlineStr"/>
       <c r="X195" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.512648+00:00</t>
+          <t>2026-10-17T11:42:59.735106+00:00</t>
         </is>
       </c>
     </row>
@@ -44297,7 +44297,7 @@
       <c r="W196" t="inlineStr"/>
       <c r="X196" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.512703+00:00</t>
+          <t>2026-10-17T11:42:59.735164+00:00</t>
         </is>
       </c>
     </row>
@@ -44393,7 +44393,7 @@
       <c r="W197" t="inlineStr"/>
       <c r="X197" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.512826+00:00</t>
+          <t>2026-10-17T11:42:59.735288+00:00</t>
         </is>
       </c>
     </row>
@@ -44489,7 +44489,7 @@
       <c r="W198" t="inlineStr"/>
       <c r="X198" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.513164+00:00</t>
+          <t>2026-10-17T11:42:59.735672+00:00</t>
         </is>
       </c>
     </row>
@@ -44585,7 +44585,7 @@
       <c r="W199" t="inlineStr"/>
       <c r="X199" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.513539+00:00</t>
+          <t>2026-10-17T11:42:59.736092+00:00</t>
         </is>
       </c>
     </row>
@@ -44681,7 +44681,7 @@
       <c r="W200" t="inlineStr"/>
       <c r="X200" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.513611+00:00</t>
+          <t>2026-10-17T11:42:59.736164+00:00</t>
         </is>
       </c>
     </row>
@@ -44777,7 +44777,7 @@
       <c r="W201" t="inlineStr"/>
       <c r="X201" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.514068+00:00</t>
+          <t>2026-10-17T11:42:59.736665+00:00</t>
         </is>
       </c>
     </row>
@@ -44873,7 +44873,7 @@
       <c r="W202" t="inlineStr"/>
       <c r="X202" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.514383+00:00</t>
+          <t>2026-10-17T11:42:59.737040+00:00</t>
         </is>
       </c>
     </row>
@@ -44969,7 +44969,7 @@
       <c r="W203" t="inlineStr"/>
       <c r="X203" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.514434+00:00</t>
+          <t>2026-10-17T11:42:59.737106+00:00</t>
         </is>
       </c>
     </row>
@@ -45065,7 +45065,7 @@
       <c r="W204" t="inlineStr"/>
       <c r="X204" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.514730+00:00</t>
+          <t>2026-10-17T11:42:59.737426+00:00</t>
         </is>
       </c>
     </row>
@@ -45161,7 +45161,7 @@
       <c r="W205" t="inlineStr"/>
       <c r="X205" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.514792+00:00</t>
+          <t>2026-10-17T11:42:59.737519+00:00</t>
         </is>
       </c>
     </row>
@@ -45257,7 +45257,7 @@
       <c r="W206" t="inlineStr"/>
       <c r="X206" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.514864+00:00</t>
+          <t>2026-10-17T11:42:59.737599+00:00</t>
         </is>
       </c>
     </row>
@@ -45353,7 +45353,7 @@
       <c r="W207" t="inlineStr"/>
       <c r="X207" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.514927+00:00</t>
+          <t>2026-10-17T11:42:59.737663+00:00</t>
         </is>
       </c>
     </row>
@@ -45449,7 +45449,7 @@
       <c r="W208" t="inlineStr"/>
       <c r="X208" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.514979+00:00</t>
+          <t>2026-10-17T11:42:59.737716+00:00</t>
         </is>
       </c>
     </row>
@@ -45545,7 +45545,7 @@
       <c r="W209" t="inlineStr"/>
       <c r="X209" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.515028+00:00</t>
+          <t>2026-10-17T11:42:59.737767+00:00</t>
         </is>
       </c>
     </row>
@@ -45641,7 +45641,7 @@
       <c r="W210" t="inlineStr"/>
       <c r="X210" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.515357+00:00</t>
+          <t>2026-10-17T11:42:59.738200+00:00</t>
         </is>
       </c>
     </row>
@@ -45737,7 +45737,7 @@
       <c r="W211" t="inlineStr"/>
       <c r="X211" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.515487+00:00</t>
+          <t>2026-10-17T11:42:59.738401+00:00</t>
         </is>
       </c>
     </row>
@@ -45833,7 +45833,7 @@
       <c r="W212" t="inlineStr"/>
       <c r="X212" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.515634+00:00</t>
+          <t>2026-10-17T11:42:59.738564+00:00</t>
         </is>
       </c>
     </row>
@@ -45929,7 +45929,7 @@
       <c r="W213" t="inlineStr"/>
       <c r="X213" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.515784+00:00</t>
+          <t>2026-10-17T11:42:59.738753+00:00</t>
         </is>
       </c>
     </row>
@@ -46025,7 +46025,7 @@
       <c r="W214" t="inlineStr"/>
       <c r="X214" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.516527+00:00</t>
+          <t>2026-10-17T11:42:59.739548+00:00</t>
         </is>
       </c>
     </row>
@@ -46121,7 +46121,7 @@
       <c r="W215" t="inlineStr"/>
       <c r="X215" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.517135+00:00</t>
+          <t>2026-10-17T11:42:59.739987+00:00</t>
         </is>
       </c>
     </row>
@@ -46217,7 +46217,7 @@
       <c r="W216" t="inlineStr"/>
       <c r="X216" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.518618+00:00</t>
+          <t>2026-10-17T11:42:59.741909+00:00</t>
         </is>
       </c>
     </row>
@@ -46313,7 +46313,7 @@
       <c r="W217" t="inlineStr"/>
       <c r="X217" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.519422+00:00</t>
+          <t>2026-10-17T11:42:59.742836+00:00</t>
         </is>
       </c>
     </row>
@@ -46409,7 +46409,7 @@
       <c r="W218" t="inlineStr"/>
       <c r="X218" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.520503+00:00</t>
+          <t>2026-10-17T11:42:59.743923+00:00</t>
         </is>
       </c>
     </row>
@@ -46505,7 +46505,7 @@
       <c r="W219" t="inlineStr"/>
       <c r="X219" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.520958+00:00</t>
+          <t>2026-10-17T11:42:59.744421+00:00</t>
         </is>
       </c>
     </row>
@@ -46601,7 +46601,7 @@
       <c r="W220" t="inlineStr"/>
       <c r="X220" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.521930+00:00</t>
+          <t>2026-10-17T11:42:59.745678+00:00</t>
         </is>
       </c>
     </row>
@@ -46697,7 +46697,7 @@
       <c r="W221" t="inlineStr"/>
       <c r="X221" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.522673+00:00</t>
+          <t>2026-10-17T11:42:59.746454+00:00</t>
         </is>
       </c>
     </row>
@@ -46793,7 +46793,7 @@
       <c r="W222" t="inlineStr"/>
       <c r="X222" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.523107+00:00</t>
+          <t>2026-10-17T11:42:59.746940+00:00</t>
         </is>
       </c>
     </row>
@@ -46889,7 +46889,7 @@
       <c r="W223" t="inlineStr"/>
       <c r="X223" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.524168+00:00</t>
+          <t>2026-10-17T11:42:59.748009+00:00</t>
         </is>
       </c>
     </row>
@@ -46985,7 +46985,7 @@
       <c r="W224" t="inlineStr"/>
       <c r="X224" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.524832+00:00</t>
+          <t>2026-10-17T11:42:59.748715+00:00</t>
         </is>
       </c>
     </row>
@@ -47081,7 +47081,7 @@
       <c r="W225" t="inlineStr"/>
       <c r="X225" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.526067+00:00</t>
+          <t>2026-10-17T11:42:59.749965+00:00</t>
         </is>
       </c>
     </row>
@@ -47177,7 +47177,7 @@
       <c r="W226" t="inlineStr"/>
       <c r="X226" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.526515+00:00</t>
+          <t>2026-10-17T11:42:59.750417+00:00</t>
         </is>
       </c>
     </row>
@@ -47273,7 +47273,7 @@
       <c r="W227" t="inlineStr"/>
       <c r="X227" t="inlineStr">
         <is>
-          <t>2026-10-17T11:37:12.527360+00:00</t>
+          <t>2026-10-17T11:42:59.751229+00:00</t>
         </is>
       </c>
     </row>
@@ -47288,7 +47288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47456,35 +47456,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>R07238</t>
+          <t>R10086</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R07238.derived.49b84e369d4bb31b</t>
+          <t>R10086.main.84777bfb7a2cd42f</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>49b84e369d4bb31b4ebdcd25265be3174105c3433e6fbb865f34a445775516a1</t>
+          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>34855493</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
-        </is>
-      </c>
+        <v>984310</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>g a.skp</t>
+          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -47496,35 +47492,35 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>R03161</t>
+          <t>R03155</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R03161.transport_archive.0ef4d4796c84feff</t>
+          <t>R03155.main.2875ce0c137df622</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0ef4d4796c84fefff7b8450bc56400f8c59f4bdcf074fc51404edff5e4e217f6</t>
+          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>726772</v>
+        <v>5745828</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC5627928/supplementaryFiles</t>
+          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>PMC5627928_supplementaryFiles.zip</t>
+          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -47536,35 +47532,35 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>R08877</t>
+          <t>R06036</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>R08877.transport_archive.ed8e864a3225e9c4</t>
+          <t>R06036.main.0bdc7b19fdb70091</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ed8e864a3225e9c4cecf84e5f4670c985de4c6d453d0b7b459ad5870e6627f97</t>
+          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>704921</v>
+        <v>927168</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10714394/supplementaryFiles</t>
+          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>PMC10714394_supplementaryFiles.zip</t>
+          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -47576,35 +47572,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>R09236</t>
+          <t>R13899</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R09236.transport_archive.f3c6856282b7e8d6</t>
+          <t>R13899.main.19143e56fa77ce99</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>f3c6856282b7e8d694d35a87eae016d8e66aa902189c7c3311a1153ea24752e0</t>
+          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>483405</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10535533/supplementaryFiles</t>
-        </is>
-      </c>
+        <v>479092</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PMC10535533_supplementaryFiles.zip</t>
+          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -47616,470 +47608,38 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R10086</t>
+          <t>R13955</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>R10086.transport_archive.4d9eddf454b786ed</t>
+          <t>R13955.main.6714f79deccd703d</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>transport_archive</t>
+          <t>main</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4d9eddf454b786eddece423a320b28d7f96959a935334ddc7c7e2fe32d39bc9b</t>
+          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>641038</v>
+        <v>14662119</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10837232/supplementaryFiles</t>
+          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>PMC10837232_supplementaryFiles.zip</t>
+          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>R12985</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>R12985.transport_archive.418d45f1ca296020</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>transport_archive</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>418d45f1ca2960209df0bfc1c3d44069413edc213239570a3d71d08d01f3e3e0</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>672244</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12937426/supplementaryFiles</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>PMC12937426_supplementaryFiles.zip</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>R06325</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>R06325.transport_archive.6eb4ef126661714a</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>transport_archive</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>6eb4ef126661714ae89bde97acdddac2c2a582864ca26ff9af569cfe609a4226</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>1730580</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8290346/supplementaryFiles</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>PMC8290346_supplementaryFiles.zip</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>R07238</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>R07238.transport_archive.3785c23cb2f4ab50</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>transport_archive</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>3785c23cb2f4ab50f5b2b5cbb581da63ced9f8d1e69a91e6faca839b6b57587d</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>14596266</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC8044681/supplementaryFiles</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>PMC8044681_supplementaryFiles.zip</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>R08646</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>R08646.transport_archive.ecda9ea461a3deb3</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>transport_archive</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ecda9ea461a3deb361931eb51186e88488c4d6ae284899e1feb1d611de42550a</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>1539133</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC10559078/supplementaryFiles</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>PMC10559078_supplementaryFiles.zip</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>R11844</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>R11844.transport_archive.60ef29cf0a557bf4</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>transport_archive</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>60ef29cf0a557bf44838f4a3f45e2dbf1b1a2001547f5c0b976b48cc64c1b6d9</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>521862</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC12125087/supplementaryFiles</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>PMC12125087_supplementaryFiles.zip</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>R05213</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>R05213.transport_archive.c61c88cf9fd489be</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>transport_archive</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>c61c88cf9fd489beab88c1b72bbfe5f13167f32c984b6dba6e48ba97c6136b7b</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>1960371</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>https://www.ebi.ac.uk/europepmc/webservices/rest/PMC6858683/supplementaryFiles</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>PMC6858683_supplementaryFiles.zip</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>R10086</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>R10086.main.84777bfb7a2cd42f</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>84777bfb7a2cd42f9696e060fc79d5de3e72d5ad8fa1e222934a7fcdf97dd365</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>984310</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>R10086_2024_Effect_of_micro-aeration_on_syntrophic_and_methanogenic_activity_in.pdf</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>R03155</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>R03155.main.2875ce0c137df622</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2875ce0c137df622bdafd5e5f4cf9be69518057654dadfcaa55a2b7c46e8625c</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>5745828</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>https://dspace.lib.ntua.gr/xmlui/bitstream/handle/123456789/44237/Msc.%20Thesis_Aristotle_Vasileiou%20THE.pdf?sequence=1&amp;isAllowed=y</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>R03155_2016_Effect_of_bioaugmentation_with_hydrolytic_bacteria_and_micro_aeration.pdf</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>R06036</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>R06036.main.0bdc7b19fdb70091</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>0bdc7b19fdb700910361bf68b9c874d8a5c51772418f9d267f9163e360dc4b27</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>927168</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>https://link.springer.com/content/pdf/10.1007/s42452-020-03247-3.pdf</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>R06036_2020_Rapid_hydrogen_generation_from_cotton_wastes_by_mean_of.pdf</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>R13899</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>R13899.main.19143e56fa77ce99</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>19143e56fa77ce99639f652b53bde1b70f61a67b18f24b9686fc371215092714</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>479092</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>R13899_2013_Effect_of_aerobic_pretreatment_of_waste_on_the_rate.pdf</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>历史已获取，当前原件未恢复</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>R13955</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>R13955.main.6714f79deccd703d</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>6714f79deccd703d9c74784b27ea4770f9095bfad44e0579a4f5de2990ae711f</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>14662119</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://lup.lub.lu.se/search/files/30364253/Thesis_Chao_Li_150_dpi.pdf</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>R13955_2017_Biogas_Production_from_Lignocellulosic_Biomass_Impact_of_pre-treatment_co-digestion.pdf</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
         <is>
           <t>历史已获取，当前原件未恢复</t>
         </is>

</xml_diff>

<commit_message>
Persist exact supplementary links embedded in verified PDFs and source outcomes
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -24118,7 +24118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X227"/>
+  <dimension ref="A1:Y227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24242,6 +24242,11 @@
           <t>recovery_checked_at_utc</t>
         </is>
       </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>extraction_20261017</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="b">
@@ -24347,7 +24352,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.362587+00:00</t>
+          <t>2026-10-17T11:47:11.041328+00:00</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 129, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -24455,7 +24465,12 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.363566+00:00</t>
+          <t>2026-10-17T11:47:11.042565+00:00</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 125, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -24555,9 +24570,10 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.363595+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.042678+00:00</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="b">
@@ -24663,7 +24679,12 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.363833+00:00</t>
+          <t>2026-10-17T11:47:11.042935+00:00</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 171, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -24771,7 +24792,12 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.364965+00:00</t>
+          <t>2026-10-17T11:47:11.044024+00:00</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 203, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -24879,7 +24905,12 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.365568+00:00</t>
+          <t>2026-10-17T11:47:11.044489+00:00</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 91, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -24987,7 +25018,12 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.371124+00:00</t>
+          <t>2026-10-17T11:47:11.050466+00:00</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 130, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25095,7 +25131,12 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.373557+00:00</t>
+          <t>2026-10-17T11:47:11.052891+00:00</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 218, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25244,12 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.374457+00:00</t>
+          <t>2026-10-17T11:47:11.053821+00:00</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 87, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25311,7 +25357,12 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.374852+00:00</t>
+          <t>2026-10-17T11:47:11.054275+00:00</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 93, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25419,7 +25470,12 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.375581+00:00</t>
+          <t>2026-10-17T11:47:11.055006+00:00</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 142, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25527,7 +25583,12 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.376216+00:00</t>
+          <t>2026-10-17T11:47:11.055653+00:00</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 80, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25635,7 +25696,12 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.377100+00:00</t>
+          <t>2026-10-17T11:47:11.056813+00:00</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 128, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25809,12 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.377359+00:00</t>
+          <t>2026-10-17T11:47:11.057158+00:00</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 421, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25851,7 +25922,12 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.378216+00:00</t>
+          <t>2026-10-17T11:47:11.058454+00:00</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 99, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -25959,7 +26035,12 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.386871+00:00</t>
+          <t>2026-10-17T11:47:11.066942+00:00</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 114, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26148,12 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.387809+00:00</t>
+          <t>2026-10-17T11:47:11.067770+00:00</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 127, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26175,7 +26261,12 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.389095+00:00</t>
+          <t>2026-10-17T11:47:11.069168+00:00</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 357, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26283,7 +26374,12 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.391663+00:00</t>
+          <t>2026-10-17T11:47:11.071918+00:00</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 103, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26391,7 +26487,12 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.392860+00:00</t>
+          <t>2026-10-17T11:47:11.072999+00:00</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 117, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26600,12 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.394174+00:00</t>
+          <t>2026-10-17T11:47:11.074354+00:00</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 299, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26713,12 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.398752+00:00</t>
+          <t>2026-10-17T11:47:11.078775+00:00</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 132, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26715,7 +26826,12 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.401000+00:00</t>
+          <t>2026-10-17T11:47:11.081131+00:00</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 152, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26823,7 +26939,12 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.402895+00:00</t>
+          <t>2026-10-17T11:47:11.084591+00:00</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 138, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -26931,7 +27052,12 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.403565+00:00</t>
+          <t>2026-10-17T11:47:11.085306+00:00</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 529, "table_count": 8, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27039,7 +27165,12 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.403947+00:00</t>
+          <t>2026-10-17T11:47:11.085796+00:00</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 188, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27147,7 +27278,12 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.406172+00:00</t>
+          <t>2026-10-17T11:47:11.088664+00:00</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 106, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27255,7 +27391,12 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.407521+00:00</t>
+          <t>2026-10-17T11:47:11.090034+00:00</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 91, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27363,7 +27504,12 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.409662+00:00</t>
+          <t>2026-10-17T11:47:11.092287+00:00</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 317, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27617,12 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.411756+00:00</t>
+          <t>2026-10-17T11:47:11.094562+00:00</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 127, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27579,7 +27730,12 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.412358+00:00</t>
+          <t>2026-10-17T11:47:11.095102+00:00</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 389, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27687,7 +27843,12 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.412911+00:00</t>
+          <t>2026-10-17T11:47:11.095842+00:00</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 150, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27795,7 +27956,12 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.414879+00:00</t>
+          <t>2026-10-17T11:47:11.097593+00:00</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 565, "table_count": 13, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -27903,7 +28069,12 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.417946+00:00</t>
+          <t>2026-10-17T11:47:11.100741+00:00</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 222, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28011,7 +28182,12 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.420136+00:00</t>
+          <t>2026-10-17T11:47:11.102968+00:00</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 57, "table_count": 0, "ocr_pages": 47, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28295,12 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.421413+00:00</t>
+          <t>2026-10-17T11:47:11.104156+00:00</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 207, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28408,12 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.424313+00:00</t>
+          <t>2026-10-17T11:47:11.107071+00:00</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 161, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28335,7 +28521,12 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.424994+00:00</t>
+          <t>2026-10-17T11:47:11.107805+00:00</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 152, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28443,7 +28634,12 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.426709+00:00</t>
+          <t>2026-10-17T11:47:11.109857+00:00</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 274, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28551,7 +28747,12 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.426989+00:00</t>
+          <t>2026-10-17T11:47:11.110161+00:00</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 133, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28659,7 +28860,12 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.428841+00:00</t>
+          <t>2026-10-17T11:47:11.112174+00:00</t>
+        </is>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 290, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28973,12 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.431699+00:00</t>
+          <t>2026-10-17T11:47:11.115103+00:00</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 248, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28875,7 +29086,12 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.433089+00:00</t>
+          <t>2026-10-17T11:47:11.116446+00:00</t>
+        </is>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 481, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -28983,7 +29199,12 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.433648+00:00</t>
+          <t>2026-10-17T11:47:11.116966+00:00</t>
+        </is>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 199, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29091,7 +29312,12 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.436352+00:00</t>
+          <t>2026-10-17T11:47:11.120084+00:00</t>
+        </is>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1180, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29199,7 +29425,12 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.437768+00:00</t>
+          <t>2026-10-17T11:47:11.121467+00:00</t>
+        </is>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 155, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29307,7 +29538,12 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.441198+00:00</t>
+          <t>2026-10-17T11:47:11.125096+00:00</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1126, "table_count": 4, "ocr_pages": 1, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29415,7 +29651,12 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.442875+00:00</t>
+          <t>2026-10-17T11:47:11.126791+00:00</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 92, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29764,12 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.444700+00:00</t>
+          <t>2026-10-17T11:47:11.128686+00:00</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 225, "table_count": 0, "ocr_pages": 4, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29631,7 +29877,12 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.445765+00:00</t>
+          <t>2026-10-17T11:47:11.129869+00:00</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 178, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29739,7 +29990,12 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.446209+00:00</t>
+          <t>2026-10-17T11:47:11.130344+00:00</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 80, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29847,7 +30103,12 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.446633+00:00</t>
+          <t>2026-10-17T11:47:11.130706+00:00</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 71, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -29955,7 +30216,12 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.448235+00:00</t>
+          <t>2026-10-17T11:47:11.132150+00:00</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 215, "table_count": 4, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30329,12 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.449734+00:00</t>
+          <t>2026-10-17T11:47:11.133591+00:00</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 214, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30171,7 +30442,12 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.451341+00:00</t>
+          <t>2026-10-17T11:47:11.135193+00:00</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 206, "table_count": 4, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30279,7 +30555,12 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.451692+00:00</t>
+          <t>2026-10-17T11:47:11.135596+00:00</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 67, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30387,7 +30668,12 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.452849+00:00</t>
+          <t>2026-10-17T11:47:11.136947+00:00</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 300, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30495,7 +30781,12 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.454360+00:00</t>
+          <t>2026-10-17T11:47:11.138455+00:00</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 700, "table_count": 7, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30894,12 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.454934+00:00</t>
+          <t>2026-10-17T11:47:11.139224+00:00</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 132, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30711,7 +31007,12 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.455862+00:00</t>
+          <t>2026-10-17T11:47:11.140494+00:00</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 73, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30819,7 +31120,12 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.456176+00:00</t>
+          <t>2026-10-17T11:47:11.140931+00:00</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 482, "table_count": 12, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -30927,7 +31233,12 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.461923+00:00</t>
+          <t>2026-10-17T11:47:11.146674+00:00</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 7267, "table_count": 8, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31035,7 +31346,12 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.462418+00:00</t>
+          <t>2026-10-17T11:47:11.147101+00:00</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 265, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31143,7 +31459,12 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.462977+00:00</t>
+          <t>2026-10-17T11:47:11.147704+00:00</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 93, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31251,7 +31572,12 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.463416+00:00</t>
+          <t>2026-10-17T11:47:11.148139+00:00</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 131, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31359,7 +31685,12 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.464466+00:00</t>
+          <t>2026-10-17T11:47:11.149188+00:00</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 321, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31467,7 +31798,12 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.467638+00:00</t>
+          <t>2026-10-17T11:47:11.152143+00:00</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 452, "table_count": 1, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31575,7 +31911,12 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.467917+00:00</t>
+          <t>2026-10-17T11:47:11.152511+00:00</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 124, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31683,7 +32024,12 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.472358+00:00</t>
+          <t>2026-10-17T11:47:11.157098+00:00</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 171, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31791,7 +32137,12 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.473135+00:00</t>
+          <t>2026-10-17T11:47:11.157942+00:00</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 367, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -31899,7 +32250,12 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.475382+00:00</t>
+          <t>2026-10-17T11:47:11.160089+00:00</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 117, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32007,7 +32363,12 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.477168+00:00</t>
+          <t>2026-10-17T11:47:11.162131+00:00</t>
+        </is>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 106, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32115,7 +32476,12 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.478100+00:00</t>
+          <t>2026-10-17T11:47:11.163009+00:00</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 121, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32223,7 +32589,12 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.479514+00:00</t>
+          <t>2026-10-17T11:47:11.164805+00:00</t>
+        </is>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1469, "table_count": 29, "ocr_pages": 1, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32702,12 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.481729+00:00</t>
+          <t>2026-10-17T11:47:11.167414+00:00</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1794, "table_count": 6, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32439,7 +32815,12 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.491521+00:00</t>
+          <t>2026-10-17T11:47:11.176350+00:00</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 3333, "table_count": 6, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32547,7 +32928,12 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.492995+00:00</t>
+          <t>2026-10-17T11:47:11.177741+00:00</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 204, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32655,7 +33041,12 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.493241+00:00</t>
+          <t>2026-10-17T11:47:11.177995+00:00</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 111, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32755,9 +33146,10 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.493263+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.178017+00:00</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="b">
@@ -32863,7 +33255,12 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.498723+00:00</t>
+          <t>2026-10-17T11:47:11.183578+00:00</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 3225, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -32967,7 +33364,12 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.499148+00:00</t>
+          <t>2026-10-17T11:47:11.184053+00:00</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 708, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -33071,7 +33473,12 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.499525+00:00</t>
+          <t>2026-10-17T11:47:11.184530+00:00</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 778, "table_count": 6, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -33175,7 +33582,12 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.499919+00:00</t>
+          <t>2026-10-17T11:47:11.185059+00:00</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 824, "table_count": 4, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -33279,7 +33691,12 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.500631+00:00</t>
+          <t>2026-10-17T11:47:11.185895+00:00</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1861, "table_count": 6, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -33383,7 +33800,12 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.502000+00:00</t>
+          <t>2026-10-17T11:47:11.187458+00:00</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 574, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -33487,7 +33909,12 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.502806+00:00</t>
+          <t>2026-10-17T11:47:11.188921+00:00</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1033, "table_count": 16, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -33591,7 +34018,12 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.503108+00:00</t>
+          <t>2026-10-17T11:47:11.189365+00:00</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 97, "table_count": 1, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -33699,7 +34131,12 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.503743+00:00</t>
+          <t>2026-10-17T11:47:11.190190+00:00</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 99, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -33799,9 +34236,10 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.503757+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.190214+00:00</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="b">
@@ -33907,7 +34345,12 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.503811+00:00</t>
+          <t>2026-10-17T11:47:11.190279+00:00</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 124, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Formulas are preserved, never executed/recalculated; unavailable cached values are explicit. Charts and embedded images are not content-indexed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34458,12 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.504036+00:00</t>
+          <t>2026-10-17T11:47:11.190538+00:00</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 187, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34123,7 +34571,12 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.504169+00:00</t>
+          <t>2026-10-17T11:47:11.190662+00:00</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>{"status": "archive_catalogued", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["ZIP member names/checksums indexed; member content indexed through separately SHA-bound derived assets. No executable/code is run."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34235,7 +34688,12 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.504283+00:00</t>
+          <t>2026-10-17T11:47:11.190782+00:00</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 843, "table_count": 5, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Formulas are preserved, never executed/recalculated; unavailable cached values are explicit. Charts and embedded images are not content-indexed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34343,7 +34801,12 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.504743+00:00</t>
+          <t>2026-10-17T11:47:11.191257+00:00</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 301, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34451,7 +34914,12 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.504962+00:00</t>
+          <t>2026-10-17T11:47:11.191492+00:00</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>{"status": "archive_catalogued", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["ZIP member names/checksums indexed; member content indexed through separately SHA-bound derived assets. No executable/code is run."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34563,7 +35031,12 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.505020+00:00</t>
+          <t>2026-10-17T11:47:11.191553+00:00</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 443, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Formulas are preserved, never executed/recalculated; unavailable cached values are explicit. Charts and embedded images are not content-indexed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34675,7 +35148,12 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.505104+00:00</t>
+          <t>2026-10-17T11:47:11.191613+00:00</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 422, "table_count": 13, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Formulas are preserved, never executed/recalculated; unavailable cached values are explicit. Charts and embedded images are not content-indexed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34787,7 +35265,12 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.505257+00:00</t>
+          <t>2026-10-17T11:47:11.191752+00:00</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 3191, "table_count": 1, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Formulas are preserved, never executed/recalculated; unavailable cached values are explicit. Charts and embedded images are not content-indexed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -34899,7 +35382,12 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.505330+00:00</t>
+          <t>2026-10-17T11:47:11.192027+00:00</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 302, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Formulas are preserved, never executed/recalculated; unavailable cached values are explicit. Charts and embedded images are not content-indexed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35007,7 +35495,12 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.506011+00:00</t>
+          <t>2026-10-17T11:47:11.192524+00:00</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 485, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Word OOXML body paragraphs/tables and section headers/footers; page numbers depend on renderer; nested tables, text boxes, footnotes and embedded objects are not guaranteed parsed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35115,7 +35608,12 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.506091+00:00</t>
+          <t>2026-10-17T11:47:11.192580+00:00</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 54, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Formulas are preserved, never executed/recalculated; unavailable cached values are explicit. Charts and embedded images are not content-indexed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35223,7 +35721,12 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.506166+00:00</t>
+          <t>2026-10-17T11:47:11.192649+00:00</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Word OOXML body paragraphs/tables and section headers/footers; page numbers depend on renderer; nested tables, text boxes, footnotes and embedded objects are not guaranteed parsed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35331,7 +35834,12 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.516379+00:00</t>
+          <t>2026-10-17T11:47:11.203833+00:00</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>{"status": "archive_catalogued", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["ZIP member names/checksums indexed; member content indexed through separately SHA-bound derived assets. No executable/code is run."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35435,9 +35943,10 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.516457+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.203924+00:00</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="b">
@@ -35543,7 +36052,12 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.664314+00:00</t>
+          <t>2026-10-17T11:47:11.364771+00:00</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 24, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Word OOXML body paragraphs/tables and section headers/footers; page numbers depend on renderer; nested tables, text boxes, footnotes and embedded objects are not guaranteed parsed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35651,7 +36165,12 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.664603+00:00</t>
+          <t>2026-10-17T11:47:11.365050+00:00</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 534, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35759,7 +36278,12 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.665853+00:00</t>
+          <t>2026-10-17T11:47:11.366447+00:00</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 12, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Word OOXML body paragraphs/tables and section headers/footers; page numbers depend on renderer; nested tables, text boxes, footnotes and embedded objects are not guaranteed parsed."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35861,7 +36385,12 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.665972+00:00</t>
+          <t>2026-10-17T11:47:11.366570+00:00</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 135, "table_count": 1, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -35955,9 +36484,10 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.665988+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.366585+00:00</t>
+        </is>
+      </c>
+      <c r="Y110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr"/>
@@ -36057,7 +36587,12 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.666219+00:00</t>
+          <t>2026-10-17T11:47:11.366839+00:00</t>
+        </is>
+      </c>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 51, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -36159,7 +36694,12 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.666329+00:00</t>
+          <t>2026-10-17T11:47:11.366940+00:00</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 112, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -36261,7 +36801,12 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.666449+00:00</t>
+          <t>2026-10-17T11:47:11.367239+00:00</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 231, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -36355,9 +36900,10 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.666461+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.367267+00:00</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr"/>
@@ -36457,7 +37003,12 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.666932+00:00</t>
+          <t>2026-10-17T11:47:11.367697+00:00</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 437, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -36551,9 +37102,10 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.666949+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.367711+00:00</t>
+        </is>
+      </c>
+      <c r="Y116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr"/>
@@ -36653,7 +37205,12 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.667173+00:00</t>
+          <t>2026-10-17T11:47:11.367929+00:00</t>
+        </is>
+      </c>
+      <c r="Y117" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 89, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -36747,9 +37304,10 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.667184+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.367939+00:00</t>
+        </is>
+      </c>
+      <c r="Y118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr"/>
@@ -36849,7 +37407,12 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.667733+00:00</t>
+          <t>2026-10-17T11:47:11.368461+00:00</t>
+        </is>
+      </c>
+      <c r="Y119" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 813, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -36943,9 +37506,10 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.667747+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.368473+00:00</t>
+        </is>
+      </c>
+      <c r="Y120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr"/>
@@ -37045,7 +37609,12 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.668023+00:00</t>
+          <t>2026-10-17T11:47:11.368815+00:00</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 164, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -37147,7 +37716,12 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.668155+00:00</t>
+          <t>2026-10-17T11:47:11.368970+00:00</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 675, "table_count": 5, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -37241,9 +37815,10 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.668166+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.368983+00:00</t>
+        </is>
+      </c>
+      <c r="Y123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr"/>
@@ -37343,7 +37918,12 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.668786+00:00</t>
+          <t>2026-10-17T11:47:11.369656+00:00</t>
+        </is>
+      </c>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 258, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -37437,9 +38017,10 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.668798+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.369670+00:00</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr"/>
@@ -37539,7 +38120,12 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.679117+00:00</t>
+          <t>2026-10-17T11:47:11.380641+00:00</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 331, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -37641,7 +38227,12 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.679386+00:00</t>
+          <t>2026-10-17T11:47:11.380884+00:00</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 455, "table_count": 4, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -37735,9 +38326,10 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.679403+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.380898+00:00</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr"/>
@@ -37837,7 +38429,12 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.679720+00:00</t>
+          <t>2026-10-17T11:47:11.381224+00:00</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 352, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -37939,7 +38536,12 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.679923+00:00</t>
+          <t>2026-10-17T11:47:11.381542+00:00</t>
+        </is>
+      </c>
+      <c r="Y130" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 592, "table_count": 4, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -38041,7 +38643,12 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.680120+00:00</t>
+          <t>2026-10-17T11:47:11.381946+00:00</t>
+        </is>
+      </c>
+      <c r="Y131" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 173, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -38135,9 +38742,10 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.680138+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.381972+00:00</t>
+        </is>
+      </c>
+      <c r="Y132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr"/>
@@ -38237,7 +38845,12 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.680497+00:00</t>
+          <t>2026-10-17T11:47:11.382366+00:00</t>
+        </is>
+      </c>
+      <c r="Y133" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 361, "table_count": 3, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -38331,9 +38944,10 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.680510+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.382419+00:00</t>
+        </is>
+      </c>
+      <c r="Y134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr"/>
@@ -38433,7 +39047,12 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.681648+00:00</t>
+          <t>2026-10-17T11:47:11.383693+00:00</t>
+        </is>
+      </c>
+      <c r="Y135" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 140, "table_count": 1, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Repository JATS XML text/structured tables; linked figures/media not all fetched. It is not a recovered historical PDF. Table rowspan/colspan retained as locators, not expanded into a rectangular semantic grid."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -38541,7 +39160,12 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.682701+00:00</t>
+          <t>2026-10-17T11:47:11.384880+00:00</t>
+        </is>
+      </c>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 117, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -38627,13 +39251,18 @@
       <c r="U137" t="inlineStr"/>
       <c r="V137" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.693667+00:00</t>
+          <t>2026-10-17T11:47:11.397066+00:00</t>
+        </is>
+      </c>
+      <c r="Y137" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1555, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -38727,13 +39356,18 @@
       <c r="U138" t="inlineStr"/>
       <c r="V138" t="inlineStr">
         <is>
-          <t>historical_only_current_original_missing</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.694193+00:00</t>
+          <t>2026-10-17T11:47:11.397878+00:00</t>
+        </is>
+      </c>
+      <c r="Y138" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 317, "table_count": 11, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -38821,9 +39455,10 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.694217+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.397956+00:00</t>
+        </is>
+      </c>
+      <c r="Y139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="b">
@@ -38915,13 +39550,18 @@
       <c r="U140" t="inlineStr"/>
       <c r="V140" t="inlineStr">
         <is>
-          <t>historical_only_current_original_missing</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.695527+00:00</t>
+          <t>2026-10-17T11:47:11.399139+00:00</t>
+        </is>
+      </c>
+      <c r="Y140" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 105, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -39015,13 +39655,18 @@
       <c r="U141" t="inlineStr"/>
       <c r="V141" t="inlineStr">
         <is>
-          <t>historical_only_current_original_missing</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.699793+00:00</t>
+          <t>2026-10-17T11:47:11.402653+00:00</t>
+        </is>
+      </c>
+      <c r="Y141" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 246, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -39115,13 +39760,18 @@
       <c r="U142" t="inlineStr"/>
       <c r="V142" t="inlineStr">
         <is>
-          <t>historical_only_current_original_missing</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.700865+00:00</t>
+          <t>2026-10-17T11:47:11.403549+00:00</t>
+        </is>
+      </c>
+      <c r="Y142" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 134, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -39213,9 +39863,10 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.700896+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.403568+00:00</t>
+        </is>
+      </c>
+      <c r="Y143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="b">
@@ -39307,13 +39958,18 @@
       <c r="U144" t="inlineStr"/>
       <c r="V144" t="inlineStr">
         <is>
-          <t>historical_only_current_original_missing</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.701616+00:00</t>
+          <t>2026-10-17T11:47:11.404216+00:00</t>
+        </is>
+      </c>
+      <c r="Y144" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 338, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -39405,9 +40061,10 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.701637+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.404231+00:00</t>
+        </is>
+      </c>
+      <c r="Y145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="b">
@@ -39503,13 +40160,18 @@
       <c r="U146" t="inlineStr"/>
       <c r="V146" t="inlineStr">
         <is>
-          <t>historical_only_current_original_missing</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.702476+00:00</t>
+          <t>2026-10-17T11:47:11.405058+00:00</t>
+        </is>
+      </c>
+      <c r="Y146" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 770, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -39597,9 +40259,10 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.702493+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.405074+00:00</t>
+        </is>
+      </c>
+      <c r="Y147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="b">
@@ -39689,9 +40352,10 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.702497+00:00</t>
-        </is>
-      </c>
+          <t>2026-10-17T11:47:11.405078+00:00</t>
+        </is>
+      </c>
+      <c r="Y148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="b">
@@ -39779,13 +40443,18 @@
       <c r="U149" t="inlineStr"/>
       <c r="V149" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W149" t="inlineStr"/>
       <c r="X149" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.703262+00:00</t>
+          <t>2026-10-17T11:47:11.406035+00:00</t>
+        </is>
+      </c>
+      <c r="Y149" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 310, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -39875,13 +40544,18 @@
       <c r="U150" t="inlineStr"/>
       <c r="V150" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W150" t="inlineStr"/>
       <c r="X150" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.704338+00:00</t>
+          <t>2026-10-17T11:47:11.407171+00:00</t>
+        </is>
+      </c>
+      <c r="Y150" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 109, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -39971,13 +40645,18 @@
       <c r="U151" t="inlineStr"/>
       <c r="V151" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W151" t="inlineStr"/>
       <c r="X151" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.704752+00:00</t>
+          <t>2026-10-17T11:47:11.407628+00:00</t>
+        </is>
+      </c>
+      <c r="Y151" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 159, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40067,13 +40746,18 @@
       <c r="U152" t="inlineStr"/>
       <c r="V152" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W152" t="inlineStr"/>
       <c r="X152" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.715101+00:00</t>
+          <t>2026-10-17T11:47:11.419092+00:00</t>
+        </is>
+      </c>
+      <c r="Y152" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 1555, "table_count": 2, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40163,13 +40847,18 @@
       <c r="U153" t="inlineStr"/>
       <c r="V153" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W153" t="inlineStr"/>
       <c r="X153" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.715277+00:00</t>
+          <t>2026-10-17T11:47:11.419269+00:00</t>
+        </is>
+      </c>
+      <c r="Y153" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40259,13 +40948,18 @@
       <c r="U154" t="inlineStr"/>
       <c r="V154" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.715597+00:00</t>
+          <t>2026-10-17T11:47:11.419471+00:00</t>
+        </is>
+      </c>
+      <c r="Y154" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40355,13 +41049,18 @@
       <c r="U155" t="inlineStr"/>
       <c r="V155" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W155" t="inlineStr"/>
       <c r="X155" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.716108+00:00</t>
+          <t>2026-10-17T11:47:11.419911+00:00</t>
+        </is>
+      </c>
+      <c r="Y155" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40451,13 +41150,18 @@
       <c r="U156" t="inlineStr"/>
       <c r="V156" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.716418+00:00</t>
+          <t>2026-10-17T11:47:11.420171+00:00</t>
+        </is>
+      </c>
+      <c r="Y156" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40547,13 +41251,18 @@
       <c r="U157" t="inlineStr"/>
       <c r="V157" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W157" t="inlineStr"/>
       <c r="X157" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.716761+00:00</t>
+          <t>2026-10-17T11:47:11.420558+00:00</t>
+        </is>
+      </c>
+      <c r="Y157" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40643,13 +41352,18 @@
       <c r="U158" t="inlineStr"/>
       <c r="V158" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W158" t="inlineStr"/>
       <c r="X158" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.717914+00:00</t>
+          <t>2026-10-17T11:47:11.421821+00:00</t>
+        </is>
+      </c>
+      <c r="Y158" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 130, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40739,13 +41453,18 @@
       <c r="U159" t="inlineStr"/>
       <c r="V159" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W159" t="inlineStr"/>
       <c r="X159" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.719750+00:00</t>
+          <t>2026-10-17T11:47:11.423593+00:00</t>
+        </is>
+      </c>
+      <c r="Y159" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 464, "table_count": 1, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40835,13 +41554,18 @@
       <c r="U160" t="inlineStr"/>
       <c r="V160" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W160" t="inlineStr"/>
       <c r="X160" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.720424+00:00</t>
+          <t>2026-10-17T11:47:11.424240+00:00</t>
+        </is>
+      </c>
+      <c r="Y160" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 316, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -40931,13 +41655,18 @@
       <c r="U161" t="inlineStr"/>
       <c r="V161" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W161" t="inlineStr"/>
       <c r="X161" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.720758+00:00</t>
+          <t>2026-10-17T11:47:11.424622+00:00</t>
+        </is>
+      </c>
+      <c r="Y161" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41027,13 +41756,18 @@
       <c r="U162" t="inlineStr"/>
       <c r="V162" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W162" t="inlineStr"/>
       <c r="X162" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.720827+00:00</t>
+          <t>2026-10-17T11:47:11.424719+00:00</t>
+        </is>
+      </c>
+      <c r="Y162" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41123,13 +41857,18 @@
       <c r="U163" t="inlineStr"/>
       <c r="V163" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W163" t="inlineStr"/>
       <c r="X163" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.720897+00:00</t>
+          <t>2026-10-17T11:47:11.424808+00:00</t>
+        </is>
+      </c>
+      <c r="Y163" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41219,13 +41958,18 @@
       <c r="U164" t="inlineStr"/>
       <c r="V164" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W164" t="inlineStr"/>
       <c r="X164" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.721180+00:00</t>
+          <t>2026-10-17T11:47:11.425771+00:00</t>
+        </is>
+      </c>
+      <c r="Y164" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41315,13 +42059,18 @@
       <c r="U165" t="inlineStr"/>
       <c r="V165" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W165" t="inlineStr"/>
       <c r="X165" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.721711+00:00</t>
+          <t>2026-10-17T11:47:11.426245+00:00</t>
+        </is>
+      </c>
+      <c r="Y165" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41411,13 +42160,18 @@
       <c r="U166" t="inlineStr"/>
       <c r="V166" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W166" t="inlineStr"/>
       <c r="X166" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.722069+00:00</t>
+          <t>2026-10-17T11:47:11.426624+00:00</t>
+        </is>
+      </c>
+      <c r="Y166" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41507,13 +42261,18 @@
       <c r="U167" t="inlineStr"/>
       <c r="V167" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W167" t="inlineStr"/>
       <c r="X167" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.722763+00:00</t>
+          <t>2026-10-17T11:47:11.427315+00:00</t>
+        </is>
+      </c>
+      <c r="Y167" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41603,13 +42362,18 @@
       <c r="U168" t="inlineStr"/>
       <c r="V168" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W168" t="inlineStr"/>
       <c r="X168" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.723366+00:00</t>
+          <t>2026-10-17T11:47:11.427688+00:00</t>
+        </is>
+      </c>
+      <c r="Y168" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41699,13 +42463,18 @@
       <c r="U169" t="inlineStr"/>
       <c r="V169" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W169" t="inlineStr"/>
       <c r="X169" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.723649+00:00</t>
+          <t>2026-10-17T11:47:11.427838+00:00</t>
+        </is>
+      </c>
+      <c r="Y169" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41795,13 +42564,18 @@
       <c r="U170" t="inlineStr"/>
       <c r="V170" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W170" t="inlineStr"/>
       <c r="X170" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.723808+00:00</t>
+          <t>2026-10-17T11:47:11.427984+00:00</t>
+        </is>
+      </c>
+      <c r="Y170" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41891,13 +42665,18 @@
       <c r="U171" t="inlineStr"/>
       <c r="V171" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W171" t="inlineStr"/>
       <c r="X171" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.723941+00:00</t>
+          <t>2026-10-17T11:47:11.428334+00:00</t>
+        </is>
+      </c>
+      <c r="Y171" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -41987,13 +42766,18 @@
       <c r="U172" t="inlineStr"/>
       <c r="V172" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W172" t="inlineStr"/>
       <c r="X172" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.724000+00:00</t>
+          <t>2026-10-17T11:47:11.428478+00:00</t>
+        </is>
+      </c>
+      <c r="Y172" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42083,13 +42867,18 @@
       <c r="U173" t="inlineStr"/>
       <c r="V173" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W173" t="inlineStr"/>
       <c r="X173" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.724069+00:00</t>
+          <t>2026-10-17T11:47:11.428560+00:00</t>
+        </is>
+      </c>
+      <c r="Y173" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42179,13 +42968,18 @@
       <c r="U174" t="inlineStr"/>
       <c r="V174" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W174" t="inlineStr"/>
       <c r="X174" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.724467+00:00</t>
+          <t>2026-10-17T11:47:11.428992+00:00</t>
+        </is>
+      </c>
+      <c r="Y174" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42275,13 +43069,18 @@
       <c r="U175" t="inlineStr"/>
       <c r="V175" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W175" t="inlineStr"/>
       <c r="X175" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.727394+00:00</t>
+          <t>2026-10-17T11:47:11.429418+00:00</t>
+        </is>
+      </c>
+      <c r="Y175" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42371,13 +43170,18 @@
       <c r="U176" t="inlineStr"/>
       <c r="V176" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W176" t="inlineStr"/>
       <c r="X176" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.727742+00:00</t>
+          <t>2026-10-17T11:47:11.429727+00:00</t>
+        </is>
+      </c>
+      <c r="Y176" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42467,13 +43271,18 @@
       <c r="U177" t="inlineStr"/>
       <c r="V177" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W177" t="inlineStr"/>
       <c r="X177" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.728091+00:00</t>
+          <t>2026-10-17T11:47:11.430240+00:00</t>
+        </is>
+      </c>
+      <c r="Y177" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42563,13 +43372,18 @@
       <c r="U178" t="inlineStr"/>
       <c r="V178" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W178" t="inlineStr"/>
       <c r="X178" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.728229+00:00</t>
+          <t>2026-10-17T11:47:11.430416+00:00</t>
+        </is>
+      </c>
+      <c r="Y178" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42659,13 +43473,18 @@
       <c r="U179" t="inlineStr"/>
       <c r="V179" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W179" t="inlineStr"/>
       <c r="X179" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.728970+00:00</t>
+          <t>2026-10-17T11:47:11.431090+00:00</t>
+        </is>
+      </c>
+      <c r="Y179" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42755,13 +43574,18 @@
       <c r="U180" t="inlineStr"/>
       <c r="V180" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.730102+00:00</t>
+          <t>2026-10-17T11:47:11.431758+00:00</t>
+        </is>
+      </c>
+      <c r="Y180" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42851,13 +43675,18 @@
       <c r="U181" t="inlineStr"/>
       <c r="V181" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W181" t="inlineStr"/>
       <c r="X181" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.730254+00:00</t>
+          <t>2026-10-17T11:47:11.431876+00:00</t>
+        </is>
+      </c>
+      <c r="Y181" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -42947,13 +43776,18 @@
       <c r="U182" t="inlineStr"/>
       <c r="V182" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W182" t="inlineStr"/>
       <c r="X182" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.730911+00:00</t>
+          <t>2026-10-17T11:47:11.432404+00:00</t>
+        </is>
+      </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43043,13 +43877,18 @@
       <c r="U183" t="inlineStr"/>
       <c r="V183" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W183" t="inlineStr"/>
       <c r="X183" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.731127+00:00</t>
+          <t>2026-10-17T11:47:11.432543+00:00</t>
+        </is>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43139,13 +43978,18 @@
       <c r="U184" t="inlineStr"/>
       <c r="V184" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W184" t="inlineStr"/>
       <c r="X184" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.731746+00:00</t>
+          <t>2026-10-17T11:47:11.432614+00:00</t>
+        </is>
+      </c>
+      <c r="Y184" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43235,13 +44079,18 @@
       <c r="U185" t="inlineStr"/>
       <c r="V185" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W185" t="inlineStr"/>
       <c r="X185" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.732360+00:00</t>
+          <t>2026-10-17T11:47:11.432890+00:00</t>
+        </is>
+      </c>
+      <c r="Y185" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43331,13 +44180,18 @@
       <c r="U186" t="inlineStr"/>
       <c r="V186" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W186" t="inlineStr"/>
       <c r="X186" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.732424+00:00</t>
+          <t>2026-10-17T11:47:11.432938+00:00</t>
+        </is>
+      </c>
+      <c r="Y186" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43427,13 +44281,18 @@
       <c r="U187" t="inlineStr"/>
       <c r="V187" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W187" t="inlineStr"/>
       <c r="X187" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.732826+00:00</t>
+          <t>2026-10-17T11:47:11.433091+00:00</t>
+        </is>
+      </c>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43523,13 +44382,18 @@
       <c r="U188" t="inlineStr"/>
       <c r="V188" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W188" t="inlineStr"/>
       <c r="X188" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.732901+00:00</t>
+          <t>2026-10-17T11:47:11.433146+00:00</t>
+        </is>
+      </c>
+      <c r="Y188" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43619,13 +44483,18 @@
       <c r="U189" t="inlineStr"/>
       <c r="V189" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W189" t="inlineStr"/>
       <c r="X189" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.733232+00:00</t>
+          <t>2026-10-17T11:47:11.433514+00:00</t>
+        </is>
+      </c>
+      <c r="Y189" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43715,13 +44584,18 @@
       <c r="U190" t="inlineStr"/>
       <c r="V190" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W190" t="inlineStr"/>
       <c r="X190" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.733323+00:00</t>
+          <t>2026-10-17T11:47:11.433584+00:00</t>
+        </is>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43811,13 +44685,18 @@
       <c r="U191" t="inlineStr"/>
       <c r="V191" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W191" t="inlineStr"/>
       <c r="X191" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.734023+00:00</t>
+          <t>2026-10-17T11:47:11.434163+00:00</t>
+        </is>
+      </c>
+      <c r="Y191" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -43907,13 +44786,18 @@
       <c r="U192" t="inlineStr"/>
       <c r="V192" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W192" t="inlineStr"/>
       <c r="X192" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.734127+00:00</t>
+          <t>2026-10-17T11:47:11.434247+00:00</t>
+        </is>
+      </c>
+      <c r="Y192" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44003,13 +44887,18 @@
       <c r="U193" t="inlineStr"/>
       <c r="V193" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W193" t="inlineStr"/>
       <c r="X193" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.734681+00:00</t>
+          <t>2026-10-17T11:47:11.434600+00:00</t>
+        </is>
+      </c>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44099,13 +44988,18 @@
       <c r="U194" t="inlineStr"/>
       <c r="V194" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W194" t="inlineStr"/>
       <c r="X194" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.734858+00:00</t>
+          <t>2026-10-17T11:47:11.434739+00:00</t>
+        </is>
+      </c>
+      <c r="Y194" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44195,13 +45089,18 @@
       <c r="U195" t="inlineStr"/>
       <c r="V195" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W195" t="inlineStr"/>
       <c r="X195" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.735106+00:00</t>
+          <t>2026-10-17T11:47:11.434992+00:00</t>
+        </is>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44291,13 +45190,18 @@
       <c r="U196" t="inlineStr"/>
       <c r="V196" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W196" t="inlineStr"/>
       <c r="X196" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.735164+00:00</t>
+          <t>2026-10-17T11:47:11.435107+00:00</t>
+        </is>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44387,13 +45291,18 @@
       <c r="U197" t="inlineStr"/>
       <c r="V197" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W197" t="inlineStr"/>
       <c r="X197" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.735288+00:00</t>
+          <t>2026-10-17T11:47:11.435251+00:00</t>
+        </is>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44483,13 +45392,18 @@
       <c r="U198" t="inlineStr"/>
       <c r="V198" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W198" t="inlineStr"/>
       <c r="X198" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.735672+00:00</t>
+          <t>2026-10-17T11:47:11.435629+00:00</t>
+        </is>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44579,13 +45493,18 @@
       <c r="U199" t="inlineStr"/>
       <c r="V199" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W199" t="inlineStr"/>
       <c r="X199" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.736092+00:00</t>
+          <t>2026-10-17T11:47:11.435974+00:00</t>
+        </is>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44675,13 +45594,18 @@
       <c r="U200" t="inlineStr"/>
       <c r="V200" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W200" t="inlineStr"/>
       <c r="X200" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.736164+00:00</t>
+          <t>2026-10-17T11:47:11.436056+00:00</t>
+        </is>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44771,13 +45695,18 @@
       <c r="U201" t="inlineStr"/>
       <c r="V201" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W201" t="inlineStr"/>
       <c r="X201" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.736665+00:00</t>
+          <t>2026-10-17T11:47:11.436532+00:00</t>
+        </is>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44867,13 +45796,18 @@
       <c r="U202" t="inlineStr"/>
       <c r="V202" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W202" t="inlineStr"/>
       <c r="X202" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.737040+00:00</t>
+          <t>2026-10-17T11:47:11.436836+00:00</t>
+        </is>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -44963,13 +45897,18 @@
       <c r="U203" t="inlineStr"/>
       <c r="V203" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W203" t="inlineStr"/>
       <c r="X203" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.737106+00:00</t>
+          <t>2026-10-17T11:47:11.436885+00:00</t>
+        </is>
+      </c>
+      <c r="Y203" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45059,13 +45998,18 @@
       <c r="U204" t="inlineStr"/>
       <c r="V204" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W204" t="inlineStr"/>
       <c r="X204" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.737426+00:00</t>
+          <t>2026-10-17T11:47:11.437181+00:00</t>
+        </is>
+      </c>
+      <c r="Y204" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45155,13 +46099,18 @@
       <c r="U205" t="inlineStr"/>
       <c r="V205" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W205" t="inlineStr"/>
       <c r="X205" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.737519+00:00</t>
+          <t>2026-10-17T11:47:11.437246+00:00</t>
+        </is>
+      </c>
+      <c r="Y205" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45251,13 +46200,18 @@
       <c r="U206" t="inlineStr"/>
       <c r="V206" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W206" t="inlineStr"/>
       <c r="X206" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.737599+00:00</t>
+          <t>2026-10-17T11:47:11.437445+00:00</t>
+        </is>
+      </c>
+      <c r="Y206" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45347,13 +46301,18 @@
       <c r="U207" t="inlineStr"/>
       <c r="V207" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W207" t="inlineStr"/>
       <c r="X207" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.737663+00:00</t>
+          <t>2026-10-17T11:47:11.437572+00:00</t>
+        </is>
+      </c>
+      <c r="Y207" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45443,13 +46402,18 @@
       <c r="U208" t="inlineStr"/>
       <c r="V208" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W208" t="inlineStr"/>
       <c r="X208" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.737716+00:00</t>
+          <t>2026-10-17T11:47:11.437631+00:00</t>
+        </is>
+      </c>
+      <c r="Y208" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45539,13 +46503,18 @@
       <c r="U209" t="inlineStr"/>
       <c r="V209" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W209" t="inlineStr"/>
       <c r="X209" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.737767+00:00</t>
+          <t>2026-10-17T11:47:11.437685+00:00</t>
+        </is>
+      </c>
+      <c r="Y209" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45635,13 +46604,18 @@
       <c r="U210" t="inlineStr"/>
       <c r="V210" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W210" t="inlineStr"/>
       <c r="X210" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.738200+00:00</t>
+          <t>2026-10-17T11:47:11.438319+00:00</t>
+        </is>
+      </c>
+      <c r="Y210" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45731,13 +46705,18 @@
       <c r="U211" t="inlineStr"/>
       <c r="V211" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W211" t="inlineStr"/>
       <c r="X211" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.738401+00:00</t>
+          <t>2026-10-17T11:47:11.438492+00:00</t>
+        </is>
+      </c>
+      <c r="Y211" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45827,13 +46806,18 @@
       <c r="U212" t="inlineStr"/>
       <c r="V212" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W212" t="inlineStr"/>
       <c r="X212" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.738564+00:00</t>
+          <t>2026-10-17T11:47:11.438648+00:00</t>
+        </is>
+      </c>
+      <c r="Y212" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -45923,13 +46907,18 @@
       <c r="U213" t="inlineStr"/>
       <c r="V213" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>retained_not_content_indexed</t>
         </is>
       </c>
       <c r="W213" t="inlineStr"/>
       <c r="X213" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.738753+00:00</t>
+          <t>2026-10-17T11:47:11.439108+00:00</t>
+        </is>
+      </c>
+      <c r="Y213" t="inlineStr">
+        <is>
+          <t>{"status": "retained_not_content_indexed", "search_chunks": 0, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["Original retained; no supported content parser for this format. Images/video/models are not claimed searchable."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46019,13 +47008,18 @@
       <c r="U214" t="inlineStr"/>
       <c r="V214" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W214" t="inlineStr"/>
       <c r="X214" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.739548+00:00</t>
+          <t>2026-10-17T11:47:11.439928+00:00</t>
+        </is>
+      </c>
+      <c r="Y214" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 139, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46115,13 +47109,18 @@
       <c r="U215" t="inlineStr"/>
       <c r="V215" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W215" t="inlineStr"/>
       <c r="X215" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.739987+00:00</t>
+          <t>2026-10-17T11:47:11.440466+00:00</t>
+        </is>
+      </c>
+      <c r="Y215" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 9, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46211,13 +47210,18 @@
       <c r="U216" t="inlineStr"/>
       <c r="V216" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W216" t="inlineStr"/>
       <c r="X216" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.741909+00:00</t>
+          <t>2026-10-17T11:47:11.442669+00:00</t>
+        </is>
+      </c>
+      <c r="Y216" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 416, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46307,13 +47311,18 @@
       <c r="U217" t="inlineStr"/>
       <c r="V217" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W217" t="inlineStr"/>
       <c r="X217" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.742836+00:00</t>
+          <t>2026-10-17T11:47:11.443578+00:00</t>
+        </is>
+      </c>
+      <c r="Y217" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 148, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46403,13 +47412,18 @@
       <c r="U218" t="inlineStr"/>
       <c r="V218" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W218" t="inlineStr"/>
       <c r="X218" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.743923+00:00</t>
+          <t>2026-10-17T11:47:11.444649+00:00</t>
+        </is>
+      </c>
+      <c r="Y218" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 168, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46499,13 +47513,18 @@
       <c r="U219" t="inlineStr"/>
       <c r="V219" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W219" t="inlineStr"/>
       <c r="X219" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.744421+00:00</t>
+          <t>2026-10-17T11:47:11.445174+00:00</t>
+        </is>
+      </c>
+      <c r="Y219" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 10, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46595,13 +47614,18 @@
       <c r="U220" t="inlineStr"/>
       <c r="V220" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W220" t="inlineStr"/>
       <c r="X220" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.745678+00:00</t>
+          <t>2026-10-17T11:47:11.446208+00:00</t>
+        </is>
+      </c>
+      <c r="Y220" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 130, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46691,13 +47715,18 @@
       <c r="U221" t="inlineStr"/>
       <c r="V221" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W221" t="inlineStr"/>
       <c r="X221" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.746454+00:00</t>
+          <t>2026-10-17T11:47:11.447024+00:00</t>
+        </is>
+      </c>
+      <c r="Y221" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 89, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46787,13 +47816,18 @@
       <c r="U222" t="inlineStr"/>
       <c r="V222" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W222" t="inlineStr"/>
       <c r="X222" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.746940+00:00</t>
+          <t>2026-10-17T11:47:11.447493+00:00</t>
+        </is>
+      </c>
+      <c r="Y222" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 8, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46883,13 +47917,18 @@
       <c r="U223" t="inlineStr"/>
       <c r="V223" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W223" t="inlineStr"/>
       <c r="X223" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.748009+00:00</t>
+          <t>2026-10-17T11:47:11.448658+00:00</t>
+        </is>
+      </c>
+      <c r="Y223" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 239, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -46979,13 +48018,18 @@
       <c r="U224" t="inlineStr"/>
       <c r="V224" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W224" t="inlineStr"/>
       <c r="X224" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.748715+00:00</t>
+          <t>2026-10-17T11:47:11.449515+00:00</t>
+        </is>
+      </c>
+      <c r="Y224" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 64, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -47075,13 +48119,18 @@
       <c r="U225" t="inlineStr"/>
       <c r="V225" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W225" t="inlineStr"/>
       <c r="X225" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.749965+00:00</t>
+          <t>2026-10-17T11:47:11.450839+00:00</t>
+        </is>
+      </c>
+      <c r="Y225" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 139, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -47171,13 +48220,18 @@
       <c r="U226" t="inlineStr"/>
       <c r="V226" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W226" t="inlineStr"/>
       <c r="X226" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.750417+00:00</t>
+          <t>2026-10-17T11:47:11.451282+00:00</t>
+        </is>
+      </c>
+      <c r="Y226" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 5, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>
@@ -47267,13 +48321,18 @@
       <c r="U227" t="inlineStr"/>
       <c r="V227" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>parsed</t>
         </is>
       </c>
       <c r="W227" t="inlineStr"/>
       <c r="X227" t="inlineStr">
         <is>
-          <t>2026-10-17T11:42:59.751229+00:00</t>
+          <t>2026-10-17T11:47:11.452115+00:00</t>
+        </is>
+      </c>
+      <c r="Y227" t="inlineStr">
+        <is>
+          <t>{"status": "parsed", "search_chunks": 163, "table_count": 0, "ocr_pages": 0, "ocr_pending_pages": [], "limitations": ["PDF logical reading order and inferred vector-grid cells may be imperfect; borderless/scan tables are not guaranteed structured.", "OCR language=eng; OCR values, symbols and units require checking against source page."], "errors": []}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore literature project and persist verified originals and recovery evidence
</commit_message>
<xml_diff>
--- a/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
+++ b/results/ad-oxygen-literature-20261006/inventory/unified_library_inventory.xlsx
@@ -18215,7 +18215,7 @@
       </c>
       <c r="G417" t="inlineStr">
         <is>
-          <t>access_failed</t>
+          <t>partial_or_access_failed</t>
         </is>
       </c>
       <c r="H417" t="b">
@@ -24352,7 +24352,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.041328+00:00</t>
+          <t>2026-10-17T11:51:25.776691+00:00</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -24465,7 +24465,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.042565+00:00</t>
+          <t>2026-10-17T11:51:25.777938+00:00</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -24570,7 +24570,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.042678+00:00</t>
+          <t>2026-10-17T11:51:25.777979+00:00</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr"/>
@@ -24679,7 +24679,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.042935+00:00</t>
+          <t>2026-10-17T11:51:25.778220+00:00</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -24792,7 +24792,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.044024+00:00</t>
+          <t>2026-10-17T11:51:25.779467+00:00</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -24905,7 +24905,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.044489+00:00</t>
+          <t>2026-10-17T11:51:25.779947+00:00</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -25018,7 +25018,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.050466+00:00</t>
+          <t>2026-10-17T11:51:25.788234+00:00</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -25131,7 +25131,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.052891+00:00</t>
+          <t>2026-10-17T11:51:25.790882+00:00</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -25244,7 +25244,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.053821+00:00</t>
+          <t>2026-10-17T11:51:25.791802+00:00</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -25357,7 +25357,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.054275+00:00</t>
+          <t>2026-10-17T11:51:25.792123+00:00</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -25470,7 +25470,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.055006+00:00</t>
+          <t>2026-10-17T11:51:25.792837+00:00</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -25583,7 +25583,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.055653+00:00</t>
+          <t>2026-10-17T11:51:25.793527+00:00</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
@@ -25696,7 +25696,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.056813+00:00</t>
+          <t>2026-10-17T11:51:25.794465+00:00</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -25809,7 +25809,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.057158+00:00</t>
+          <t>2026-10-17T11:51:25.794705+00:00</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
@@ -25922,7 +25922,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.058454+00:00</t>
+          <t>2026-10-17T11:51:25.795571+00:00</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -26035,7 +26035,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.066942+00:00</t>
+          <t>2026-10-17T11:51:25.807178+00:00</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
@@ -26148,7 +26148,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.067770+00:00</t>
+          <t>2026-10-17T11:51:25.808007+00:00</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -26261,7 +26261,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.069168+00:00</t>
+          <t>2026-10-17T11:51:25.809198+00:00</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -26374,7 +26374,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.071918+00:00</t>
+          <t>2026-10-17T11:51:25.811928+00:00</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
@@ -26487,7 +26487,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.072999+00:00</t>
+          <t>2026-10-17T11:51:25.813249+00:00</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -26600,7 +26600,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.074354+00:00</t>
+          <t>2026-10-17T11:51:25.814616+00:00</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
@@ -26713,7 +26713,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.078775+00:00</t>
+          <t>2026-10-17T11:51:25.821932+00:00</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -26826,7 +26826,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.081131+00:00</t>
+          <t>2026-10-17T11:51:25.824178+00:00</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -26939,7 +26939,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.084591+00:00</t>
+          <t>2026-10-17T11:51:25.826123+00:00</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
@@ -27052,7 +27052,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.085306+00:00</t>
+          <t>2026-10-17T11:51:25.826805+00:00</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
@@ -27165,7 +27165,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.085796+00:00</t>
+          <t>2026-10-17T11:51:25.827158+00:00</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
@@ -27278,7 +27278,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.088664+00:00</t>
+          <t>2026-10-17T11:51:25.829146+00:00</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
@@ -27391,7 +27391,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.090034+00:00</t>
+          <t>2026-10-17T11:51:25.830422+00:00</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
@@ -27504,7 +27504,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.092287+00:00</t>
+          <t>2026-10-17T11:51:25.832651+00:00</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
@@ -27617,7 +27617,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.094562+00:00</t>
+          <t>2026-10-17T11:51:25.834760+00:00</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
@@ -27730,7 +27730,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.095102+00:00</t>
+          <t>2026-10-17T11:51:25.835415+00:00</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
@@ -27843,7 +27843,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.095842+00:00</t>
+          <t>2026-10-17T11:51:25.835983+00:00</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
@@ -27956,7 +27956,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.097593+00:00</t>
+          <t>2026-10-17T11:51:25.837712+00:00</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -28069,7 +28069,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.100741+00:00</t>
+          <t>2026-10-17T11:51:25.840680+00:00</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
@@ -28182,7 +28182,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.102968+00:00</t>
+          <t>2026-10-17T11:51:25.842852+00:00</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -28295,7 +28295,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.104156+00:00</t>
+          <t>2026-10-17T11:51:25.844105+00:00</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
@@ -28408,7 +28408,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.107071+00:00</t>
+          <t>2026-10-17T11:51:25.846968+00:00</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -28521,7 +28521,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.107805+00:00</t>
+          <t>2026-10-17T11:51:25.847674+00:00</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
@@ -28634,7 +28634,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.109857+00:00</t>
+          <t>2026-10-17T11:51:25.849237+00:00</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
@@ -28747,7 +28747,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.110161+00:00</t>
+          <t>2026-10-17T11:51:25.849514+00:00</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -28860,7 +28860,7 @@
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.112174+00:00</t>
+          <t>2026-10-17T11:51:25.851519+00:00</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
@@ -28973,7 +28973,7 @@
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.115103+00:00</t>
+          <t>2026-10-17T11:51:25.854481+00:00</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
@@ -29086,7 +29086,7 @@
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.116446+00:00</t>
+          <t>2026-10-17T11:51:25.855870+00:00</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
@@ -29199,7 +29199,7 @@
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.116966+00:00</t>
+          <t>2026-10-17T11:51:25.856427+00:00</t>
         </is>
       </c>
       <c r="Y45" t="inlineStr">
@@ -29312,7 +29312,7 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.120084+00:00</t>
+          <t>2026-10-17T11:51:25.859012+00:00</t>
         </is>
       </c>
       <c r="Y46" t="inlineStr">
@@ -29425,7 +29425,7 @@
       </c>
       <c r="X47" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.121467+00:00</t>
+          <t>2026-10-17T11:51:25.860146+00:00</t>
         </is>
       </c>
       <c r="Y47" t="inlineStr">
@@ -29538,7 +29538,7 @@
       </c>
       <c r="X48" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.125096+00:00</t>
+          <t>2026-10-17T11:51:25.863679+00:00</t>
         </is>
       </c>
       <c r="Y48" t="inlineStr">
@@ -29651,7 +29651,7 @@
       </c>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.126791+00:00</t>
+          <t>2026-10-17T11:51:25.865506+00:00</t>
         </is>
       </c>
       <c r="Y49" t="inlineStr">
@@ -29764,7 +29764,7 @@
       </c>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.128686+00:00</t>
+          <t>2026-10-17T11:51:25.867546+00:00</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="X51" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.129869+00:00</t>
+          <t>2026-10-17T11:51:25.868500+00:00</t>
         </is>
       </c>
       <c r="Y51" t="inlineStr">
@@ -29990,7 +29990,7 @@
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.130344+00:00</t>
+          <t>2026-10-17T11:51:25.868933+00:00</t>
         </is>
       </c>
       <c r="Y52" t="inlineStr">
@@ -30103,7 +30103,7 @@
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.130706+00:00</t>
+          <t>2026-10-17T11:51:25.869308+00:00</t>
         </is>
       </c>
       <c r="Y53" t="inlineStr">
@@ -30216,7 +30216,7 @@
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.132150+00:00</t>
+          <t>2026-10-17T11:51:25.871071+00:00</t>
         </is>
       </c>
       <c r="Y54" t="inlineStr">
@@ -30329,7 +30329,7 @@
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.133591+00:00</t>
+          <t>2026-10-17T11:51:25.872528+00:00</t>
         </is>
       </c>
       <c r="Y55" t="inlineStr">
@@ -30442,7 +30442,7 @@
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.135193+00:00</t>
+          <t>2026-10-17T11:51:25.874209+00:00</t>
         </is>
       </c>
       <c r="Y56" t="inlineStr">
@@ -30555,7 +30555,7 @@
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.135596+00:00</t>
+          <t>2026-10-17T11:51:25.874724+00:00</t>
         </is>
       </c>
       <c r="Y57" t="inlineStr">
@@ -30668,7 +30668,7 @@
       </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.136947+00:00</t>
+          <t>2026-10-17T11:51:25.876334+00:00</t>
         </is>
       </c>
       <c r="Y58" t="inlineStr">
@@ -30781,7 +30781,7 @@
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.138455+00:00</t>
+          <t>2026-10-17T11:51:25.879197+00:00</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr">
@@ -30894,7 +30894,7 @@
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.139224+00:00</t>
+          <t>2026-10-17T11:51:25.880627+00:00</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr">
@@ -31007,7 +31007,7 @@
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.140494+00:00</t>
+          <t>2026-10-17T11:51:25.881625+00:00</t>
         </is>
       </c>
       <c r="Y61" t="inlineStr">
@@ -31120,7 +31120,7 @@
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.140931+00:00</t>
+          <t>2026-10-17T11:51:25.881945+00:00</t>
         </is>
       </c>
       <c r="Y62" t="inlineStr">
@@ -31233,7 +31233,7 @@
       </c>
       <c r="X63" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.146674+00:00</t>
+          <t>2026-10-17T11:51:25.887878+00:00</t>
         </is>
       </c>
       <c r="Y63" t="inlineStr">
@@ -31346,7 +31346,7 @@
       </c>
       <c r="X64" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.147101+00:00</t>
+          <t>2026-10-17T11:51:25.888395+00:00</t>
         </is>
       </c>
       <c r="Y64" t="inlineStr">
@@ -31459,7 +31459,7 @@
       </c>
       <c r="X65" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.147704+00:00</t>
+          <t>2026-10-17T11:51:25.889042+00:00</t>
         </is>
       </c>
       <c r="Y65" t="inlineStr">
@@ -31572,7 +31572,7 @@
       </c>
       <c r="X66" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.148139+00:00</t>
+          <t>2026-10-17T11:51:25.889538+00:00</t>
         </is>
       </c>
       <c r="Y66" t="inlineStr">
@@ -31685,7 +31685,7 @@
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.149188+00:00</t>
+          <t>2026-10-17T11:51:25.890633+00:00</t>
         </is>
       </c>
       <c r="Y67" t="inlineStr">
@@ -31798,7 +31798,7 @@
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.152143+00:00</t>
+          <t>2026-10-17T11:51:25.893739+00:00</t>
         </is>
       </c>
       <c r="Y68" t="inlineStr">
@@ -31911,7 +31911,7 @@
       </c>
       <c r="X69" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.152511+00:00</t>
+          <t>2026-10-17T11:51:25.894021+00:00</t>
         </is>
       </c>
       <c r="Y69" t="inlineStr">
@@ -32024,7 +32024,7 @@
       </c>
       <c r="X70" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.157098+00:00</t>
+          <t>2026-10-17T11:51:25.899681+00:00</t>
         </is>
       </c>
       <c r="Y70" t="inlineStr">
@@ -32137,7 +32137,7 @@
       </c>
       <c r="X71" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.157942+00:00</t>
+          <t>2026-10-17T11:51:25.901422+00:00</t>
         </is>
       </c>
       <c r="Y71" t="inlineStr">
@@ -32250,7 +32250,7 @@
       </c>
       <c r="X72" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.160089+00:00</t>
+          <t>2026-10-17T11:51:25.904607+00:00</t>
         </is>
       </c>
       <c r="Y72" t="inlineStr">
@@ -32363,7 +32363,7 @@
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.162131+00:00</t>
+          <t>2026-10-17T11:51:25.907757+00:00</t>
         </is>
       </c>
       <c r="Y73" t="inlineStr">
@@ -32476,7 +32476,7 @@
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.163009+00:00</t>
+          <t>2026-10-17T11:51:25.909311+00:00</t>
         </is>
       </c>
       <c r="Y74" t="inlineStr">
@@ -32589,7 +32589,7 @@
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.164805+00:00</t>
+          <t>2026-10-17T11:51:25.911055+00:00</t>
         </is>
       </c>
       <c r="Y75" t="inlineStr">
@@ -32702,7 +32702,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.167414+00:00</t>
+          <t>2026-10-17T11:51:25.913455+00:00</t>
         </is>
       </c>
       <c r="Y76" t="inlineStr">
@@ -32815,7 +32815,7 @@
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.176350+00:00</t>
+          <t>2026-10-17T11:51:25.926192+00:00</t>
         </is>
       </c>
       <c r="Y77" t="inlineStr">
@@ -32928,7 +32928,7 @@
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.177741+00:00</t>
+          <t>2026-10-17T11:51:25.927707+00:00</t>
         </is>
       </c>
       <c r="Y78" t="inlineStr">
@@ -33041,7 +33041,7 @@
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.177995+00:00</t>
+          <t>2026-10-17T11:51:25.927877+00:00</t>
         </is>
       </c>
       <c r="Y79" t="inlineStr">
@@ -33146,7 +33146,7 @@
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.178017+00:00</t>
+          <t>2026-10-17T11:51:25.927894+00:00</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr"/>
@@ -33255,7 +33255,7 @@
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.183578+00:00</t>
+          <t>2026-10-17T11:51:25.932920+00:00</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
@@ -33364,7 +33364,7 @@
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.184053+00:00</t>
+          <t>2026-10-17T11:51:25.933357+00:00</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -33473,7 +33473,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.184530+00:00</t>
+          <t>2026-10-17T11:51:25.934772+00:00</t>
         </is>
       </c>
       <c r="Y83" t="inlineStr">
@@ -33582,7 +33582,7 @@
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.185059+00:00</t>
+          <t>2026-10-17T11:51:25.935405+00:00</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
@@ -33691,7 +33691,7 @@
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.185895+00:00</t>
+          <t>2026-10-17T11:51:25.936135+00:00</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr">
@@ -33800,7 +33800,7 @@
       </c>
       <c r="X86" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.187458+00:00</t>
+          <t>2026-10-17T11:51:25.937633+00:00</t>
         </is>
       </c>
       <c r="Y86" t="inlineStr">
@@ -33909,7 +33909,7 @@
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.188921+00:00</t>
+          <t>2026-10-17T11:51:25.938526+00:00</t>
         </is>
       </c>
       <c r="Y87" t="inlineStr">
@@ -34018,7 +34018,7 @@
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.189365+00:00</t>
+          <t>2026-10-17T11:51:25.938953+00:00</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
@@ -34131,7 +34131,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.190190+00:00</t>
+          <t>2026-10-17T11:51:25.940202+00:00</t>
         </is>
       </c>
       <c r="Y89" t="inlineStr">
@@ -34236,7 +34236,7 @@
       </c>
       <c r="X90" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.190214+00:00</t>
+          <t>2026-10-17T11:51:25.940238+00:00</t>
         </is>
       </c>
       <c r="Y90" t="inlineStr"/>
@@ -34345,7 +34345,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.190279+00:00</t>
+          <t>2026-10-17T11:51:25.940340+00:00</t>
         </is>
       </c>
       <c r="Y91" t="inlineStr">
@@ -34458,7 +34458,7 @@
       </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.190538+00:00</t>
+          <t>2026-10-17T11:51:25.940569+00:00</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -34571,7 +34571,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.190662+00:00</t>
+          <t>2026-10-17T11:51:25.940690+00:00</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -34688,7 +34688,7 @@
       </c>
       <c r="X94" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.190782+00:00</t>
+          <t>2026-10-17T11:51:25.940888+00:00</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr">
@@ -34801,7 +34801,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.191257+00:00</t>
+          <t>2026-10-17T11:51:25.941407+00:00</t>
         </is>
       </c>
       <c r="Y95" t="inlineStr">
@@ -34914,7 +34914,7 @@
       </c>
       <c r="X96" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.191492+00:00</t>
+          <t>2026-10-17T11:51:25.941648+00:00</t>
         </is>
       </c>
       <c r="Y96" t="inlineStr">
@@ -35031,7 +35031,7 @@
       </c>
       <c r="X97" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.191553+00:00</t>
+          <t>2026-10-17T11:51:25.941708+00:00</t>
         </is>
       </c>
       <c r="Y97" t="inlineStr">
@@ -35148,7 +35148,7 @@
       </c>
       <c r="X98" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.191613+00:00</t>
+          <t>2026-10-17T11:51:25.941772+00:00</t>
         </is>
       </c>
       <c r="Y98" t="inlineStr">
@@ -35265,7 +35265,7 @@
       </c>
       <c r="X99" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.191752+00:00</t>
+          <t>2026-10-17T11:51:25.942004+00:00</t>
         </is>
       </c>
       <c r="Y99" t="inlineStr">
@@ -35382,7 +35382,7 @@
       </c>
       <c r="X100" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.192027+00:00</t>
+          <t>2026-10-17T11:51:25.942202+00:00</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr">
@@ -35495,7 +35495,7 @@
       </c>
       <c r="X101" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.192524+00:00</t>
+          <t>2026-10-17T11:51:25.942707+00:00</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr">
@@ -35608,7 +35608,7 @@
       </c>
       <c r="X102" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.192580+00:00</t>
+          <t>2026-10-17T11:51:25.942763+00:00</t>
         </is>
       </c>
       <c r="Y102" t="inlineStr">
@@ -35721,7 +35721,7 @@
       </c>
       <c r="X103" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.192649+00:00</t>
+          <t>2026-10-17T11:51:25.942832+00:00</t>
         </is>
       </c>
       <c r="Y103" t="inlineStr">
@@ -35834,7 +35834,7 @@
       </c>
       <c r="X104" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.203833+00:00</t>
+          <t>2026-10-17T11:51:25.961036+00:00</t>
         </is>
       </c>
       <c r="Y104" t="inlineStr">
@@ -35943,7 +35943,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.203924+00:00</t>
+          <t>2026-10-17T11:51:25.961147+00:00</t>
         </is>
       </c>
       <c r="Y105" t="inlineStr"/>
@@ -36052,7 +36052,7 @@
       </c>
       <c r="X106" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.364771+00:00</t>
+          <t>2026-10-17T11:51:26.138459+00:00</t>
         </is>
       </c>
       <c r="Y106" t="inlineStr">
@@ -36165,7 +36165,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.365050+00:00</t>
+          <t>2026-10-17T11:51:26.138731+00:00</t>
         </is>
       </c>
       <c r="Y107" t="inlineStr">
@@ -36278,7 +36278,7 @@
       </c>
       <c r="X108" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.366447+00:00</t>
+          <t>2026-10-17T11:51:26.141424+00:00</t>
         </is>
       </c>
       <c r="Y108" t="inlineStr">
@@ -36385,7 +36385,7 @@
       </c>
       <c r="X109" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.366570+00:00</t>
+          <t>2026-10-17T11:51:26.141601+00:00</t>
         </is>
       </c>
       <c r="Y109" t="inlineStr">
@@ -36484,7 +36484,7 @@
       </c>
       <c r="X110" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.366585+00:00</t>
+          <t>2026-10-17T11:51:26.141619+00:00</t>
         </is>
       </c>
       <c r="Y110" t="inlineStr"/>
@@ -36587,7 +36587,7 @@
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.366839+00:00</t>
+          <t>2026-10-17T11:51:26.141827+00:00</t>
         </is>
       </c>
       <c r="Y111" t="inlineStr">
@@ -36694,7 +36694,7 @@
       </c>
       <c r="X112" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.366940+00:00</t>
+          <t>2026-10-17T11:51:26.141914+00:00</t>
         </is>
       </c>
       <c r="Y112" t="inlineStr">
@@ -36801,7 +36801,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.367239+00:00</t>
+          <t>2026-10-17T11:51:26.142021+00:00</t>
         </is>
       </c>
       <c r="Y113" t="inlineStr">
@@ -36900,7 +36900,7 @@
       </c>
       <c r="X114" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.367267+00:00</t>
+          <t>2026-10-17T11:51:26.142033+00:00</t>
         </is>
       </c>
       <c r="Y114" t="inlineStr"/>
@@ -37003,7 +37003,7 @@
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.367697+00:00</t>
+          <t>2026-10-17T11:51:26.142431+00:00</t>
         </is>
       </c>
       <c r="Y115" t="inlineStr">
@@ -37102,7 +37102,7 @@
       </c>
       <c r="X116" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.367711+00:00</t>
+          <t>2026-10-17T11:51:26.142445+00:00</t>
         </is>
       </c>
       <c r="Y116" t="inlineStr"/>
@@ -37205,7 +37205,7 @@
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.367929+00:00</t>
+          <t>2026-10-17T11:51:26.142667+00:00</t>
         </is>
       </c>
       <c r="Y117" t="inlineStr">
@@ -37304,7 +37304,7 @@
       </c>
       <c r="X118" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.367939+00:00</t>
+          <t>2026-10-17T11:51:26.142678+00:00</t>
         </is>
       </c>
       <c r="Y118" t="inlineStr"/>
@@ -37407,7 +37407,7 @@
       </c>
       <c r="X119" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.368461+00:00</t>
+          <t>2026-10-17T11:51:26.143684+00:00</t>
         </is>
       </c>
       <c r="Y119" t="inlineStr">
@@ -37506,7 +37506,7 @@
       </c>
       <c r="X120" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.368473+00:00</t>
+          <t>2026-10-17T11:51:26.143712+00:00</t>
         </is>
       </c>
       <c r="Y120" t="inlineStr"/>
@@ -37609,7 +37609,7 @@
       </c>
       <c r="X121" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.368815+00:00</t>
+          <t>2026-10-17T11:51:26.144074+00:00</t>
         </is>
       </c>
       <c r="Y121" t="inlineStr">
@@ -37716,7 +37716,7 @@
       </c>
       <c r="X122" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.368970+00:00</t>
+          <t>2026-10-17T11:51:26.144231+00:00</t>
         </is>
       </c>
       <c r="Y122" t="inlineStr">
@@ -37815,7 +37815,7 @@
       </c>
       <c r="X123" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.368983+00:00</t>
+          <t>2026-10-17T11:51:26.144245+00:00</t>
         </is>
       </c>
       <c r="Y123" t="inlineStr"/>
@@ -37918,7 +37918,7 @@
       </c>
       <c r="X124" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.369656+00:00</t>
+          <t>2026-10-17T11:51:26.144966+00:00</t>
         </is>
       </c>
       <c r="Y124" t="inlineStr">
@@ -38017,7 +38017,7 @@
       </c>
       <c r="X125" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.369670+00:00</t>
+          <t>2026-10-17T11:51:26.144979+00:00</t>
         </is>
       </c>
       <c r="Y125" t="inlineStr"/>
@@ -38120,7 +38120,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.380641+00:00</t>
+          <t>2026-10-17T11:51:26.158882+00:00</t>
         </is>
       </c>
       <c r="Y126" t="inlineStr">
@@ -38227,7 +38227,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.380884+00:00</t>
+          <t>2026-10-17T11:51:26.159146+00:00</t>
         </is>
       </c>
       <c r="Y127" t="inlineStr">
@@ -38326,7 +38326,7 @@
       </c>
       <c r="X128" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.380898+00:00</t>
+          <t>2026-10-17T11:51:26.159162+00:00</t>
         </is>
       </c>
       <c r="Y128" t="inlineStr"/>
@@ -38429,7 +38429,7 @@
       </c>
       <c r="X129" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.381224+00:00</t>
+          <t>2026-10-17T11:51:26.159487+00:00</t>
         </is>
       </c>
       <c r="Y129" t="inlineStr">
@@ -38536,7 +38536,7 @@
       </c>
       <c r="X130" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.381542+00:00</t>
+          <t>2026-10-17T11:51:26.159691+00:00</t>
         </is>
       </c>
       <c r="Y130" t="inlineStr">
@@ -38643,7 +38643,7 @@
       </c>
       <c r="X131" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.381946+00:00</t>
+          <t>2026-10-17T11:51:26.159985+00:00</t>
         </is>
       </c>
       <c r="Y131" t="inlineStr">
@@ -38742,7 +38742,7 @@
       </c>
       <c r="X132" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.381972+00:00</t>
+          <t>2026-10-17T11:51:26.160009+00:00</t>
         </is>
       </c>
       <c r="Y132" t="inlineStr"/>
@@ -38845,7 +38845,7 @@
       </c>
       <c r="X133" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.382366+00:00</t>
+          <t>2026-10-17T11:51:26.160389+00:00</t>
         </is>
       </c>
       <c r="Y133" t="inlineStr">
@@ -38944,7 +38944,7 @@
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.382419+00:00</t>
+          <t>2026-10-17T11:51:26.160405+00:00</t>
         </is>
       </c>
       <c r="Y134" t="inlineStr"/>
@@ -39047,7 +39047,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.383693+00:00</t>
+          <t>2026-10-17T11:51:26.161643+00:00</t>
         </is>
       </c>
       <c r="Y135" t="inlineStr">
@@ -39160,7 +39160,7 @@
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.384880+00:00</t>
+          <t>2026-10-17T11:51:26.163026+00:00</t>
         </is>
       </c>
       <c r="Y136" t="inlineStr">
@@ -39257,7 +39257,7 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.397066+00:00</t>
+          <t>2026-10-17T11:51:26.174235+00:00</t>
         </is>
       </c>
       <c r="Y137" t="inlineStr">
@@ -39362,7 +39362,7 @@
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.397878+00:00</t>
+          <t>2026-10-17T11:51:26.174973+00:00</t>
         </is>
       </c>
       <c r="Y138" t="inlineStr">
@@ -39455,7 +39455,7 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.397956+00:00</t>
+          <t>2026-10-17T11:51:26.174999+00:00</t>
         </is>
       </c>
       <c r="Y139" t="inlineStr"/>
@@ -39556,7 +39556,7 @@
       <c r="W140" t="inlineStr"/>
       <c r="X140" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.399139+00:00</t>
+          <t>2026-10-17T11:51:26.176208+00:00</t>
         </is>
       </c>
       <c r="Y140" t="inlineStr">
@@ -39661,7 +39661,7 @@
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.402653+00:00</t>
+          <t>2026-10-17T11:51:26.180061+00:00</t>
         </is>
       </c>
       <c r="Y141" t="inlineStr">
@@ -39766,7 +39766,7 @@
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.403549+00:00</t>
+          <t>2026-10-17T11:51:26.181104+00:00</t>
         </is>
       </c>
       <c r="Y142" t="inlineStr">
@@ -39863,7 +39863,7 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.403568+00:00</t>
+          <t>2026-10-17T11:51:26.181131+00:00</t>
         </is>
       </c>
       <c r="Y143" t="inlineStr"/>
@@ -39964,7 +39964,7 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.404216+00:00</t>
+          <t>2026-10-17T11:51:26.182058+00:00</t>
         </is>
       </c>
       <c r="Y144" t="inlineStr">
@@ -40061,7 +40061,7 @@
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.404231+00:00</t>
+          <t>2026-10-17T11:51:26.182087+00:00</t>
         </is>
       </c>
       <c r="Y145" t="inlineStr"/>
@@ -40166,7 +40166,7 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.405058+00:00</t>
+          <t>2026-10-17T11:51:26.182947+00:00</t>
         </is>
       </c>
       <c r="Y146" t="inlineStr">
@@ -40259,7 +40259,7 @@
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.405074+00:00</t>
+          <t>2026-10-17T11:51:26.182967+00:00</t>
         </is>
       </c>
       <c r="Y147" t="inlineStr"/>
@@ -40352,7 +40352,7 @@
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.405078+00:00</t>
+          <t>2026-10-17T11:51:26.182970+00:00</t>
         </is>
       </c>
       <c r="Y148" t="inlineStr"/>
@@ -40449,7 +40449,7 @@
       <c r="W149" t="inlineStr"/>
       <c r="X149" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.406035+00:00</t>
+          <t>2026-10-17T11:51:26.183766+00:00</t>
         </is>
       </c>
       <c r="Y149" t="inlineStr">
@@ -40550,7 +40550,7 @@
       <c r="W150" t="inlineStr"/>
       <c r="X150" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.407171+00:00</t>
+          <t>2026-10-17T11:51:26.184986+00:00</t>
         </is>
       </c>
       <c r="Y150" t="inlineStr">
@@ -40651,7 +40651,7 @@
       <c r="W151" t="inlineStr"/>
       <c r="X151" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.407628+00:00</t>
+          <t>2026-10-17T11:51:26.185554+00:00</t>
         </is>
       </c>
       <c r="Y151" t="inlineStr">
@@ -40752,7 +40752,7 @@
       <c r="W152" t="inlineStr"/>
       <c r="X152" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.419092+00:00</t>
+          <t>2026-10-17T11:51:26.196374+00:00</t>
         </is>
       </c>
       <c r="Y152" t="inlineStr">
@@ -40853,7 +40853,7 @@
       <c r="W153" t="inlineStr"/>
       <c r="X153" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.419269+00:00</t>
+          <t>2026-10-17T11:51:26.196608+00:00</t>
         </is>
       </c>
       <c r="Y153" t="inlineStr">
@@ -40954,7 +40954,7 @@
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.419471+00:00</t>
+          <t>2026-10-17T11:51:26.196779+00:00</t>
         </is>
       </c>
       <c r="Y154" t="inlineStr">
@@ -41055,7 +41055,7 @@
       <c r="W155" t="inlineStr"/>
       <c r="X155" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.419911+00:00</t>
+          <t>2026-10-17T11:51:26.197221+00:00</t>
         </is>
       </c>
       <c r="Y155" t="inlineStr">
@@ -41156,7 +41156,7 @@
       <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.420171+00:00</t>
+          <t>2026-10-17T11:51:26.197758+00:00</t>
         </is>
       </c>
       <c r="Y156" t="inlineStr">
@@ -41257,7 +41257,7 @@
       <c r="W157" t="inlineStr"/>
       <c r="X157" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.420558+00:00</t>
+          <t>2026-10-17T11:51:26.198109+00:00</t>
         </is>
       </c>
       <c r="Y157" t="inlineStr">
@@ -41358,7 +41358,7 @@
       <c r="W158" t="inlineStr"/>
       <c r="X158" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.421821+00:00</t>
+          <t>2026-10-17T11:51:26.199446+00:00</t>
         </is>
       </c>
       <c r="Y158" t="inlineStr">
@@ -41459,7 +41459,7 @@
       <c r="W159" t="inlineStr"/>
       <c r="X159" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.423593+00:00</t>
+          <t>2026-10-17T11:51:26.201537+00:00</t>
         </is>
       </c>
       <c r="Y159" t="inlineStr">
@@ -41560,7 +41560,7 @@
       <c r="W160" t="inlineStr"/>
       <c r="X160" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.424240+00:00</t>
+          <t>2026-10-17T11:51:26.202228+00:00</t>
         </is>
       </c>
       <c r="Y160" t="inlineStr">
@@ -41661,7 +41661,7 @@
       <c r="W161" t="inlineStr"/>
       <c r="X161" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.424622+00:00</t>
+          <t>2026-10-17T11:51:26.202558+00:00</t>
         </is>
       </c>
       <c r="Y161" t="inlineStr">
@@ -41762,7 +41762,7 @@
       <c r="W162" t="inlineStr"/>
       <c r="X162" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.424719+00:00</t>
+          <t>2026-10-17T11:51:26.202621+00:00</t>
         </is>
       </c>
       <c r="Y162" t="inlineStr">
@@ -41863,7 +41863,7 @@
       <c r="W163" t="inlineStr"/>
       <c r="X163" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.424808+00:00</t>
+          <t>2026-10-17T11:51:26.202688+00:00</t>
         </is>
       </c>
       <c r="Y163" t="inlineStr">
@@ -41964,7 +41964,7 @@
       <c r="W164" t="inlineStr"/>
       <c r="X164" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.425771+00:00</t>
+          <t>2026-10-17T11:51:26.203055+00:00</t>
         </is>
       </c>
       <c r="Y164" t="inlineStr">
@@ -42065,7 +42065,7 @@
       <c r="W165" t="inlineStr"/>
       <c r="X165" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.426245+00:00</t>
+          <t>2026-10-17T11:51:26.203524+00:00</t>
         </is>
       </c>
       <c r="Y165" t="inlineStr">
@@ -42166,7 +42166,7 @@
       <c r="W166" t="inlineStr"/>
       <c r="X166" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.426624+00:00</t>
+          <t>2026-10-17T11:51:26.203966+00:00</t>
         </is>
       </c>
       <c r="Y166" t="inlineStr">
@@ -42267,7 +42267,7 @@
       <c r="W167" t="inlineStr"/>
       <c r="X167" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.427315+00:00</t>
+          <t>2026-10-17T11:51:26.205949+00:00</t>
         </is>
       </c>
       <c r="Y167" t="inlineStr">
@@ -42368,7 +42368,7 @@
       <c r="W168" t="inlineStr"/>
       <c r="X168" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.427688+00:00</t>
+          <t>2026-10-17T11:51:26.206530+00:00</t>
         </is>
       </c>
       <c r="Y168" t="inlineStr">
@@ -42469,7 +42469,7 @@
       <c r="W169" t="inlineStr"/>
       <c r="X169" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.427838+00:00</t>
+          <t>2026-10-17T11:51:26.206797+00:00</t>
         </is>
       </c>
       <c r="Y169" t="inlineStr">
@@ -42570,7 +42570,7 @@
       <c r="W170" t="inlineStr"/>
       <c r="X170" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.427984+00:00</t>
+          <t>2026-10-17T11:51:26.207012+00:00</t>
         </is>
       </c>
       <c r="Y170" t="inlineStr">
@@ -42671,7 +42671,7 @@
       <c r="W171" t="inlineStr"/>
       <c r="X171" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.428334+00:00</t>
+          <t>2026-10-17T11:51:26.207158+00:00</t>
         </is>
       </c>
       <c r="Y171" t="inlineStr">
@@ -42772,7 +42772,7 @@
       <c r="W172" t="inlineStr"/>
       <c r="X172" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.428478+00:00</t>
+          <t>2026-10-17T11:51:26.207221+00:00</t>
         </is>
       </c>
       <c r="Y172" t="inlineStr">
@@ -42873,7 +42873,7 @@
       <c r="W173" t="inlineStr"/>
       <c r="X173" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.428560+00:00</t>
+          <t>2026-10-17T11:51:26.207314+00:00</t>
         </is>
       </c>
       <c r="Y173" t="inlineStr">
@@ -42974,7 +42974,7 @@
       <c r="W174" t="inlineStr"/>
       <c r="X174" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.428992+00:00</t>
+          <t>2026-10-17T11:51:26.207735+00:00</t>
         </is>
       </c>
       <c r="Y174" t="inlineStr">
@@ -43075,7 +43075,7 @@
       <c r="W175" t="inlineStr"/>
       <c r="X175" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.429418+00:00</t>
+          <t>2026-10-17T11:51:26.208478+00:00</t>
         </is>
       </c>
       <c r="Y175" t="inlineStr">
@@ -43176,7 +43176,7 @@
       <c r="W176" t="inlineStr"/>
       <c r="X176" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.429727+00:00</t>
+          <t>2026-10-17T11:51:26.209237+00:00</t>
         </is>
       </c>
       <c r="Y176" t="inlineStr">
@@ -43277,7 +43277,7 @@
       <c r="W177" t="inlineStr"/>
       <c r="X177" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.430240+00:00</t>
+          <t>2026-10-17T11:51:26.210007+00:00</t>
         </is>
       </c>
       <c r="Y177" t="inlineStr">
@@ -43378,7 +43378,7 @@
       <c r="W178" t="inlineStr"/>
       <c r="X178" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.430416+00:00</t>
+          <t>2026-10-17T11:51:26.210169+00:00</t>
         </is>
       </c>
       <c r="Y178" t="inlineStr">
@@ -43479,7 +43479,7 @@
       <c r="W179" t="inlineStr"/>
       <c r="X179" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.431090+00:00</t>
+          <t>2026-10-17T11:51:26.211027+00:00</t>
         </is>
       </c>
       <c r="Y179" t="inlineStr">
@@ -43580,7 +43580,7 @@
       <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.431758+00:00</t>
+          <t>2026-10-17T11:51:26.211682+00:00</t>
         </is>
       </c>
       <c r="Y180" t="inlineStr">
@@ -43681,7 +43681,7 @@
       <c r="W181" t="inlineStr"/>
       <c r="X181" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.431876+00:00</t>
+          <t>2026-10-17T11:51:26.211794+00:00</t>
         </is>
       </c>
       <c r="Y181" t="inlineStr">
@@ -43782,7 +43782,7 @@
       <c r="W182" t="inlineStr"/>
       <c r="X182" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.432404+00:00</t>
+          <t>2026-10-17T11:51:26.212377+00:00</t>
         </is>
       </c>
       <c r="Y182" t="inlineStr">
@@ -43883,7 +43883,7 @@
       <c r="W183" t="inlineStr"/>
       <c r="X183" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.432543+00:00</t>
+          <t>2026-10-17T11:51:26.212633+00:00</t>
         </is>
       </c>
       <c r="Y183" t="inlineStr">
@@ -43984,7 +43984,7 @@
       <c r="W184" t="inlineStr"/>
       <c r="X184" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.432614+00:00</t>
+          <t>2026-10-17T11:51:26.213354+00:00</t>
         </is>
       </c>
       <c r="Y184" t="inlineStr">
@@ -44085,7 +44085,7 @@
       <c r="W185" t="inlineStr"/>
       <c r="X185" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.432890+00:00</t>
+          <t>2026-10-17T11:51:26.213677+00:00</t>
         </is>
       </c>
       <c r="Y185" t="inlineStr">
@@ -44186,7 +44186,7 @@
       <c r="W186" t="inlineStr"/>
       <c r="X186" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.432938+00:00</t>
+          <t>2026-10-17T11:51:26.213740+00:00</t>
         </is>
       </c>
       <c r="Y186" t="inlineStr">
@@ -44287,7 +44287,7 @@
       <c r="W187" t="inlineStr"/>
       <c r="X187" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.433091+00:00</t>
+          <t>2026-10-17T11:51:26.214024+00:00</t>
         </is>
       </c>
       <c r="Y187" t="inlineStr">
@@ -44388,7 +44388,7 @@
       <c r="W188" t="inlineStr"/>
       <c r="X188" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.433146+00:00</t>
+          <t>2026-10-17T11:51:26.214080+00:00</t>
         </is>
       </c>
       <c r="Y188" t="inlineStr">
@@ -44489,7 +44489,7 @@
       <c r="W189" t="inlineStr"/>
       <c r="X189" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.433514+00:00</t>
+          <t>2026-10-17T11:51:26.214437+00:00</t>
         </is>
       </c>
       <c r="Y189" t="inlineStr">
@@ -44590,7 +44590,7 @@
       <c r="W190" t="inlineStr"/>
       <c r="X190" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.433584+00:00</t>
+          <t>2026-10-17T11:51:26.214511+00:00</t>
         </is>
       </c>
       <c r="Y190" t="inlineStr">
@@ -44691,7 +44691,7 @@
       <c r="W191" t="inlineStr"/>
       <c r="X191" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.434163+00:00</t>
+          <t>2026-10-17T11:51:26.215418+00:00</t>
         </is>
       </c>
       <c r="Y191" t="inlineStr">
@@ -44792,7 +44792,7 @@
       <c r="W192" t="inlineStr"/>
       <c r="X192" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.434247+00:00</t>
+          <t>2026-10-17T11:51:26.215650+00:00</t>
         </is>
       </c>
       <c r="Y192" t="inlineStr">
@@ -44893,7 +44893,7 @@
       <c r="W193" t="inlineStr"/>
       <c r="X193" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.434600+00:00</t>
+          <t>2026-10-17T11:51:26.216235+00:00</t>
         </is>
       </c>
       <c r="Y193" t="inlineStr">
@@ -44994,7 +44994,7 @@
       <c r="W194" t="inlineStr"/>
       <c r="X194" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.434739+00:00</t>
+          <t>2026-10-17T11:51:26.216429+00:00</t>
         </is>
       </c>
       <c r="Y194" t="inlineStr">
@@ -45095,7 +45095,7 @@
       <c r="W195" t="inlineStr"/>
       <c r="X195" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.434992+00:00</t>
+          <t>2026-10-17T11:51:26.216779+00:00</t>
         </is>
       </c>
       <c r="Y195" t="inlineStr">
@@ -45196,7 +45196,7 @@
       <c r="W196" t="inlineStr"/>
       <c r="X196" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.435107+00:00</t>
+          <t>2026-10-17T11:51:26.216856+00:00</t>
         </is>
       </c>
       <c r="Y196" t="inlineStr">
@@ -45297,7 +45297,7 @@
       <c r="W197" t="inlineStr"/>
       <c r="X197" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.435251+00:00</t>
+          <t>2026-10-17T11:51:26.216984+00:00</t>
         </is>
       </c>
       <c r="Y197" t="inlineStr">
@@ -45398,7 +45398,7 @@
       <c r="W198" t="inlineStr"/>
       <c r="X198" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.435629+00:00</t>
+          <t>2026-10-17T11:51:26.217535+00:00</t>
         </is>
       </c>
       <c r="Y198" t="inlineStr">
@@ -45499,7 +45499,7 @@
       <c r="W199" t="inlineStr"/>
       <c r="X199" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.435974+00:00</t>
+          <t>2026-10-17T11:51:26.217900+00:00</t>
         </is>
       </c>
       <c r="Y199" t="inlineStr">
@@ -45600,7 +45600,7 @@
       <c r="W200" t="inlineStr"/>
       <c r="X200" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.436056+00:00</t>
+          <t>2026-10-17T11:51:26.217974+00:00</t>
         </is>
       </c>
       <c r="Y200" t="inlineStr">
@@ -45701,7 +45701,7 @@
       <c r="W201" t="inlineStr"/>
       <c r="X201" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.436532+00:00</t>
+          <t>2026-10-17T11:51:26.218551+00:00</t>
         </is>
       </c>
       <c r="Y201" t="inlineStr">
@@ -45802,7 +45802,7 @@
       <c r="W202" t="inlineStr"/>
       <c r="X202" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.436836+00:00</t>
+          <t>2026-10-17T11:51:26.218977+00:00</t>
         </is>
       </c>
       <c r="Y202" t="inlineStr">
@@ -45903,7 +45903,7 @@
       <c r="W203" t="inlineStr"/>
       <c r="X203" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.436885+00:00</t>
+          <t>2026-10-17T11:51:26.219035+00:00</t>
         </is>
       </c>
       <c r="Y203" t="inlineStr">
@@ -46004,7 +46004,7 @@
       <c r="W204" t="inlineStr"/>
       <c r="X204" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.437181+00:00</t>
+          <t>2026-10-17T11:51:26.219360+00:00</t>
         </is>
       </c>
       <c r="Y204" t="inlineStr">
@@ -46105,7 +46105,7 @@
       <c r="W205" t="inlineStr"/>
       <c r="X205" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.437246+00:00</t>
+          <t>2026-10-17T11:51:26.219431+00:00</t>
         </is>
       </c>
       <c r="Y205" t="inlineStr">
@@ -46206,7 +46206,7 @@
       <c r="W206" t="inlineStr"/>
       <c r="X206" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.437445+00:00</t>
+          <t>2026-10-17T11:51:26.219508+00:00</t>
         </is>
       </c>
       <c r="Y206" t="inlineStr">
@@ -46307,7 +46307,7 @@
       <c r="W207" t="inlineStr"/>
       <c r="X207" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.437572+00:00</t>
+          <t>2026-10-17T11:51:26.219724+00:00</t>
         </is>
       </c>
       <c r="Y207" t="inlineStr">
@@ -46408,7 +46408,7 @@
       <c r="W208" t="inlineStr"/>
       <c r="X208" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.437631+00:00</t>
+          <t>2026-10-17T11:51:26.219783+00:00</t>
         </is>
       </c>
       <c r="Y208" t="inlineStr">
@@ -46509,7 +46509,7 @@
       <c r="W209" t="inlineStr"/>
       <c r="X209" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.437685+00:00</t>
+          <t>2026-10-17T11:51:26.219835+00:00</t>
         </is>
       </c>
       <c r="Y209" t="inlineStr">
@@ -46610,7 +46610,7 @@
       <c r="W210" t="inlineStr"/>
       <c r="X210" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.438319+00:00</t>
+          <t>2026-10-17T11:51:26.220485+00:00</t>
         </is>
       </c>
       <c r="Y210" t="inlineStr">
@@ -46711,7 +46711,7 @@
       <c r="W211" t="inlineStr"/>
       <c r="X211" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.438492+00:00</t>
+          <t>2026-10-17T11:51:26.220646+00:00</t>
         </is>
       </c>
       <c r="Y211" t="inlineStr">
@@ -46812,7 +46812,7 @@
       <c r="W212" t="inlineStr"/>
       <c r="X212" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.438648+00:00</t>
+          <t>2026-10-17T11:51:26.220803+00:00</t>
         </is>
       </c>
       <c r="Y212" t="inlineStr">
@@ -46913,7 +46913,7 @@
       <c r="W213" t="inlineStr"/>
       <c r="X213" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.439108+00:00</t>
+          <t>2026-10-17T11:51:26.220954+00:00</t>
         </is>
       </c>
       <c r="Y213" t="inlineStr">
@@ -47014,7 +47014,7 @@
       <c r="W214" t="inlineStr"/>
       <c r="X214" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.439928+00:00</t>
+          <t>2026-10-17T11:51:26.221800+00:00</t>
         </is>
       </c>
       <c r="Y214" t="inlineStr">
@@ -47115,7 +47115,7 @@
       <c r="W215" t="inlineStr"/>
       <c r="X215" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.440466+00:00</t>
+          <t>2026-10-17T11:51:26.222597+00:00</t>
         </is>
       </c>
       <c r="Y215" t="inlineStr">
@@ -47216,7 +47216,7 @@
       <c r="W216" t="inlineStr"/>
       <c r="X216" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.442669+00:00</t>
+          <t>2026-10-17T11:51:26.226513+00:00</t>
         </is>
       </c>
       <c r="Y216" t="inlineStr">
@@ -47317,7 +47317,7 @@
       <c r="W217" t="inlineStr"/>
       <c r="X217" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.443578+00:00</t>
+          <t>2026-10-17T11:51:26.227664+00:00</t>
         </is>
       </c>
       <c r="Y217" t="inlineStr">
@@ -47418,7 +47418,7 @@
       <c r="W218" t="inlineStr"/>
       <c r="X218" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.444649+00:00</t>
+          <t>2026-10-17T11:51:26.229119+00:00</t>
         </is>
       </c>
       <c r="Y218" t="inlineStr">
@@ -47519,7 +47519,7 @@
       <c r="W219" t="inlineStr"/>
       <c r="X219" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.445174+00:00</t>
+          <t>2026-10-17T11:51:26.229673+00:00</t>
         </is>
       </c>
       <c r="Y219" t="inlineStr">
@@ -47620,7 +47620,7 @@
       <c r="W220" t="inlineStr"/>
       <c r="X220" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.446208+00:00</t>
+          <t>2026-10-17T11:51:26.230992+00:00</t>
         </is>
       </c>
       <c r="Y220" t="inlineStr">
@@ -47721,7 +47721,7 @@
       <c r="W221" t="inlineStr"/>
       <c r="X221" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.447024+00:00</t>
+          <t>2026-10-17T11:51:26.231784+00:00</t>
         </is>
       </c>
       <c r="Y221" t="inlineStr">
@@ -47822,7 +47822,7 @@
       <c r="W222" t="inlineStr"/>
       <c r="X222" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.447493+00:00</t>
+          <t>2026-10-17T11:51:26.232580+00:00</t>
         </is>
       </c>
       <c r="Y222" t="inlineStr">
@@ -47923,7 +47923,7 @@
       <c r="W223" t="inlineStr"/>
       <c r="X223" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.448658+00:00</t>
+          <t>2026-10-17T11:51:26.233866+00:00</t>
         </is>
       </c>
       <c r="Y223" t="inlineStr">
@@ -48024,7 +48024,7 @@
       <c r="W224" t="inlineStr"/>
       <c r="X224" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.449515+00:00</t>
+          <t>2026-10-17T11:51:26.234698+00:00</t>
         </is>
       </c>
       <c r="Y224" t="inlineStr">
@@ -48125,7 +48125,7 @@
       <c r="W225" t="inlineStr"/>
       <c r="X225" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.450839+00:00</t>
+          <t>2026-10-17T11:51:26.236084+00:00</t>
         </is>
       </c>
       <c r="Y225" t="inlineStr">
@@ -48226,7 +48226,7 @@
       <c r="W226" t="inlineStr"/>
       <c r="X226" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.451282+00:00</t>
+          <t>2026-10-17T11:51:26.239282+00:00</t>
         </is>
       </c>
       <c r="Y226" t="inlineStr">
@@ -48327,7 +48327,7 @@
       <c r="W227" t="inlineStr"/>
       <c r="X227" t="inlineStr">
         <is>
-          <t>2026-10-17T11:47:11.452115+00:00</t>
+          <t>2026-10-17T11:51:26.240355+00:00</t>
         </is>
       </c>
       <c r="Y227" t="inlineStr">

</xml_diff>